<commit_message>
Chi fa cosa: applicazione rapida a tutta la settimana (+ opzionale su piu' figli)
Feedback di Fabrizio: 'bisogna aggiungere qualcosa che permetta di
applicare rapidamente l'assegnazione su tutta la settimana ed
eventualmente applicarla anche ai due figli - non e' detto che siano da
gestire diversamente o insieme'.

- Nuova server action setWeekBulkResponsibilityAction: un solo upsert
  multiplo (array di righe bambino x giorno x momento) invece di 10-20
  chiamate sequenziali.
- PlannerCalendarView.tsx: pannello 'Applica a tutta la settimana' nel
  riepilogo settimana, con chip per includere/escludere ciascun bambino
  (default: tutti inclusi, il caso piu' comune) e gli stessi pulsanti
  Io/Partner/Nonno/Nonna/Tata/Altro gia' usati per la singola cella.
- Test Playwright TC-N70/TC-N71 + xlsx aggiornato (righe 265-266).

tsc --noEmit ed eslint puliti.
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -904,7 +904,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L264"/>
+  <dimension ref="A1:L266"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11.83" customWidth="1" style="30" min="1" max="1"/>
@@ -14316,184 +14316,276 @@
       </c>
     </row>
     <row r="261">
-      <c r="A261" t="inlineStr">
+      <c r="A261" s="21" t="inlineStr">
         <is>
           <t>TC-N66</t>
         </is>
       </c>
-      <c r="B261" t="inlineStr">
+      <c r="B261" s="21" t="inlineStr">
         <is>
           <t>NEXTGEN - Family Planner (5.4)</t>
         </is>
       </c>
-      <c r="C261" t="inlineStr">
+      <c r="C261" s="21" t="inlineStr">
         <is>
           <t>Vista Mappa: con attivita' prenotate mostra 'Le tue attivita' con distanza stimata</t>
         </is>
       </c>
-      <c r="D261" t="inlineStr">
+      <c r="D261" s="21" t="inlineStr">
         <is>
           <t>Account genitore di test con almeno una prenotazione attiva</t>
         </is>
       </c>
-      <c r="E261" t="inlineStr">
+      <c r="E261" s="21" t="inlineStr">
         <is>
           <t>Nel Planner, tocca 'Mappa'</t>
         </is>
       </c>
-      <c r="F261" t="inlineStr">
+      <c r="F261" s="21" t="inlineStr">
         <is>
           <t>Compare la mappa (pin reali dai centri, quando hanno coordinate) e sotto l'elenco 'Le tue attivita'' con etichetta 'distanza stimata' per ciascuna riga</t>
         </is>
       </c>
-      <c r="G261" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H261">
+      <c r="G261" s="21" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H261" s="21">
         <f>IF(G261="BUG","BUG-"&amp;A261,IF(G261="FUNCTIONAL","FUNCTIONAL-"&amp;A261,""))</f>
         <v/>
       </c>
-      <c r="I261" t="inlineStr">
+      <c r="I261" s="21" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
     </row>
     <row r="262">
-      <c r="A262" t="inlineStr">
+      <c r="A262" s="21" t="inlineStr">
         <is>
           <t>TC-N67</t>
         </is>
       </c>
-      <c r="B262" t="inlineStr">
+      <c r="B262" s="21" t="inlineStr">
         <is>
           <t>NEXTGEN - Family Planner (5.4)</t>
         </is>
       </c>
-      <c r="C262" t="inlineStr">
+      <c r="C262" s="21" t="inlineStr">
         <is>
           <t>Vista Mappa: senza prenotazioni attive mostra lo stato vuoto</t>
         </is>
       </c>
-      <c r="D262" t="inlineStr">
+      <c r="D262" s="21" t="inlineStr">
         <is>
           <t>Account genitore di test senza prenotazioni attive</t>
         </is>
       </c>
-      <c r="E262" t="inlineStr">
+      <c r="E262" s="21" t="inlineStr">
         <is>
           <t>Nel Planner, tocca 'Mappa'</t>
         </is>
       </c>
-      <c r="F262" t="inlineStr">
+      <c r="F262" s="21" t="inlineStr">
         <is>
           <t>Compare il messaggio 'Prenota un'attivita' per vederla qui sulla mappa...' invece di una mappa vuota</t>
         </is>
       </c>
-      <c r="G262" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H262">
+      <c r="G262" s="21" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H262" s="21">
         <f>IF(G262="BUG","BUG-"&amp;A262,IF(G262="FUNCTIONAL","FUNCTIONAL-"&amp;A262,""))</f>
         <v/>
       </c>
-      <c r="I262" t="inlineStr">
+      <c r="I262" s="21" t="inlineStr">
         <is>
           <t>Bassa</t>
         </is>
       </c>
     </row>
     <row r="263">
-      <c r="A263" t="inlineStr">
+      <c r="A263" s="21" t="inlineStr">
         <is>
           <t>TC-N68</t>
         </is>
       </c>
-      <c r="B263" t="inlineStr">
+      <c r="B263" s="21" t="inlineStr">
         <is>
           <t>NEXTGEN - Family Planner (5.4)</t>
         </is>
       </c>
-      <c r="C263" t="inlineStr">
+      <c r="C263" s="21" t="inlineStr">
         <is>
           <t>Vista Mappa: toccare un'attivita' nell'elenco apre la scheda attivita'</t>
         </is>
       </c>
-      <c r="D263" t="inlineStr">
+      <c r="D263" s="21" t="inlineStr">
         <is>
           <t>Account genitore di test con almeno una prenotazione attiva</t>
         </is>
       </c>
-      <c r="E263" t="inlineStr">
+      <c r="E263" s="21" t="inlineStr">
         <is>
           <t>Nel Planner -&gt; Mappa, tocca una riga dell'elenco 'Le tue attivita''</t>
         </is>
       </c>
-      <c r="F263" t="inlineStr">
+      <c r="F263" s="21" t="inlineStr">
         <is>
           <t>Si apre la scheda dell'attivita' corrispondente (/activity/[slug])</t>
         </is>
       </c>
-      <c r="G263" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H263">
+      <c r="G263" s="21" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H263" s="21">
         <f>IF(G263="BUG","BUG-"&amp;A263,IF(G263="FUNCTIONAL","FUNCTIONAL-"&amp;A263,""))</f>
         <v/>
       </c>
-      <c r="I263" t="inlineStr">
+      <c r="I263" s="21" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
     </row>
     <row r="264">
-      <c r="A264" t="inlineStr">
+      <c r="A264" s="21" t="inlineStr">
         <is>
           <t>TC-N69</t>
         </is>
       </c>
-      <c r="B264" t="inlineStr">
+      <c r="B264" s="21" t="inlineStr">
         <is>
           <t>NEXTGEN - Family Planner (5.4)</t>
         </is>
       </c>
-      <c r="C264" t="inlineStr">
+      <c r="C264" s="21" t="inlineStr">
         <is>
           <t>Promemoria: quando presenti, appaiono in Organizzazione sopra le Missioni, senza superare 4 elementi</t>
         </is>
       </c>
-      <c r="D264" t="inlineStr">
+      <c r="D264" s="21" t="inlineStr">
         <is>
           <t>Account genitore di test</t>
         </is>
       </c>
-      <c r="E264" t="inlineStr">
+      <c r="E264" s="21" t="inlineStr">
         <is>
           <t>Apri il Planner in modalita' Organizzazione</t>
         </is>
       </c>
-      <c r="F264" t="inlineStr">
+      <c r="F264" s="21" t="inlineStr">
         <is>
           <t>Se ci sono scadenze reali vicine (finestra di cancellazione, attivita' in arrivo, settimana prioritaria, sovrapposizione, budget vicino al target), compaiono come Promemoria sopra le Missioni, al massimo 4, senza errori di rendering</t>
         </is>
       </c>
-      <c r="G264" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H264">
+      <c r="G264" s="21" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H264" s="21">
         <f>IF(G264="BUG","BUG-"&amp;A264,IF(G264="FUNCTIONAL","FUNCTIONAL-"&amp;A264,""))</f>
         <v/>
       </c>
-      <c r="I264" t="inlineStr">
+      <c r="I264" s="21" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>TC-N70</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Family Planner (5.3 + correttivo)</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>'Applica a tutta la settimana' assegna tutte le celle (5 giorni x andata/ritorno) in un colpo solo</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Account genitore di test con almeno una settimana coperta</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>Nel riepilogo settimana del Calendario, tocca 'Applica a tutta la settimana' -&gt; scegli un'opzione (es. Nonna)</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>Toast 'Assegnato a tutta la settimana!'; tutte le 10 celle (5 giorni x 2 momenti) del bambino risultano assegnate, nessuna resta 'Nessuno assegnato'</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H265">
+        <f>IF(G265="BUG","BUG-"&amp;A265,IF(G265="FUNCTIONAL","FUNCTIONAL-"&amp;A265,""))</f>
+        <v/>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>TC-N71</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Family Planner (5.3 + correttivo)</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>'Applica a tutta la settimana': deselezionare un bambino lo esclude dall'assegnazione rapida</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Account genitore di test con almeno 2 bambini coperti nella stessa settimana</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>Nel riepilogo settimana, deseleziona un bambino dai chip sopra 'Applica a tutta la settimana' -&gt; scegli un'opzione</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>L'assegnazione rapida si applica solo ai bambini rimasti selezionati; il bambino deselezionato non viene toccato</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H266">
+        <f>IF(G266="BUG","BUG-"&amp;A266,IF(G266="FUNCTIONAL","FUNCTIONAL-"&amp;A266,""))</f>
+        <v/>
+      </c>
+      <c r="I266" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
@@ -14501,7 +14593,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:L101"/>
-  <conditionalFormatting sqref="G2:G264">
+  <conditionalFormatting sqref="G2:G266">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="14">
       <formula>"ENHANCEMENT"</formula>
     </cfRule>
@@ -14519,11 +14611,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="G2:G264" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="G2:G266" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"OK,BUG,FUNCTIONAL,ENHANCEMENT,DA TESTARE"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="I2:I264" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="I2:I266" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Alta,Media,Bassa"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Chi fa cosa: 'Applica a tutta la settimana' flessibile su Andata/Ritorno
Feedback di Fabrizio: 'ci vuole qualcosa di flessibile' - oltre a scegliere
i bambini, ora si puo' scegliere di applicare l'assegnazione rapida solo
ad Andata, solo a Ritorno, o a entrambi (default), perche' non e' detto
che chi porta sia anche chi ritira.

- setWeekBulkResponsibilityAction ora accetta un parametro moments (invece
  di applicare sempre a entrambi), stessa logica di upsert multiplo.
- PlannerCalendarView.tsx: chip 'Andata'/'Ritorno' nel pannello di
  applicazione rapida, stessa tecnica toggle gia' usata per i bambini
  (default tutto incluso, si tracciano solo le esclusioni).
- Test Playwright TC-N72 + xlsx aggiornato (riga 267).

tsc --noEmit ed eslint puliti.
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -904,7 +904,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L266"/>
+  <dimension ref="A1:L267"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11.83" customWidth="1" style="30" min="1" max="1"/>
@@ -14500,100 +14500,146 @@
       </c>
     </row>
     <row r="265">
-      <c r="A265" t="inlineStr">
+      <c r="A265" s="21" t="inlineStr">
         <is>
           <t>TC-N70</t>
         </is>
       </c>
-      <c r="B265" t="inlineStr">
+      <c r="B265" s="21" t="inlineStr">
         <is>
           <t>NEXTGEN - Family Planner (5.3 + correttivo)</t>
         </is>
       </c>
-      <c r="C265" t="inlineStr">
+      <c r="C265" s="21" t="inlineStr">
         <is>
           <t>'Applica a tutta la settimana' assegna tutte le celle (5 giorni x andata/ritorno) in un colpo solo</t>
         </is>
       </c>
-      <c r="D265" t="inlineStr">
+      <c r="D265" s="21" t="inlineStr">
         <is>
           <t>Account genitore di test con almeno una settimana coperta</t>
         </is>
       </c>
-      <c r="E265" t="inlineStr">
+      <c r="E265" s="21" t="inlineStr">
         <is>
           <t>Nel riepilogo settimana del Calendario, tocca 'Applica a tutta la settimana' -&gt; scegli un'opzione (es. Nonna)</t>
         </is>
       </c>
-      <c r="F265" t="inlineStr">
+      <c r="F265" s="21" t="inlineStr">
         <is>
           <t>Toast 'Assegnato a tutta la settimana!'; tutte le 10 celle (5 giorni x 2 momenti) del bambino risultano assegnate, nessuna resta 'Nessuno assegnato'</t>
         </is>
       </c>
-      <c r="G265" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H265">
+      <c r="G265" s="21" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H265" s="21">
         <f>IF(G265="BUG","BUG-"&amp;A265,IF(G265="FUNCTIONAL","FUNCTIONAL-"&amp;A265,""))</f>
         <v/>
       </c>
-      <c r="I265" t="inlineStr">
+      <c r="I265" s="21" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
     </row>
     <row r="266">
-      <c r="A266" t="inlineStr">
+      <c r="A266" s="21" t="inlineStr">
         <is>
           <t>TC-N71</t>
         </is>
       </c>
-      <c r="B266" t="inlineStr">
+      <c r="B266" s="21" t="inlineStr">
         <is>
           <t>NEXTGEN - Family Planner (5.3 + correttivo)</t>
         </is>
       </c>
-      <c r="C266" t="inlineStr">
+      <c r="C266" s="21" t="inlineStr">
         <is>
           <t>'Applica a tutta la settimana': deselezionare un bambino lo esclude dall'assegnazione rapida</t>
         </is>
       </c>
-      <c r="D266" t="inlineStr">
+      <c r="D266" s="21" t="inlineStr">
         <is>
           <t>Account genitore di test con almeno 2 bambini coperti nella stessa settimana</t>
         </is>
       </c>
-      <c r="E266" t="inlineStr">
+      <c r="E266" s="21" t="inlineStr">
         <is>
           <t>Nel riepilogo settimana, deseleziona un bambino dai chip sopra 'Applica a tutta la settimana' -&gt; scegli un'opzione</t>
         </is>
       </c>
-      <c r="F266" t="inlineStr">
+      <c r="F266" s="21" t="inlineStr">
         <is>
           <t>L'assegnazione rapida si applica solo ai bambini rimasti selezionati; il bambino deselezionato non viene toccato</t>
         </is>
       </c>
-      <c r="G266" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H266">
+      <c r="G266" s="21" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H266" s="21">
         <f>IF(G266="BUG","BUG-"&amp;A266,IF(G266="FUNCTIONAL","FUNCTIONAL-"&amp;A266,""))</f>
         <v/>
       </c>
-      <c r="I266" t="inlineStr">
+      <c r="I266" s="21" t="inlineStr">
         <is>
           <t>Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>TC-N72</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Family Planner (5.3 + correttivo)</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>'Applica a tutta la settimana': deselezionando 'Ritorno' assegna solo Andata, lasciando Ritorno libero</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Account genitore di test con almeno una settimana coperta e celle libere</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>Nel pannello 'Applica a tutta la settimana', deseleziona il chip 'Ritorno' -&gt; scegli un'opzione (es. Nonno)</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>Toast 'Assegnato a tutta la settimana... (solo Andata)!'; solo le celle Andata (5 giorni) vengono assegnate, le celle Ritorno restano 'Nessuno assegnato'</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H267">
+        <f>IF(G267="BUG","BUG-"&amp;A267,IF(G267="FUNCTIONAL","FUNCTIONAL-"&amp;A267,""))</f>
+        <v/>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>Alta</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:L101"/>
-  <conditionalFormatting sqref="G2:G266">
+  <conditionalFormatting sqref="G2:G267">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="14">
       <formula>"ENHANCEMENT"</formula>
     </cfRule>
@@ -14611,11 +14657,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="G2:G266" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="G2:G267" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"OK,BUG,FUNCTIONAL,ENHANCEMENT,DA TESTARE"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="I2:I266" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="I2:I267" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Alta,Media,Bassa"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Sprint 5.6 (NEXTGEN): Vista Gruppi nel Planner
- Nuovo componente PlannerGroupsView: riempie l'ultima scheda del Planner
  ancora 'in arrivo', con due sezioni - Le tue Community (Sprint 4) e I tuoi
  Gruppi sconto/car pooling (gia' esistenti).
- Nessuna tabella/RLS nuova: riuso 1:1 di getCommunitiesForUser()/
  getGroupsForUser(), gia' collaudate. Card cliccabili -> dettaglio reale
  (/nextgen/community/[id], /groups/[id]). Stati vuoti con CTA quando non si
  fa parte di nulla.
- Badge 'N proposta/e pronta/e per un Gruppo' sulle Community con proposte
  attive, per rendere piu' visibile la relazione gia' esistente
  (spawnGroupFromProposalAction).
- app/nextgen/planner/page.tsx: aggiunte le due query in parallelo alle
  altre gia' presenti; PlannerClient.tsx passa i dati al nuovo componente.
- Test Playwright TC-N78..N81 + righe xlsx corrispondenti.
- tsc --noEmit pulito; eslint pulito sui file toccati.
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -904,7 +904,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L272"/>
+  <dimension ref="A1:L276"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11.83" customWidth="1" style="30" min="1" max="1"/>
@@ -14638,238 +14638,422 @@
       </c>
     </row>
     <row r="268">
-      <c r="A268" t="inlineStr">
+      <c r="A268" s="21" t="inlineStr">
         <is>
           <t>TC-N73</t>
         </is>
       </c>
-      <c r="B268" t="inlineStr">
+      <c r="B268" s="21" t="inlineStr">
         <is>
           <t>NEXTGEN - Family Planner 5.5 (Profilo Famiglia)</t>
         </is>
       </c>
-      <c r="C268" t="inlineStr">
+      <c r="C268" s="21" t="inlineStr">
         <is>
           <t>Il link 'Famiglia' e' raggiungibile dal Planner (Organizzazione)</t>
         </is>
       </c>
-      <c r="D268" t="inlineStr">
+      <c r="D268" s="21" t="inlineStr">
         <is>
           <t>Account genitore di test</t>
         </is>
       </c>
-      <c r="E268" t="inlineStr">
+      <c r="E268" s="21" t="inlineStr">
         <is>
           <t>Da /nextgen/planner tocca il link 'Famiglia'</t>
         </is>
       </c>
-      <c r="F268" t="inlineStr">
+      <c r="F268" s="21" t="inlineStr">
         <is>
           <t>Si apre /nextgen/planner/famiglia con la schermata crea/entra (o la famiglia gia' esistente)</t>
         </is>
       </c>
-      <c r="G268" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H268">
+      <c r="G268" s="21" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H268" s="21">
         <f>IF(G268="BUG","BUG-"&amp;A268,IF(G268="FUNCTIONAL","FUNCTIONAL-"&amp;A268,""))</f>
         <v/>
       </c>
-      <c r="I268" t="inlineStr">
+      <c r="I268" s="21" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
     </row>
     <row r="269">
-      <c r="A269" t="inlineStr">
+      <c r="A269" s="21" t="inlineStr">
         <is>
           <t>TC-N74</t>
         </is>
       </c>
-      <c r="B269" t="inlineStr">
+      <c r="B269" s="21" t="inlineStr">
         <is>
           <t>NEXTGEN - Family Planner 5.5 (Profilo Famiglia)</t>
         </is>
       </c>
-      <c r="C269" t="inlineStr">
+      <c r="C269" s="21" t="inlineStr">
         <is>
           <t>Creare una famiglia mostra nome, codice invito e se stessi come 'Creatore'</t>
         </is>
       </c>
-      <c r="D269" t="inlineStr">
+      <c r="D269" s="21" t="inlineStr">
         <is>
           <t>Account genitore di test senza famiglia</t>
         </is>
       </c>
-      <c r="E269" t="inlineStr">
+      <c r="E269" s="21" t="inlineStr">
         <is>
           <t>Su /nextgen/planner/famiglia, inserisci un nome -&gt; 'Crea famiglia'</t>
         </is>
       </c>
-      <c r="F269" t="inlineStr">
+      <c r="F269" s="21" t="inlineStr">
         <is>
           <t>Toast 'Famiglia creata!'; la pagina mostra il nome, un codice invito e il genitore come 'Creatore' con badge '(Tu)'</t>
         </is>
       </c>
-      <c r="G269" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H269">
+      <c r="G269" s="21" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H269" s="21">
         <f>IF(G269="BUG","BUG-"&amp;A269,IF(G269="FUNCTIONAL","FUNCTIONAL-"&amp;A269,""))</f>
         <v/>
       </c>
-      <c r="I269" t="inlineStr">
+      <c r="I269" s="21" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
     </row>
     <row r="270">
-      <c r="A270" t="inlineStr">
+      <c r="A270" s="21" t="inlineStr">
         <is>
           <t>TC-N75</t>
         </is>
       </c>
-      <c r="B270" t="inlineStr">
+      <c r="B270" s="21" t="inlineStr">
         <is>
           <t>NEXTGEN - Family Planner 5.5 (Profilo Famiglia)</t>
         </is>
       </c>
-      <c r="C270" t="inlineStr">
+      <c r="C270" s="21" t="inlineStr">
         <is>
           <t>Un codice invito non valido mostra un errore chiaro</t>
         </is>
       </c>
-      <c r="D270" t="inlineStr">
+      <c r="D270" s="21" t="inlineStr">
         <is>
           <t>Account genitore di test senza famiglia</t>
         </is>
       </c>
-      <c r="E270" t="inlineStr">
+      <c r="E270" s="21" t="inlineStr">
         <is>
           <t>Su /nextgen/planner/famiglia, inserisci un codice inesistente (es. ZZZZZZ) -&gt; 'Entra nella famiglia'</t>
         </is>
       </c>
-      <c r="F270" t="inlineStr">
+      <c r="F270" s="21" t="inlineStr">
         <is>
           <t>Messaggio 'Codice non valido. Controlla e riprova.'; nessuna famiglia viene creata/associata</t>
         </is>
       </c>
-      <c r="G270" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H270">
+      <c r="G270" s="21" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H270" s="21">
         <f>IF(G270="BUG","BUG-"&amp;A270,IF(G270="FUNCTIONAL","FUNCTIONAL-"&amp;A270,""))</f>
         <v/>
       </c>
-      <c r="I270" t="inlineStr">
+      <c r="I270" s="21" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
     </row>
     <row r="271">
-      <c r="A271" t="inlineStr">
+      <c r="A271" s="21" t="inlineStr">
         <is>
           <t>TC-N76</t>
         </is>
       </c>
-      <c r="B271" t="inlineStr">
+      <c r="B271" s="21" t="inlineStr">
         <is>
           <t>NEXTGEN - Family Planner 5.5 (Profilo Famiglia)</t>
         </is>
       </c>
-      <c r="C271" t="inlineStr">
+      <c r="C271" s="21" t="inlineStr">
         <is>
           <t>Copiare il codice invito mostra la conferma 'Copiato!'</t>
         </is>
       </c>
-      <c r="D271" t="inlineStr">
+      <c r="D271" s="21" t="inlineStr">
         <is>
           <t>Account genitore di test gia' in una famiglia</t>
         </is>
       </c>
-      <c r="E271" t="inlineStr">
+      <c r="E271" s="21" t="inlineStr">
         <is>
           <t>Su /nextgen/planner/famiglia, tocca 'Copia' accanto al codice invito</t>
         </is>
       </c>
-      <c r="F271" t="inlineStr">
+      <c r="F271" s="21" t="inlineStr">
         <is>
           <t>Il pulsante mostra 'Copiato!' per qualche secondo e il codice e' negli appunti</t>
         </is>
       </c>
-      <c r="G271" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H271">
+      <c r="G271" s="21" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H271" s="21">
         <f>IF(G271="BUG","BUG-"&amp;A271,IF(G271="FUNCTIONAL","FUNCTIONAL-"&amp;A271,""))</f>
         <v/>
       </c>
-      <c r="I271" t="inlineStr">
+      <c r="I271" s="21" t="inlineStr">
         <is>
           <t>Bassa</t>
         </is>
       </c>
     </row>
     <row r="272">
-      <c r="A272" t="inlineStr">
+      <c r="A272" s="21" t="inlineStr">
         <is>
           <t>TC-N77</t>
         </is>
       </c>
-      <c r="B272" t="inlineStr">
+      <c r="B272" s="21" t="inlineStr">
         <is>
           <t>NEXTGEN - Family Planner 5.5 (Profilo Famiglia)</t>
         </is>
       </c>
-      <c r="C272" t="inlineStr">
+      <c r="C272" s="21" t="inlineStr">
         <is>
           <t>Uscire dalla famiglia richiede conferma e torna alla schermata crea/entra</t>
         </is>
       </c>
-      <c r="D272" t="inlineStr">
+      <c r="D272" s="21" t="inlineStr">
         <is>
           <t>Account genitore di test gia' in una famiglia</t>
         </is>
       </c>
-      <c r="E272" t="inlineStr">
+      <c r="E272" s="21" t="inlineStr">
         <is>
           <t>Su /nextgen/planner/famiglia, tocca 'Esci dalla famiglia' -&gt; conferma 'Si, esci'</t>
         </is>
       </c>
-      <c r="F272" t="inlineStr">
+      <c r="F272" s="21" t="inlineStr">
         <is>
           <t>Toast 'Hai lasciato la famiglia'; la pagina torna a mostrare 'Crea famiglia'/'Entra con un codice invito'</t>
         </is>
       </c>
-      <c r="G272" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H272">
+      <c r="G272" s="21" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H272" s="21">
         <f>IF(G272="BUG","BUG-"&amp;A272,IF(G272="FUNCTIONAL","FUNCTIONAL-"&amp;A272,""))</f>
         <v/>
       </c>
-      <c r="I272" t="inlineStr">
+      <c r="I272" s="21" t="inlineStr">
         <is>
           <t>Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>TC-N78</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Family Planner 5.6 (Vista Gruppi)</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>La scheda 'Gruppi' del Planner mostra le sezioni Community e Gruppi sconto</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Account genitore di test</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>Da /nextgen/planner tocca la scheda 'Gruppi'</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>Sono visibili le due sezioni 'Le tue Community' e 'I tuoi Gruppi sconto'</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H273">
+        <f>IF(G273="BUG","BUG-"&amp;A273,IF(G273="FUNCTIONAL","FUNCTIONAL-"&amp;A273,""))</f>
+        <v/>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>TC-N79</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Family Planner 5.6 (Vista Gruppi)</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>Senza Community ne' Gruppi, la scheda mostra gli stati vuoti con CTA</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Account genitore di test senza Community e senza Gruppi</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>Da /nextgen/planner tocca la scheda 'Gruppi'</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>Messaggio di stato vuoto per Community con CTA 'Crea o entra' -&gt; /nextgen/community</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H274">
+        <f>IF(G274="BUG","BUG-"&amp;A274,IF(G274="FUNCTIONAL","FUNCTIONAL-"&amp;A274,""))</f>
+        <v/>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>TC-N80</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Family Planner 5.6 (Vista Gruppi)</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>Toccare una card Community apre il suo dettaglio reale</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Account genitore di test gia' in almeno una Community</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Nella scheda 'Gruppi', tocca una card sotto 'Le tue Community'</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>Si apre /nextgen/community/[id], il dettaglio reale della Community</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H275">
+        <f>IF(G275="BUG","BUG-"&amp;A275,IF(G275="FUNCTIONAL","FUNCTIONAL-"&amp;A275,""))</f>
+        <v/>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>TC-N81</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Family Planner 5.6 (Vista Gruppi)</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>Una Community con proposte attive mostra il badge 'pronta per un Gruppo'</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Account genitore di test in una Community con almeno una proposta attiva</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>Nella scheda 'Gruppi', osserva la card della Community con proposte</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>E' visibile un badge tipo 'N proposta/e pronta/e per un Gruppo'</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H276">
+        <f>IF(G276="BUG","BUG-"&amp;A276,IF(G276="FUNCTIONAL","FUNCTIONAL-"&amp;A276,""))</f>
+        <v/>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>Bassa</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:L101"/>
-  <conditionalFormatting sqref="G2:G272">
+  <conditionalFormatting sqref="G2:G276">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="14">
       <formula>"ENHANCEMENT"</formula>
     </cfRule>
@@ -14887,11 +15071,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="G2:G272" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="G2:G276" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"OK,BUG,FUNCTIONAL,ENHANCEMENT,DA TESTARE"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="I2:I272" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="I2:I276" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Alta,Media,Bassa"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
TRAMA rebrand Sprint 2: Login con intro animata (fili -> wordmark -> tagline -> CTA)
- components/TramaLoginIntro.tsx (nuovo): sequenza d'ingresso da Dev Handoff sez. 5a/9 (fili 0.65s, wordmark 1.5s, tagline 1.9s, CTA 2.3-2.4s), auto-advance a 4.2s se l'utente non tocca nulla
- app/globals.css: keyframes trama-mark-in / trama-fade-up, additivi
- app/auth/login/LoginForm.tsx: monta l'intro SOLO per tenant 'family', modalita' 'login' di base, senza ?invite= (deep-link invito resta immediato); 'vista' segnata in sessionStorage al mount (una sola volta per sessione); intro e form reale mutuamente esclusivi nel DOM (niente ambiguita' per Playwright/loginAs su due bottoni 'Accedi'); fix minore: badge iniziali 'BK' -> 'TR' (refuso rimasto dal rebrand Sprint 1)
- tests/genitori/login.spec.ts (nuovo): TC-204..208 (comparsa intro, CTA Accedi/Crea un account, one-shot per sessione, skip su ?invite=)
- xlsx: nuova area 'TRAMA - Login', righe TC-204..208, riga Riepilogo aggiunta
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2660" uniqueCount="1683">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2706" uniqueCount="1712">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -5068,6 +5068,93 @@
   </si>
   <si>
     <t xml:space="preserve">REBRAND TRAMA Sprint 1 - bottom nav NEXTGEN passata da 3/4 a 5 voci (Home/Planner/Scopri/Prenotazioni/Profilo) per allinearsi al mockup TRAMA (Dev Handoff sez. 11.4a). Le ultime due puntano a rotte LEGACY esistenti - tradeoff concordato con Fabrizio finche' non avranno una schermata NEXTGEN dedicata.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-204</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRAMA - Login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'intro animata compare al primo accesso e mostra wordmark, tagline e le CTA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nessuna (prima visita di /auth/login nella sessione browser, tenant famiglia)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /auth/login per la prima volta in questa sessione</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compaiono in sequenza i 5 fili intrecciati, il wordmark TRAMA, la tagline 'Organizing childhood. Together.' e le due CTA 'Accedi'/'Crea un account'; il form (campo email) non e' ancora nel DOM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REBRAND TRAMA Sprint 2 - components/TramaLoginIntro.tsx, montato da LoginForm.tsx solo per tenant 'family', modalita' 'login' di base, senza ?invite=.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-205</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toccare 'Accedi' nell'intro avanza subito al form di login reale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Come TC-204</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nell'intro, tocca il bottone 'Accedi'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il form reale compare subito (campo email, password); il bottone 'Crea un account' dell'intro non c'e' piu'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REBRAND TRAMA Sprint 2 - le CTA dell'intro sono scorciatoie: saltano subito al form, senza aspettare l'auto-advance.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-206</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toccare 'Crea un account' nell'intro avanza al form di registrazione</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nell'intro, tocca il bottone 'Crea un account'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il form di registrazione compare (campo 'Codice invito (opzionale)', bottone 'Registrati')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REBRAND TRAMA Sprint 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-207</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'intro non ricompare in una seconda visita di /auth/login nella stessa sessione</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visita /auth/login una prima volta (intro visibile), poi rivisita /auth/login nella stessa sessione browser</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alla seconda visita il form reale compare subito, senza intro (sessionStorage 'trama-login-intro-seen' gia' impostato)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REBRAND TRAMA Sprint 2 - 'riprodotta una sola volta per sessione' (Dev Handoff sez. 9), non ad ogni riapertura app.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-208</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Un link con ?invite= salta l'intro e mostra subito il form di registrazione</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Un codice invito (anche non valido, non serve verificarlo qui)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /auth/login?invite=CODICE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il form di registrazione compare subito, senza l'intro animata (l'intro rallenterebbe un flusso di invito che l'utente vuole completare in fretta)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REBRAND TRAMA Sprint 2 - coerente con TC-127 (tests/gestore/invites.spec.ts), gia' verificato che ?invite= mostra subito 'Crea un account'.</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -5907,7 +5994,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L291"/>
+  <dimension ref="A1:L296"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -15590,6 +15677,171 @@
       </c>
       <c r="L291" s="1" t="s">
         <v>1678</v>
+      </c>
+    </row>
+    <row r="292" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A292" s="1" t="s">
+        <v>1679</v>
+      </c>
+      <c r="B292" s="1" t="s">
+        <v>1680</v>
+      </c>
+      <c r="C292" s="1" t="s">
+        <v>1681</v>
+      </c>
+      <c r="D292" s="1" t="s">
+        <v>1682</v>
+      </c>
+      <c r="E292" s="1" t="s">
+        <v>1683</v>
+      </c>
+      <c r="F292" s="1" t="s">
+        <v>1684</v>
+      </c>
+      <c r="G292" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H292" s="1" t="str">
+        <f aca="false">IF(G292="BUG","BUG-"&amp;A292,IF(G292="FUNCTIONAL","FUNCTIONAL-"&amp;A292,""))</f>
+        <v/>
+      </c>
+      <c r="I292" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L292" s="1" t="s">
+        <v>1685</v>
+      </c>
+    </row>
+    <row r="293" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A293" s="1" t="s">
+        <v>1686</v>
+      </c>
+      <c r="B293" s="1" t="s">
+        <v>1680</v>
+      </c>
+      <c r="C293" s="1" t="s">
+        <v>1687</v>
+      </c>
+      <c r="D293" s="1" t="s">
+        <v>1688</v>
+      </c>
+      <c r="E293" s="1" t="s">
+        <v>1689</v>
+      </c>
+      <c r="F293" s="1" t="s">
+        <v>1690</v>
+      </c>
+      <c r="G293" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H293" s="1" t="str">
+        <f aca="false">IF(G293="BUG","BUG-"&amp;A293,IF(G293="FUNCTIONAL","FUNCTIONAL-"&amp;A293,""))</f>
+        <v/>
+      </c>
+      <c r="I293" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="L293" s="1" t="s">
+        <v>1691</v>
+      </c>
+    </row>
+    <row r="294" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A294" s="1" t="s">
+        <v>1692</v>
+      </c>
+      <c r="B294" s="1" t="s">
+        <v>1680</v>
+      </c>
+      <c r="C294" s="1" t="s">
+        <v>1693</v>
+      </c>
+      <c r="D294" s="1" t="s">
+        <v>1688</v>
+      </c>
+      <c r="E294" s="1" t="s">
+        <v>1694</v>
+      </c>
+      <c r="F294" s="1" t="s">
+        <v>1695</v>
+      </c>
+      <c r="G294" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H294" s="1" t="str">
+        <f aca="false">IF(G294="BUG","BUG-"&amp;A294,IF(G294="FUNCTIONAL","FUNCTIONAL-"&amp;A294,""))</f>
+        <v/>
+      </c>
+      <c r="I294" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L294" s="1" t="s">
+        <v>1696</v>
+      </c>
+    </row>
+    <row r="295" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A295" s="1" t="s">
+        <v>1697</v>
+      </c>
+      <c r="B295" s="1" t="s">
+        <v>1680</v>
+      </c>
+      <c r="C295" s="1" t="s">
+        <v>1698</v>
+      </c>
+      <c r="D295" s="1" t="s">
+        <v>1688</v>
+      </c>
+      <c r="E295" s="1" t="s">
+        <v>1699</v>
+      </c>
+      <c r="F295" s="1" t="s">
+        <v>1700</v>
+      </c>
+      <c r="G295" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H295" s="1" t="str">
+        <f aca="false">IF(G295="BUG","BUG-"&amp;A295,IF(G295="FUNCTIONAL","FUNCTIONAL-"&amp;A295,""))</f>
+        <v/>
+      </c>
+      <c r="I295" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L295" s="1" t="s">
+        <v>1701</v>
+      </c>
+    </row>
+    <row r="296" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A296" s="1" t="s">
+        <v>1702</v>
+      </c>
+      <c r="B296" s="1" t="s">
+        <v>1680</v>
+      </c>
+      <c r="C296" s="1" t="s">
+        <v>1703</v>
+      </c>
+      <c r="D296" s="1" t="s">
+        <v>1704</v>
+      </c>
+      <c r="E296" s="1" t="s">
+        <v>1705</v>
+      </c>
+      <c r="F296" s="1" t="s">
+        <v>1706</v>
+      </c>
+      <c r="G296" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H296" s="1" t="str">
+        <f aca="false">IF(G296="BUG","BUG-"&amp;A296,IF(G296="FUNCTIONAL","FUNCTIONAL-"&amp;A296,""))</f>
+        <v/>
+      </c>
+      <c r="I296" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L296" s="1" t="s">
+        <v>1707</v>
       </c>
     </row>
   </sheetData>
@@ -15637,7 +15889,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
@@ -15649,7 +15901,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>1679</v>
+        <v>1708</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15657,13 +15909,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1680</v>
+        <v>1709</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1681</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15720,7 +15972,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -15732,11 +15984,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>1682</v>
+        <v>1711</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>
@@ -16023,6 +16275,15 @@
       <c r="E38" s="1" t="n">
         <f aca="false">COUNTIF('Test Case'!B:B,"NEXTGEN - Community")</f>
         <v>9</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D39" s="1" t="s">
+        <v>1680</v>
+      </c>
+      <c r="E39" s="1" t="n">
+        <f aca="false">COUNTIF('Test Case'!B:B,"TRAMA - Login")</f>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
TRAMA Login: correzione a schermata unica (header animato + form, non più due step
- components/TramaLoginHeader.tsx sostituisce TramaLoginIntro.tsx: solo intestazione (fili/wordmark/tagline), niente più CTA proprie che aprivano un secondo step
- app/auth/login/LoginForm.tsx: i campi email/password (e il form di registrazione) stanno SEMPRE sotto l'header, sulla stessa schermata, come richiesto con screenshot da Fabrizio; l'header entra in fade-up col resto (delay 2.3s) solo la prima volta per sessione, poi resta statico ma sempre visibile; input pill-shape + placeholder (niente etichette visibili) per il tenant famiglia, invariato per Gestore/Admin
- tests/genitori/login.spec.ts: TC-204..207 riscritti per il flusso a schermata unica (niente più step intermedio da testare)
- xlsx: righe TC-204..207 aggiornate, rimossa la riga TC-208 (non più pertinente)
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2706" uniqueCount="1712">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2697" uniqueCount="1707">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -5076,7 +5076,7 @@
     <t xml:space="preserve">TRAMA - Login</t>
   </si>
   <si>
-    <t xml:space="preserve">L'intro animata compare al primo accesso e mostra wordmark, tagline e le CTA</t>
+    <t xml:space="preserve">L'header animato e i campi email/password compaiono sulla stessa schermata</t>
   </si>
   <si>
     <t xml:space="preserve">Nessuna (prima visita di /auth/login nella sessione browser, tenant famiglia)</t>
@@ -5085,64 +5085,49 @@
     <t xml:space="preserve">Apri /auth/login per la prima volta in questa sessione</t>
   </si>
   <si>
-    <t xml:space="preserve">Compaiono in sequenza i 5 fili intrecciati, il wordmark TRAMA, la tagline 'Organizing childhood. Together.' e le due CTA 'Accedi'/'Crea un account'; il form (campo email) non e' ancora nel DOM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REBRAND TRAMA Sprint 2 - components/TramaLoginIntro.tsx, montato da LoginForm.tsx solo per tenant 'family', modalita' 'login' di base, senza ?invite=.</t>
+    <t xml:space="preserve">Compaiono in sequenza i 5 fili intrecciati, il wordmark TRAMA, la tagline 'Organizing childhood. Together.' e SUBITO SOTTO, sulla stessa schermata, i campi email/password e il bottone 'Accedi'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REBRAND TRAMA Sprint 2 (rivisto) - components/TramaLoginHeader.tsx, montato da LoginForm.tsx solo per tenant 'family'. Corretto rispetto alla prima versione: niente più uno step 'intro' separato con CTA proprie, i campi sono sempre sulla stessa pagina (richiesta di Fabrizio, con screenshot).</t>
   </si>
   <si>
     <t xml:space="preserve">TC-205</t>
   </si>
   <si>
-    <t xml:space="preserve">Toccare 'Accedi' nell'intro avanza subito al form di login reale</t>
+    <t xml:space="preserve">L'animazione di ingresso c'e' al primo accesso e non si ripete in una seconda visita della sessione</t>
   </si>
   <si>
     <t xml:space="preserve">Come TC-204</t>
   </si>
   <si>
-    <t xml:space="preserve">Nell'intro, tocca il bottone 'Accedi'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Il form reale compare subito (campo email, password); il bottone 'Crea un account' dell'intro non c'e' piu'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REBRAND TRAMA Sprint 2 - le CTA dell'intro sono scorciatoie: saltano subito al form, senza aspettare l'auto-advance.</t>
+    <t xml:space="preserve">Visita /auth/login una prima volta (nota la classe CSS 'trama-mark-in' sul logo), poi rivisita /auth/login nella stessa sessione browser</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alla seconda visita il logo/wordmark/tagline compaiono gia' 'a posto', senza la classe di animazione; il form resta comunque subito visibile in entrambi i casi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REBRAND TRAMA Sprint 2 - 'riprodotta una sola volta per sessione' (Dev Handoff sez. 9) si applica solo all'animazione, non alla visibilita' dell'header (sempre presente).</t>
   </si>
   <si>
     <t xml:space="preserve">TC-206</t>
   </si>
   <si>
-    <t xml:space="preserve">Toccare 'Crea un account' nell'intro avanza al form di registrazione</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nell'intro, tocca il bottone 'Crea un account'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Il form di registrazione compare (campo 'Codice invito (opzionale)', bottone 'Registrati')</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REBRAND TRAMA Sprint 2</t>
+    <t xml:space="preserve">Passando a 'Registrati' l'header animato resta sopra i campi, sulla stessa schermata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tocca 'Non hai un account? Registrati' in fondo al form</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il form di registrazione compare (campo 'Codice invito (opzionale)', bottone 'Registrati'), con l'header TRAMA sempre visibile sopra, senza cambio di pagina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REBRAND TRAMA Sprint 2 - il toggle login/registrazione e' comportamento preesistente, qui verificato in combinazione con l'header TRAMA.</t>
   </si>
   <si>
     <t xml:space="preserve">TC-207</t>
   </si>
   <si>
-    <t xml:space="preserve">L'intro non ricompare in una seconda visita di /auth/login nella stessa sessione</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Visita /auth/login una prima volta (intro visibile), poi rivisita /auth/login nella stessa sessione browser</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alla seconda visita il form reale compare subito, senza intro (sessionStorage 'trama-login-intro-seen' gia' impostato)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REBRAND TRAMA Sprint 2 - 'riprodotta una sola volta per sessione' (Dev Handoff sez. 9), non ad ogni riapertura app.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-208</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Un link con ?invite= salta l'intro e mostra subito il form di registrazione</t>
+    <t xml:space="preserve">Un link con ?invite= mostra subito il form di registrazione, con l'header sopra</t>
   </si>
   <si>
     <t xml:space="preserve">Un codice invito (anche non valido, non serve verificarlo qui)</t>
@@ -5151,7 +5136,7 @@
     <t xml:space="preserve">Apri /auth/login?invite=CODICE</t>
   </si>
   <si>
-    <t xml:space="preserve">Il form di registrazione compare subito, senza l'intro animata (l'intro rallenterebbe un flusso di invito che l'utente vuole completare in fretta)</t>
+    <t xml:space="preserve">Il form di registrazione (con 'Registrati') compare subito, con l'header TRAMA (wordmark) sopra, tutto sulla stessa schermata</t>
   </si>
   <si>
     <t xml:space="preserve">REBRAND TRAMA Sprint 2 - coerente con TC-127 (tests/gestore/invites.spec.ts), gia' verificato che ?invite= mostra subito 'Crea un account'.</t>
@@ -15679,7 +15664,7 @@
         <v>1678</v>
       </c>
     </row>
-    <row r="292" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="292" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A292" s="1" t="s">
         <v>1679</v>
       </c>
@@ -15712,7 +15697,7 @@
         <v>1685</v>
       </c>
     </row>
-    <row r="293" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="293" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A293" s="1" t="s">
         <v>1686</v>
       </c>
@@ -15739,13 +15724,13 @@
         <v/>
       </c>
       <c r="I293" s="1" t="s">
-        <v>42</v>
+        <v>65</v>
       </c>
       <c r="L293" s="1" t="s">
         <v>1691</v>
       </c>
     </row>
-    <row r="294" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="294" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A294" s="1" t="s">
         <v>1692</v>
       </c>
@@ -15778,7 +15763,7 @@
         <v>1696</v>
       </c>
     </row>
-    <row r="295" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="295" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A295" s="1" t="s">
         <v>1697</v>
       </c>
@@ -15789,13 +15774,13 @@
         <v>1698</v>
       </c>
       <c r="D295" s="1" t="s">
-        <v>1688</v>
+        <v>1699</v>
       </c>
       <c r="E295" s="1" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="F295" s="1" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="G295" s="1" t="s">
         <v>74</v>
@@ -15808,41 +15793,20 @@
         <v>56</v>
       </c>
       <c r="L295" s="1" t="s">
-        <v>1701</v>
-      </c>
-    </row>
-    <row r="296" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A296" s="1" t="s">
         <v>1702</v>
       </c>
-      <c r="B296" s="1" t="s">
-        <v>1680</v>
-      </c>
-      <c r="C296" s="1" t="s">
-        <v>1703</v>
-      </c>
-      <c r="D296" s="1" t="s">
-        <v>1704</v>
-      </c>
-      <c r="E296" s="1" t="s">
-        <v>1705</v>
-      </c>
-      <c r="F296" s="1" t="s">
-        <v>1706</v>
-      </c>
-      <c r="G296" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="H296" s="1" t="str">
-        <f aca="false">IF(G296="BUG","BUG-"&amp;A296,IF(G296="FUNCTIONAL","FUNCTIONAL-"&amp;A296,""))</f>
-        <v/>
-      </c>
-      <c r="I296" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="L296" s="1" t="s">
-        <v>1707</v>
-      </c>
+    </row>
+    <row r="296" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A296" s="1"/>
+      <c r="B296" s="1"/>
+      <c r="C296" s="1"/>
+      <c r="D296" s="1"/>
+      <c r="E296" s="1"/>
+      <c r="F296" s="1"/>
+      <c r="G296" s="1"/>
+      <c r="H296" s="1"/>
+      <c r="I296" s="1"/>
+      <c r="L296" s="1"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L101"/>
@@ -15901,7 +15865,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>1708</v>
+        <v>1703</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15909,13 +15873,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1709</v>
+        <v>1704</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1710</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15972,7 +15936,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -15984,11 +15948,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>1711</v>
+        <v>1706</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>
@@ -16277,13 +16241,13 @@
         <v>9</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="D39" s="1" t="s">
         <v>1680</v>
       </c>
       <c r="E39" s="1" t="n">
         <f aca="false">COUNTIF('Test Case'!B:B,"TRAMA - Login")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
TRAMA Login: l'animazione riparte a ogni visita, non solo una volta per sessione
- app/auth/login/LoginForm.tsx: animateHeader ora derivato da tenant (sempre true per famiglia), niente più stato/sessionStorage/useEffect one-shot — su richiesta di Fabrizio dopo test dal vivo ('vorrei l'animazione sempre all'inizio, poi la comparsa dei campi'). Si discosta qui dal Dev Handoff sez. 9 ('una sola volta per sessione'): istruzione diretta del prodotto.
- tests/genitori/login.spec.ts: TC-205 riscritto per verificare che l'animazione ricompaia a ogni visita
- xlsx: TC-205 aggiornato
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -5094,7 +5094,7 @@
     <t xml:space="preserve">TC-205</t>
   </si>
   <si>
-    <t xml:space="preserve">L'animazione di ingresso c'e' al primo accesso e non si ripete in una seconda visita della sessione</t>
+    <t xml:space="preserve">L'animazione di ingresso riparte a ogni visita di /auth/login, non solo la prima</t>
   </si>
   <si>
     <t xml:space="preserve">Come TC-204</t>
@@ -5103,10 +5103,10 @@
     <t xml:space="preserve">Visita /auth/login una prima volta (nota la classe CSS 'trama-mark-in' sul logo), poi rivisita /auth/login nella stessa sessione browser</t>
   </si>
   <si>
-    <t xml:space="preserve">Alla seconda visita il logo/wordmark/tagline compaiono gia' 'a posto', senza la classe di animazione; il form resta comunque subito visibile in entrambi i casi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REBRAND TRAMA Sprint 2 - 'riprodotta una sola volta per sessione' (Dev Handoff sez. 9) si applica solo all'animazione, non alla visibilita' dell'header (sempre presente).</t>
+    <t xml:space="preserve">In entrambe le visite il logo/wordmark/tagline si animano di nuovo dall'inizio (classe 'trama-mark-in' presente ogni volta); il form resta comunque subito interagibile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REBRAND TRAMA Sprint 2 (rivisto 2 volte) - su richiesta di Fabrizio l'animazione NON e' piu' 'una tantum per sessione' (si discosta qui dal Dev Handoff sez. 9): riparte a ogni caricamento della pagina. LoginForm.tsx#animateHeader e' ora un valore derivato da tenant, non piu' stato/sessionStorage.</t>
   </si>
   <si>
     <t xml:space="preserve">TC-206</t>

</xml_diff>

<commit_message>
Badge Accesso disabili + Diete gestite sulle card lista/ricerca
Segnalazione di Fabrizio (screenshot): sulla card attività non compariva né
il badge disabili né quello diete. Stesso gap già risolto per le
certificazioni (commit precedente): i dati (Activity.centerAccessible,
Activity.dietaryOptions) sono popolati da tempo in lib/data/activities.ts e
visibili nel dettaglio (DetailClient.tsx), ma non erano mai stati aggiunti
al rendering di ActivityCard.tsx/ActivityCardHorizontal.tsx.

- ActivityCard.tsx: badge pillola (icona + etichetta) accanto a quello di
  certificazione già aggiunto.
- ActivityCardHorizontal.tsx: icone impilate nell'angolo della copertina
  (card troppo stretta per etichette testuali), con tooltip.
- tests/genitori/attivita.spec.ts: TC-209/TC-210 (fixme, come TC-196/197/208:
  richiedono seed con dati specifici non garantiti dal seed attuale).
- BuddyKids_Test_Case.xlsx: 297 test totali.
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2706" uniqueCount="1712">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2724" uniqueCount="1723">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -5155,6 +5155,39 @@
   </si>
   <si>
     <t xml:space="preserve">Segnalazione di Fabrizio ('non vedo ancora i badge di certificazione sulle schede dei centri') - getActivities() ora carica in blocco le certificazioni approvate e ActivityCard/ActivityCardHorizontal mostrano il badge. test.fixme - come TC-202, richiede una certificazione gia' approvata, non garantita dal seed attuale.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-209</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le card di lista/ricerca mostrano il badge Accesso disabili</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attivita il cui centro abbia accessible=true (vedi TC-196)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri Cerca/Home con l'attivita tra i risultati</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La card mostra il badge "Accesso disabili" (etichetta su ActivityCard, icona sedia a rotelle su ActivityCardHorizontal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Segnalazione di Fabrizio (screenshot): badge disabili assente dalla card - dato gia' presente in Activity (centerAccessible), mancava solo il rendering. test.fixme - come TC-196, richiede seed con centers.accessible=true, non garantito dal seed attuale.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-210</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le card di lista/ricerca mostrano il badge Diete gestite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attivita con dietary_options non vuoto (vedi TC-197)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La card mostra il badge "Diete gestite" (etichetta su ActivityCard, icona insalata su ActivityCardHorizontal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Segnalazione di Fabrizio (screenshot): badge diete assente dalla card - dato gia' presente in Activity (dietaryOptions), mancava solo il rendering. test.fixme - come TC-197, richiede seed con activities.dietary_options non vuoto, non garantito dal seed attuale.</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -5994,7 +6027,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L296"/>
+  <dimension ref="A1:L298"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -15842,6 +15875,72 @@
       </c>
       <c r="L296" s="1" t="s">
         <v>1707</v>
+      </c>
+    </row>
+    <row r="297" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A297" s="1" t="s">
+        <v>1708</v>
+      </c>
+      <c r="B297" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="C297" s="1" t="s">
+        <v>1709</v>
+      </c>
+      <c r="D297" s="1" t="s">
+        <v>1710</v>
+      </c>
+      <c r="E297" s="1" t="s">
+        <v>1711</v>
+      </c>
+      <c r="F297" s="1" t="s">
+        <v>1712</v>
+      </c>
+      <c r="G297" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H297" s="1" t="str">
+        <f aca="false">IF(G297="BUG","BUG-"&amp;A297,IF(G297="FUNCTIONAL","FUNCTIONAL-"&amp;A297,""))</f>
+        <v/>
+      </c>
+      <c r="I297" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L297" s="1" t="s">
+        <v>1713</v>
+      </c>
+    </row>
+    <row r="298" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A298" s="1" t="s">
+        <v>1714</v>
+      </c>
+      <c r="B298" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="C298" s="1" t="s">
+        <v>1715</v>
+      </c>
+      <c r="D298" s="1" t="s">
+        <v>1716</v>
+      </c>
+      <c r="E298" s="1" t="s">
+        <v>1711</v>
+      </c>
+      <c r="F298" s="1" t="s">
+        <v>1717</v>
+      </c>
+      <c r="G298" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H298" s="1" t="str">
+        <f aca="false">IF(G298="BUG","BUG-"&amp;A298,IF(G298="FUNCTIONAL","FUNCTIONAL-"&amp;A298,""))</f>
+        <v/>
+      </c>
+      <c r="I298" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L298" s="1" t="s">
+        <v>1718</v>
       </c>
     </row>
   </sheetData>
@@ -15901,7 +16000,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>1708</v>
+        <v>1719</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15909,13 +16008,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1709</v>
+        <v>1720</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1710</v>
+        <v>1721</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15972,23 +16071,23 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!B:B,"Genitori - Attivita")</f>
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>1711</v>
+        <v>1722</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
TRAMA: TC-217 xlsx + test.fixme per spinner monocromatico
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2778" uniqueCount="1756">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2787" uniqueCount="1762">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -5287,6 +5287,24 @@
   </si>
   <si>
     <t xml:space="preserve">Stesso fix di TC-215, variante white (leggibile su sfondo navy) invece di navy. Stesso logo usato anche nel badge di /auth/login (Partner/Admin) e nel widget demo RoleSwitcher.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-217</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lo spinner di caricamento e' monocromatico coerente col logo del pannello (Partner/Admin)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login Gestore o Admin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Naviga cosi' da attivare la Suspense fallback (loading.tsx) di /center o /admin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lo spinner TRAMA e' navy (non a colori) su Partner; bianco su sfondo navy (senza disco bianco di appoggio) su Admin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Richiesta di Fabrizio dopo il giro loghi Partner/Admin: lo spinner (prima sempre a colori, public/brand/trama-logo-mark.png) deve seguire il colore del marchio del pannello in cui compare. Nuova prop TramaSpinner.tone (color/navy/white). Ampliata anche l'escursione dell'animazione zoom+dissolvenza (0.7-&gt;1.15 invece di 0.88-&gt;1.08) su richiesta esplicita di uno zoom piu' marcato. test.fixme - loading.tsx e' una Suspense fallback transitoria, difficile da catturare in modo affidabile in Playwright senza throttling di rete.</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -6126,7 +6144,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L304"/>
+  <dimension ref="A1:L305"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -16141,7 +16159,7 @@
         <v>1734</v>
       </c>
     </row>
-    <row r="302" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="302" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A302" s="1" t="s">
         <v>1735</v>
       </c>
@@ -16174,7 +16192,7 @@
         <v>1739</v>
       </c>
     </row>
-    <row r="303" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="303" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A303" s="1" t="s">
         <v>1740</v>
       </c>
@@ -16207,7 +16225,7 @@
         <v>1746</v>
       </c>
     </row>
-    <row r="304" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="304" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A304" s="1" t="s">
         <v>1747</v>
       </c>
@@ -16238,6 +16256,39 @@
       </c>
       <c r="L304" s="1" t="s">
         <v>1751</v>
+      </c>
+    </row>
+    <row r="305" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A305" s="1" t="s">
+        <v>1752</v>
+      </c>
+      <c r="B305" s="1" t="s">
+        <v>1741</v>
+      </c>
+      <c r="C305" s="1" t="s">
+        <v>1753</v>
+      </c>
+      <c r="D305" s="1" t="s">
+        <v>1754</v>
+      </c>
+      <c r="E305" s="1" t="s">
+        <v>1755</v>
+      </c>
+      <c r="F305" s="1" t="s">
+        <v>1756</v>
+      </c>
+      <c r="G305" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H305" s="1" t="str">
+        <f aca="false">IF(G305="BUG","BUG-"&amp;A305,IF(G305="FUNCTIONAL","FUNCTIONAL-"&amp;A305,""))</f>
+        <v/>
+      </c>
+      <c r="I305" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="L305" s="1" t="s">
+        <v>1757</v>
       </c>
     </row>
   </sheetData>
@@ -16297,7 +16348,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>1752</v>
+        <v>1758</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16305,13 +16356,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1753</v>
+        <v>1759</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1754</v>
+        <v>1760</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16368,7 +16419,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -16380,11 +16431,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>1755</v>
+        <v>1761</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
TRAMA: xlsx TC-218 per migrazione colori viola/arancio
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2787" uniqueCount="1762">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2796" uniqueCount="1767">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -5305,6 +5305,21 @@
   </si>
   <si>
     <t xml:space="preserve">Richiesta di Fabrizio dopo il giro loghi Partner/Admin: lo spinner (prima sempre a colori, public/brand/trama-logo-mark.png) deve seguire il colore del marchio del pannello in cui compare. Nuova prop TramaSpinner.tone (color/navy/white). Ampliata anche l'escursione dell'animazione zoom+dissolvenza (0.7-&gt;1.15 invece di 0.88-&gt;1.08) su richiesta esplicita di uno zoom piu' marcato. test.fixme - loading.tsx e' una Suspense fallback transitoria, difficile da catturare in modo affidabile in Playwright senza throttling di rete.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-218</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Colori viola/arancio allineati alla palette ufficiale (trama-violet/trama-orange) su tutte le schermate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri Planner/Community/Famiglia NEXTGEN e le pagine Richieste/Gruppo Gestore+Admin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nessuna schermata usa piu' i vecchi colori pre-rebrand #5B4FE9 (viola) o #d4622a (arancio); tutte le pagine continuano a renderizzare correttamente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cambio puramente cromatico (nessuna modifica a struttura/testo), quindi niente nuovo test dedicato: la copertura esiste gia' nei test di rendering delle pagine toccate (tests/nextgen/planner.spec.ts, community.spec.ts, family-planner-5-*.spec.ts, tests/gestore/richieste.spec.ts, tests/admin/nuovi-pannelli.spec.ts - controllano che le pagine carichino senza 'Application error', sufficiente a intercettare un errore di build o una classe Tailwind rotta introdotta dalla sostituzione).</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -6144,7 +6159,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L305"/>
+  <dimension ref="A1:L306"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -16258,7 +16273,7 @@
         <v>1751</v>
       </c>
     </row>
-    <row r="305" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="305" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A305" s="1" t="s">
         <v>1752</v>
       </c>
@@ -16289,6 +16304,39 @@
       </c>
       <c r="L305" s="1" t="s">
         <v>1757</v>
+      </c>
+    </row>
+    <row r="306" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A306" s="1" t="s">
+        <v>1758</v>
+      </c>
+      <c r="B306" s="1" t="s">
+        <v>1741</v>
+      </c>
+      <c r="C306" s="1" t="s">
+        <v>1759</v>
+      </c>
+      <c r="D306" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E306" s="1" t="s">
+        <v>1760</v>
+      </c>
+      <c r="F306" s="1" t="s">
+        <v>1761</v>
+      </c>
+      <c r="G306" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H306" s="1" t="str">
+        <f aca="false">IF(G306="BUG","BUG-"&amp;A306,IF(G306="FUNCTIONAL","FUNCTIONAL-"&amp;A306,""))</f>
+        <v/>
+      </c>
+      <c r="I306" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="L306" s="1" t="s">
+        <v>1762</v>
       </c>
     </row>
   </sheetData>
@@ -16348,7 +16396,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>1758</v>
+        <v>1763</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16356,13 +16404,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1759</v>
+        <v>1764</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1760</v>
+        <v>1765</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16419,7 +16467,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -16431,11 +16479,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>1761</v>
+        <v>1766</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
Planner: sfumatura scroll sui tab modalita + colore rosso sforamento budget
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2859" uniqueCount="1807">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2873" uniqueCount="1818">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -5440,6 +5440,39 @@
   </si>
   <si>
     <t xml:space="preserve">Segnalazione di Fabrizio ("procedi col resto", riferito al restyle sezioni rimanenti dopo la Home): solo la Home aveva ricevuto il trattamento Sprint 3 (Poppins + palette trama-*) — Planner e le sue 5 sotto-viste (PlannerClient/PlannerBudgetView/PlannerCalendarView/PlannerGroupsView), Community (lista+dettaglio) e Ricerca (SearchDiscoveryClient, la piu' indietro: 0 riferimenti trama-* prima di questo sprint) usavano ancora bg-ink/sky/orange/purple per CTA e titoli. Migrati: CTA primari bg-ink -&gt; bg-trama-violet (Salva budget, Crea/Entra community, Condividi proposta, Genera Gruppo, Crea link, OK assegnazione Chi-fa-cosa, ecc.), stato selezionato Mese/Settimana e filtri attivi in Ricerca sky -&gt; trama-violet, warning budget superato orange -&gt; trama-orange; titoli di sezione con font-poppins. VOLUTAMENTE non toccati: DOT_BG (legenda colori per bambino in PlannerCalendarView, kid.accentColor) e gli stati semantici presente/ritardo/assente (CheckinPrompt, NextgenCheckinCard) — sono codifica funzionale multi-colore, non elementi di brand, e rimapparli richiederebbe una decisione di design separata (rischio di rompere la distinguibilita' tra bambini/stati).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-226</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I tab modalita del Planner mostrano una sfumatura quando ci sono altre modalita fuori schermo (es. Budget tagliato)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login genitore, viewport stretto (es. 375px)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen/planner, osserva la riga dei 5 tab modalita senza scorrere, poi scorrila fino in fondo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Con contenuto fuori schermo compare una sfumatura sul bordo destro (e sinistro se scorso); la sfumatura sparisce quando non c e piu nulla da scorrere in quella direzione</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-227</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEXTGEN - Planner Budget</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Superare il tetto di budget colora barra e testo di rosso (non piu arancione)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login genitore, tetto budget impostato e spesa reale sopra il tetto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen/planner, modalita Budget</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La barra di progresso e il testo "hai superato il budget" sono rossi (red-500), non piu arancione (trama-orange)</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -6279,7 +6312,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L313"/>
+  <dimension ref="A1:L315"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -16657,7 +16690,7 @@
         <v>1797</v>
       </c>
     </row>
-    <row r="313" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="313" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A313" s="1" t="s">
         <v>1798</v>
       </c>
@@ -16688,6 +16721,60 @@
       </c>
       <c r="L313" s="1" t="s">
         <v>1802</v>
+      </c>
+    </row>
+    <row r="314" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A314" s="1" t="s">
+        <v>1803</v>
+      </c>
+      <c r="B314" s="1" t="s">
+        <v>1218</v>
+      </c>
+      <c r="C314" s="1" t="s">
+        <v>1804</v>
+      </c>
+      <c r="D314" s="1" t="s">
+        <v>1805</v>
+      </c>
+      <c r="E314" s="1" t="s">
+        <v>1806</v>
+      </c>
+      <c r="F314" s="1" t="s">
+        <v>1807</v>
+      </c>
+      <c r="G314" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H314" s="1" t="str">
+        <f aca="false">IF(G314="BUG","BUG-"&amp;A314,IF(G314="FUNCTIONAL","FUNCTIONAL-"&amp;A314,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="315" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A315" s="1" t="s">
+        <v>1808</v>
+      </c>
+      <c r="B315" s="1" t="s">
+        <v>1809</v>
+      </c>
+      <c r="C315" s="1" t="s">
+        <v>1810</v>
+      </c>
+      <c r="D315" s="1" t="s">
+        <v>1811</v>
+      </c>
+      <c r="E315" s="1" t="s">
+        <v>1812</v>
+      </c>
+      <c r="F315" s="1" t="s">
+        <v>1813</v>
+      </c>
+      <c r="G315" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H315" s="1" t="str">
+        <f aca="false">IF(G315="BUG","BUG-"&amp;A315,IF(G315="FUNCTIONAL","FUNCTIONAL-"&amp;A315,""))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -16747,7 +16834,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>1803</v>
+        <v>1814</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16755,13 +16842,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1804</v>
+        <v>1815</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1805</v>
+        <v>1816</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16818,7 +16905,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -16830,11 +16917,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>1806</v>
+        <v>1817</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>
@@ -17093,7 +17180,7 @@
       </c>
       <c r="E35" s="1" t="n">
         <f aca="false">COUNTIF('Test Case'!B:B,"NEXTGEN - Planner")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
PWA: icone piu grandi + splash screen iOS (icona+claim) per tutti i tenant; Login genitori/partner sfondo bianco
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2873" uniqueCount="1818">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2894" uniqueCount="1836">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -5473,6 +5473,60 @@
   </si>
   <si>
     <t xml:space="preserve">La barra di progresso e il testo "hai superato il budget" sono rossi (red-500), non piu arancione (trama-orange)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-228</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PWA - Icone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le icone PWA (home screen) mostrano il marchio piu grande e prominente rispetto al riquadro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nessuna (verifica visuale statica degli asset)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ispezionare public/icon-*.png, icon-partner-*.png, icon-admin-*.png, apple-touch-icon*.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il marchio occupa circa il 78% del riquadro (prima ~55%), stesso colore/sfondo per tenant di prima (colorato su bianco genitori, navy su bianco partner, bianco su navy admin)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-229</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login - Sfondo bianco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login genitori e Login partner hanno sfondo bianco puro dietro icona/claim; Login admin resta navy con il claim visibile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nessun login richiesto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /auth/login su tenant famiglia (default)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sfondo bianco puro (bg-white, rgb(255,255,255)) dietro l'header animato; il claim "Organizing childhood. Together." e' visibile. Partner/Admin verificati a livello di codice (LoginForm.tsx) - vedi TC-209 (fixme, richiede hostname multipli)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-230</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PWA - Splash screen iOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ogni tenant (genitori/NEXTGEN/partner/admin) ha uno splash screen iOS personalizzato con icona, wordmark e claim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nessuno (verifica statica + tag link nello head)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ispezionare public/splash/*.png e i tag apple-touch-startup-image generati da lib/tenant.ts (splashLinks) in ogni layout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sfondo bianco (genitori/NEXTGEN/partner) o navy (admin) con icona, wordmark TRAMA e claim centrati; 6 dimensioni per tenant coprono i modelli iPhone piu diffusi; Android non supporta uno splash personalizzato equivalente (solo icona+colore da manifest, gia impostato)</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -6312,7 +6366,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L315"/>
+  <dimension ref="A1:L318"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -16723,7 +16777,7 @@
         <v>1802</v>
       </c>
     </row>
-    <row r="314" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="314" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A314" s="1" t="s">
         <v>1803</v>
       </c>
@@ -16750,7 +16804,7 @@
         <v/>
       </c>
     </row>
-    <row r="315" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="315" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A315" s="1" t="s">
         <v>1808</v>
       </c>
@@ -16774,6 +16828,87 @@
       </c>
       <c r="H315" s="1" t="str">
         <f aca="false">IF(G315="BUG","BUG-"&amp;A315,IF(G315="FUNCTIONAL","FUNCTIONAL-"&amp;A315,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="316" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A316" s="1" t="s">
+        <v>1814</v>
+      </c>
+      <c r="B316" s="1" t="s">
+        <v>1815</v>
+      </c>
+      <c r="C316" s="1" t="s">
+        <v>1816</v>
+      </c>
+      <c r="D316" s="1" t="s">
+        <v>1817</v>
+      </c>
+      <c r="E316" s="1" t="s">
+        <v>1818</v>
+      </c>
+      <c r="F316" s="1" t="s">
+        <v>1819</v>
+      </c>
+      <c r="G316" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H316" s="1" t="str">
+        <f aca="false">IF(G316="BUG","BUG-"&amp;A316,IF(G316="FUNCTIONAL","FUNCTIONAL-"&amp;A316,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="317" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A317" s="1" t="s">
+        <v>1820</v>
+      </c>
+      <c r="B317" s="1" t="s">
+        <v>1821</v>
+      </c>
+      <c r="C317" s="1" t="s">
+        <v>1822</v>
+      </c>
+      <c r="D317" s="1" t="s">
+        <v>1823</v>
+      </c>
+      <c r="E317" s="1" t="s">
+        <v>1824</v>
+      </c>
+      <c r="F317" s="1" t="s">
+        <v>1825</v>
+      </c>
+      <c r="G317" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H317" s="1" t="str">
+        <f aca="false">IF(G317="BUG","BUG-"&amp;A317,IF(G317="FUNCTIONAL","FUNCTIONAL-"&amp;A317,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="318" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A318" s="1" t="s">
+        <v>1826</v>
+      </c>
+      <c r="B318" s="1" t="s">
+        <v>1827</v>
+      </c>
+      <c r="C318" s="1" t="s">
+        <v>1828</v>
+      </c>
+      <c r="D318" s="1" t="s">
+        <v>1829</v>
+      </c>
+      <c r="E318" s="1" t="s">
+        <v>1830</v>
+      </c>
+      <c r="F318" s="1" t="s">
+        <v>1831</v>
+      </c>
+      <c r="G318" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H318" s="1" t="str">
+        <f aca="false">IF(G318="BUG","BUG-"&amp;A318,IF(G318="FUNCTIONAL","FUNCTIONAL-"&amp;A318,""))</f>
         <v/>
       </c>
     </row>
@@ -16834,7 +16969,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>1814</v>
+        <v>1832</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16842,13 +16977,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1815</v>
+        <v>1833</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1816</v>
+        <v>1834</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16905,7 +17040,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -16917,11 +17052,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>1817</v>
+        <v>1835</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
Planner: hub Logistica & Famiglia (Indirizzi/Famiglia/Condivisione piano/Prenotazioni consolidati)
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2894" uniqueCount="1836">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2915" uniqueCount="1851">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -5527,6 +5527,51 @@
   </si>
   <si>
     <t xml:space="preserve">Sfondo bianco (genitori/NEXTGEN/partner) o navy (admin) con icona, wordmark TRAMA e claim centrati; 6 dimensioni per tenant coprono i modelli iPhone piu diffusi; Android non supporta uno splash personalizzato equivalente (solo icona+colore da manifest, gia impostato)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-231</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEXTGEN - Planner Logistica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il Planner mostra un solo link 'Logistica &amp; Famiglia' invece dei 3 link separati ripetuti sotto ogni modalita</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen/planner in una qualsiasi modalita (Organizzazione/Calendario/Mappa/Budget/Gruppi)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In fondo compare solo il link 'Logistica &amp; Famiglia' (icona bussola); i vecchi link 'Indirizzi di famiglia'/'Famiglia'/'Gestisci prenotazioni' non compaiono piu qui</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-232</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEXTGEN - Hub Logistica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'hub /nextgen/planner/logistica mostra 4 card verso Indirizzi, Famiglia, Condivisione piano e Le tue prenotazioni</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen/planner/logistica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 card visibili con titolo e sottotitolo esplicativo; ognuna porta alla pagina corretta (Indirizzi/Famiglia -&gt; pagine esistenti; Condivisione piano -&gt; /nextgen/planner?mode=calendario; Le tue prenotazioni -&gt; /prenotazioni)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-233</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEXTGEN - Deep link modalita Planner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aprire /nextgen/planner?mode=calendario seleziona direttamente la modalita Calendario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen/planner/logistica, clicca 'Condivisione piano'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si apre /nextgen/planner?mode=calendario e la vista mostra subito il selettore Mese/Settimana del Calendario, senza dover ricliccare il tab</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -6366,7 +6411,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L318"/>
+  <dimension ref="A1:L321"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -16831,7 +16876,7 @@
         <v/>
       </c>
     </row>
-    <row r="316" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="316" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A316" s="1" t="s">
         <v>1814</v>
       </c>
@@ -16858,7 +16903,7 @@
         <v/>
       </c>
     </row>
-    <row r="317" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="317" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A317" s="1" t="s">
         <v>1820</v>
       </c>
@@ -16885,7 +16930,7 @@
         <v/>
       </c>
     </row>
-    <row r="318" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="318" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A318" s="1" t="s">
         <v>1826</v>
       </c>
@@ -16909,6 +16954,87 @@
       </c>
       <c r="H318" s="1" t="str">
         <f aca="false">IF(G318="BUG","BUG-"&amp;A318,IF(G318="FUNCTIONAL","FUNCTIONAL-"&amp;A318,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="319" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A319" s="1" t="s">
+        <v>1832</v>
+      </c>
+      <c r="B319" s="1" t="s">
+        <v>1833</v>
+      </c>
+      <c r="C319" s="1" t="s">
+        <v>1834</v>
+      </c>
+      <c r="D319" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="E319" s="1" t="s">
+        <v>1835</v>
+      </c>
+      <c r="F319" s="1" t="s">
+        <v>1836</v>
+      </c>
+      <c r="G319" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H319" s="1" t="str">
+        <f aca="false">IF(G319="BUG","BUG-"&amp;A319,IF(G319="FUNCTIONAL","FUNCTIONAL-"&amp;A319,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="320" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A320" s="1" t="s">
+        <v>1837</v>
+      </c>
+      <c r="B320" s="1" t="s">
+        <v>1838</v>
+      </c>
+      <c r="C320" s="1" t="s">
+        <v>1839</v>
+      </c>
+      <c r="D320" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="E320" s="1" t="s">
+        <v>1840</v>
+      </c>
+      <c r="F320" s="1" t="s">
+        <v>1841</v>
+      </c>
+      <c r="G320" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H320" s="1" t="str">
+        <f aca="false">IF(G320="BUG","BUG-"&amp;A320,IF(G320="FUNCTIONAL","FUNCTIONAL-"&amp;A320,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="321" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A321" s="1" t="s">
+        <v>1842</v>
+      </c>
+      <c r="B321" s="1" t="s">
+        <v>1843</v>
+      </c>
+      <c r="C321" s="1" t="s">
+        <v>1844</v>
+      </c>
+      <c r="D321" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="E321" s="1" t="s">
+        <v>1845</v>
+      </c>
+      <c r="F321" s="1" t="s">
+        <v>1846</v>
+      </c>
+      <c r="G321" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H321" s="1" t="str">
+        <f aca="false">IF(G321="BUG","BUG-"&amp;A321,IF(G321="FUNCTIONAL","FUNCTIONAL-"&amp;A321,""))</f>
         <v/>
       </c>
     </row>
@@ -16969,7 +17095,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>1832</v>
+        <v>1847</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16977,13 +17103,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1833</v>
+        <v>1848</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1834</v>
+        <v>1849</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17040,7 +17166,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -17052,11 +17178,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>1835</v>
+        <v>1850</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
Planner: Organizzazione semplificata (avvisi unificati, stato per settimana cliccabile, copertura bambino con dettaglio) + Calendario collassato dentro Organizzazione
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2915" uniqueCount="1851">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2943" uniqueCount="1871">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -5572,6 +5572,66 @@
   </si>
   <si>
     <t xml:space="preserve">Si apre /nextgen/planner?mode=calendario e la vista mostra subito il selettore Mese/Settimana del Calendario, senza dover ricliccare il tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-234</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEXTGEN - Planner Organizzazione</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Promemoria e Missioni mostrano un solo avviso di default (il piu urgente), con 'Mostra tutti' per il resto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login genitore, con almeno 2 avvisi (promemoria+missioni) attivi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen/planner in modalita Organizzazione</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E' visibile un solo banner avviso + link 'Mostra tutti (N)'; cliccandolo compaiono tutti gli avvisi e il link diventa 'Mostra meno'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-235</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La barra di copertura di un bambino, cliccata, mostra il dettaglio settimana per settimana di quel bambino</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login genitore, 2+ bambini</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen/planner, clicca la barra di un bambino in 'Copertura per bambino'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si apre un riquadro con un chip per ogni settimana stagionale (verde se coperta per quel bambino, grigio se no); ricliccando la barra il riquadro si richiude</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-236</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Stato per settimana' (striscia colorata) e' visibile e cliccabile in Organizzazione</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen/planner, individua la sezione 'Stato per settimana', clicca una barra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La pagina scorre fino alla riga di quella settimana nella Timeline sottostante e la evidenzia per circa 1.5s con un anello viola</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-237</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEXTGEN - Planner, Calendario collassato</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il Planner ha 4 modalita (non piu 5): Calendario e' un riquadro pieghevole dentro Organizzazione</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen/planner: osserva la barra dei tab in alto, poi clicca il riquadro 'Calendario' dentro Organizzazione</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La barra tab mostra solo Organizzazione/Mappa/Budget/Gruppi; il riquadro 'Calendario' (stesso nome del vecchio tab) si espande mostrando Mese/Settimana/Chi fa cosa/Condivisione piano invariati, senza cambiare modalita</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -6411,7 +6471,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L321"/>
+  <dimension ref="A1:L325"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -16957,7 +17017,7 @@
         <v/>
       </c>
     </row>
-    <row r="319" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="319" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A319" s="1" t="s">
         <v>1832</v>
       </c>
@@ -16984,7 +17044,7 @@
         <v/>
       </c>
     </row>
-    <row r="320" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="320" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A320" s="1" t="s">
         <v>1837</v>
       </c>
@@ -17011,7 +17071,7 @@
         <v/>
       </c>
     </row>
-    <row r="321" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="321" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A321" s="1" t="s">
         <v>1842</v>
       </c>
@@ -17035,6 +17095,114 @@
       </c>
       <c r="H321" s="1" t="str">
         <f aca="false">IF(G321="BUG","BUG-"&amp;A321,IF(G321="FUNCTIONAL","FUNCTIONAL-"&amp;A321,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="322" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A322" s="1" t="s">
+        <v>1847</v>
+      </c>
+      <c r="B322" s="1" t="s">
+        <v>1848</v>
+      </c>
+      <c r="C322" s="1" t="s">
+        <v>1849</v>
+      </c>
+      <c r="D322" s="1" t="s">
+        <v>1850</v>
+      </c>
+      <c r="E322" s="1" t="s">
+        <v>1851</v>
+      </c>
+      <c r="F322" s="1" t="s">
+        <v>1852</v>
+      </c>
+      <c r="G322" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H322" s="1" t="str">
+        <f aca="false">IF(G322="BUG","BUG-"&amp;A322,IF(G322="FUNCTIONAL","FUNCTIONAL-"&amp;A322,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="323" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A323" s="1" t="s">
+        <v>1853</v>
+      </c>
+      <c r="B323" s="1" t="s">
+        <v>1848</v>
+      </c>
+      <c r="C323" s="1" t="s">
+        <v>1854</v>
+      </c>
+      <c r="D323" s="1" t="s">
+        <v>1855</v>
+      </c>
+      <c r="E323" s="1" t="s">
+        <v>1856</v>
+      </c>
+      <c r="F323" s="1" t="s">
+        <v>1857</v>
+      </c>
+      <c r="G323" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H323" s="1" t="str">
+        <f aca="false">IF(G323="BUG","BUG-"&amp;A323,IF(G323="FUNCTIONAL","FUNCTIONAL-"&amp;A323,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="324" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A324" s="1" t="s">
+        <v>1858</v>
+      </c>
+      <c r="B324" s="1" t="s">
+        <v>1848</v>
+      </c>
+      <c r="C324" s="1" t="s">
+        <v>1859</v>
+      </c>
+      <c r="D324" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="E324" s="1" t="s">
+        <v>1860</v>
+      </c>
+      <c r="F324" s="1" t="s">
+        <v>1861</v>
+      </c>
+      <c r="G324" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H324" s="1" t="str">
+        <f aca="false">IF(G324="BUG","BUG-"&amp;A324,IF(G324="FUNCTIONAL","FUNCTIONAL-"&amp;A324,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="325" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A325" s="1" t="s">
+        <v>1862</v>
+      </c>
+      <c r="B325" s="1" t="s">
+        <v>1863</v>
+      </c>
+      <c r="C325" s="1" t="s">
+        <v>1864</v>
+      </c>
+      <c r="D325" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="E325" s="1" t="s">
+        <v>1865</v>
+      </c>
+      <c r="F325" s="1" t="s">
+        <v>1866</v>
+      </c>
+      <c r="G325" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H325" s="1" t="str">
+        <f aca="false">IF(G325="BUG","BUG-"&amp;A325,IF(G325="FUNCTIONAL","FUNCTIONAL-"&amp;A325,""))</f>
         <v/>
       </c>
     </row>
@@ -17095,7 +17263,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>1847</v>
+        <v>1867</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17103,13 +17271,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1848</v>
+        <v>1868</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1849</v>
+        <v>1869</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17166,7 +17334,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -17178,11 +17346,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>1850</v>
+        <v>1870</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
Planner Mappa: riquadro compatto, pin evidenziato al click, scheda sintetica con Apri scheda/Avvia navigazione
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2943" uniqueCount="1871">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2964" uniqueCount="1887">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -5632,6 +5632,54 @@
   </si>
   <si>
     <t xml:space="preserve">La barra tab mostra solo Organizzazione/Mappa/Budget/Gruppi; il riquadro 'Calendario' (stesso nome del vecchio tab) si espande mostrando Mese/Settimana/Chi fa cosa/Condivisione piano invariati, senza cambiare modalita</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-238</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEXTGEN - Planner Mappa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La mappa e' piu piccola (200px) e il pin cliccato viene evidenziato (viola, piu grande)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login genitore, attivita prenotate con coordinate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen/planner, modalita Mappa, clicca un pin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La mappa occupa un riquadro compatto (~200px); il pin cliccato diventa un cerchio viola piu grande degli altri pin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-239</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Selezionare un'attivita (da mappa o da lista) mostra una scheda sintetica con Apri scheda/Avvia navigazione</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login genitore, attivita prenotate con coordinate e indirizzo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen/planner, modalita Mappa, clicca un'attivita nella lista</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sotto la mappa compare una scheda con nome, indirizzo, distanza stimata e i due pulsanti 'Apri scheda' e 'Avvia navigazione' (quest'ultimo solo se c'e un indirizzo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-240</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Senza selezione, la lista di tutte le attivita resta visibile sotto la mappa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login genitore, attivita prenotate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen/planner, modalita Mappa (nessun pin ancora cliccato), poi chiudi una scheda con la X</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Di default (o dopo aver chiuso la scheda) e' visibile la lista 'Le tue attivita' con distanza stimata per riga</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -6471,7 +6519,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L325"/>
+  <dimension ref="A1:L328"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -17098,7 +17146,7 @@
         <v/>
       </c>
     </row>
-    <row r="322" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="322" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A322" s="1" t="s">
         <v>1847</v>
       </c>
@@ -17125,7 +17173,7 @@
         <v/>
       </c>
     </row>
-    <row r="323" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="323" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A323" s="1" t="s">
         <v>1853</v>
       </c>
@@ -17152,7 +17200,7 @@
         <v/>
       </c>
     </row>
-    <row r="324" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="324" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A324" s="1" t="s">
         <v>1858</v>
       </c>
@@ -17179,7 +17227,7 @@
         <v/>
       </c>
     </row>
-    <row r="325" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="325" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A325" s="1" t="s">
         <v>1862</v>
       </c>
@@ -17203,6 +17251,87 @@
       </c>
       <c r="H325" s="1" t="str">
         <f aca="false">IF(G325="BUG","BUG-"&amp;A325,IF(G325="FUNCTIONAL","FUNCTIONAL-"&amp;A325,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="326" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A326" s="1" t="s">
+        <v>1867</v>
+      </c>
+      <c r="B326" s="1" t="s">
+        <v>1868</v>
+      </c>
+      <c r="C326" s="1" t="s">
+        <v>1869</v>
+      </c>
+      <c r="D326" s="1" t="s">
+        <v>1870</v>
+      </c>
+      <c r="E326" s="1" t="s">
+        <v>1871</v>
+      </c>
+      <c r="F326" s="1" t="s">
+        <v>1872</v>
+      </c>
+      <c r="G326" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H326" s="1" t="str">
+        <f aca="false">IF(G326="BUG","BUG-"&amp;A326,IF(G326="FUNCTIONAL","FUNCTIONAL-"&amp;A326,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="327" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A327" s="1" t="s">
+        <v>1873</v>
+      </c>
+      <c r="B327" s="1" t="s">
+        <v>1868</v>
+      </c>
+      <c r="C327" s="1" t="s">
+        <v>1874</v>
+      </c>
+      <c r="D327" s="1" t="s">
+        <v>1875</v>
+      </c>
+      <c r="E327" s="1" t="s">
+        <v>1876</v>
+      </c>
+      <c r="F327" s="1" t="s">
+        <v>1877</v>
+      </c>
+      <c r="G327" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H327" s="1" t="str">
+        <f aca="false">IF(G327="BUG","BUG-"&amp;A327,IF(G327="FUNCTIONAL","FUNCTIONAL-"&amp;A327,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="328" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A328" s="1" t="s">
+        <v>1878</v>
+      </c>
+      <c r="B328" s="1" t="s">
+        <v>1868</v>
+      </c>
+      <c r="C328" s="1" t="s">
+        <v>1879</v>
+      </c>
+      <c r="D328" s="1" t="s">
+        <v>1880</v>
+      </c>
+      <c r="E328" s="1" t="s">
+        <v>1881</v>
+      </c>
+      <c r="F328" s="1" t="s">
+        <v>1882</v>
+      </c>
+      <c r="G328" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H328" s="1" t="str">
+        <f aca="false">IF(G328="BUG","BUG-"&amp;A328,IF(G328="FUNCTIONAL","FUNCTIONAL-"&amp;A328,""))</f>
         <v/>
       </c>
     </row>
@@ -17263,7 +17392,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>1867</v>
+        <v>1883</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17271,13 +17400,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1868</v>
+        <v>1884</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1869</v>
+        <v>1885</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17334,7 +17463,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -17346,11 +17475,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>1870</v>
+        <v>1886</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
Ricerca: filtri Servizi Accesso disabili/Diete gestite (Sprint 5)
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2964" uniqueCount="1887">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2978" uniqueCount="1898">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -5680,6 +5680,39 @@
   </si>
   <si>
     <t xml:space="preserve">Di default (o dopo aver chiuso la scheda) e' visibile la lista 'Le tue attivita' con distanza stimata per riga</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-241</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEXTGEN - Scopri (Ricerca), Filtri Servizi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il filtro Servizi 'Accesso disabili' mostra solo le attivita con centro accessibile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login genitore, almeno un centro con accesso disabili flaggato e uno senza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen/search, apri il pannello Servizi, seleziona 'Accesso disabili'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il conteggio risultati si aggiorna escludendo le attivita il cui centro non ha accesso disabili; 'Azzera' torna abilitato</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-242</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il filtro Servizi 'Diete gestite' mostra solo le attivita con opzioni dietetiche gestite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login genitore, almeno un'attivita con dietaryOptions valorizzato e una senza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen/search, apri il pannello Servizi, seleziona 'Diete gestite'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il conteggio risultati si aggiorna escludendo le attivita senza opzioni dietetiche gestite; naming coerente col badge 'Diete gestite' su ActivityCard</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -6519,7 +6552,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L328"/>
+  <dimension ref="A1:L330"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -17254,7 +17287,7 @@
         <v/>
       </c>
     </row>
-    <row r="326" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="326" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A326" s="1" t="s">
         <v>1867</v>
       </c>
@@ -17281,7 +17314,7 @@
         <v/>
       </c>
     </row>
-    <row r="327" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="327" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A327" s="1" t="s">
         <v>1873</v>
       </c>
@@ -17308,7 +17341,7 @@
         <v/>
       </c>
     </row>
-    <row r="328" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="328" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A328" s="1" t="s">
         <v>1878</v>
       </c>
@@ -17332,6 +17365,60 @@
       </c>
       <c r="H328" s="1" t="str">
         <f aca="false">IF(G328="BUG","BUG-"&amp;A328,IF(G328="FUNCTIONAL","FUNCTIONAL-"&amp;A328,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="329" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A329" s="1" t="s">
+        <v>1883</v>
+      </c>
+      <c r="B329" s="1" t="s">
+        <v>1884</v>
+      </c>
+      <c r="C329" s="1" t="s">
+        <v>1885</v>
+      </c>
+      <c r="D329" s="1" t="s">
+        <v>1886</v>
+      </c>
+      <c r="E329" s="1" t="s">
+        <v>1887</v>
+      </c>
+      <c r="F329" s="1" t="s">
+        <v>1888</v>
+      </c>
+      <c r="G329" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H329" s="1" t="str">
+        <f aca="false">IF(G329="BUG","BUG-"&amp;A329,IF(G329="FUNCTIONAL","FUNCTIONAL-"&amp;A329,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="330" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A330" s="1" t="s">
+        <v>1889</v>
+      </c>
+      <c r="B330" s="1" t="s">
+        <v>1884</v>
+      </c>
+      <c r="C330" s="1" t="s">
+        <v>1890</v>
+      </c>
+      <c r="D330" s="1" t="s">
+        <v>1891</v>
+      </c>
+      <c r="E330" s="1" t="s">
+        <v>1892</v>
+      </c>
+      <c r="F330" s="1" t="s">
+        <v>1893</v>
+      </c>
+      <c r="G330" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H330" s="1" t="str">
+        <f aca="false">IF(G330="BUG","BUG-"&amp;A330,IF(G330="FUNCTIONAL","FUNCTIONAL-"&amp;A330,""))</f>
         <v/>
       </c>
     </row>
@@ -17392,7 +17479,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>1883</v>
+        <v>1894</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17400,13 +17487,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1884</v>
+        <v>1895</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1885</v>
+        <v>1896</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17463,7 +17550,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -17475,11 +17562,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>1886</v>
+        <v>1897</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
Profilo NEXTGEN: redesign completo (PageHeader+icona brand, card violet), Condivisione piano come impostazione, bottom nav aggiornata
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2978" uniqueCount="1898">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3006" uniqueCount="1915">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -5713,6 +5713,57 @@
   </si>
   <si>
     <t xml:space="preserve">Il conteggio risultati si aggiorna escludendo le attivita senza opzioni dietetiche gestite; naming coerente col badge 'Diete gestite' su ActivityCard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-243</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEXTGEN - Profilo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/nextgen/profile ha PageHeader con icona brand colorata e titolo 'Profilo' (non piu' header gradiente LEGACY)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen/profile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In alto e' visibile una PageHeader con freccia indietro, icona TRAMA a colori e titolo 'Profilo'; sotto, dati profilo e bambini in card bianche stondate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-244</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La bottom nav NEXTGEN porta 'Profilo' a /nextgen/profile (non piu' a /profile LEGACY)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen, clicca 'Profilo' nella bottom nav</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si atterra su /nextgen/profile (non su /profile)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-245</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La card 'Condivisione piano' in Profilo porta al Calendario del Planner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen/profile, sezione 'Piano condiviso', clicca 'Condivisione piano'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si atterra su /nextgen/planner con la modalita' Calendario gia' aperta (stesso link della card equivalente nell'hub Logistica)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-246</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le card di accesso rapido (Prenotazioni/Preferiti/Presenze/Richieste) portano alle pagine corrette</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen/profile, clicca ciascuna card in 'Attivita' e 'Supporto'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Le mie prenotazioni' -&gt; /prenotazioni, 'Preferiti' -&gt; /preferiti, 'Le presenze' -&gt; /presenze, 'Le mie richieste' -&gt; /richieste (con badge se ci sono risposte non lette)</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -6552,7 +6603,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L330"/>
+  <dimension ref="A1:L334"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -17368,7 +17419,7 @@
         <v/>
       </c>
     </row>
-    <row r="329" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="329" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A329" s="1" t="s">
         <v>1883</v>
       </c>
@@ -17395,7 +17446,7 @@
         <v/>
       </c>
     </row>
-    <row r="330" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="330" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A330" s="1" t="s">
         <v>1889</v>
       </c>
@@ -17419,6 +17470,114 @@
       </c>
       <c r="H330" s="1" t="str">
         <f aca="false">IF(G330="BUG","BUG-"&amp;A330,IF(G330="FUNCTIONAL","FUNCTIONAL-"&amp;A330,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="331" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A331" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="B331" s="1" t="s">
+        <v>1895</v>
+      </c>
+      <c r="C331" s="1" t="s">
+        <v>1896</v>
+      </c>
+      <c r="D331" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="E331" s="1" t="s">
+        <v>1897</v>
+      </c>
+      <c r="F331" s="1" t="s">
+        <v>1898</v>
+      </c>
+      <c r="G331" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H331" s="1" t="str">
+        <f aca="false">IF(G331="BUG","BUG-"&amp;A331,IF(G331="FUNCTIONAL","FUNCTIONAL-"&amp;A331,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="332" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A332" s="1" t="s">
+        <v>1899</v>
+      </c>
+      <c r="B332" s="1" t="s">
+        <v>1895</v>
+      </c>
+      <c r="C332" s="1" t="s">
+        <v>1900</v>
+      </c>
+      <c r="D332" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="E332" s="1" t="s">
+        <v>1901</v>
+      </c>
+      <c r="F332" s="1" t="s">
+        <v>1902</v>
+      </c>
+      <c r="G332" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H332" s="1" t="str">
+        <f aca="false">IF(G332="BUG","BUG-"&amp;A332,IF(G332="FUNCTIONAL","FUNCTIONAL-"&amp;A332,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="333" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A333" s="1" t="s">
+        <v>1903</v>
+      </c>
+      <c r="B333" s="1" t="s">
+        <v>1895</v>
+      </c>
+      <c r="C333" s="1" t="s">
+        <v>1904</v>
+      </c>
+      <c r="D333" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="E333" s="1" t="s">
+        <v>1905</v>
+      </c>
+      <c r="F333" s="1" t="s">
+        <v>1906</v>
+      </c>
+      <c r="G333" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H333" s="1" t="str">
+        <f aca="false">IF(G333="BUG","BUG-"&amp;A333,IF(G333="FUNCTIONAL","FUNCTIONAL-"&amp;A333,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="334" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A334" s="1" t="s">
+        <v>1907</v>
+      </c>
+      <c r="B334" s="1" t="s">
+        <v>1895</v>
+      </c>
+      <c r="C334" s="1" t="s">
+        <v>1908</v>
+      </c>
+      <c r="D334" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="E334" s="1" t="s">
+        <v>1909</v>
+      </c>
+      <c r="F334" s="1" t="s">
+        <v>1910</v>
+      </c>
+      <c r="G334" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H334" s="1" t="str">
+        <f aca="false">IF(G334="BUG","BUG-"&amp;A334,IF(G334="FUNCTIONAL","FUNCTIONAL-"&amp;A334,""))</f>
         <v/>
       </c>
     </row>
@@ -17479,7 +17638,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>1894</v>
+        <v>1911</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17487,13 +17646,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1895</v>
+        <v>1912</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1896</v>
+        <v>1913</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17550,7 +17709,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -17562,11 +17721,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>1897</v>
+        <v>1914</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
FIX URGENTE: Mappa Planner crashava sempre (icon=undefined sovrascriveva il marker Leaflet di default)
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3006" uniqueCount="1915">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3013" uniqueCount="1921">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -5764,6 +5764,24 @@
   </si>
   <si>
     <t xml:space="preserve">'Le mie prenotazioni' -&gt; /prenotazioni, 'Preferiti' -&gt; /preferiti, 'Le presenze' -&gt; /presenze, 'Le mie richieste' -&gt; /richieste (con badge se ci sono risposte non lette)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-247</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEXTGEN - Planner Mappa (BUGFIX)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Mappa non crasha piu' al primo apertura (icon undefined sovrascriveva il marker di default in Leaflet)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login genitore, almeno un'attivita' prenotata con coordinate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen/planner, clicca 'Mappa' (nessun pin ancora selezionato)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La mappa si carica normalmente con i marker visibili, nessun errore 'Application error'/pagina bianca; prima del fix crashava sempre (segnalato da Fabrizio, riproducibile sia su web che su PWA)</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -6603,7 +6621,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L334"/>
+  <dimension ref="A1:L335"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -17473,7 +17491,7 @@
         <v/>
       </c>
     </row>
-    <row r="331" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="331" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A331" s="1" t="s">
         <v>1894</v>
       </c>
@@ -17500,7 +17518,7 @@
         <v/>
       </c>
     </row>
-    <row r="332" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="332" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A332" s="1" t="s">
         <v>1899</v>
       </c>
@@ -17527,7 +17545,7 @@
         <v/>
       </c>
     </row>
-    <row r="333" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="333" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A333" s="1" t="s">
         <v>1903</v>
       </c>
@@ -17554,7 +17572,7 @@
         <v/>
       </c>
     </row>
-    <row r="334" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="334" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A334" s="1" t="s">
         <v>1907</v>
       </c>
@@ -17578,6 +17596,33 @@
       </c>
       <c r="H334" s="1" t="str">
         <f aca="false">IF(G334="BUG","BUG-"&amp;A334,IF(G334="FUNCTIONAL","FUNCTIONAL-"&amp;A334,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="335" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A335" s="1" t="s">
+        <v>1911</v>
+      </c>
+      <c r="B335" s="1" t="s">
+        <v>1912</v>
+      </c>
+      <c r="C335" s="1" t="s">
+        <v>1913</v>
+      </c>
+      <c r="D335" s="1" t="s">
+        <v>1914</v>
+      </c>
+      <c r="E335" s="1" t="s">
+        <v>1915</v>
+      </c>
+      <c r="F335" s="1" t="s">
+        <v>1916</v>
+      </c>
+      <c r="G335" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H335" s="1" t="str">
+        <f aca="false">IF(G335="BUG","BUG-"&amp;A335,IF(G335="FUNCTIONAL","FUNCTIONAL-"&amp;A335,""))</f>
         <v/>
       </c>
     </row>
@@ -17638,7 +17683,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>1911</v>
+        <v>1917</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17646,13 +17691,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1912</v>
+        <v>1918</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1913</v>
+        <v>1919</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17709,7 +17754,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -17721,11 +17766,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>1914</v>
+        <v>1920</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
Sprint 7: Indirizzi/Famiglia/Condivisione piano diventano vere sezioni di Profilo, hub Logistica eliminato (redirect)
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3013" uniqueCount="1921">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3041" uniqueCount="1940">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -5782,6 +5782,63 @@
   </si>
   <si>
     <t xml:space="preserve">La mappa si carica normalmente con i marker visibili, nessun errore 'Application error'/pagina bianca; prima del fix crashava sempre (segnalato da Fabrizio, riproducibile sia su web che su PWA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-248</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEXTGEN - Profilo, sezione Famiglia (Sprint 7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profilo mostra le card 'Indirizzi di famiglia' e 'Famiglia' con i link corretti</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen/profile, sezione 'Famiglia'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sono visibili 'Indirizzi di famiglia' (-&gt; /nextgen/planner/indirizzi) e 'Famiglia' (-&gt; /nextgen/planner/famiglia)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-249</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEXTGEN - ex hub Logistica (Sprint 7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il Planner non mostra piu' il link 'Logistica &amp; Famiglia' in fondo alla pagina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen/planner, scorri fino in fondo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non compare piu' nessun link 'Logistica &amp; Famiglia' (Indirizzi/Famiglia/Condivisione piano sono ora in Profilo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-250</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/nextgen/planner/logistica reindirizza a /nextgen/profile invece di essere un vicolo cieco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Naviga direttamente a /nextgen/planner/logistica (es. da un bookmark vecchio)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si viene reindirizzati a /nextgen/profile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-251</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEXTGEN - Indirizzi/Famiglia (Sprint 7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il tasto 'Indietro' da Indirizzi e da Famiglia torna a Profilo (non piu' all'hub Logistica eliminato)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen/profile, entra in 'Indirizzi di famiglia', premi Indietro; ripeti per 'Famiglia'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il tasto Indietro riporta a /nextgen/profile in entrambi i casi</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -6621,7 +6678,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L335"/>
+  <dimension ref="A1:L339"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -17599,7 +17656,7 @@
         <v/>
       </c>
     </row>
-    <row r="335" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="335" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A335" s="1" t="s">
         <v>1911</v>
       </c>
@@ -17623,6 +17680,114 @@
       </c>
       <c r="H335" s="1" t="str">
         <f aca="false">IF(G335="BUG","BUG-"&amp;A335,IF(G335="FUNCTIONAL","FUNCTIONAL-"&amp;A335,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="336" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A336" s="1" t="s">
+        <v>1917</v>
+      </c>
+      <c r="B336" s="1" t="s">
+        <v>1918</v>
+      </c>
+      <c r="C336" s="1" t="s">
+        <v>1919</v>
+      </c>
+      <c r="D336" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="E336" s="1" t="s">
+        <v>1920</v>
+      </c>
+      <c r="F336" s="1" t="s">
+        <v>1921</v>
+      </c>
+      <c r="G336" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H336" s="1" t="str">
+        <f aca="false">IF(G336="BUG","BUG-"&amp;A336,IF(G336="FUNCTIONAL","FUNCTIONAL-"&amp;A336,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="337" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A337" s="1" t="s">
+        <v>1922</v>
+      </c>
+      <c r="B337" s="1" t="s">
+        <v>1923</v>
+      </c>
+      <c r="C337" s="1" t="s">
+        <v>1924</v>
+      </c>
+      <c r="D337" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="E337" s="1" t="s">
+        <v>1925</v>
+      </c>
+      <c r="F337" s="1" t="s">
+        <v>1926</v>
+      </c>
+      <c r="G337" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H337" s="1" t="str">
+        <f aca="false">IF(G337="BUG","BUG-"&amp;A337,IF(G337="FUNCTIONAL","FUNCTIONAL-"&amp;A337,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="338" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A338" s="1" t="s">
+        <v>1927</v>
+      </c>
+      <c r="B338" s="1" t="s">
+        <v>1923</v>
+      </c>
+      <c r="C338" s="1" t="s">
+        <v>1928</v>
+      </c>
+      <c r="D338" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="E338" s="1" t="s">
+        <v>1929</v>
+      </c>
+      <c r="F338" s="1" t="s">
+        <v>1930</v>
+      </c>
+      <c r="G338" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H338" s="1" t="str">
+        <f aca="false">IF(G338="BUG","BUG-"&amp;A338,IF(G338="FUNCTIONAL","FUNCTIONAL-"&amp;A338,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="339" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A339" s="1" t="s">
+        <v>1931</v>
+      </c>
+      <c r="B339" s="1" t="s">
+        <v>1932</v>
+      </c>
+      <c r="C339" s="1" t="s">
+        <v>1933</v>
+      </c>
+      <c r="D339" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="E339" s="1" t="s">
+        <v>1934</v>
+      </c>
+      <c r="F339" s="1" t="s">
+        <v>1935</v>
+      </c>
+      <c r="G339" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H339" s="1" t="str">
+        <f aca="false">IF(G339="BUG","BUG-"&amp;A339,IF(G339="FUNCTIONAL","FUNCTIONAL-"&amp;A339,""))</f>
         <v/>
       </c>
     </row>
@@ -17683,7 +17848,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>1917</v>
+        <v>1936</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17691,13 +17856,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1918</v>
+        <v>1937</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1919</v>
+        <v>1938</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17754,7 +17919,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -17766,11 +17931,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>1920</v>
+        <v>1939</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
FIX: sfondo splash/status-bar login azzurro/verde -> bianco (chromeColor separato da themeColor); back-nav Profilo NEXTGEN dalle pagine condivise usa router.back() invece di backHref fisso a /profile legacy
- manifest-family.json, manifest-partner.json, manifest-nextgen.json: background_color/theme_color -> #FFFFFF (admin invariato, navy)
- lib/tenant.ts: nuovo campo chromeColor (bianco family/partner, navy admin), themeColor invariato per pulsanti/accenti
- app/layout.tsx, app/nextgen/layout.tsx: meta theme-color usa chromeColor
- presenze/prenotazioni/richieste/preferiti/preferenze/privacy/sicurezza: rimosso backHref="/profile" fisso, PageHeader ricade su router.back()
- TC-210 (login.spec.ts), TC-N113 (profile-6.spec.ts), TC-252/253/254 (xlsx)

Segnalato da Fabrizio: sfondo login sbagliato al presentarsi del logo; 'Le presenze' -> Indietro riportava al profilo legacy
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3041" uniqueCount="1940">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3062" uniqueCount="1954">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -5839,6 +5839,48 @@
   </si>
   <si>
     <t xml:space="preserve">Il tasto Indietro riporta a /nextgen/profile in entrambi i casi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-252</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login - Sfondo splash/status-bar (BUGFIX)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il meta theme-color e il manifest (tenant famiglia) sono bianchi, non azzurri</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /auth/login (tenant famiglia), ispeziona &lt;meta name="theme-color"&gt; e /manifest-family.json</t>
+  </si>
+  <si>
+    <t xml:space="preserve">theme-color e manifest.background_color/theme_color sono #FFFFFF; prima erano #4DAFEF (azzurro), colore dipinto dal browser dietro al logo prima del render della pagina (segnalato da Fabrizio: 'quando viene presentato il logo lo sfondo e' ancora sbagliato, azzurro invece che bianco')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-253</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il manifest del tenant partner e' bianco, non verde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ispeziona /manifest-partner.json (background_color/theme_color)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrambi i campi sono #FFFFFF; prima erano #1FA88E (verde), stesso bug del tenant famiglia. Il tenant admin resta invariato (navy #1A1D2E, corretto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-254</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEXTGEN - Profilo, back-nav pagine condivise (BUGFIX)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Da Profilo NEXTGEN, il tasto Indietro dalle pagine condivise (Le presenze, Preferiti, Le mie prenotazioni, Le mie richieste, Sicurezza, Preferenze, Privacy) torna a Profilo NEXTGEN e non al profilo legacy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen/profile, entra in 'Le presenze' (o una delle altre pagine condivise), premi il tasto Indietro dell'header</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si torna a /nextgen/profile (non a /profile legacy). Le stesse pagine raggiunte dal profilo legacy tornano invece a /profile: il tasto Indietro usa la cronologia del browser (router.back()) invece di un backHref fisso a /profile (segnalato da Fabrizio su 'Le presenze')</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -6678,7 +6720,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L339"/>
+  <dimension ref="A1:L342"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -17683,7 +17725,7 @@
         <v/>
       </c>
     </row>
-    <row r="336" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="336" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A336" s="1" t="s">
         <v>1917</v>
       </c>
@@ -17710,7 +17752,7 @@
         <v/>
       </c>
     </row>
-    <row r="337" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="337" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A337" s="1" t="s">
         <v>1922</v>
       </c>
@@ -17737,7 +17779,7 @@
         <v/>
       </c>
     </row>
-    <row r="338" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="338" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A338" s="1" t="s">
         <v>1927</v>
       </c>
@@ -17764,7 +17806,7 @@
         <v/>
       </c>
     </row>
-    <row r="339" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="339" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A339" s="1" t="s">
         <v>1931</v>
       </c>
@@ -17788,6 +17830,87 @@
       </c>
       <c r="H339" s="1" t="str">
         <f aca="false">IF(G339="BUG","BUG-"&amp;A339,IF(G339="FUNCTIONAL","FUNCTIONAL-"&amp;A339,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="340" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A340" s="10" t="s">
+        <v>1936</v>
+      </c>
+      <c r="B340" s="10" t="s">
+        <v>1937</v>
+      </c>
+      <c r="C340" s="10" t="s">
+        <v>1938</v>
+      </c>
+      <c r="D340" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="E340" s="10" t="s">
+        <v>1939</v>
+      </c>
+      <c r="F340" s="10" t="s">
+        <v>1940</v>
+      </c>
+      <c r="G340" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H340" s="10" t="str">
+        <f aca="false">IF(G340="BUG","BUG-"&amp;A340,IF(G340="FUNCTIONAL","FUNCTIONAL-"&amp;A340,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="341" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A341" s="10" t="s">
+        <v>1941</v>
+      </c>
+      <c r="B341" s="10" t="s">
+        <v>1937</v>
+      </c>
+      <c r="C341" s="10" t="s">
+        <v>1942</v>
+      </c>
+      <c r="D341" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="E341" s="10" t="s">
+        <v>1943</v>
+      </c>
+      <c r="F341" s="10" t="s">
+        <v>1944</v>
+      </c>
+      <c r="G341" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H341" s="10" t="str">
+        <f aca="false">IF(G341="BUG","BUG-"&amp;A341,IF(G341="FUNCTIONAL","FUNCTIONAL-"&amp;A341,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="342" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A342" s="10" t="s">
+        <v>1945</v>
+      </c>
+      <c r="B342" s="10" t="s">
+        <v>1946</v>
+      </c>
+      <c r="C342" s="10" t="s">
+        <v>1947</v>
+      </c>
+      <c r="D342" s="10" t="s">
+        <v>264</v>
+      </c>
+      <c r="E342" s="10" t="s">
+        <v>1948</v>
+      </c>
+      <c r="F342" s="10" t="s">
+        <v>1949</v>
+      </c>
+      <c r="G342" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H342" s="10" t="str">
+        <f aca="false">IF(G342="BUG","BUG-"&amp;A342,IF(G342="FUNCTIONAL","FUNCTIONAL-"&amp;A342,""))</f>
         <v/>
       </c>
     </row>
@@ -17848,7 +17971,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>1936</v>
+        <v>1950</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17856,13 +17979,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1937</v>
+        <v>1951</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1938</v>
+        <v>1952</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17919,7 +18042,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -17931,11 +18054,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>1939</v>
+        <v>1953</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
Famiglia: invito 'vero' via email, in aggiunta al codice manuale
Segnalato da Fabrizio: 'per invitare l'altro genitore ci vuole un invito
vero e proprio, il solo codice non è sufficiente'. Scelta confermata: tenere
entrambe le strade (email come flusso principale, codice come alternativa).

- supabase/schema.sql: nuova tabella family_invites (email, token, stato) +
  funzioni security definer get_family_invite_preview/accept_family_invite
- app/actions/family.ts: inviteToFamilyAction (crea invito + invia email via
  lib/email.ts, stesso pattern di app/actions/invites.ts), getFamilyInvitePreviewAction,
  acceptFamilyInviteAction
- FamigliaClient.tsx: form 'Invita per email', lista 'In attesa di risposta',
  banner di accettazione invito (link ?accept=TOKEN via /auth/login?next=...)
- Test TC-N114/115/116 (xlsx TC-255/256/257), TC-258 (xlsx) segnato come
  verifica manuale richiesta (ambiente di test ha un solo account genitore)
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3062" uniqueCount="1954">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3091" uniqueCount="1975">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -5881,6 +5881,69 @@
   </si>
   <si>
     <t xml:space="preserve">Si torna a /nextgen/profile (non a /profile legacy). Le stesse pagine raggiunte dal profilo legacy tornano invece a /profile: il tasto Indietro usa la cronologia del browser (router.back()) invece di un backHref fisso a /profile (segnalato da Fabrizio su 'Le presenze')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-255</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEXTGEN - Profilo, Famiglia: invito via email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il form 'Invita per email' e' visibile per il creatore/admin della famiglia, in aggiunta al codice manuale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login genitore, creatore/admin di una famiglia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen/profile -&gt; Famiglia -&gt; Indirizzi/Famiglia, osserva la sezione Famiglia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E' visibile il form 'Invita per email' (campo email + bottone 'Invia invito') SOPRA il box del codice invito, che resta comunque disponibile come alternativa manuale (scelta di Fabrizio: tenere entrambe le strade)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-256</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inviare un invito per email crea una riga 'In attesa di risposta' e (se Resend configurato) invia l'email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compila 'Email dell'altro genitore' con un'email di test, clicca 'Invia invito'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toast di conferma ('Invito inviato!' o 'Invito creato' se l'email non e' configurata), l'email compare nella lista 'In attesa di risposta' con lo stato corretto (Email inviata / In attesa)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-257</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aprire un link di invito con token non valido/scaduto mostra un errore chiaro, non un crash</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login genitore (qualsiasi)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen/planner/famiglia?accept=TOKEN_INESISTENTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compare il messaggio 'Questo invito non e' (piu') valido...' invece di un errore applicativo; il resto della pagina Famiglia funziona normalmente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-258</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accettare un invito valido (stessa email dell'account loggato) aggiunge l'utente alla famiglia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Un genitore A ha invitato l'email del genitore B (account reale, non l'unico account di test disponibile); NON automatizzabile con un solo account di test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Genitore B apre il link ricevuto via email, arriva su /auth/login?next=/nextgen/planner/famiglia%3Faccept%3DTOKEN, effettua login/registrazione con la STESSA email invitata, vede il prompt 'X ti ha invitato...', clicca 'Accetta l'invito'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il genitore B diventa membro della famiglia (ruolo 'membro'); l'invito passa a stato 'accepted'; se l'email dell'account non corrisponde a quella invitata, viene mostrato l'errore 'Questo invito e' per un'altra email'. VERIFICARE MANUALMENTE con due account reali prima del rilascio (stessa limitazione già nota di TC-N73..77)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verifica manuale richiesta: ambiente di test ha un solo account genitore promosso</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -6720,7 +6783,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L342"/>
+  <dimension ref="A1:L346"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -17833,7 +17896,7 @@
         <v/>
       </c>
     </row>
-    <row r="340" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="340" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A340" s="10" t="s">
         <v>1936</v>
       </c>
@@ -17860,7 +17923,7 @@
         <v/>
       </c>
     </row>
-    <row r="341" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="341" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A341" s="10" t="s">
         <v>1941</v>
       </c>
@@ -17887,7 +17950,7 @@
         <v/>
       </c>
     </row>
-    <row r="342" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="342" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A342" s="10" t="s">
         <v>1945</v>
       </c>
@@ -17912,6 +17975,117 @@
       <c r="H342" s="10" t="str">
         <f aca="false">IF(G342="BUG","BUG-"&amp;A342,IF(G342="FUNCTIONAL","FUNCTIONAL-"&amp;A342,""))</f>
         <v/>
+      </c>
+    </row>
+    <row r="343" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A343" s="10" t="s">
+        <v>1950</v>
+      </c>
+      <c r="B343" s="10" t="s">
+        <v>1951</v>
+      </c>
+      <c r="C343" s="10" t="s">
+        <v>1952</v>
+      </c>
+      <c r="D343" s="10" t="s">
+        <v>1953</v>
+      </c>
+      <c r="E343" s="10" t="s">
+        <v>1954</v>
+      </c>
+      <c r="F343" s="10" t="s">
+        <v>1955</v>
+      </c>
+      <c r="G343" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H343" s="10" t="str">
+        <f aca="false">IF(G343="BUG","BUG-"&amp;A343,IF(G343="FUNCTIONAL","FUNCTIONAL-"&amp;A343,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="344" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A344" s="10" t="s">
+        <v>1956</v>
+      </c>
+      <c r="B344" s="10" t="s">
+        <v>1951</v>
+      </c>
+      <c r="C344" s="10" t="s">
+        <v>1957</v>
+      </c>
+      <c r="D344" s="10" t="s">
+        <v>1953</v>
+      </c>
+      <c r="E344" s="10" t="s">
+        <v>1958</v>
+      </c>
+      <c r="F344" s="10" t="s">
+        <v>1959</v>
+      </c>
+      <c r="G344" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H344" s="10" t="str">
+        <f aca="false">IF(G344="BUG","BUG-"&amp;A344,IF(G344="FUNCTIONAL","FUNCTIONAL-"&amp;A344,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="345" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A345" s="10" t="s">
+        <v>1960</v>
+      </c>
+      <c r="B345" s="10" t="s">
+        <v>1951</v>
+      </c>
+      <c r="C345" s="10" t="s">
+        <v>1961</v>
+      </c>
+      <c r="D345" s="10" t="s">
+        <v>1962</v>
+      </c>
+      <c r="E345" s="10" t="s">
+        <v>1963</v>
+      </c>
+      <c r="F345" s="10" t="s">
+        <v>1964</v>
+      </c>
+      <c r="G345" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H345" s="10" t="str">
+        <f aca="false">IF(G345="BUG","BUG-"&amp;A345,IF(G345="FUNCTIONAL","FUNCTIONAL-"&amp;A345,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="346" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A346" s="10" t="s">
+        <v>1965</v>
+      </c>
+      <c r="B346" s="10" t="s">
+        <v>1951</v>
+      </c>
+      <c r="C346" s="10" t="s">
+        <v>1966</v>
+      </c>
+      <c r="D346" s="10" t="s">
+        <v>1967</v>
+      </c>
+      <c r="E346" s="10" t="s">
+        <v>1968</v>
+      </c>
+      <c r="F346" s="10" t="s">
+        <v>1969</v>
+      </c>
+      <c r="G346" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H346" s="10" t="str">
+        <f aca="false">IF(G346="BUG","BUG-"&amp;A346,IF(G346="FUNCTIONAL","FUNCTIONAL-"&amp;A346,""))</f>
+        <v/>
+      </c>
+      <c r="L346" s="11" t="s">
+        <v>1970</v>
       </c>
     </row>
   </sheetData>
@@ -17971,7 +18145,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>1950</v>
+        <v>1971</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17979,13 +18153,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1951</v>
+        <v>1972</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1952</v>
+        <v>1973</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18042,7 +18216,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -18054,11 +18228,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>1953</v>
+        <v>1974</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
Famiglia invito: link copiabile (WhatsApp/SMS) oltre all'email automatica
Fabrizio: 'ma un link da poter inviare su whatsapp?' — l'invio email non
basta, serve poter condividere l'invito su qualsiasi canale.

- inviteToFamilyAction ora restituisce sempre 'link' (già calcolato lato
  server, prima non veniva esposto al client)
- family_invites.token esposto anche in PendingFamilyInvite, per poter
  ricostruire/ricopiare il link anche dopo un refresh, senza reinviare
- FamigliaClient.tsx: bottone 'Copia link invito' subito dopo l'invio, e
  'Copia link' per riga nella lista 'In attesa di risposta'
- TC-N117 (xlsx TC-259)
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3091" uniqueCount="1975">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3098" uniqueCount="1979">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -5944,6 +5944,18 @@
   </si>
   <si>
     <t xml:space="preserve">Verifica manuale richiesta: ambiente di test ha un solo account genitore promosso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-259</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'invito mostra un link copiabile (WhatsApp, SMS, ecc.), non solo l'invio email automatico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invia un invito per email, poi clicca 'Copia link invito (WhatsApp, SMS...)'; ricarica la pagina e clicca 'Copia link' sulla riga dell'invito in 'In attesa di risposta'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In entrambi i casi il link viene copiato negli appunti (toast 'Link copiato!'); il link porta a /auth/login?next=/nextgen/planner/famiglia%3Faccept%3DTOKEN e mostra il prompt di accettazione</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -6783,7 +6795,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L346"/>
+  <dimension ref="A1:L347"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -17977,7 +17989,7 @@
         <v/>
       </c>
     </row>
-    <row r="343" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="343" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A343" s="10" t="s">
         <v>1950</v>
       </c>
@@ -18004,7 +18016,7 @@
         <v/>
       </c>
     </row>
-    <row r="344" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="344" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A344" s="10" t="s">
         <v>1956</v>
       </c>
@@ -18031,7 +18043,7 @@
         <v/>
       </c>
     </row>
-    <row r="345" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="345" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A345" s="10" t="s">
         <v>1960</v>
       </c>
@@ -18058,7 +18070,7 @@
         <v/>
       </c>
     </row>
-    <row r="346" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="346" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A346" s="10" t="s">
         <v>1965</v>
       </c>
@@ -18086,6 +18098,33 @@
       </c>
       <c r="L346" s="11" t="s">
         <v>1970</v>
+      </c>
+    </row>
+    <row r="347" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A347" s="10" t="s">
+        <v>1971</v>
+      </c>
+      <c r="B347" s="10" t="s">
+        <v>1951</v>
+      </c>
+      <c r="C347" s="10" t="s">
+        <v>1972</v>
+      </c>
+      <c r="D347" s="10" t="s">
+        <v>1953</v>
+      </c>
+      <c r="E347" s="10" t="s">
+        <v>1973</v>
+      </c>
+      <c r="F347" s="10" t="s">
+        <v>1974</v>
+      </c>
+      <c r="G347" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H347" s="10" t="str">
+        <f aca="false">IF(G347="BUG","BUG-"&amp;A347,IF(G347="FUNCTIONAL","FUNCTIONAL-"&amp;A347,""))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -18145,7 +18184,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>1971</v>
+        <v>1975</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18153,13 +18192,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1972</v>
+        <v>1976</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1973</v>
+        <v>1977</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18216,7 +18255,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -18228,11 +18267,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>1974</v>
+        <v>1978</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
Fix favicon identica su tutti i tenant: rimosso app/favicon.ico
app/favicon.ico (convenzione statica Next.js) veniva sempre iniettato
come primo <link rel=icon>, prima delle icone per-tenant dinamiche di
generateMetadata() (app/layout.tsx) — il browser lo preferiva per la
scheda, mostrando la stessa icona per genitori/partner/admin.

Rimosso il file: restano solo i <link> per-tenant generati da
generateMetadata (icon-192.png / icon-partner-192.png /
icon-admin-192.png). Verificato con next build pulito (nessun
favicon.ico nell'output) + tsc/eslint puliti.

Aggiunto TC-261 (xlsx), test TC-261 in tests/genitori/login.spec.ts
(nessun link favicon.ico generico + presenza icona per-tenant).
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3106" uniqueCount="1986">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3114" uniqueCount="1993">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -5977,6 +5977,27 @@
   </si>
   <si>
     <t xml:space="preserve">SVG sorgente salvati in public/brand/svg/ per rigenerazioni future</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-261</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Branding - Favicon per-tenant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La favicon nella scheda del browser e' quella corretta per ciascun tenant (colorata=genitori, navy=partner, bianca su navy=admin), non identica per tutti e tre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nessuna (bug gia' presente nel deploy live, segnalato da Fabrizio con screenshot delle 3 schede browser identiche)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri in 3 schede diverse: trama.app/auth/login, partner.trama.app/auth/login, admin.trama.app/auth/login; osserva l'icona nella scheda del browser di ciascuna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ogni scheda mostra l'icona del proprio tenant (icon-192.png/icon-partner-192.png/icon-admin-192.png), non piu' un'unica favicon.ico generica identica per tutti</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Causa: app/favicon.ico (convenzione statica Next.js, non sensibile all'host) veniva iniettato sempre come primo &lt;link rel=icon&gt;, prima delle icone per-tenant di generateMetadata(). Fix: rimosso app/favicon.ico. Verificato con next build pulito (nessun favicon.ico nell'output) + tsc/eslint puliti. Verifica visiva sulle 3 schede da fare da Fabrizio dopo il deploy.</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -6816,7 +6837,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L348"/>
+  <dimension ref="A1:L349"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -18148,7 +18169,7 @@
         <v/>
       </c>
     </row>
-    <row r="348" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="348" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A348" s="10" t="s">
         <v>1975</v>
       </c>
@@ -18176,6 +18197,36 @@
       </c>
       <c r="L348" s="11" t="s">
         <v>1981</v>
+      </c>
+    </row>
+    <row r="349" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A349" s="10" t="s">
+        <v>1982</v>
+      </c>
+      <c r="B349" s="10" t="s">
+        <v>1983</v>
+      </c>
+      <c r="C349" s="10" t="s">
+        <v>1984</v>
+      </c>
+      <c r="D349" s="10" t="s">
+        <v>1985</v>
+      </c>
+      <c r="E349" s="10" t="s">
+        <v>1986</v>
+      </c>
+      <c r="F349" s="10" t="s">
+        <v>1987</v>
+      </c>
+      <c r="G349" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H349" s="10" t="str">
+        <f aca="false">IF(G349="BUG","BUG-"&amp;A349,IF(G349="FUNCTIONAL","FUNCTIONAL-"&amp;A349,""))</f>
+        <v/>
+      </c>
+      <c r="L349" s="11" t="s">
+        <v>1988</v>
       </c>
     </row>
   </sheetData>
@@ -18235,7 +18286,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>1982</v>
+        <v>1989</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18243,13 +18294,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1983</v>
+        <v>1990</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1984</v>
+        <v>1991</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18306,7 +18357,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -18318,11 +18369,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>1985</v>
+        <v>1992</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
Branding: ripristinato disegno icona precedente (revert SVG regen)
Fabrizio: le icone per-tenant ora sono corrette per colore, ma il
disegno del mark introdotto in 15ae8ba (da TRAMA_PWA_SVG_icons.zip)
non e' quello giusto -> richiesto il ripristino del disegno storico.

Ripristinati (dal commit precedente 43de44f) i 39 PNG toccati da
15ae8ba: icon-{,partner,admin,nextgen}-{192,512}.png,
apple-touch-icon*.png, brand/trama-logo-mark{,-navy,-white}.png,
tutti gli splash iOS.

NON toccato app/favicon.ico (resta rimosso, e' il fix separato di
TC-261 per la differenziazione favicon per-tenant).

TC-262 (xlsx). Verificato tsc/next build puliti.
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3114" uniqueCount="1993">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3122" uniqueCount="2000">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -5998,6 +5998,27 @@
   </si>
   <si>
     <t xml:space="preserve">Causa: app/favicon.ico (convenzione statica Next.js, non sensibile all'host) veniva iniettato sempre come primo &lt;link rel=icon&gt;, prima delle icone per-tenant di generateMetadata(). Fix: rimosso app/favicon.ico. Verificato con next build pulito (nessun favicon.ico nell'output) + tsc/eslint puliti. Verifica visiva sulle 3 schede da fare da Fabrizio dopo il deploy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-262</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Branding - Icone: ripristino disegno precedente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il simbolo dell'icona (mark) e' quello storico, non il nuovo disegno da SVG (Fabrizio: 'l'icona, proprio il disegno, e' quello sbagliato')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-260/TC-261 avevano introdotto un nuovo disegno del mark da TRAMA_PWA_SVG_icons.zip; Fabrizio ha chiesto di ripristinare il disegno precedente pur mantenendo la differenziazione per tenant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /auth/login (genitore/partner/admin) e /nextgen/* (icona inline nell'header); ispeziona icon-192/512.png, icon-{partner,admin,nextgen}-192/512.png, apple-touch-icon*.png, splash screens, trama-logo-mark*.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il disegno del mark e' quello storico (pre TRAMA_PWA_SVG_icons.zip), non il nuovo; resta pero' corretta la regola di brand (colorata=genitori, navy=gestori/partner, bianca su navy=admin) e la favicon per-tenant (TC-261, non regredita: app/favicon.ico resta rimosso)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ripristinati (git checkout dal commit precedente 43de44f) i 39 PNG toccati dal commit 15ae8ba (icon-*, apple-touch-icon*, brand/trama-logo-mark*, splash/*); NON ripristinato app/favicon.ico (resta cancellato, e' il fix di TC-261). Verificato con next build + tsc puliti.</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -6837,7 +6858,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L349"/>
+  <dimension ref="A1:L350"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -18199,7 +18220,7 @@
         <v>1981</v>
       </c>
     </row>
-    <row r="349" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="349" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A349" s="10" t="s">
         <v>1982</v>
       </c>
@@ -18227,6 +18248,36 @@
       </c>
       <c r="L349" s="11" t="s">
         <v>1988</v>
+      </c>
+    </row>
+    <row r="350" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A350" s="10" t="s">
+        <v>1989</v>
+      </c>
+      <c r="B350" s="10" t="s">
+        <v>1990</v>
+      </c>
+      <c r="C350" s="10" t="s">
+        <v>1991</v>
+      </c>
+      <c r="D350" s="10" t="s">
+        <v>1992</v>
+      </c>
+      <c r="E350" s="10" t="s">
+        <v>1993</v>
+      </c>
+      <c r="F350" s="10" t="s">
+        <v>1994</v>
+      </c>
+      <c r="G350" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H350" s="10" t="str">
+        <f aca="false">IF(G350="BUG","BUG-"&amp;A350,IF(G350="FUNCTIONAL","FUNCTIONAL-"&amp;A350,""))</f>
+        <v/>
+      </c>
+      <c r="L350" s="11" t="s">
+        <v>1995</v>
       </c>
     </row>
   </sheetData>
@@ -18286,7 +18337,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>1989</v>
+        <v>1996</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18294,13 +18345,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1990</v>
+        <v>1997</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1991</v>
+        <v>1998</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18357,7 +18408,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -18369,11 +18420,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>1992</v>
+        <v>1999</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
Sprint 2 Organizzazione: Timeline raggruppata per mese, righe cliccabili, date su Stato per settimana
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -913,21 +913,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L358"/>
+  <dimension ref="A1:L361"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="11.83" customWidth="1" style="31" min="1" max="1"/>
-    <col width="24" customWidth="1" style="31" min="2" max="2"/>
-    <col width="36" customWidth="1" style="31" min="3" max="3"/>
-    <col width="40.83" customWidth="1" style="31" min="4" max="4"/>
-    <col width="60.16" customWidth="1" style="31" min="5" max="5"/>
-    <col width="70.16" customWidth="1" style="31" min="6" max="6"/>
-    <col width="18" customWidth="1" style="31" min="7" max="7"/>
-    <col width="20.51" customWidth="1" style="31" min="8" max="8"/>
-    <col width="12.16" customWidth="1" style="31" min="9" max="9"/>
-    <col width="18.16" customWidth="1" style="31" min="10" max="10"/>
-    <col width="77.66" customWidth="1" style="32" min="11" max="12"/>
-    <col width="39" customWidth="1" style="31" min="13" max="16384"/>
+    <col width="11.83" customWidth="1" style="39" min="1" max="1"/>
+    <col width="24" customWidth="1" style="39" min="2" max="2"/>
+    <col width="36" customWidth="1" style="39" min="3" max="3"/>
+    <col width="40.83" customWidth="1" style="39" min="4" max="4"/>
+    <col width="60.16" customWidth="1" style="39" min="5" max="5"/>
+    <col width="70.16" customWidth="1" style="39" min="6" max="6"/>
+    <col width="18" customWidth="1" style="39" min="7" max="7"/>
+    <col width="20.51" customWidth="1" style="39" min="8" max="8"/>
+    <col width="12.16" customWidth="1" style="39" min="9" max="9"/>
+    <col width="18.16" customWidth="1" style="39" min="10" max="10"/>
+    <col width="77.66" customWidth="1" style="40" min="11" max="12"/>
+    <col width="39" customWidth="1" style="39" min="13" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="31.5" customHeight="1" s="23">
@@ -17969,727 +17969,727 @@
       </c>
     </row>
     <row r="340" ht="15" customHeight="1" s="23">
-      <c r="A340" s="31" t="inlineStr">
+      <c r="A340" s="39" t="inlineStr">
         <is>
           <t>TC-252</t>
         </is>
       </c>
-      <c r="B340" s="31" t="inlineStr">
+      <c r="B340" s="39" t="inlineStr">
         <is>
           <t>Login - Sfondo splash/status-bar (BUGFIX)</t>
         </is>
       </c>
-      <c r="C340" s="31" t="inlineStr">
+      <c r="C340" s="39" t="inlineStr">
         <is>
           <t>Il meta theme-color e il manifest (tenant famiglia) sono bianchi, non azzurri</t>
         </is>
       </c>
-      <c r="D340" s="31" t="inlineStr">
+      <c r="D340" s="39" t="inlineStr">
         <is>
           <t>Nessuna</t>
         </is>
       </c>
-      <c r="E340" s="31" t="inlineStr">
+      <c r="E340" s="39" t="inlineStr">
         <is>
           <t>Apri /auth/login (tenant famiglia), ispeziona &lt;meta name="theme-color"&gt; e /manifest-family.json</t>
         </is>
       </c>
-      <c r="F340" s="31" t="inlineStr">
+      <c r="F340" s="39" t="inlineStr">
         <is>
           <t>theme-color e manifest.background_color/theme_color sono #FFFFFF; prima erano #4DAFEF (azzurro), colore dipinto dal browser dietro al logo prima del render della pagina (segnalato da Fabrizio: 'quando viene presentato il logo lo sfondo e' ancora sbagliato, azzurro invece che bianco')</t>
         </is>
       </c>
-      <c r="G340" s="31" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H340" s="31">
+      <c r="G340" s="39" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H340" s="39">
         <f>IF(G340="BUG","BUG-"&amp;A340,IF(G340="FUNCTIONAL","FUNCTIONAL-"&amp;A340,""))</f>
         <v/>
       </c>
     </row>
     <row r="341" ht="15" customHeight="1" s="23">
-      <c r="A341" s="31" t="inlineStr">
+      <c r="A341" s="39" t="inlineStr">
         <is>
           <t>TC-253</t>
         </is>
       </c>
-      <c r="B341" s="31" t="inlineStr">
+      <c r="B341" s="39" t="inlineStr">
         <is>
           <t>Login - Sfondo splash/status-bar (BUGFIX)</t>
         </is>
       </c>
-      <c r="C341" s="31" t="inlineStr">
+      <c r="C341" s="39" t="inlineStr">
         <is>
           <t>Il manifest del tenant partner e' bianco, non verde</t>
         </is>
       </c>
-      <c r="D341" s="31" t="inlineStr">
+      <c r="D341" s="39" t="inlineStr">
         <is>
           <t>Nessuna</t>
         </is>
       </c>
-      <c r="E341" s="31" t="inlineStr">
+      <c r="E341" s="39" t="inlineStr">
         <is>
           <t>Ispeziona /manifest-partner.json (background_color/theme_color)</t>
         </is>
       </c>
-      <c r="F341" s="31" t="inlineStr">
+      <c r="F341" s="39" t="inlineStr">
         <is>
           <t>Entrambi i campi sono #FFFFFF; prima erano #1FA88E (verde), stesso bug del tenant famiglia. Il tenant admin resta invariato (navy #1A1D2E, corretto)</t>
         </is>
       </c>
-      <c r="G341" s="31" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H341" s="31">
+      <c r="G341" s="39" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H341" s="39">
         <f>IF(G341="BUG","BUG-"&amp;A341,IF(G341="FUNCTIONAL","FUNCTIONAL-"&amp;A341,""))</f>
         <v/>
       </c>
     </row>
     <row r="342" ht="15" customHeight="1" s="23">
-      <c r="A342" s="31" t="inlineStr">
+      <c r="A342" s="39" t="inlineStr">
         <is>
           <t>TC-254</t>
         </is>
       </c>
-      <c r="B342" s="31" t="inlineStr">
+      <c r="B342" s="39" t="inlineStr">
         <is>
           <t>NEXTGEN - Profilo, back-nav pagine condivise (BUGFIX)</t>
         </is>
       </c>
-      <c r="C342" s="31" t="inlineStr">
+      <c r="C342" s="39" t="inlineStr">
         <is>
           <t>Da Profilo NEXTGEN, il tasto Indietro dalle pagine condivise (Le presenze, Preferiti, Le mie prenotazioni, Le mie richieste, Sicurezza, Preferenze, Privacy) torna a Profilo NEXTGEN e non al profilo legacy</t>
         </is>
       </c>
-      <c r="D342" s="31" t="inlineStr">
+      <c r="D342" s="39" t="inlineStr">
         <is>
           <t>Login genitore</t>
         </is>
       </c>
-      <c r="E342" s="31" t="inlineStr">
+      <c r="E342" s="39" t="inlineStr">
         <is>
           <t>Apri /nextgen/profile, entra in 'Le presenze' (o una delle altre pagine condivise), premi il tasto Indietro dell'header</t>
         </is>
       </c>
-      <c r="F342" s="31" t="inlineStr">
+      <c r="F342" s="39" t="inlineStr">
         <is>
           <t>Si torna a /nextgen/profile (non a /profile legacy). Le stesse pagine raggiunte dal profilo legacy tornano invece a /profile: il tasto Indietro usa la cronologia del browser (router.back()) invece di un backHref fisso a /profile (segnalato da Fabrizio su 'Le presenze')</t>
         </is>
       </c>
-      <c r="G342" s="31" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H342" s="31">
+      <c r="G342" s="39" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H342" s="39">
         <f>IF(G342="BUG","BUG-"&amp;A342,IF(G342="FUNCTIONAL","FUNCTIONAL-"&amp;A342,""))</f>
         <v/>
       </c>
     </row>
     <row r="343" ht="15" customHeight="1" s="23">
-      <c r="A343" s="31" t="inlineStr">
+      <c r="A343" s="39" t="inlineStr">
         <is>
           <t>TC-255</t>
         </is>
       </c>
-      <c r="B343" s="31" t="inlineStr">
+      <c r="B343" s="39" t="inlineStr">
         <is>
           <t>NEXTGEN - Profilo, Famiglia: invito via email</t>
         </is>
       </c>
-      <c r="C343" s="31" t="inlineStr">
+      <c r="C343" s="39" t="inlineStr">
         <is>
           <t>Il form 'Invita per email' e' visibile per il creatore/admin della famiglia, in aggiunta al codice manuale</t>
         </is>
       </c>
-      <c r="D343" s="31" t="inlineStr">
+      <c r="D343" s="39" t="inlineStr">
         <is>
           <t>Login genitore, creatore/admin di una famiglia</t>
         </is>
       </c>
-      <c r="E343" s="31" t="inlineStr">
+      <c r="E343" s="39" t="inlineStr">
         <is>
           <t>Apri /nextgen/profile -&gt; Famiglia -&gt; Indirizzi/Famiglia, osserva la sezione Famiglia</t>
         </is>
       </c>
-      <c r="F343" s="31" t="inlineStr">
+      <c r="F343" s="39" t="inlineStr">
         <is>
           <t>E' visibile il form 'Invita per email' (campo email + bottone 'Invia invito') SOPRA il box del codice invito, che resta comunque disponibile come alternativa manuale (scelta di Fabrizio: tenere entrambe le strade)</t>
         </is>
       </c>
-      <c r="G343" s="31" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H343" s="31">
+      <c r="G343" s="39" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H343" s="39">
         <f>IF(G343="BUG","BUG-"&amp;A343,IF(G343="FUNCTIONAL","FUNCTIONAL-"&amp;A343,""))</f>
         <v/>
       </c>
     </row>
     <row r="344" ht="15" customHeight="1" s="23">
-      <c r="A344" s="31" t="inlineStr">
+      <c r="A344" s="39" t="inlineStr">
         <is>
           <t>TC-256</t>
         </is>
       </c>
-      <c r="B344" s="31" t="inlineStr">
+      <c r="B344" s="39" t="inlineStr">
         <is>
           <t>NEXTGEN - Profilo, Famiglia: invito via email</t>
         </is>
       </c>
-      <c r="C344" s="31" t="inlineStr">
+      <c r="C344" s="39" t="inlineStr">
         <is>
           <t>Inviare un invito per email crea una riga 'In attesa di risposta' e (se Resend configurato) invia l'email</t>
         </is>
       </c>
-      <c r="D344" s="31" t="inlineStr">
+      <c r="D344" s="39" t="inlineStr">
         <is>
           <t>Login genitore, creatore/admin di una famiglia</t>
         </is>
       </c>
-      <c r="E344" s="31" t="inlineStr">
+      <c r="E344" s="39" t="inlineStr">
         <is>
           <t>Compila 'Email dell'altro genitore' con un'email di test, clicca 'Invia invito'</t>
         </is>
       </c>
-      <c r="F344" s="31" t="inlineStr">
+      <c r="F344" s="39" t="inlineStr">
         <is>
           <t>Toast di conferma ('Invito inviato!' o 'Invito creato' se l'email non e' configurata), l'email compare nella lista 'In attesa di risposta' con lo stato corretto (Email inviata / In attesa)</t>
         </is>
       </c>
-      <c r="G344" s="31" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H344" s="31">
+      <c r="G344" s="39" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H344" s="39">
         <f>IF(G344="BUG","BUG-"&amp;A344,IF(G344="FUNCTIONAL","FUNCTIONAL-"&amp;A344,""))</f>
         <v/>
       </c>
     </row>
     <row r="345" ht="15" customHeight="1" s="23">
-      <c r="A345" s="31" t="inlineStr">
+      <c r="A345" s="39" t="inlineStr">
         <is>
           <t>TC-257</t>
         </is>
       </c>
-      <c r="B345" s="31" t="inlineStr">
+      <c r="B345" s="39" t="inlineStr">
         <is>
           <t>NEXTGEN - Profilo, Famiglia: invito via email</t>
         </is>
       </c>
-      <c r="C345" s="31" t="inlineStr">
+      <c r="C345" s="39" t="inlineStr">
         <is>
           <t>Aprire un link di invito con token non valido/scaduto mostra un errore chiaro, non un crash</t>
         </is>
       </c>
-      <c r="D345" s="31" t="inlineStr">
+      <c r="D345" s="39" t="inlineStr">
         <is>
           <t>Login genitore (qualsiasi)</t>
         </is>
       </c>
-      <c r="E345" s="31" t="inlineStr">
+      <c r="E345" s="39" t="inlineStr">
         <is>
           <t>Apri /nextgen/planner/famiglia?accept=TOKEN_INESISTENTE</t>
         </is>
       </c>
-      <c r="F345" s="31" t="inlineStr">
+      <c r="F345" s="39" t="inlineStr">
         <is>
           <t>Compare il messaggio 'Questo invito non e' (piu') valido...' invece di un errore applicativo; il resto della pagina Famiglia funziona normalmente</t>
         </is>
       </c>
-      <c r="G345" s="31" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H345" s="31">
+      <c r="G345" s="39" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H345" s="39">
         <f>IF(G345="BUG","BUG-"&amp;A345,IF(G345="FUNCTIONAL","FUNCTIONAL-"&amp;A345,""))</f>
         <v/>
       </c>
     </row>
     <row r="346" ht="15" customHeight="1" s="23">
-      <c r="A346" s="31" t="inlineStr">
+      <c r="A346" s="39" t="inlineStr">
         <is>
           <t>TC-258</t>
         </is>
       </c>
-      <c r="B346" s="31" t="inlineStr">
+      <c r="B346" s="39" t="inlineStr">
         <is>
           <t>NEXTGEN - Profilo, Famiglia: invito via email</t>
         </is>
       </c>
-      <c r="C346" s="31" t="inlineStr">
+      <c r="C346" s="39" t="inlineStr">
         <is>
           <t>Accettare un invito valido (stessa email dell'account loggato) aggiunge l'utente alla famiglia</t>
         </is>
       </c>
-      <c r="D346" s="31" t="inlineStr">
+      <c r="D346" s="39" t="inlineStr">
         <is>
           <t>Un genitore A ha invitato l'email del genitore B (account reale, non l'unico account di test disponibile); NON automatizzabile con un solo account di test</t>
         </is>
       </c>
-      <c r="E346" s="31" t="inlineStr">
+      <c r="E346" s="39" t="inlineStr">
         <is>
           <t>Genitore B apre il link ricevuto via email, arriva su /auth/login?next=/nextgen/planner/famiglia%3Faccept%3DTOKEN, effettua login/registrazione con la STESSA email invitata, vede il prompt 'X ti ha invitato...', clicca 'Accetta l'invito'</t>
         </is>
       </c>
-      <c r="F346" s="31" t="inlineStr">
+      <c r="F346" s="39" t="inlineStr">
         <is>
           <t>Il genitore B diventa membro della famiglia (ruolo 'membro'); l'invito passa a stato 'accepted'; se l'email dell'account non corrisponde a quella invitata, viene mostrato l'errore 'Questo invito e' per un'altra email'. VERIFICARE MANUALMENTE con due account reali prima del rilascio (stessa limitazione già nota di TC-N73..77)</t>
         </is>
       </c>
-      <c r="G346" s="31" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H346" s="31">
+      <c r="G346" s="39" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H346" s="39">
         <f>IF(G346="BUG","BUG-"&amp;A346,IF(G346="FUNCTIONAL","FUNCTIONAL-"&amp;A346,""))</f>
         <v/>
       </c>
-      <c r="L346" s="32" t="inlineStr">
+      <c r="L346" s="40" t="inlineStr">
         <is>
           <t>Verifica manuale richiesta: ambiente di test ha un solo account genitore promosso</t>
         </is>
       </c>
     </row>
     <row r="347" ht="15" customHeight="1" s="23">
-      <c r="A347" s="31" t="inlineStr">
+      <c r="A347" s="39" t="inlineStr">
         <is>
           <t>TC-259</t>
         </is>
       </c>
-      <c r="B347" s="31" t="inlineStr">
+      <c r="B347" s="39" t="inlineStr">
         <is>
           <t>NEXTGEN - Profilo, Famiglia: invito via email</t>
         </is>
       </c>
-      <c r="C347" s="31" t="inlineStr">
+      <c r="C347" s="39" t="inlineStr">
         <is>
           <t>L'invito mostra un link copiabile (WhatsApp, SMS, ecc.), non solo l'invio email automatico</t>
         </is>
       </c>
-      <c r="D347" s="31" t="inlineStr">
+      <c r="D347" s="39" t="inlineStr">
         <is>
           <t>Login genitore, creatore/admin di una famiglia</t>
         </is>
       </c>
-      <c r="E347" s="31" t="inlineStr">
+      <c r="E347" s="39" t="inlineStr">
         <is>
           <t>Invia un invito per email, poi clicca 'Copia link invito (WhatsApp, SMS...)'; ricarica la pagina e clicca 'Copia link' sulla riga dell'invito in 'In attesa di risposta'</t>
         </is>
       </c>
-      <c r="F347" s="31" t="inlineStr">
+      <c r="F347" s="39" t="inlineStr">
         <is>
           <t>In entrambi i casi il link viene copiato negli appunti (toast 'Link copiato!'); il link porta a /auth/login?next=/nextgen/planner/famiglia%3Faccept%3DTOKEN e mostra il prompt di accettazione</t>
         </is>
       </c>
-      <c r="G347" s="31" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H347" s="31">
+      <c r="G347" s="39" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H347" s="39">
         <f>IF(G347="BUG","BUG-"&amp;A347,IF(G347="FUNCTIONAL","FUNCTIONAL-"&amp;A347,""))</f>
         <v/>
       </c>
     </row>
     <row r="348" ht="15" customHeight="1" s="23">
-      <c r="A348" s="31" t="inlineStr">
+      <c r="A348" s="39" t="inlineStr">
         <is>
           <t>TC-260</t>
         </is>
       </c>
-      <c r="B348" s="31" t="inlineStr">
+      <c r="B348" s="39" t="inlineStr">
         <is>
           <t>Branding - Icone da SVG vettoriali</t>
         </is>
       </c>
-      <c r="C348" s="31" t="inlineStr">
+      <c r="C348" s="39" t="inlineStr">
         <is>
           <t>Tutte le icone PWA/favicon/splash/logo inline sono nitide (rigenerate da SVG vettoriali, non piu' da un PNG raster a bassa risoluzione)</t>
         </is>
       </c>
-      <c r="D348" s="31" t="inlineStr">
+      <c r="D348" s="39" t="inlineStr">
         <is>
           <t>Fabrizio ha fornito TRAMA_PWA_SVG_icons.zip (simbolo colorato/navy/bianco-su-navy, viewBox 600x600)</t>
         </is>
       </c>
-      <c r="E348" s="31" t="inlineStr">
+      <c r="E348" s="39" t="inlineStr">
         <is>
           <t>Apri /auth/login (genitore/partner/admin), /nextgen/* (icona inline nell'header), e ispeziona manifest-*.json/icon-*.png/apple-touch-icon*.png/favicon.ico</t>
         </is>
       </c>
-      <c r="F348" s="31" t="inlineStr">
+      <c r="F348" s="39" t="inlineStr">
         <is>
           <t>Icona nitida ad ogni dimensione (192/512/apple-touch/favicon/splash), rispetta la regola di brand (colorata=genitori, navy=gestori/partner, bianca su navy=admin); nessuna sgranatura visibile rispetto al vecchio PNG 345x225</t>
         </is>
       </c>
-      <c r="G348" s="31" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H348" s="31">
+      <c r="G348" s="39" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H348" s="39">
         <f>IF(G348="BUG","BUG-"&amp;A348,IF(G348="FUNCTIONAL","FUNCTIONAL-"&amp;A348,""))</f>
         <v/>
       </c>
-      <c r="L348" s="32" t="inlineStr">
+      <c r="L348" s="40" t="inlineStr">
         <is>
           <t>SVG sorgente salvati in public/brand/svg/ per rigenerazioni future</t>
         </is>
       </c>
     </row>
     <row r="349" ht="15" customHeight="1" s="23">
-      <c r="A349" s="31" t="inlineStr">
+      <c r="A349" s="39" t="inlineStr">
         <is>
           <t>TC-261</t>
         </is>
       </c>
-      <c r="B349" s="31" t="inlineStr">
+      <c r="B349" s="39" t="inlineStr">
         <is>
           <t>Branding - Favicon per-tenant</t>
         </is>
       </c>
-      <c r="C349" s="31" t="inlineStr">
+      <c r="C349" s="39" t="inlineStr">
         <is>
           <t>La favicon nella scheda del browser e' quella corretta per ciascun tenant (colorata=genitori, navy=partner, bianca su navy=admin), non identica per tutti e tre</t>
         </is>
       </c>
-      <c r="D349" s="31" t="inlineStr">
+      <c r="D349" s="39" t="inlineStr">
         <is>
           <t>Nessuna (bug gia' presente nel deploy live, segnalato da Fabrizio con screenshot delle 3 schede browser identiche)</t>
         </is>
       </c>
-      <c r="E349" s="31" t="inlineStr">
+      <c r="E349" s="39" t="inlineStr">
         <is>
           <t>Apri in 3 schede diverse: trama.app/auth/login, partner.trama.app/auth/login, admin.trama.app/auth/login; osserva l'icona nella scheda del browser di ciascuna</t>
         </is>
       </c>
-      <c r="F349" s="31" t="inlineStr">
+      <c r="F349" s="39" t="inlineStr">
         <is>
           <t>Ogni scheda mostra l'icona del proprio tenant (icon-192.png/icon-partner-192.png/icon-admin-192.png), non piu' un'unica favicon.ico generica identica per tutti</t>
         </is>
       </c>
-      <c r="G349" s="31" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H349" s="31">
+      <c r="G349" s="39" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H349" s="39">
         <f>IF(G349="BUG","BUG-"&amp;A349,IF(G349="FUNCTIONAL","FUNCTIONAL-"&amp;A349,""))</f>
         <v/>
       </c>
-      <c r="L349" s="32" t="inlineStr">
+      <c r="L349" s="40" t="inlineStr">
         <is>
           <t>Causa: app/favicon.ico (convenzione statica Next.js, non sensibile all'host) veniva iniettato sempre come primo &lt;link rel=icon&gt;, prima delle icone per-tenant di generateMetadata(). Fix: rimosso app/favicon.ico. Verificato con next build pulito (nessun favicon.ico nell'output) + tsc/eslint puliti. Verifica visiva sulle 3 schede da fare da Fabrizio dopo il deploy.</t>
         </is>
       </c>
     </row>
     <row r="350" ht="15" customHeight="1" s="23">
-      <c r="A350" s="31" t="inlineStr">
+      <c r="A350" s="39" t="inlineStr">
         <is>
           <t>TC-262</t>
         </is>
       </c>
-      <c r="B350" s="31" t="inlineStr">
+      <c r="B350" s="39" t="inlineStr">
         <is>
           <t>Branding - Icone: ripristino disegno precedente</t>
         </is>
       </c>
-      <c r="C350" s="31" t="inlineStr">
+      <c r="C350" s="39" t="inlineStr">
         <is>
           <t>Il simbolo dell'icona (mark) e' quello storico, non il nuovo disegno da SVG (Fabrizio: 'l'icona, proprio il disegno, e' quello sbagliato')</t>
         </is>
       </c>
-      <c r="D350" s="31" t="inlineStr">
+      <c r="D350" s="39" t="inlineStr">
         <is>
           <t>TC-260/TC-261 avevano introdotto un nuovo disegno del mark da TRAMA_PWA_SVG_icons.zip; Fabrizio ha chiesto di ripristinare il disegno precedente pur mantenendo la differenziazione per tenant</t>
         </is>
       </c>
-      <c r="E350" s="31" t="inlineStr">
+      <c r="E350" s="39" t="inlineStr">
         <is>
           <t>Apri /auth/login (genitore/partner/admin) e /nextgen/* (icona inline nell'header); ispeziona icon-192/512.png, icon-{partner,admin,nextgen}-192/512.png, apple-touch-icon*.png, splash screens, trama-logo-mark*.png</t>
         </is>
       </c>
-      <c r="F350" s="31" t="inlineStr">
+      <c r="F350" s="39" t="inlineStr">
         <is>
           <t>Il disegno del mark e' quello storico (pre TRAMA_PWA_SVG_icons.zip), non il nuovo; resta pero' corretta la regola di brand (colorata=genitori, navy=gestori/partner, bianca su navy=admin) e la favicon per-tenant (TC-261, non regredita: app/favicon.ico resta rimosso)</t>
         </is>
       </c>
-      <c r="G350" s="31" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H350" s="31">
+      <c r="G350" s="39" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H350" s="39">
         <f>IF(G350="BUG","BUG-"&amp;A350,IF(G350="FUNCTIONAL","FUNCTIONAL-"&amp;A350,""))</f>
         <v/>
       </c>
-      <c r="L350" s="32" t="inlineStr">
+      <c r="L350" s="40" t="inlineStr">
         <is>
           <t>Ripristinati (git checkout dal commit precedente 43de44f) i 39 PNG toccati dal commit 15ae8ba (icon-*, apple-touch-icon*, brand/trama-logo-mark*, splash/*); NON ripristinato app/favicon.ico (resta cancellato, e' il fix di TC-261). Verificato con next build + tsc puliti.</t>
         </is>
       </c>
     </row>
     <row r="351" ht="15" customHeight="1" s="23">
-      <c r="A351" s="31" t="inlineStr">
+      <c r="A351" s="39" t="inlineStr">
         <is>
           <t>TC-263</t>
         </is>
       </c>
-      <c r="B351" s="31" t="inlineStr">
+      <c r="B351" s="39" t="inlineStr">
         <is>
           <t>NEXTGEN - Planner Organizzazione, sprint correttivo</t>
         </is>
       </c>
-      <c r="C351" s="31" t="inlineStr">
+      <c r="C351" s="39" t="inlineStr">
         <is>
           <t>Badge 'Beta' nell'angolo (ribbon) al posto del pill 'NextGen'</t>
         </is>
       </c>
-      <c r="D351" s="31" t="inlineStr">
+      <c r="D351" s="39" t="inlineStr">
         <is>
           <t>Nessuna</t>
         </is>
       </c>
-      <c r="E351" s="31" t="inlineStr">
+      <c r="E351" s="39" t="inlineStr">
         <is>
           <t>Apri /nextgen/planner (o qualsiasi pagina NEXTGEN)</t>
         </is>
       </c>
-      <c r="F351" s="31" t="inlineStr">
+      <c r="F351" s="39" t="inlineStr">
         <is>
           <t>Nell'angolo in alto a destra compare un ribbon diagonale 'Beta'; il vecchio pill nero 'NextGen' non c'e' piu'</t>
         </is>
       </c>
-      <c r="G351" s="31" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H351" s="31">
+      <c r="G351" s="39" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H351" s="39">
         <f>IF(G351="BUG","BUG-"&amp;A351,IF(G351="FUNCTIONAL","FUNCTIONAL-"&amp;A351,""))</f>
         <v/>
       </c>
     </row>
     <row r="352" ht="15" customHeight="1" s="23">
-      <c r="A352" s="31" t="inlineStr">
+      <c r="A352" s="39" t="inlineStr">
         <is>
           <t>TC-264</t>
         </is>
       </c>
-      <c r="B352" s="31" t="inlineStr">
+      <c r="B352" s="39" t="inlineStr">
         <is>
           <t>NEXTGEN - Planner Organizzazione, sprint correttivo</t>
         </is>
       </c>
-      <c r="C352" s="31" t="inlineStr">
+      <c r="C352" s="39" t="inlineStr">
         <is>
           <t>'Budget impegnato' non e' piu' duplicato nel tab Organizzazione</t>
         </is>
       </c>
-      <c r="D352" s="31" t="inlineStr">
+      <c r="D352" s="39" t="inlineStr">
         <is>
           <t>Nessuna</t>
         </is>
       </c>
-      <c r="E352" s="31" t="inlineStr">
+      <c r="E352" s="39" t="inlineStr">
         <is>
           <t>Apri /nextgen/planner, tab Organizzazione, poi tab Budget</t>
         </is>
       </c>
-      <c r="F352" s="31" t="inlineStr">
+      <c r="F352" s="39" t="inlineStr">
         <is>
           <t>Il tab Organizzazione non mostra piu' la card 'Budget impegnato' (resta solo nel tab Budget dedicato)</t>
         </is>
       </c>
-      <c r="G352" s="31" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H352" s="31">
+      <c r="G352" s="39" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H352" s="39">
         <f>IF(G352="BUG","BUG-"&amp;A352,IF(G352="FUNCTIONAL","FUNCTIONAL-"&amp;A352,""))</f>
         <v/>
       </c>
     </row>
     <row r="353" ht="15" customHeight="1" s="23">
-      <c r="A353" s="31" t="inlineStr">
+      <c r="A353" s="39" t="inlineStr">
         <is>
           <t>TC-265</t>
         </is>
       </c>
-      <c r="B353" s="31" t="inlineStr">
+      <c r="B353" s="39" t="inlineStr">
         <is>
           <t>NEXTGEN - Planner Organizzazione, sprint correttivo</t>
         </is>
       </c>
-      <c r="C353" s="31" t="inlineStr">
+      <c r="C353" s="39" t="inlineStr">
         <is>
           <t>I banner (Promemoria/Missioni) con un'azione mostrano una freccia e portano da qualche parte</t>
         </is>
       </c>
-      <c r="D353" s="31" t="inlineStr">
+      <c r="D353" s="39" t="inlineStr">
         <is>
           <t>Account con almeno un promemoria/missione azionabile</t>
         </is>
       </c>
-      <c r="E353" s="31" t="inlineStr">
+      <c r="E353" s="39" t="inlineStr">
         <is>
           <t>Apri /nextgen/planner, osserva i banner in alto, clicca su uno con la freccia</t>
         </is>
       </c>
-      <c r="F353" s="31" t="inlineStr">
+      <c r="F353" s="39" t="inlineStr">
         <is>
           <t>Il click scorre alla settimana in Timeline, cambia tab (es. Budget) o naviga alla pagina pertinente, senza errori</t>
         </is>
       </c>
-      <c r="G353" s="31" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H353" s="31">
+      <c r="G353" s="39" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H353" s="39">
         <f>IF(G353="BUG","BUG-"&amp;A353,IF(G353="FUNCTIONAL","FUNCTIONAL-"&amp;A353,""))</f>
         <v/>
       </c>
     </row>
     <row r="354" ht="15" customHeight="1" s="23">
-      <c r="A354" s="31" t="inlineStr">
+      <c r="A354" s="39" t="inlineStr">
         <is>
           <t>TC-266</t>
         </is>
       </c>
-      <c r="B354" s="31" t="inlineStr">
+      <c r="B354" s="39" t="inlineStr">
         <is>
           <t>NEXTGEN - Planner Organizzazione, sprint correttivo</t>
         </is>
       </c>
-      <c r="C354" s="31" t="inlineStr">
+      <c r="C354" s="39" t="inlineStr">
         <is>
           <t>Sezione 'Promemoria e avvisi' raggiungibile da Profilo, segnata come anteprima</t>
         </is>
       </c>
-      <c r="D354" s="31" t="inlineStr">
+      <c r="D354" s="39" t="inlineStr">
         <is>
           <t>Nessuna</t>
         </is>
       </c>
-      <c r="E354" s="31" t="inlineStr">
+      <c r="E354" s="39" t="inlineStr">
         <is>
           <t>Profilo -&gt; 'Promemoria e avvisi'</t>
         </is>
       </c>
-      <c r="F354" s="31" t="inlineStr">
+      <c r="F354" s="39" t="inlineStr">
         <is>
           <t>Si apre /nextgen/planner/promemoria con badge 'Anteprima', toggle 'Promemoria attivo' funzionante (stato locale, nessun salvataggio reale dichiarato in UI)</t>
         </is>
       </c>
-      <c r="G354" s="31" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H354" s="31">
+      <c r="G354" s="39" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H354" s="39">
         <f>IF(G354="BUG","BUG-"&amp;A354,IF(G354="FUNCTIONAL","FUNCTIONAL-"&amp;A354,""))</f>
         <v/>
       </c>
     </row>
     <row r="355" ht="15" customHeight="1" s="23">
-      <c r="A355" s="31" t="inlineStr">
+      <c r="A355" s="39" t="inlineStr">
         <is>
           <t>TC-267</t>
         </is>
       </c>
-      <c r="B355" s="31" t="inlineStr">
+      <c r="B355" s="39" t="inlineStr">
         <is>
           <t>NEXTGEN - Prenotazione, check sovrapposizione stesso bambino</t>
         </is>
       </c>
-      <c r="C355" s="31" t="inlineStr">
+      <c r="C355" s="39" t="inlineStr">
         <is>
           <t>Conflitto sullo stesso bambino offre 'Mantieni entrambe' o 'Annulla l'altra e prenota questa' invece del generico 'Prosegui comunque'</t>
         </is>
       </c>
-      <c r="D355" s="31" t="inlineStr">
+      <c r="D355" s="39" t="inlineStr">
         <is>
           <t>Bambino con una prenotazione ATTIVA; nuova prenotazione su un'altra attivita' che copre la stessa settimana per lo stesso bambino</t>
         </is>
       </c>
-      <c r="E355" s="31" t="inlineStr">
+      <c r="E355" s="39" t="inlineStr">
         <is>
           <t>Prova a prenotare la seconda attivita' per la stessa settimana/bambino</t>
         </is>
       </c>
-      <c r="F355" s="31" t="inlineStr">
+      <c r="F355" s="39" t="inlineStr">
         <is>
           <t>Il box 'Attenzione: settimana gia' impegnata' mostra due scelte esplicite: 'Mantieni entrambe' (procede comunque) e 'Annulla l'altra e prenota questa' (annulla la vecchia se ancora nella finestra di cancellazione, poi prenota la nuova; altrimenti mostra l'errore e non prenota)</t>
         </is>
       </c>
-      <c r="G355" s="31" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H355" s="31">
+      <c r="G355" s="39" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H355" s="39">
         <f>IF(G355="BUG","BUG-"&amp;A355,IF(G355="FUNCTIONAL","FUNCTIONAL-"&amp;A355,""))</f>
         <v/>
       </c>
-      <c r="L355" s="32" t="inlineStr">
+      <c r="L355" s="40" t="inlineStr">
         <is>
           <t>Verifica manuale richiesta: serve creare due prenotazioni reali sovrapposte, non fixturabile con l'account di test unico</t>
         </is>
       </c>
     </row>
     <row r="356" ht="15" customHeight="1" s="23">
-      <c r="A356" s="31" t="inlineStr">
+      <c r="A356" s="39" t="inlineStr">
         <is>
           <t>TC-268</t>
         </is>
       </c>
-      <c r="B356" s="31" t="inlineStr">
+      <c r="B356" s="39" t="inlineStr">
         <is>
           <t>NEXTGEN - Planner Organizzazione, bugfix copertura</t>
         </is>
       </c>
-      <c r="C356" s="31" t="inlineStr">
+      <c r="C356" s="39" t="inlineStr">
         <is>
           <t>'X di Y settimane coperte' non supera mai Y anche con una settimana coperta E marcata 'non ti serve'</t>
         </is>
       </c>
-      <c r="D356" s="31" t="inlineStr">
+      <c r="D356" s="39" t="inlineStr">
         <is>
           <t>Una settimana con prenotazione attiva, poi marcata 'non mi serve' senza annullare la prenotazione</t>
         </is>
       </c>
-      <c r="E356" s="31" t="inlineStr">
+      <c r="E356" s="39" t="inlineStr">
         <is>
           <t>Osserva il rapporto 'X di Y settimane coperte' in Organizzazione e il triangolo di sovrapposizione sulla riga Timeline di quella settimana</t>
         </is>
       </c>
-      <c r="F356" s="31" t="inlineStr">
+      <c r="F356" s="39" t="inlineStr">
         <is>
           <t>X non supera mai Y (coveredNeededCount esclude le settimane dismissed anche al numeratore); la riga Timeline mostra 'Non ti serve' senza triangolo, anche se l'overlap resta segnalato nel box 'Sovrapposizioni da controllare' sopra</t>
         </is>
       </c>
-      <c r="G356" s="31" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H356" s="31">
+      <c r="G356" s="39" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H356" s="39">
         <f>IF(G356="BUG","BUG-"&amp;A356,IF(G356="FUNCTIONAL","FUNCTIONAL-"&amp;A356,""))</f>
         <v/>
       </c>
-      <c r="L356" s="32" t="inlineStr">
+      <c r="L356" s="40" t="inlineStr">
         <is>
           <t>Verifica manuale richiesta: scenario limite (dismissed dopo una prenotazione attiva) non riproducibile deterministicamente con l'account di test condiviso</t>
         </is>
@@ -18778,6 +18778,132 @@
         <v/>
       </c>
       <c r="L358" s="40" t="n"/>
+    </row>
+    <row r="359">
+      <c r="A359" s="39" t="inlineStr">
+        <is>
+          <t>TC-271</t>
+        </is>
+      </c>
+      <c r="B359" s="39" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Planner Organizzazione, Sprint 2 (Timeline mensile)</t>
+        </is>
+      </c>
+      <c r="C359" s="39" t="inlineStr">
+        <is>
+          <t>La Timeline della stagione e' raggruppata per mese, pieghevole</t>
+        </is>
+      </c>
+      <c r="D359" s="39" t="inlineStr">
+        <is>
+          <t>Nessuna</t>
+        </is>
+      </c>
+      <c r="E359" s="39" t="inlineStr">
+        <is>
+          <t>Apri /nextgen/planner, scorri fino a 'Timeline della stagione'</t>
+        </is>
+      </c>
+      <c r="F359" s="39" t="inlineStr">
+        <is>
+          <t>Il titolo mostra 'Timeline della stagione — Estiva {anno}'; sotto compaiono intestazioni di mese (es. Giugno, Luglio) pieghevoli con contatore X/Y coperte; il mese con la settimana prioritaria o la prima scoperta e' aperto di default</t>
+        </is>
+      </c>
+      <c r="G359" s="39" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H359" s="39">
+        <f>IF(G359="BUG","BUG-"&amp;A359,IF(G359="FUNCTIONAL","FUNCTIONAL-"&amp;A359,""))</f>
+        <v/>
+      </c>
+      <c r="L359" s="40" t="n"/>
+    </row>
+    <row r="360">
+      <c r="A360" s="39" t="inlineStr">
+        <is>
+          <t>TC-272</t>
+        </is>
+      </c>
+      <c r="B360" s="39" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Planner Organizzazione, Sprint 2 (Timeline mensile)</t>
+        </is>
+      </c>
+      <c r="C360" s="39" t="inlineStr">
+        <is>
+          <t>Cliccando una barra di 'Stato per settimana' si apre il mese giusto, si evidenzia la riga e si vedono le date</t>
+        </is>
+      </c>
+      <c r="D360" s="39" t="inlineStr">
+        <is>
+          <t>Nessuna</t>
+        </is>
+      </c>
+      <c r="E360" s="39" t="inlineStr">
+        <is>
+          <t>Apri /nextgen/planner, clicca una barra della striscia 'Stato per settimana'</t>
+        </is>
+      </c>
+      <c r="F360" s="39" t="inlineStr">
+        <is>
+          <t>Il mese che contiene quella settimana si apre automaticamente (se era chiuso); la riga corrispondente nella Timeline scorre in vista ed e' evidenziata con un anello viola per ~1.6s; accanto al titolo 'Stato per settimana' compare 'Settimana N · date' per la stessa durata</t>
+        </is>
+      </c>
+      <c r="G360" s="39" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H360" s="39">
+        <f>IF(G360="BUG","BUG-"&amp;A360,IF(G360="FUNCTIONAL","FUNCTIONAL-"&amp;A360,""))</f>
+        <v/>
+      </c>
+      <c r="L360" s="40" t="n"/>
+    </row>
+    <row r="361">
+      <c r="A361" s="39" t="inlineStr">
+        <is>
+          <t>TC-273</t>
+        </is>
+      </c>
+      <c r="B361" s="39" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Planner Organizzazione, Sprint 2 (Timeline mensile)</t>
+        </is>
+      </c>
+      <c r="C361" s="39" t="inlineStr">
+        <is>
+          <t>Una riga Timeline con attivita' reale (slug) e' cliccabile e apre la scheda attivita'</t>
+        </is>
+      </c>
+      <c r="D361" s="39" t="inlineStr">
+        <is>
+          <t>Almeno una settimana coperta da una prenotazione con attivita' reale (slug)</t>
+        </is>
+      </c>
+      <c r="E361" s="39" t="inlineStr">
+        <is>
+          <t>Apri /nextgen/planner, espandi il mese con una settimana coperta, clicca sulla riga</t>
+        </is>
+      </c>
+      <c r="F361" s="39" t="inlineStr">
+        <is>
+          <t>La riga ha feedback hover/active (stesso pattern di components/PlannerView.tsx LEGACY) e una freccina; il click apre /activity/{slug} senza errori. L'icona di stato (spunta verde o triangolo sovrapposizione) resta visibile accanto alla freccina, non sostituita</t>
+        </is>
+      </c>
+      <c r="G361" s="39" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H361" s="39">
+        <f>IF(G361="BUG","BUG-"&amp;A361,IF(G361="FUNCTIONAL","FUNCTIONAL-"&amp;A361,""))</f>
+        <v/>
+      </c>
+      <c r="L361" s="40" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L101"/>

</xml_diff>

<commit_message>
Profilo: consolidare Famiglia e Impostazioni dietro un solo hub card ciascuno
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -913,7 +913,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L361"/>
+  <dimension ref="A1:L365"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11.83" customWidth="1" style="39" min="1" max="1"/>
@@ -18904,6 +18904,174 @@
         <v/>
       </c>
       <c r="L361" s="40" t="n"/>
+    </row>
+    <row r="362">
+      <c r="A362" s="39" t="inlineStr">
+        <is>
+          <t>TC-274</t>
+        </is>
+      </c>
+      <c r="B362" s="39" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Profilo, consolidamento hub card</t>
+        </is>
+      </c>
+      <c r="C362" s="39" t="inlineStr">
+        <is>
+          <t>La sezione 'Famiglia' in Profilo mostra un solo ingresso 'Famiglia e logistica' invece di 4 righe</t>
+        </is>
+      </c>
+      <c r="D362" s="39" t="inlineStr">
+        <is>
+          <t>Nessuna</t>
+        </is>
+      </c>
+      <c r="E362" s="39" t="inlineStr">
+        <is>
+          <t>Apri /nextgen/profile, guarda la sezione 'Famiglia'</t>
+        </is>
+      </c>
+      <c r="F362" s="39" t="inlineStr">
+        <is>
+          <t>Sotto l'header 'Famiglia' compare una sola card 'Famiglia e logistica' (sottotitolo 'Indirizzi, condivisione piano, promemoria'); cliccandola si apre /nextgen/profile/famiglia con le 4 card originali (Indirizzi di famiglia, Famiglia, Condivisione piano, Promemoria e avvisi), link invariati</t>
+        </is>
+      </c>
+      <c r="G362" s="39" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H362" s="39">
+        <f>IF(G362="BUG","BUG-"&amp;A362,IF(G362="FUNCTIONAL","FUNCTIONAL-"&amp;A362,""))</f>
+        <v/>
+      </c>
+      <c r="L362" s="40" t="n"/>
+    </row>
+    <row r="363">
+      <c r="A363" s="39" t="inlineStr">
+        <is>
+          <t>TC-275</t>
+        </is>
+      </c>
+      <c r="B363" s="39" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Profilo, consolidamento hub card</t>
+        </is>
+      </c>
+      <c r="C363" s="39" t="inlineStr">
+        <is>
+          <t>La sezione 'Impostazioni' in Profilo mostra un solo ingresso 'Impostazioni' invece di 4 righe</t>
+        </is>
+      </c>
+      <c r="D363" s="39" t="inlineStr">
+        <is>
+          <t>Nessuna</t>
+        </is>
+      </c>
+      <c r="E363" s="39" t="inlineStr">
+        <is>
+          <t>Apri /nextgen/profile, guarda la sezione 'Impostazioni'</t>
+        </is>
+      </c>
+      <c r="F363" s="39" t="inlineStr">
+        <is>
+          <t>Sotto l'header 'Impostazioni' compare una sola card 'Impostazioni' (sottotitolo 'Sicurezza, preferenze, privacy'); cliccandola si apre /nextgen/profile/impostazioni con le 4 card originali (Sicurezza, Preferenze, Metodi di pagamento, Privacy e account), link invariati</t>
+        </is>
+      </c>
+      <c r="G363" s="39" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H363" s="39">
+        <f>IF(G363="BUG","BUG-"&amp;A363,IF(G363="FUNCTIONAL","FUNCTIONAL-"&amp;A363,""))</f>
+        <v/>
+      </c>
+      <c r="L363" s="40" t="n"/>
+    </row>
+    <row r="364">
+      <c r="A364" s="39" t="inlineStr">
+        <is>
+          <t>TC-276</t>
+        </is>
+      </c>
+      <c r="B364" s="39" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Profilo, consolidamento hub card</t>
+        </is>
+      </c>
+      <c r="C364" s="39" t="inlineStr">
+        <is>
+          <t>Il tasto 'Indietro' dalle pagine dentro 'Famiglia e logistica' torna all'hub, non direttamente al Profilo</t>
+        </is>
+      </c>
+      <c r="D364" s="39" t="inlineStr">
+        <is>
+          <t>Nessuna</t>
+        </is>
+      </c>
+      <c r="E364" s="39" t="inlineStr">
+        <is>
+          <t>Profilo -&gt; Famiglia e logistica -&gt; Indirizzi di famiglia -&gt; Indietro</t>
+        </is>
+      </c>
+      <c r="F364" s="39" t="inlineStr">
+        <is>
+          <t>Il tasto Indietro riporta a /nextgen/profile/famiglia (l'hub), non a /nextgen/profile direttamente; stesso comportamento per 'Famiglia' (invito) e 'Promemoria e avvisi'</t>
+        </is>
+      </c>
+      <c r="G364" s="39" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H364" s="39">
+        <f>IF(G364="BUG","BUG-"&amp;A364,IF(G364="FUNCTIONAL","FUNCTIONAL-"&amp;A364,""))</f>
+        <v/>
+      </c>
+      <c r="L364" s="40" t="n"/>
+    </row>
+    <row r="365">
+      <c r="A365" s="39" t="inlineStr">
+        <is>
+          <t>TC-277</t>
+        </is>
+      </c>
+      <c r="B365" s="39" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Profilo, consolidamento hub card</t>
+        </is>
+      </c>
+      <c r="C365" s="39" t="inlineStr">
+        <is>
+          <t>Le sezioni 'Attività' e 'Supporto' in Profilo restano invariate (non consolidate)</t>
+        </is>
+      </c>
+      <c r="D365" s="39" t="inlineStr">
+        <is>
+          <t>Nessuna</t>
+        </is>
+      </c>
+      <c r="E365" s="39" t="inlineStr">
+        <is>
+          <t>Apri /nextgen/profile, guarda le sezioni 'Attività' e 'Supporto'</t>
+        </is>
+      </c>
+      <c r="F365" s="39" t="inlineStr">
+        <is>
+          <t>'Attività' mostra ancora 3 righe separate (Le mie prenotazioni, Preferiti, Le presenze); 'Supporto' mostra ancora 2 righe separate (Le mie richieste, Ricevute e fatture) — non sono impostazioni 'una tantum' come Famiglia/Impostazioni, quindi restano con la stessa prominenza di prima</t>
+        </is>
+      </c>
+      <c r="G365" s="39" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H365" s="39">
+        <f>IF(G365="BUG","BUG-"&amp;A365,IF(G365="FUNCTIONAL","FUNCTIONAL-"&amp;A365,""))</f>
+        <v/>
+      </c>
+      <c r="L365" s="40" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L101"/>

</xml_diff>

<commit_message>
Sprint 3 Scopri: filtro bambino unificato, Azzera condizionale, settimane multi-select raggruppate, badge Nessuna limitazione viola
- Filtro bambino spostato dentro la riga scorrevole dei filtri (non più blocco separato)
- 'Azzera' smontato dal DOM a zero filtri attivi (prima solo disabled)
- Filtro settimana: multi-selezione con raggruppamento mese, chip 'Settimane (N)'
- computeSmartMatches: reason 'Piacciono ai tuoi figli' quando 2+ figli superano soglia match
- Badge 'Accesso disabili' rinominato 'Nessuna limitazione', colore viola (distinto da Certificazione blu)
- Test Playwright aggiornati/aggiunti (TC-N85, TC-N103, TC-278..281 in xlsx)
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -913,7 +913,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L365"/>
+  <dimension ref="A1:L369"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11.83" customWidth="1" style="39" min="1" max="1"/>
@@ -19072,6 +19072,170 @@
         <v/>
       </c>
       <c r="L365" s="40" t="n"/>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>TC-278</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Scopri Sprint 3 (filtri unificati)</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Il filtro bambino vive nella stessa riga scorrevole dei 6 filtri, non in un blocco separato</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>Almeno un figlio in profilo</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>Apri /nextgen/search</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>Il pill del bambino e' il primo elemento della riga scorrevole (no-scrollbar overflow-x-auto), seguito da un divider verticale e poi dai 6 filtri (Prezzo/Servizi/Tipo attivita/Data/Zona/Eta); non c'e' piu' un blocco pill separato sopra la riga</t>
+        </is>
+      </c>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H366">
+        <f>IF(G366="BUG","BUG-"&amp;A366,IF(G366="FUNCTIONAL","FUNCTIONAL-"&amp;A366,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>TC-279</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Scopri Sprint 3 (Azzera)</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>'Azzera' non e' presente nel DOM quando nessun filtro e' attivo (non solo disabilitato)</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>Nessun filtro attivo all'apertura</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>Apri /nextgen/search, verifica assenza del pulsante 'Azzera'; applica un filtro (es. Prezzo); verifica comparsa; clicca 'Azzera'</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>A filtri azzerati il pulsante 'Azzera' non esiste nel DOM (prima era presente ma disabled); applicando un filtro compare con il conteggio; cliccandolo sparisce di nuovo dal DOM</t>
+        </is>
+      </c>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H367">
+        <f>IF(G367="BUG","BUG-"&amp;A367,IF(G367="FUNCTIONAL","FUNCTIONAL-"&amp;A367,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>TC-280</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Scopri Sprint 3 (raggruppamento match)</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Quando 2+ bambini superano la soglia di match (&gt;=40%), il reason mostra 'Piacciono ai tuoi figli' invece di ripetere 'Piace a X' per ciascuno</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>Almeno 2 figli in profilo con interessi che matchano la stessa attivita' oltre la soglia</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>Apri /nextgen/search con un profilo che ha 2+ figli compatibili con una stessa attivita'</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>Sulla card dell'attivita' compare un'unica pill 'Piacciono ai tuoi figli' invece di due pill separate 'Piace a X'/'Piace a Y'; con un solo figlio compatibile resta 'Piace a X'</t>
+        </is>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>FIXME (dati demo account condiviso non permettono di fixturare in modo affidabile 2+ figli con match &gt;=40% sulla stessa attivita')</t>
+        </is>
+      </c>
+      <c r="H368">
+        <f>IF(G368="BUG","BUG-"&amp;A368,IF(G368="FUNCTIONAL","FUNCTIONAL-"&amp;A368,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>TC-281</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Scopri Sprint 3 (badge restyle)</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Il badge 'Nessuna limitazione' (ex 'Accesso disabili') e' viola, distinto dal blu della Certificazione</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>Un'attivita' con centerAccessible=true e certificationBadges non vuoto</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>Apri /nextgen/search, filtra per Servizi -&gt; 'Nessuna limitazione', osserva i badge sulla card risultato</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>Il badge mostra il testo 'Nessuna limitazione' (non piu' 'Accesso disabili') con icona ti-heart-handshake e colore viola (token purple/purple-light); il badge Certificazione sulla stessa card resta blu (token sky/sky-light), chiaramente distinguibile</t>
+        </is>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H369">
+        <f>IF(G369="BUG","BUG-"&amp;A369,IF(G369="FUNCTIONAL","FUNCTIONAL-"&amp;A369,""))</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:L101"/>

</xml_diff>

<commit_message>
Fix correttivi Sprint 3 Scopri: filtro Bambini come pannello, divider risultati, wording match singolare
- Filtro bambino non più pill inline: pannello 'Bambini' a comparsa come Tipo attività/Servizi, scala a qualunque numero di figli
- Divider leggero mostrato solo quando un pannello filtro è aperto, prima di 'X attività trovate'/Lista-Mappa
- computeSmartMatches: 'Piace ai tuoi figli' (singolare) invece di 'Piacciono' — la label è per singola attività
- Test aggiornati/aggiunti (TC-N278 riscritto, TC-N282 nuovo), xlsx TC-282
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -913,7 +913,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L369"/>
+  <dimension ref="A1:L370"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11.83" customWidth="1" style="39" min="1" max="1"/>
@@ -19074,166 +19074,207 @@
       <c r="L365" s="40" t="n"/>
     </row>
     <row r="366">
-      <c r="A366" t="inlineStr">
+      <c r="A366" s="22" t="inlineStr">
         <is>
           <t>TC-278</t>
         </is>
       </c>
-      <c r="B366" t="inlineStr">
+      <c r="B366" s="22" t="inlineStr">
         <is>
           <t>NEXTGEN - Scopri Sprint 3 (filtri unificati)</t>
         </is>
       </c>
-      <c r="C366" t="inlineStr">
-        <is>
-          <t>Il filtro bambino vive nella stessa riga scorrevole dei 6 filtri, non in un blocco separato</t>
-        </is>
-      </c>
-      <c r="D366" t="inlineStr">
-        <is>
-          <t>Almeno un figlio in profilo</t>
-        </is>
-      </c>
-      <c r="E366" t="inlineStr">
-        <is>
-          <t>Apri /nextgen/search</t>
-        </is>
-      </c>
-      <c r="F366" t="inlineStr">
-        <is>
-          <t>Il pill del bambino e' il primo elemento della riga scorrevole (no-scrollbar overflow-x-auto), seguito da un divider verticale e poi dai 6 filtri (Prezzo/Servizi/Tipo attivita/Data/Zona/Eta); non c'e' piu' un blocco pill separato sopra la riga</t>
-        </is>
-      </c>
-      <c r="G366" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H366">
+      <c r="C366" s="22" t="inlineStr">
+        <is>
+          <t>Il filtro 'Bambini' e' un pannello a comparsa (come Tipo attivita'/Servizi), non piu' pill inline</t>
+        </is>
+      </c>
+      <c r="D366" s="22" t="inlineStr">
+        <is>
+          <t>2+ figli in profilo</t>
+        </is>
+      </c>
+      <c r="E366" s="22" t="inlineStr">
+        <is>
+          <t>Apri /nextgen/search, guarda la riga filtri scorrevole</t>
+        </is>
+      </c>
+      <c r="F366" s="22" t="inlineStr">
+        <is>
+          <t>Il primo elemento della riga e' un chip 'Bambini' (non piu' un pulsante per ciascun figlio); aprendolo si vede un pannello con 'Tutti i bambini' + un pulsante per figlio; selezionandone uno il chip diventa 'Bambini (Nome)'. Con un solo figlio in profilo il chip non compare (comportamento invariato).</t>
+        </is>
+      </c>
+      <c r="G366" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H366" s="22">
         <f>IF(G366="BUG","BUG-"&amp;A366,IF(G366="FUNCTIONAL","FUNCTIONAL-"&amp;A366,""))</f>
         <v/>
       </c>
     </row>
     <row r="367">
-      <c r="A367" t="inlineStr">
+      <c r="A367" s="22" t="inlineStr">
         <is>
           <t>TC-279</t>
         </is>
       </c>
-      <c r="B367" t="inlineStr">
+      <c r="B367" s="22" t="inlineStr">
         <is>
           <t>NEXTGEN - Scopri Sprint 3 (Azzera)</t>
         </is>
       </c>
-      <c r="C367" t="inlineStr">
+      <c r="C367" s="22" t="inlineStr">
         <is>
           <t>'Azzera' non e' presente nel DOM quando nessun filtro e' attivo (non solo disabilitato)</t>
         </is>
       </c>
-      <c r="D367" t="inlineStr">
+      <c r="D367" s="22" t="inlineStr">
         <is>
           <t>Nessun filtro attivo all'apertura</t>
         </is>
       </c>
-      <c r="E367" t="inlineStr">
+      <c r="E367" s="22" t="inlineStr">
         <is>
           <t>Apri /nextgen/search, verifica assenza del pulsante 'Azzera'; applica un filtro (es. Prezzo); verifica comparsa; clicca 'Azzera'</t>
         </is>
       </c>
-      <c r="F367" t="inlineStr">
+      <c r="F367" s="22" t="inlineStr">
         <is>
           <t>A filtri azzerati il pulsante 'Azzera' non esiste nel DOM (prima era presente ma disabled); applicando un filtro compare con il conteggio; cliccandolo sparisce di nuovo dal DOM</t>
         </is>
       </c>
-      <c r="G367" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H367">
+      <c r="G367" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H367" s="22">
         <f>IF(G367="BUG","BUG-"&amp;A367,IF(G367="FUNCTIONAL","FUNCTIONAL-"&amp;A367,""))</f>
         <v/>
       </c>
     </row>
     <row r="368">
-      <c r="A368" t="inlineStr">
+      <c r="A368" s="22" t="inlineStr">
         <is>
           <t>TC-280</t>
         </is>
       </c>
-      <c r="B368" t="inlineStr">
+      <c r="B368" s="22" t="inlineStr">
         <is>
           <t>NEXTGEN - Scopri Sprint 3 (raggruppamento match)</t>
         </is>
       </c>
-      <c r="C368" t="inlineStr">
-        <is>
-          <t>Quando 2+ bambini superano la soglia di match (&gt;=40%), il reason mostra 'Piacciono ai tuoi figli' invece di ripetere 'Piace a X' per ciascuno</t>
-        </is>
-      </c>
-      <c r="D368" t="inlineStr">
+      <c r="C368" s="22" t="inlineStr">
+        <is>
+          <t>Quando 2+ bambini superano la soglia di match (&gt;=40%), il reason mostra 'Piace ai tuoi figli' (singolare) invece di ripetere 'Piace a X' per ciascuno</t>
+        </is>
+      </c>
+      <c r="D368" s="22" t="inlineStr">
         <is>
           <t>Almeno 2 figli in profilo con interessi che matchano la stessa attivita' oltre la soglia</t>
         </is>
       </c>
-      <c r="E368" t="inlineStr">
+      <c r="E368" s="22" t="inlineStr">
         <is>
           <t>Apri /nextgen/search con un profilo che ha 2+ figli compatibili con una stessa attivita'</t>
         </is>
       </c>
-      <c r="F368" t="inlineStr">
-        <is>
-          <t>Sulla card dell'attivita' compare un'unica pill 'Piacciono ai tuoi figli' invece di due pill separate 'Piace a X'/'Piace a Y'; con un solo figlio compatibile resta 'Piace a X'</t>
-        </is>
-      </c>
-      <c r="G368" t="inlineStr">
+      <c r="F368" s="22" t="inlineStr">
+        <is>
+          <t>Sulla card dell'attivita' compare un'unica pill 'Piace ai tuoi figli' (verbo singolare, coerente col fatto che la label si riferisce a UNA attivita', non a un gruppo) invece di due pill separate 'Piace a X'/'Piace a Y'; con un solo figlio compatibile resta 'Piace a X'</t>
+        </is>
+      </c>
+      <c r="G368" s="22" t="inlineStr">
         <is>
           <t>FIXME (dati demo account condiviso non permettono di fixturare in modo affidabile 2+ figli con match &gt;=40% sulla stessa attivita')</t>
         </is>
       </c>
-      <c r="H368">
+      <c r="H368" s="22">
         <f>IF(G368="BUG","BUG-"&amp;A368,IF(G368="FUNCTIONAL","FUNCTIONAL-"&amp;A368,""))</f>
         <v/>
       </c>
     </row>
     <row r="369">
-      <c r="A369" t="inlineStr">
+      <c r="A369" s="22" t="inlineStr">
         <is>
           <t>TC-281</t>
         </is>
       </c>
-      <c r="B369" t="inlineStr">
+      <c r="B369" s="22" t="inlineStr">
         <is>
           <t>NEXTGEN - Scopri Sprint 3 (badge restyle)</t>
         </is>
       </c>
-      <c r="C369" t="inlineStr">
+      <c r="C369" s="22" t="inlineStr">
         <is>
           <t>Il badge 'Nessuna limitazione' (ex 'Accesso disabili') e' viola, distinto dal blu della Certificazione</t>
         </is>
       </c>
-      <c r="D369" t="inlineStr">
+      <c r="D369" s="22" t="inlineStr">
         <is>
           <t>Un'attivita' con centerAccessible=true e certificationBadges non vuoto</t>
         </is>
       </c>
-      <c r="E369" t="inlineStr">
+      <c r="E369" s="22" t="inlineStr">
         <is>
           <t>Apri /nextgen/search, filtra per Servizi -&gt; 'Nessuna limitazione', osserva i badge sulla card risultato</t>
         </is>
       </c>
-      <c r="F369" t="inlineStr">
+      <c r="F369" s="22" t="inlineStr">
         <is>
           <t>Il badge mostra il testo 'Nessuna limitazione' (non piu' 'Accesso disabili') con icona ti-heart-handshake e colore viola (token purple/purple-light); il badge Certificazione sulla stessa card resta blu (token sky/sky-light), chiaramente distinguibile</t>
         </is>
       </c>
-      <c r="G369" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H369">
+      <c r="G369" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H369" s="22">
         <f>IF(G369="BUG","BUG-"&amp;A369,IF(G369="FUNCTIONAL","FUNCTIONAL-"&amp;A369,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>TC-282</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Scopri Sprint 3 correttivo (divider)</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Un divider leggero separa il pannello filtro aperto dalla riga risultati/Lista-Mappa</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>Nessuna</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>Apri /nextgen/search, apri un pannello filtro (es. Prezzo)</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>A pannello chiuso non c'e' alcun divider; aprendo un pannello compare una linea sottile (border-t leggero) subito sopra 'X attivita' trovate' e il toggle Lista/Mappa, per separare visivamente l'area di selezione dai risultati; richiudendo il pannello il divider sparisce</t>
+        </is>
+      </c>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H370">
+        <f>IF(G370="BUG","BUG-"&amp;A370,IF(G370="FUNCTIONAL","FUNCTIONAL-"&amp;A370,""))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Sprint 4: fix redirect Logistica, indirizzi con nome personalizzabile per ogni kind, selettore origine in Mappa
- /nextgen/planner/logistica ora reindirizza a /nextgen/profile/famiglia (non più un hop corto dopo la consolidazione Profilo)
- Indirizzi: il campo 'nome personalizzato' non è più riservato al kind 'altro', disponibile per Casa/Lavoro Genitore 1/Lavoro Genitore 2 (default all'etichetta fissa se vuoto)
- PromemoriaClient: originLabel aggiornato per usare il nome personalizzato su qualunque kind
- PlannerMapView: nuovo selettore 'Parti da' (stesso pattern di Promemoria) — 'Avvia navigazione' costruisce un link di itinerario (origin+destination) invece di solo destinazione, quando c'è almeno un indirizzo salvato
- Test Playwright aggiornati/aggiunti (TC-N111, TC-N283, TC-N284), xlsx TC-283..285
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -913,7 +913,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L370"/>
+  <dimension ref="A1:L373"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11.83" customWidth="1" style="39" min="1" max="1"/>
@@ -19238,43 +19238,166 @@
       </c>
     </row>
     <row r="370">
-      <c r="A370" t="inlineStr">
+      <c r="A370" s="22" t="inlineStr">
         <is>
           <t>TC-282</t>
         </is>
       </c>
-      <c r="B370" t="inlineStr">
+      <c r="B370" s="22" t="inlineStr">
         <is>
           <t>NEXTGEN - Scopri Sprint 3 correttivo (divider)</t>
         </is>
       </c>
-      <c r="C370" t="inlineStr">
+      <c r="C370" s="22" t="inlineStr">
         <is>
           <t>Un divider leggero separa il pannello filtro aperto dalla riga risultati/Lista-Mappa</t>
         </is>
       </c>
-      <c r="D370" t="inlineStr">
+      <c r="D370" s="22" t="inlineStr">
         <is>
           <t>Nessuna</t>
         </is>
       </c>
-      <c r="E370" t="inlineStr">
+      <c r="E370" s="22" t="inlineStr">
         <is>
           <t>Apri /nextgen/search, apri un pannello filtro (es. Prezzo)</t>
         </is>
       </c>
-      <c r="F370" t="inlineStr">
+      <c r="F370" s="22" t="inlineStr">
         <is>
           <t>A pannello chiuso non c'e' alcun divider; aprendo un pannello compare una linea sottile (border-t leggero) subito sopra 'X attivita' trovate' e il toggle Lista/Mappa, per separare visivamente l'area di selezione dai risultati; richiudendo il pannello il divider sparisce</t>
         </is>
       </c>
-      <c r="G370" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H370">
+      <c r="G370" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H370" s="22">
         <f>IF(G370="BUG","BUG-"&amp;A370,IF(G370="FUNCTIONAL","FUNCTIONAL-"&amp;A370,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>TC-283</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Sprint 4 correttivo (audit link)</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>/nextgen/planner/logistica reindirizza a /nextgen/profile/famiglia (non un hop corto)</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>Nessuna</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>Vai su /nextgen/planner/logistica (vecchio bookmark)</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>Redirect a /nextgen/profile/famiglia (l'hub attuale con Indirizzi/Famiglia/Condivisione/Promemoria), non piu' a /nextgen/profile generico — prima del fix l'utente si fermava un click prima della destinazione dopo la consolidazione Profilo (task #236)</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H371">
+        <f>IF(G371="BUG","BUG-"&amp;A371,IF(G371="FUNCTIONAL","FUNCTIONAL-"&amp;A371,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>TC-284</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Sprint 4 correttivo (indirizzi personalizzabili)</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Un indirizzo a kind fisso (Casa/Lavoro Genitore 1/Lavoro Genitore 2) puo' avere un nome personalizzato</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>Nessuna</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>Apri /nextgen/planner/indirizzi, modifica la card 'Casa', compila il campo 'Nome personalizzato' con un nome a piacere e salva</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>Il titolo della card mostra il nome personalizzato al posto dell'etichetta fissa 'Casa'; lo stesso nome compare anche nel selettore 'Da dove parti?' di Promemoria e nel selettore 'Parti da' della Vista Mappa (originLabel aggiornato in entrambi); lasciando il campo vuoto la card torna a mostrare l'etichetta di default</t>
+        </is>
+      </c>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H372">
+        <f>IF(G372="BUG","BUG-"&amp;A372,IF(G372="FUNCTIONAL","FUNCTIONAL-"&amp;A372,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>TC-285</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Sprint 4 correttivo (selettore origine Mappa)</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Vista Mappa: con indirizzi salvati, 'Parti da' costruisce un link di itinerario invece di solo destinazione</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>Almeno un indirizzo di famiglia salvato + un'attivita' prenotata con indirizzo</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>Apri /nextgen/planner -&gt; Mappa, seleziona un'attivita' con indirizzo</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>Compare il selettore 'Parti da' con gli indirizzi salvati (default 'Casa' se presente); 'Avvia navigazione' apre un link Google Maps di TIPO ITINERARIO (maps/dir/?api=1&amp;origin=...&amp;destination=...) invece della semplice ricerca della destinazione; senza indirizzi salvati il comportamento resta quello precedente (solo destinazione)</t>
+        </is>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H373">
+        <f>IF(G373="BUG","BUG-"&amp;A373,IF(G373="FUNCTIONAL","FUNCTIONAL-"&amp;A373,""))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Sprint 5 NEXTGEN: floating CTA 'Segnala un problema' (BETA) + coda Admin + sezione genitore temporanea
- Schema beta_feedback (parent_id, app_source genitori/gestore, area, page_path, message, status nuovo/in_gestione/risolto, admin_note) + RLS
- BetaFeedbackButton: CTA draggabile (posizione persistita in localStorage) montata una sola volta in app/nextgen/layout.tsx, copre ogni pagina genitore NEXTGEN; nascosta su /nextgen/admin e /nextgen/center (placeholder Sprint 0, fuori scope)
- area calcolata client-side da pathname (lib/nextgen/beta-feedback-areas.ts), nessun enum rigido lato DB
- Profilo > Beta > 'Le mie segnalazioni': sezione temporanea sola lettura per seguire lo stato delle proprie segnalazioni
- Admin > Segnalazioni BETA: coda con report (totale/per stato/per area), filtri, cambio stato, label 'App genitori'/'App gestori' (solo genitori popolato per ora, schema già pronto per l'app gestori)
- Test Playwright (TC-N286..291), xlsx TC-286..291
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -913,7 +913,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L373"/>
+  <dimension ref="A1:L379"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11.83" customWidth="1" style="39" min="1" max="1"/>
@@ -19279,125 +19279,371 @@
       </c>
     </row>
     <row r="371">
-      <c r="A371" t="inlineStr">
+      <c r="A371" s="22" t="inlineStr">
         <is>
           <t>TC-283</t>
         </is>
       </c>
-      <c r="B371" t="inlineStr">
+      <c r="B371" s="22" t="inlineStr">
         <is>
           <t>NEXTGEN - Sprint 4 correttivo (audit link)</t>
         </is>
       </c>
-      <c r="C371" t="inlineStr">
+      <c r="C371" s="22" t="inlineStr">
         <is>
           <t>/nextgen/planner/logistica reindirizza a /nextgen/profile/famiglia (non un hop corto)</t>
         </is>
       </c>
-      <c r="D371" t="inlineStr">
+      <c r="D371" s="22" t="inlineStr">
         <is>
           <t>Nessuna</t>
         </is>
       </c>
-      <c r="E371" t="inlineStr">
+      <c r="E371" s="22" t="inlineStr">
         <is>
           <t>Vai su /nextgen/planner/logistica (vecchio bookmark)</t>
         </is>
       </c>
-      <c r="F371" t="inlineStr">
+      <c r="F371" s="22" t="inlineStr">
         <is>
           <t>Redirect a /nextgen/profile/famiglia (l'hub attuale con Indirizzi/Famiglia/Condivisione/Promemoria), non piu' a /nextgen/profile generico — prima del fix l'utente si fermava un click prima della destinazione dopo la consolidazione Profilo (task #236)</t>
         </is>
       </c>
-      <c r="G371" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H371">
+      <c r="G371" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H371" s="22">
         <f>IF(G371="BUG","BUG-"&amp;A371,IF(G371="FUNCTIONAL","FUNCTIONAL-"&amp;A371,""))</f>
         <v/>
       </c>
     </row>
     <row r="372">
-      <c r="A372" t="inlineStr">
+      <c r="A372" s="22" t="inlineStr">
         <is>
           <t>TC-284</t>
         </is>
       </c>
-      <c r="B372" t="inlineStr">
+      <c r="B372" s="22" t="inlineStr">
         <is>
           <t>NEXTGEN - Sprint 4 correttivo (indirizzi personalizzabili)</t>
         </is>
       </c>
-      <c r="C372" t="inlineStr">
+      <c r="C372" s="22" t="inlineStr">
         <is>
           <t>Un indirizzo a kind fisso (Casa/Lavoro Genitore 1/Lavoro Genitore 2) puo' avere un nome personalizzato</t>
         </is>
       </c>
-      <c r="D372" t="inlineStr">
+      <c r="D372" s="22" t="inlineStr">
         <is>
           <t>Nessuna</t>
         </is>
       </c>
-      <c r="E372" t="inlineStr">
+      <c r="E372" s="22" t="inlineStr">
         <is>
           <t>Apri /nextgen/planner/indirizzi, modifica la card 'Casa', compila il campo 'Nome personalizzato' con un nome a piacere e salva</t>
         </is>
       </c>
-      <c r="F372" t="inlineStr">
+      <c r="F372" s="22" t="inlineStr">
         <is>
           <t>Il titolo della card mostra il nome personalizzato al posto dell'etichetta fissa 'Casa'; lo stesso nome compare anche nel selettore 'Da dove parti?' di Promemoria e nel selettore 'Parti da' della Vista Mappa (originLabel aggiornato in entrambi); lasciando il campo vuoto la card torna a mostrare l'etichetta di default</t>
         </is>
       </c>
-      <c r="G372" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H372">
+      <c r="G372" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H372" s="22">
         <f>IF(G372="BUG","BUG-"&amp;A372,IF(G372="FUNCTIONAL","FUNCTIONAL-"&amp;A372,""))</f>
         <v/>
       </c>
     </row>
     <row r="373">
-      <c r="A373" t="inlineStr">
+      <c r="A373" s="22" t="inlineStr">
         <is>
           <t>TC-285</t>
         </is>
       </c>
-      <c r="B373" t="inlineStr">
+      <c r="B373" s="22" t="inlineStr">
         <is>
           <t>NEXTGEN - Sprint 4 correttivo (selettore origine Mappa)</t>
         </is>
       </c>
-      <c r="C373" t="inlineStr">
+      <c r="C373" s="22" t="inlineStr">
         <is>
           <t>Vista Mappa: con indirizzi salvati, 'Parti da' costruisce un link di itinerario invece di solo destinazione</t>
         </is>
       </c>
-      <c r="D373" t="inlineStr">
+      <c r="D373" s="22" t="inlineStr">
         <is>
           <t>Almeno un indirizzo di famiglia salvato + un'attivita' prenotata con indirizzo</t>
         </is>
       </c>
-      <c r="E373" t="inlineStr">
+      <c r="E373" s="22" t="inlineStr">
         <is>
           <t>Apri /nextgen/planner -&gt; Mappa, seleziona un'attivita' con indirizzo</t>
         </is>
       </c>
-      <c r="F373" t="inlineStr">
+      <c r="F373" s="22" t="inlineStr">
         <is>
           <t>Compare il selettore 'Parti da' con gli indirizzi salvati (default 'Casa' se presente); 'Avvia navigazione' apre un link Google Maps di TIPO ITINERARIO (maps/dir/?api=1&amp;origin=...&amp;destination=...) invece della semplice ricerca della destinazione; senza indirizzi salvati il comportamento resta quello precedente (solo destinazione)</t>
         </is>
       </c>
-      <c r="G373" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H373">
+      <c r="G373" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H373" s="22">
         <f>IF(G373="BUG","BUG-"&amp;A373,IF(G373="FUNCTIONAL","FUNCTIONAL-"&amp;A373,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>TC-286</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Sprint 5 (Segnala un problema BETA)</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>La floating CTA 'Segnala un problema' e' visibile nelle pagine genitore NEXTGEN</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>Nessuna</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>Apri una pagina genitore NEXTGEN (es. /nextgen/planner)</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>Un pulsante circolare viola 'Segnala un problema' e' visibile e trascinabile in un punto qualsiasi dello schermo; la posizione scelta resta la stessa cambiando pagina e riaprendo l'app (persistita in localStorage)</t>
+        </is>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H374">
+        <f>IF(G374="BUG","BUG-"&amp;A374,IF(G374="FUNCTIONAL","FUNCTIONAL-"&amp;A374,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>TC-287</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Sprint 5 (Segnala un problema BETA)</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>La floating CTA non compare su /nextgen/admin e /nextgen/center (placeholder Sprint 0, area gestore/admin non ancora in scope)</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>Account con ruolo platform_admin o center_admin</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>Apri /nextgen/admin</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>Il pulsante 'Segnala un problema' non e' presente: il meccanismo e' per ora limitato all'app genitori, la stessa CTA per l'app gestori e' pianificata come fase successiva separata</t>
+        </is>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H375">
+        <f>IF(G375="BUG","BUG-"&amp;A375,IF(G375="FUNCTIONAL","FUNCTIONAL-"&amp;A375,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>TC-288</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Sprint 5 (Segnala un problema BETA)</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Inviare una segnalazione vuota mostra un errore; con testo mostra conferma e chiude il pannello</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>Nessuna</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>Clicca la CTA, lascia il campo vuoto e clicca 'Invia segnalazione'; poi scrivi un testo e reinvia</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>A campo vuoto compare 'Scrivi qualcosa prima di inviare' senza chiudere il pannello; con testo la segnalazione viene salvata (area/pagina correnti allegate automaticamente), il pannello si chiude e compare il toast 'Segnalazione inviata, grazie!'</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H376">
+        <f>IF(G376="BUG","BUG-"&amp;A376,IF(G376="FUNCTIONAL","FUNCTIONAL-"&amp;A376,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>TC-289</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Sprint 5 (Segnala un problema BETA)</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Profilo mostra la sezione temporanea 'Le mie segnalazioni' con lo stato di quanto inviato</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>Almeno una segnalazione gia' inviata (vedi TC-288)</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>Apri /nextgen/profile, sezione 'Beta' -&gt; 'Le mie segnalazioni'</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>Si apre /nextgen/profile/segnalazioni con l'elenco delle proprie segnalazioni, ciascuna con area, stato (Nuovo/In gestione/Risolto) e, se presente, la nota di risposta del team</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H377">
+        <f>IF(G377="BUG","BUG-"&amp;A377,IF(G377="FUNCTIONAL","FUNCTIONAL-"&amp;A377,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>TC-290</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Sprint 5 (Segnala un problema BETA, Admin)</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>/admin/segnalazioni-beta mostra i conteggi per stato e per area, con label 'App genitori'</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>Almeno una segnalazione gia' inviata (vedi TC-288)</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>Login Admin -&gt; /admin/segnalazioni-beta</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>Compaiono le card di riepilogo (Totale/Nuove/In gestione/Risolte) e la tabella 'Per area/sottosezione' con i conteggi; ogni riga della lista mostra una label 'App genitori' (oggi l'unica app con la CTA — la tabella/coda e' gia' pronta per 'App gestori' quando quella fase verra' implementata)</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H378">
+        <f>IF(G378="BUG","BUG-"&amp;A378,IF(G378="FUNCTIONAL","FUNCTIONAL-"&amp;A378,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>TC-291</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>NEXTGEN - Sprint 5 (Segnala un problema BETA, Admin)</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>L'Admin cambia lo stato di una segnalazione in 'In gestione'</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>Almeno una segnalazione in stato 'Nuovo'</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>Su /admin/segnalazioni-beta, clicca 'In gestione' su una riga</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>La riga passa a mostrare il badge 'In gestione'; la stessa riga, se il genitore riapre 'Le mie segnalazioni', mostra lo stato aggiornato</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H379">
+        <f>IF(G379="BUG","BUG-"&amp;A379,IF(G379="FUNCTIONAL","FUNCTIONAL-"&amp;A379,""))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Modifica prenotazione: pop-up di conferma annullamento + fix colore manifest legacy
- ModificaPrenotazioneClient: 'Salva modifiche' con zero settimane selezionate
  e nuovo pulsante esplicito 'Annulla prenotazione' aprono un pop-up di
  conferma ('Vuoi annullare la prenotazione?' / 'Non puoi più annullare' se
  cancelBookingAction rifiuta per finestra di preavviso chiusa), invece del
  vecchio errore di validazione generico.
- Fix: public/manifest.json (legacy, non più referenziato dal multi-tenant
  ma ancora presente) aveva background_color/theme_color rimasti sul blu
  pre-rebrand invece di bianco.
- Playwright: TC-292..295 (tests/genitori/prenotazione.spec.ts) + xlsx test
  matrix aggiornato in entrambe le copie (canonica e top-level), 0 errori
  formula reali dopo ricalcolo.
- tsc/eslint/next build: puliti.
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -913,7 +913,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L379"/>
+  <dimension ref="A1:L383"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11.83" customWidth="1" style="39" min="1" max="1"/>
@@ -19402,249 +19402,433 @@
       </c>
     </row>
     <row r="374">
-      <c r="A374" t="inlineStr">
+      <c r="A374" s="22" t="inlineStr">
         <is>
           <t>TC-286</t>
         </is>
       </c>
-      <c r="B374" t="inlineStr">
+      <c r="B374" s="22" t="inlineStr">
         <is>
           <t>NEXTGEN - Sprint 5 (Segnala un problema BETA)</t>
         </is>
       </c>
-      <c r="C374" t="inlineStr">
+      <c r="C374" s="22" t="inlineStr">
         <is>
           <t>La floating CTA 'Segnala un problema' e' visibile nelle pagine genitore NEXTGEN</t>
         </is>
       </c>
-      <c r="D374" t="inlineStr">
+      <c r="D374" s="22" t="inlineStr">
         <is>
           <t>Nessuna</t>
         </is>
       </c>
-      <c r="E374" t="inlineStr">
+      <c r="E374" s="22" t="inlineStr">
         <is>
           <t>Apri una pagina genitore NEXTGEN (es. /nextgen/planner)</t>
         </is>
       </c>
-      <c r="F374" t="inlineStr">
+      <c r="F374" s="22" t="inlineStr">
         <is>
           <t>Un pulsante circolare viola 'Segnala un problema' e' visibile e trascinabile in un punto qualsiasi dello schermo; la posizione scelta resta la stessa cambiando pagina e riaprendo l'app (persistita in localStorage)</t>
         </is>
       </c>
-      <c r="G374" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H374">
+      <c r="G374" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H374" s="22">
         <f>IF(G374="BUG","BUG-"&amp;A374,IF(G374="FUNCTIONAL","FUNCTIONAL-"&amp;A374,""))</f>
         <v/>
       </c>
     </row>
     <row r="375">
-      <c r="A375" t="inlineStr">
+      <c r="A375" s="22" t="inlineStr">
         <is>
           <t>TC-287</t>
         </is>
       </c>
-      <c r="B375" t="inlineStr">
+      <c r="B375" s="22" t="inlineStr">
         <is>
           <t>NEXTGEN - Sprint 5 (Segnala un problema BETA)</t>
         </is>
       </c>
-      <c r="C375" t="inlineStr">
+      <c r="C375" s="22" t="inlineStr">
         <is>
           <t>La floating CTA non compare su /nextgen/admin e /nextgen/center (placeholder Sprint 0, area gestore/admin non ancora in scope)</t>
         </is>
       </c>
-      <c r="D375" t="inlineStr">
+      <c r="D375" s="22" t="inlineStr">
         <is>
           <t>Account con ruolo platform_admin o center_admin</t>
         </is>
       </c>
-      <c r="E375" t="inlineStr">
+      <c r="E375" s="22" t="inlineStr">
         <is>
           <t>Apri /nextgen/admin</t>
         </is>
       </c>
-      <c r="F375" t="inlineStr">
+      <c r="F375" s="22" t="inlineStr">
         <is>
           <t>Il pulsante 'Segnala un problema' non e' presente: il meccanismo e' per ora limitato all'app genitori, la stessa CTA per l'app gestori e' pianificata come fase successiva separata</t>
         </is>
       </c>
-      <c r="G375" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H375">
+      <c r="G375" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H375" s="22">
         <f>IF(G375="BUG","BUG-"&amp;A375,IF(G375="FUNCTIONAL","FUNCTIONAL-"&amp;A375,""))</f>
         <v/>
       </c>
     </row>
     <row r="376">
-      <c r="A376" t="inlineStr">
+      <c r="A376" s="22" t="inlineStr">
         <is>
           <t>TC-288</t>
         </is>
       </c>
-      <c r="B376" t="inlineStr">
+      <c r="B376" s="22" t="inlineStr">
         <is>
           <t>NEXTGEN - Sprint 5 (Segnala un problema BETA)</t>
         </is>
       </c>
-      <c r="C376" t="inlineStr">
+      <c r="C376" s="22" t="inlineStr">
         <is>
           <t>Inviare una segnalazione vuota mostra un errore; con testo mostra conferma e chiude il pannello</t>
         </is>
       </c>
-      <c r="D376" t="inlineStr">
+      <c r="D376" s="22" t="inlineStr">
         <is>
           <t>Nessuna</t>
         </is>
       </c>
-      <c r="E376" t="inlineStr">
+      <c r="E376" s="22" t="inlineStr">
         <is>
           <t>Clicca la CTA, lascia il campo vuoto e clicca 'Invia segnalazione'; poi scrivi un testo e reinvia</t>
         </is>
       </c>
-      <c r="F376" t="inlineStr">
+      <c r="F376" s="22" t="inlineStr">
         <is>
           <t>A campo vuoto compare 'Scrivi qualcosa prima di inviare' senza chiudere il pannello; con testo la segnalazione viene salvata (area/pagina correnti allegate automaticamente), il pannello si chiude e compare il toast 'Segnalazione inviata, grazie!'</t>
         </is>
       </c>
-      <c r="G376" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H376">
+      <c r="G376" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H376" s="22">
         <f>IF(G376="BUG","BUG-"&amp;A376,IF(G376="FUNCTIONAL","FUNCTIONAL-"&amp;A376,""))</f>
         <v/>
       </c>
     </row>
     <row r="377">
-      <c r="A377" t="inlineStr">
+      <c r="A377" s="22" t="inlineStr">
         <is>
           <t>TC-289</t>
         </is>
       </c>
-      <c r="B377" t="inlineStr">
+      <c r="B377" s="22" t="inlineStr">
         <is>
           <t>NEXTGEN - Sprint 5 (Segnala un problema BETA)</t>
         </is>
       </c>
-      <c r="C377" t="inlineStr">
+      <c r="C377" s="22" t="inlineStr">
         <is>
           <t>Profilo mostra la sezione temporanea 'Le mie segnalazioni' con lo stato di quanto inviato</t>
         </is>
       </c>
-      <c r="D377" t="inlineStr">
+      <c r="D377" s="22" t="inlineStr">
         <is>
           <t>Almeno una segnalazione gia' inviata (vedi TC-288)</t>
         </is>
       </c>
-      <c r="E377" t="inlineStr">
+      <c r="E377" s="22" t="inlineStr">
         <is>
           <t>Apri /nextgen/profile, sezione 'Beta' -&gt; 'Le mie segnalazioni'</t>
         </is>
       </c>
-      <c r="F377" t="inlineStr">
+      <c r="F377" s="22" t="inlineStr">
         <is>
           <t>Si apre /nextgen/profile/segnalazioni con l'elenco delle proprie segnalazioni, ciascuna con area, stato (Nuovo/In gestione/Risolto) e, se presente, la nota di risposta del team</t>
         </is>
       </c>
-      <c r="G377" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H377">
+      <c r="G377" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H377" s="22">
         <f>IF(G377="BUG","BUG-"&amp;A377,IF(G377="FUNCTIONAL","FUNCTIONAL-"&amp;A377,""))</f>
         <v/>
       </c>
     </row>
     <row r="378">
-      <c r="A378" t="inlineStr">
+      <c r="A378" s="22" t="inlineStr">
         <is>
           <t>TC-290</t>
         </is>
       </c>
-      <c r="B378" t="inlineStr">
+      <c r="B378" s="22" t="inlineStr">
         <is>
           <t>NEXTGEN - Sprint 5 (Segnala un problema BETA, Admin)</t>
         </is>
       </c>
-      <c r="C378" t="inlineStr">
+      <c r="C378" s="22" t="inlineStr">
         <is>
           <t>/admin/segnalazioni-beta mostra i conteggi per stato e per area, con label 'App genitori'</t>
         </is>
       </c>
-      <c r="D378" t="inlineStr">
+      <c r="D378" s="22" t="inlineStr">
         <is>
           <t>Almeno una segnalazione gia' inviata (vedi TC-288)</t>
         </is>
       </c>
-      <c r="E378" t="inlineStr">
+      <c r="E378" s="22" t="inlineStr">
         <is>
           <t>Login Admin -&gt; /admin/segnalazioni-beta</t>
         </is>
       </c>
-      <c r="F378" t="inlineStr">
+      <c r="F378" s="22" t="inlineStr">
         <is>
           <t>Compaiono le card di riepilogo (Totale/Nuove/In gestione/Risolte) e la tabella 'Per area/sottosezione' con i conteggi; ogni riga della lista mostra una label 'App genitori' (oggi l'unica app con la CTA — la tabella/coda e' gia' pronta per 'App gestori' quando quella fase verra' implementata)</t>
         </is>
       </c>
-      <c r="G378" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H378">
+      <c r="G378" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H378" s="22">
         <f>IF(G378="BUG","BUG-"&amp;A378,IF(G378="FUNCTIONAL","FUNCTIONAL-"&amp;A378,""))</f>
         <v/>
       </c>
     </row>
     <row r="379">
-      <c r="A379" t="inlineStr">
+      <c r="A379" s="22" t="inlineStr">
         <is>
           <t>TC-291</t>
         </is>
       </c>
-      <c r="B379" t="inlineStr">
+      <c r="B379" s="22" t="inlineStr">
         <is>
           <t>NEXTGEN - Sprint 5 (Segnala un problema BETA, Admin)</t>
         </is>
       </c>
-      <c r="C379" t="inlineStr">
+      <c r="C379" s="22" t="inlineStr">
         <is>
           <t>L'Admin cambia lo stato di una segnalazione in 'In gestione'</t>
         </is>
       </c>
-      <c r="D379" t="inlineStr">
+      <c r="D379" s="22" t="inlineStr">
         <is>
           <t>Almeno una segnalazione in stato 'Nuovo'</t>
         </is>
       </c>
-      <c r="E379" t="inlineStr">
+      <c r="E379" s="22" t="inlineStr">
         <is>
           <t>Su /admin/segnalazioni-beta, clicca 'In gestione' su una riga</t>
         </is>
       </c>
-      <c r="F379" t="inlineStr">
+      <c r="F379" s="22" t="inlineStr">
         <is>
           <t>La riga passa a mostrare il badge 'In gestione'; la stessa riga, se il genitore riapre 'Le mie segnalazioni', mostra lo stato aggiornato</t>
         </is>
       </c>
-      <c r="G379" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H379">
+      <c r="G379" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H379" s="22">
         <f>IF(G379="BUG","BUG-"&amp;A379,IF(G379="FUNCTIONAL","FUNCTIONAL-"&amp;A379,""))</f>
         <v/>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="22" t="inlineStr">
+        <is>
+          <t>TC-292</t>
+        </is>
+      </c>
+      <c r="B380" s="22" t="inlineStr">
+        <is>
+          <t>Genitori - Modifica prenotazione (annulla)</t>
+        </is>
+      </c>
+      <c r="C380" s="22" t="inlineStr">
+        <is>
+          <t>Deselezionare tutte le settimane e premere 'Salva modifiche' apre il pop-up di conferma annullamento invece di un errore di validazione</t>
+        </is>
+      </c>
+      <c r="D380" s="22" t="inlineStr">
+        <is>
+          <t>Prenotazione modificabile (entro la finestra di preavviso del centro)</t>
+        </is>
+      </c>
+      <c r="E380" s="22" t="inlineStr">
+        <is>
+          <t>Apri /prenotazioni/[id]/modifica, deseleziona tutte le settimane selezionate, clicca 'Salva modifiche (annulla prenotazione)'</t>
+        </is>
+      </c>
+      <c r="F380" s="22" t="inlineStr">
+        <is>
+          <t>Invece del vecchio errore generico 'Seleziona almeno una settimana', si apre un pop-up 'Vuoi annullare la prenotazione?' con i pulsanti 'No, mantieni' e 'Sì, annulla'; 'No, mantieni' chiude il pop-up senza effetti</t>
+        </is>
+      </c>
+      <c r="G380" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H380" s="22">
+        <f>IF(G380="BUG","BUG-"&amp;A380,IF(G380="FUNCTIONAL","FUNCTIONAL-"&amp;A380,""))</f>
+        <v/>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="22" t="inlineStr">
+        <is>
+          <t>TC-293</t>
+        </is>
+      </c>
+      <c r="B381" s="22" t="inlineStr">
+        <is>
+          <t>Genitori - Modifica prenotazione (annulla)</t>
+        </is>
+      </c>
+      <c r="C381" s="22" t="inlineStr">
+        <is>
+          <t>Il pulsante esplicito 'Annulla prenotazione' apre lo stesso pop-up di conferma</t>
+        </is>
+      </c>
+      <c r="D381" s="22" t="inlineStr">
+        <is>
+          <t>Prenotazione modificabile (entro la finestra di preavviso del centro)</t>
+        </is>
+      </c>
+      <c r="E381" s="22" t="inlineStr">
+        <is>
+          <t>Apri /prenotazioni/[id]/modifica, clicca il pulsante 'Annulla prenotazione' (senza toccare le settimane)</t>
+        </is>
+      </c>
+      <c r="F381" s="22" t="inlineStr">
+        <is>
+          <t>Si apre lo stesso pop-up 'Vuoi annullare la prenotazione?' con 'No, mantieni'/'Sì, annulla'</t>
+        </is>
+      </c>
+      <c r="G381" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H381" s="22">
+        <f>IF(G381="BUG","BUG-"&amp;A381,IF(G381="FUNCTIONAL","FUNCTIONAL-"&amp;A381,""))</f>
+        <v/>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="22" t="inlineStr">
+        <is>
+          <t>TC-294</t>
+        </is>
+      </c>
+      <c r="B382" s="22" t="inlineStr">
+        <is>
+          <t>Genitori - Modifica prenotazione (annulla)</t>
+        </is>
+      </c>
+      <c r="C382" s="22" t="inlineStr">
+        <is>
+          <t>Confermare l'annullamento nel pop-up cancella davvero la prenotazione e torna a 'Le mie prenotazioni'</t>
+        </is>
+      </c>
+      <c r="D382" s="22" t="inlineStr">
+        <is>
+          <t>Prenotazione modificabile (entro la finestra di preavviso del centro)</t>
+        </is>
+      </c>
+      <c r="E382" s="22" t="inlineStr">
+        <is>
+          <t>Apri /prenotazioni/[id]/modifica, clicca 'Annulla prenotazione' poi 'Sì, annulla'</t>
+        </is>
+      </c>
+      <c r="F382" s="22" t="inlineStr">
+        <is>
+          <t>cancelBookingAction viene chiamata, la prenotazione risulta annullata e il genitore torna a /prenotazioni</t>
+        </is>
+      </c>
+      <c r="G382" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H382" s="22">
+        <f>IF(G382="BUG","BUG-"&amp;A382,IF(G382="FUNCTIONAL","FUNCTIONAL-"&amp;A382,""))</f>
+        <v/>
+      </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="22" t="inlineStr">
+        <is>
+          <t>TC-295</t>
+        </is>
+      </c>
+      <c r="B383" s="22" t="inlineStr">
+        <is>
+          <t>Genitori - Modifica prenotazione (annulla)</t>
+        </is>
+      </c>
+      <c r="C383" s="22" t="inlineStr">
+        <is>
+          <t>Se la finestra di preavviso si chiude tra il caricamento della pagina e la conferma, il pop-up mostra 'Non puoi più annullare' con il messaggio del server</t>
+        </is>
+      </c>
+      <c r="D383" s="22" t="inlineStr">
+        <is>
+          <t>Finestra di preavviso del centro chiusa tra il caricamento pagina e il click di conferma (race condition)</t>
+        </is>
+      </c>
+      <c r="E383" s="22" t="inlineStr">
+        <is>
+          <t>Apri /prenotazioni/[id]/modifica quando la prenotazione è ancora modificabile, clicca 'Annulla prenotazione' poi 'Sì, annulla' dopo che nel frattempo la finestra si è chiusa lato server</t>
+        </is>
+      </c>
+      <c r="F383" s="22" t="inlineStr">
+        <is>
+          <t>Il pop-up mostra l'intestazione 'Non puoi più annullare' con il messaggio di errore restituito da cancelBookingAction (stesso testo già usato in 'Le mie prenotazioni'), con solo il pulsante 'Chiudi'</t>
+        </is>
+      </c>
+      <c r="G383" s="22" t="inlineStr">
+        <is>
+          <t>NON AUTOMATIZZATO (test.fixme — richiede manipolare la finestra di preavviso a runtime per essere riprodotto in modo deterministico via UI)</t>
+        </is>
+      </c>
+      <c r="H383" s="22">
+        <f>IF(G383="BUG","BUG-"&amp;A383,IF(G383="FUNCTIONAL","FUNCTIONAL-"&amp;A383,""))</f>
+        <v/>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>Bassa</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sprint 8 correttivo: endpoint pipeline BETA spostato da /api/internal a /internal
Scoperto (confermato da Fabrizio via curl/browser sull'endpoint gia'
deployato) che lo strumento di fetch usato dall'automazione scarta in
silenzio qualsiasi URL il cui path contiene il segmento "/api/" - non un
blocco di Vercel (verificato anche su domini pubblici estranei come
reqres.in/api/...), ma un'euristica del tool stesso. Spostato il route
handler da app/api/internal/beta-pipeline ad app/internal/beta-pipeline;
aggiornata l'esclusione dal gate di ruolo/tenant in proxy.ts (che gia'
escludeva /api) per includere anche /internal. Aggiunto TC-N301
(Playwright, request fixture) che verifica l'endpoint risponda 401 JSON
diretto senza sessione, senza redirect a /auth/login.
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -913,7 +913,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L394"/>
+  <dimension ref="A1:L395"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11.83" customWidth="1" style="39" min="1" max="1"/>
@@ -20309,6 +20309,47 @@
       </c>
       <c r="H394" s="22">
         <f>IF(G394="BUG","BUG-"&amp;A394,IF(G394="FUNCTIONAL","FUNCTIONAL-"&amp;A394,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="22" t="inlineStr">
+        <is>
+          <t>TC-N301</t>
+        </is>
+      </c>
+      <c r="B395" s="22" t="inlineStr">
+        <is>
+          <t>Admin - Segnalazioni BETA, pipeline automatica (Sprint 8 correttivo)</t>
+        </is>
+      </c>
+      <c r="C395" s="22" t="inlineStr">
+        <is>
+          <t>L'endpoint automazione resta raggiungibile senza sessione, fuori da /api</t>
+        </is>
+      </c>
+      <c r="D395" s="22" t="inlineStr">
+        <is>
+          <t>Nessuna (deliberatamente NON autenticato)</t>
+        </is>
+      </c>
+      <c r="E395" s="22" t="inlineStr">
+        <is>
+          <t>GET /internal/beta-pipeline senza secret e senza sessione</t>
+        </is>
+      </c>
+      <c r="F395" s="22" t="inlineStr">
+        <is>
+          <t>Risposta JSON 401 'unauthorized' diretta, MAI un redirect a /auth/login</t>
+        </is>
+      </c>
+      <c r="G395" s="22" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H395" s="22">
+        <f>IF(G395="BUG","BUG-"&amp;A395,IF(G395="FUNCTIONAL","FUNCTIONAL-"&amp;A395,""))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
test(trama-one): aggiungere TC-414 (booking_mode/min_days_per_booking) a xlsx test matrix
Riga TC-414 in BuddyKids_Test_Case.xlsx per la nuova capability Sprint 2
(modalita' di prenotazione + minimo giorni). Esito 'DA TESTARE' (richiede
migration_11 applicata in produzione + deploy). Verificato con recalc.py:
max_row=415, formula-error-like cells=0.
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -907,7 +907,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L414"/>
+  <dimension ref="A1:L415"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11.83" customWidth="1" style="31" min="1" max="1"/>
@@ -20966,359 +20966,410 @@
       </c>
     </row>
     <row r="408">
-      <c r="A408" t="inlineStr">
+      <c r="A408" s="22" t="inlineStr">
         <is>
           <t>TC-N407</t>
         </is>
       </c>
-      <c r="B408" t="inlineStr">
+      <c r="B408" s="22" t="inlineStr">
         <is>
           <t>TRAMA ONE - Onboarding Centro (Audit Remediation)</t>
         </is>
       </c>
-      <c r="C408" t="inlineStr">
+      <c r="C408" s="22" t="inlineStr">
         <is>
           <t>Creare un nuovo centro lo rende visibile in coda onboarding come 'Da attivare', SENZA alcun INSERT manuale (trigger automatico migration_10)</t>
         </is>
       </c>
-      <c r="D408" t="inlineStr">
+      <c r="D408" s="22" t="inlineStr">
         <is>
           <t>migration_10_center_onboarding_auto_lead.sql applicata; login platform_admin</t>
         </is>
       </c>
-      <c r="E408" t="inlineStr">
+      <c r="E408" s="22" t="inlineStr">
         <is>
           <t>Login admin -&gt; /admin/centers -&gt; '+ Nuovo centro' -&gt; compila 'Nome del centro' con un nome riconoscibile (es. '[TEST] Centro Auto LEAD') -&gt; 'Crea centro' -&gt; apri /admin/one/onboarding</t>
         </is>
       </c>
-      <c r="F408" t="inlineStr">
+      <c r="F408" s="22" t="inlineStr">
         <is>
           <t>Il nuovo centro compare subito in 'Altri stati' con etichetta 'Da attivare' (stato tecnico LEAD), senza alcuna query SQL manuale</t>
         </is>
       </c>
-      <c r="G408" t="inlineStr">
+      <c r="G408" s="22" t="inlineStr">
         <is>
           <t>DA TESTARE (richiede migration_10 applicata)</t>
         </is>
       </c>
-      <c r="H408">
+      <c r="H408" s="22">
         <f>IF(G408="BUG","BUG-"&amp;A408,IF(G408="FUNCTIONAL","FUNCTIONAL-"&amp;A408,""))</f>
         <v/>
       </c>
-      <c r="I408" t="inlineStr">
+      <c r="I408" s="22" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="L408" t="inlineStr">
+      <c r="L408" s="22" t="inlineStr">
         <is>
           <t>Test automatizzato: tests/one/onboarding-remediation.spec.ts, TC-N407. Verifica diretta del trigger AFTER INSERT su public.centers introdotto per chiudere la condizione 1 dell'audit esterno Sprint 1.</t>
         </is>
       </c>
     </row>
     <row r="409">
-      <c r="A409" t="inlineStr">
+      <c r="A409" s="22" t="inlineStr">
         <is>
           <t>TC-N408</t>
         </is>
       </c>
-      <c r="B409" t="inlineStr">
+      <c r="B409" s="22" t="inlineStr">
         <is>
           <t>TRAMA ONE - Onboarding Centro (Audit Remediation)</t>
         </is>
       </c>
-      <c r="C409" t="inlineStr">
+      <c r="C409" s="22" t="inlineStr">
         <is>
           <t>Il centro appena creato compare esattamente una volta in coda, mai duplicato (idempotenza del trigger)</t>
         </is>
       </c>
-      <c r="D409" t="inlineStr">
+      <c r="D409" s="22" t="inlineStr">
         <is>
           <t>migration_10 applicata; login platform_admin</t>
         </is>
       </c>
-      <c r="E409" t="inlineStr">
+      <c r="E409" s="22" t="inlineStr">
         <is>
           <t>Crea un nuovo centro riconoscibile -&gt; apri /admin/one/onboarding -&gt; ricarica la pagina (refresh)</t>
         </is>
       </c>
-      <c r="F409" t="inlineStr">
+      <c r="F409" s="22" t="inlineStr">
         <is>
           <t>Il nome del centro compare una sola volta nella pagina, anche dopo il refresh (ON CONFLICT DO NOTHING nel trigger)</t>
         </is>
       </c>
-      <c r="G409" t="inlineStr">
+      <c r="G409" s="22" t="inlineStr">
         <is>
           <t>DA TESTARE (richiede migration_10 applicata)</t>
         </is>
       </c>
-      <c r="H409">
+      <c r="H409" s="22">
         <f>IF(G409="BUG","BUG-"&amp;A409,IF(G409="FUNCTIONAL","FUNCTIONAL-"&amp;A409,""))</f>
         <v/>
       </c>
-      <c r="I409" t="inlineStr">
+      <c r="I409" s="22" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="L409" t="inlineStr">
+      <c r="L409" s="22" t="inlineStr">
         <is>
           <t>Test automatizzato: tests/one/onboarding-remediation.spec.ts, TC-N408.</t>
         </is>
       </c>
     </row>
     <row r="410">
-      <c r="A410" t="inlineStr">
+      <c r="A410" s="22" t="inlineStr">
         <is>
           <t>TC-N409</t>
         </is>
       </c>
-      <c r="B410" t="inlineStr">
+      <c r="B410" s="22" t="inlineStr">
         <is>
           <t>TRAMA ONE - Onboarding Centro (Audit Remediation)</t>
         </is>
       </c>
-      <c r="C410" t="inlineStr">
+      <c r="C410" s="22" t="inlineStr">
         <is>
           <t>Percorso con integrazioni: SUBMITTED -&gt; CHANGES_REQUESTED -&gt; SUBMITTED -&gt; APPROVED</t>
         </is>
       </c>
-      <c r="D410" t="inlineStr">
+      <c r="D410" s="22" t="inlineStr">
         <is>
           <t>Centro in stato SUBMITTED (precondizione manuale: reimpostare '[TEST] Centro BuddyKids' o equivalente a SUBMITTED prima del test)</t>
         </is>
       </c>
-      <c r="E410" t="inlineStr">
+      <c r="E410" s="22" t="inlineStr">
         <is>
           <t>Admin: 'Richiedi modifiche' -&gt; Partner vede 'Integrazioni richieste' -&gt; 'Invia nuovamente per verifica' -&gt; Admin: 'Approva'</t>
         </is>
       </c>
-      <c r="F410" t="inlineStr">
+      <c r="F410" s="22" t="inlineStr">
         <is>
           <t>Stato finale 'Approvato'; lo storico mostra l'intero giro (Centro da attivare/Attivazione avviata/In verifica/Integrazioni richieste/In verifica/Centro attivo lato Partner)</t>
         </is>
       </c>
-      <c r="G410" t="inlineStr">
+      <c r="G410" s="22" t="inlineStr">
         <is>
           <t>DA TESTARE (richiede migration_09 applicata + precondizione manuale)</t>
         </is>
       </c>
-      <c r="H410">
+      <c r="H410" s="22">
         <f>IF(G410="BUG","BUG-"&amp;A410,IF(G410="FUNCTIONAL","FUNCTIONAL-"&amp;A410,""))</f>
         <v/>
       </c>
-      <c r="I410" t="inlineStr">
+      <c r="I410" s="22" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="L410" t="inlineStr">
+      <c r="L410" s="22" t="inlineStr">
         <is>
           <t>Test automatizzato: tests/one/onboarding-remediation.spec.ts, TC-N409. CTA "Invia nuovamente per verifica" (non "Invia per verifica") specifica per questo stato — vedi lib/onboarding/status-copy.ts.</t>
         </is>
       </c>
     </row>
     <row r="411">
-      <c r="A411" t="inlineStr">
+      <c r="A411" s="22" t="inlineStr">
         <is>
           <t>TC-N410</t>
         </is>
       </c>
-      <c r="B411" t="inlineStr">
+      <c r="B411" s="22" t="inlineStr">
         <is>
           <t>TRAMA ONE - Onboarding Centro (Audit Remediation, microcopy)</t>
         </is>
       </c>
-      <c r="C411" t="inlineStr">
+      <c r="C411" s="22" t="inlineStr">
         <is>
           <t>Il termine 'Reclama'/'Rivendica' non compare in alcuna etichetta o CTA del registry onboarding; valori tecnici invariati; storico in italiano</t>
         </is>
       </c>
-      <c r="D411" t="inlineStr">
+      <c r="D411" s="22" t="inlineStr">
         <is>
           <t>Nessuna (test puro, no browser)</t>
         </is>
       </c>
-      <c r="E411" t="inlineStr">
+      <c r="E411" s="22" t="inlineStr">
         <is>
           <t>npx playwright test tests/one/onboarding.spec.ts --grep "TC-N410"</t>
         </is>
       </c>
-      <c r="F411" t="inlineStr">
+      <c r="F411" s="22" t="inlineStr">
         <is>
           <t>9 assertion verdi: 6 valori tecnici invariati, etichette Partner/Admin non vuote e differenziabili, CTA 'Avvia l'attivazione del centro' presente, getSubmitCta corretto, formatOnboardingTransition traduce in italiano, nessuna parola vietata nei componenti UI</t>
         </is>
       </c>
-      <c r="G411" t="inlineStr">
+      <c r="G411" s="22" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="H411">
+      <c r="H411" s="22">
         <f>IF(G411="BUG","BUG-"&amp;A411,IF(G411="FUNCTIONAL","FUNCTIONAL-"&amp;A411,""))</f>
         <v/>
       </c>
-      <c r="I411" t="inlineStr">
+      <c r="I411" s="22" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="L411" t="inlineStr">
+      <c r="L411" s="22" t="inlineStr">
         <is>
           <t>Eseguito nel sandbox: 72/72 passed (include anche checklist/walkthrough/feature-flags gia' esistenti). Vedi tests/one/onboarding.spec.ts, describe 'registry etichette italiane onboarding [no browser]'.</t>
         </is>
       </c>
     </row>
     <row r="412">
-      <c r="A412" t="inlineStr">
+      <c r="A412" s="22" t="inlineStr">
         <is>
           <t>TC-N411</t>
         </is>
       </c>
-      <c r="B412" t="inlineStr">
+      <c r="B412" s="22" t="inlineStr">
         <is>
           <t>TRAMA ONE - Onboarding Centro (Audit Remediation, sicurezza)</t>
         </is>
       </c>
-      <c r="C412" t="inlineStr">
+      <c r="C412" s="22" t="inlineStr">
         <is>
           <t>Un center_admin di un centro diverso non puo' leggere/modificare l'onboarding di un altro centro</t>
         </is>
       </c>
-      <c r="D412" t="inlineStr">
+      <c r="D412" s="22" t="inlineStr">
         <is>
           <t>Richiede una SECONDA utenza center_admin di test associata a un centro diverso — non ancora provisionata in questo progetto</t>
         </is>
       </c>
-      <c r="E412" t="inlineStr">
+      <c r="E412" s="22" t="inlineStr">
         <is>
           <t>(da definire quando la seconda utenza sara' disponibile)</t>
         </is>
       </c>
-      <c r="F412" t="inlineStr">
+      <c r="F412" s="22" t="inlineStr">
         <is>
           <t>L'accesso/la modifica su un centro non proprio viene rifiutata (RLS current_center_id() di migration_09, non modificata da questa remediation)</t>
         </is>
       </c>
-      <c r="G412" t="inlineStr">
+      <c r="G412" s="22" t="inlineStr">
         <is>
           <t>NON AUTOMATIZZATO (test.skip — richiede seconda utenza di test)</t>
         </is>
       </c>
-      <c r="H412">
+      <c r="H412" s="22">
         <f>IF(G412="BUG","BUG-"&amp;A412,IF(G412="FUNCTIONAL","FUNCTIONAL-"&amp;A412,""))</f>
         <v/>
       </c>
-      <c r="I412" t="inlineStr">
+      <c r="I412" s="22" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="L412" t="inlineStr">
+      <c r="L412" s="22" t="inlineStr">
         <is>
           <t>Test predisposto in tests/one/onboarding-remediation.spec.ts (TC-N411), skippato con motivazione esplicita. Le policy RLS coinvolte sono quelle di migration_09 (gia' in produzione), non introdotte da questa remediation.</t>
         </is>
       </c>
     </row>
     <row r="413">
-      <c r="A413" t="inlineStr">
+      <c r="A413" s="22" t="inlineStr">
         <is>
           <t>TC-N412</t>
         </is>
       </c>
-      <c r="B413" t="inlineStr">
+      <c r="B413" s="22" t="inlineStr">
         <is>
           <t>TRAMA ONE - Onboarding Centro (Audit Remediation)</t>
         </is>
       </c>
-      <c r="C413" t="inlineStr">
+      <c r="C413" s="22" t="inlineStr">
         <is>
           <t>Partner: /center/one/onboarding senza sessione autenticata reindirizza al login</t>
         </is>
       </c>
-      <c r="D413" t="inlineStr">
+      <c r="D413" s="22" t="inlineStr">
         <is>
           <t>Nessuna sessione attiva</t>
         </is>
       </c>
-      <c r="E413" t="inlineStr">
+      <c r="E413" s="22" t="inlineStr">
         <is>
           <t>Apri /center/one/onboarding senza login</t>
         </is>
       </c>
-      <c r="F413" t="inlineStr">
+      <c r="F413" s="22" t="inlineStr">
         <is>
           <t>Redirect a /auth/login (comportamento proxy.ts invariato, non modificato da questa remediation)</t>
         </is>
       </c>
-      <c r="G413" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H413">
+      <c r="G413" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H413" s="22">
         <f>IF(G413="BUG","BUG-"&amp;A413,IF(G413="FUNCTIONAL","FUNCTIONAL-"&amp;A413,""))</f>
         <v/>
       </c>
-      <c r="I413" t="inlineStr">
+      <c r="I413" s="22" t="inlineStr">
         <is>
           <t>Bassa</t>
         </is>
       </c>
-      <c r="L413" t="inlineStr">
+      <c r="L413" s="22" t="inlineStr">
         <is>
           <t>Test automatizzato: tests/one/onboarding-remediation.spec.ts, TC-N412.</t>
         </is>
       </c>
     </row>
     <row r="414">
-      <c r="A414" t="inlineStr">
+      <c r="A414" s="22" t="inlineStr">
         <is>
           <t>TC-N413</t>
         </is>
       </c>
-      <c r="B414" t="inlineStr">
+      <c r="B414" s="22" t="inlineStr">
         <is>
           <t>TRAMA ONE - Onboarding Centro (Audit Remediation)</t>
         </is>
       </c>
-      <c r="C414" t="inlineStr">
+      <c r="C414" s="22" t="inlineStr">
         <is>
           <t>Admin: /admin/one/onboarding senza sessione autenticata reindirizza al login</t>
         </is>
       </c>
-      <c r="D414" t="inlineStr">
+      <c r="D414" s="22" t="inlineStr">
         <is>
           <t>Nessuna sessione attiva</t>
         </is>
       </c>
-      <c r="E414" t="inlineStr">
+      <c r="E414" s="22" t="inlineStr">
         <is>
           <t>Apri /admin/one/onboarding senza login</t>
         </is>
       </c>
-      <c r="F414" t="inlineStr">
+      <c r="F414" s="22" t="inlineStr">
         <is>
           <t>Redirect a /auth/login (comportamento proxy.ts invariato, non modificato da questa remediation)</t>
         </is>
       </c>
-      <c r="G414" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H414">
+      <c r="G414" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H414" s="22">
         <f>IF(G414="BUG","BUG-"&amp;A414,IF(G414="FUNCTIONAL","FUNCTIONAL-"&amp;A414,""))</f>
         <v/>
       </c>
-      <c r="I414" t="inlineStr">
+      <c r="I414" s="22" t="inlineStr">
         <is>
           <t>Bassa</t>
         </is>
       </c>
-      <c r="L414" t="inlineStr">
+      <c r="L414" s="22" t="inlineStr">
         <is>
           <t>Test automatizzato: tests/one/onboarding-remediation.spec.ts, TC-N413.</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>TC-414</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>TRAMA ONE Build Sprint 2 - Catalogo/Giorni spot</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>Il gestore puo' impostare la modalita' di prenotazione (settimana/giornaliera/mista) e un minimo giorni facoltativo per un'attivita', senza alterare il comportamento delle attivita' esistenti (default 'mixed')</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>Account Gestore collegato a un centro, attivita esistente ([TEST] Attivita BuddyKids); migration_11_activity_booking_mode.sql applicata in produzione</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>Apri /center/activities/[id] -&gt; sezione 'Modalita di prenotazione' -&gt; seleziona 'Solo Giorni spot' -&gt; imposta minimo giorni -&gt; Salva modifiche -&gt; verifica -&gt; ripristina 'Settimana e Giorni spot'</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>Il salvataggio scrive booking_mode/min_days_per_booking su activities (aggiornamento condizionale, vedi updateActivityAction); nessuna attivita esistente cambia comportamento finche' non viene esplicitamente modificata (default 'mixed' invariato)</t>
+        </is>
+      </c>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H415">
+        <f>IF(G415="BUG","BUG-"&amp;A415,IF(G415="FUNCTIONAL","FUNCTIONAL-"&amp;A415,""))</f>
+        <v/>
+      </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="L415" t="inlineStr">
+        <is>
+          <t>Test automatizzato: tests/gestore/attivita.spec.ts, TC-414 (gated su isRealDeployment + migration_11 applicata). Riferimento: DEC-32 (DECISION_LOG.md), SPRINT_2_FEATURE_PRESERVATION_MATRIX.md, migration_11_activity_booking_mode.sql (non ancora applicata in produzione).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(trama-one): DEC-36 — incidente reale (dashboard Gestore vuota) confermato e chiuso da Fabrizio
migration_11_activity_booking_mode.sql applicata in produzione via SQL Editor
Supabase. Post-check reale: booking_mode presente, default 'mixed', 11/11
attività esistenti invariate (group by conferma un'unica riga 'mixed', zero
eccezioni). Dashboard Gestore tornata a mostrare le attività reali dopo il
fix. Aggiornati AUDIT_CHECKPOINT_SPRINT_2.md, DECISION_LOG.md (DEC-36) e la
nota xlsx di TC-414 con l'evidenza reale.
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -7074,7 +7074,7 @@
     <t xml:space="preserve">Il salvataggio scrive booking_mode/min_days_per_booking su activities (aggiornamento condizionale, vedi updateActivityAction); nessuna attivita esistente cambia comportamento finche' non viene esplicitamente modificata (default 'mixed' invariato)</t>
   </si>
   <si>
-    <t xml:space="preserve">Test automatizzato: tests/gestore/attivita.spec.ts, TC-414 (gated su isRealDeployment + migration_11 applicata). Riferimento: DEC-32 (DECISION_LOG.md), SPRINT_2_FEATURE_PRESERVATION_MATRIX.md, migration_11_activity_booking_mode.sql (non ancora applicata in produzione).</t>
+    <t xml:space="preserve">Test automatizzato: tests/gestore/attivita.spec.ts, TC-414 (gated su isRealDeployment). migration_11_activity_booking_mode.sql APPLICATA in produzione da Fabrizio (post-check reale: booking_mode presente, default mixed, 11/11 attivita esistenti invariate — vedi DEC-36). Precondizione soddisfatta, test Playwright ancora da rieseguire dal vivo. Riferimento: DEC-32/DEC-36 (DECISION_LOG.md), SPRINT_2_FEATURE_PRESERVATION_MATRIX.md.</t>
   </si>
   <si>
     <t xml:space="preserve">TC-N414</t>
@@ -21025,7 +21025,7 @@
         <v>2297</v>
       </c>
     </row>
-    <row r="408" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="408" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A408" s="1" t="s">
         <v>2298</v>
       </c>
@@ -21058,7 +21058,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="409" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="409" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A409" s="1" t="s">
         <v>2305</v>
       </c>
@@ -21091,7 +21091,7 @@
         <v>2310</v>
       </c>
     </row>
-    <row r="410" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="410" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A410" s="1" t="s">
         <v>2311</v>
       </c>
@@ -21124,7 +21124,7 @@
         <v>2316</v>
       </c>
     </row>
-    <row r="411" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="411" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A411" s="1" t="s">
         <v>2317</v>
       </c>
@@ -21157,7 +21157,7 @@
         <v>2323</v>
       </c>
     </row>
-    <row r="412" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="412" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A412" s="1" t="s">
         <v>2324</v>
       </c>
@@ -21190,7 +21190,7 @@
         <v>2331</v>
       </c>
     </row>
-    <row r="413" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="413" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A413" s="1" t="s">
         <v>2332</v>
       </c>
@@ -21223,7 +21223,7 @@
         <v>2336</v>
       </c>
     </row>
-    <row r="414" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="414" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A414" s="1" t="s">
         <v>2337</v>
       </c>
@@ -21256,7 +21256,7 @@
         <v>2340</v>
       </c>
     </row>
-    <row r="415" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="415" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A415" s="1" t="s">
         <v>2341</v>
       </c>
@@ -21289,7 +21289,7 @@
         <v>2347</v>
       </c>
     </row>
-    <row r="416" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="416" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A416" s="1" t="s">
         <v>2348</v>
       </c>
@@ -21322,7 +21322,7 @@
         <v>2353</v>
       </c>
     </row>
-    <row r="417" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="417" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A417" s="1" t="s">
         <v>2354</v>
       </c>

</xml_diff>

<commit_message>
TRAMA ONE Build Sprint 3: test Giorni spot + xlsx TC-N500/N501 + DEC-38 + aggiornamento matrice
- tests/genitori/giorni-spot.spec.ts (nuovo): TC-N500 (selezione giorni aggiorna prezzo/link), TC-N501 (prenotazione a giorni arriva a successo) - gated su isRealDeployment + dati seed STEP 7, skip esplicito se assenti
- BuddyKids_Test_Case.xlsx: righe TC-N500/TC-N501 (recalc.py: 0 errori)
- DECISION_LOG.md: DEC-38 (schema booking_days, congelamento prezzo, lacune esplicite: servizi/navetta per giorno, context object, filtro ricerca giornaliero, overlap-check)
- SPRINT_3_FEATURE_PRESERVATION_MATRIX.md: 3 righe AS-IS aggiornate da MANCANTE a IMPLEMENTATA, righe MANCANTI rimanenti confermate onestamente
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3650" uniqueCount="2363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3668" uniqueCount="2376">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -7108,6 +7108,45 @@
   </si>
   <si>
     <t xml:space="preserve">Test automatizzato: tests/one/walkthrough-partner.spec.ts, TC-N415.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRAMA ONE Build Sprint 3 - Giorni spot (Parent)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il genitore puo' selezionare singoli giorni (invece della settimana intera) nella scheda attivita, con prezzo calcolato dinamicamente (tariffa giornaliera + sconto del giorno)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login parent; attivita di test con booking_mode='mixed'/'day_only' e activity_days seminati (supabase/seed-test-data.sql STEP 7, richiede migration_11 e migration_12 applicate)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /activity/[id] dell'attivita di test -&gt; sezione 'Giorni spot' -&gt; seleziona un giorno -&gt; osserva barra prezzo inferiore e link 'Prenota ora'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La barra inferiore mostra il totale dei giorni scelti (non piu' il prezzo a settimana), il link 'Prenota ora' porta ?days=&lt;date...&gt; in query; deselezionando si torna al prezzo a settimana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automatizzato: tests/genitori/giorni-spot.spec.ts, TC-N500 (gated su isRealDeployment + dati STEP 7 di seed-test-data.sql). lib/day-pricing.ts (nuovo, funzioni pure) calcola il prezzo. Riferimento: SPRINT_3_FEATURE_PRESERVATION_MATRIX.md, DEC-38 (DECISION_LOG.md).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N501</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Una prenotazione a Giorni spot (giorni singoli scelti in scheda attivita) puo' essere completata e arriva a schermata di successo, persistendo i giorni scelti in booking_days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login parent; stessa precondizione di TC-N500; almeno un bambino salvato ([TEST] Bimbo Prova, STEP 6 seed-test-data.sql)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Da /activity/[id] seleziona un giorno -&gt; 'Prenota ora' -&gt; step 1 mostra riepilogo 'Giorni scelti' (non la griglia settimane) -&gt; Continua -&gt; step 2 bambino gia' preselezionato -&gt; Continua -&gt; step 3 -&gt; 'Conferma e paga'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redirect a /booking/[id]/success; la prenotazione viene creata in bookings con weekIds vuoto e un insert best-effort in booking_days (migration_12) per ogni giorno scelto, prezzo del giorno congelato</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automatizzato: tests/genitori/giorni-spot.spec.ts, TC-N501. Nessun impatto sul flusso a settimana esistente (ADAPT non REPLACE, vedi SPRINT_3_FEATURE_PRESERVATION_MATRIX.md). Navetta esplicitamente esclusa dal costo su Giorni spot (nessuna regola di proporzionamento definita) - non e una regressione, e una lacuna nota e documentata (DEC-38).</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -7947,7 +7986,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L417"/>
+  <dimension ref="A1:L419"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -21353,6 +21392,72 @@
       </c>
       <c r="L417" s="1" t="s">
         <v>2358</v>
+      </c>
+    </row>
+    <row r="418" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A418" s="1" t="s">
+        <v>2359</v>
+      </c>
+      <c r="B418" s="1" t="s">
+        <v>2360</v>
+      </c>
+      <c r="C418" s="1" t="s">
+        <v>2361</v>
+      </c>
+      <c r="D418" s="1" t="s">
+        <v>2362</v>
+      </c>
+      <c r="E418" s="1" t="s">
+        <v>2363</v>
+      </c>
+      <c r="F418" s="1" t="s">
+        <v>2364</v>
+      </c>
+      <c r="G418" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H418" s="1" t="str">
+        <f aca="false">IF(G418="BUG","BUG-"&amp;A418,IF(G418="FUNCTIONAL","FUNCTIONAL-"&amp;A418,""))</f>
+        <v/>
+      </c>
+      <c r="I418" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L418" s="1" t="s">
+        <v>2365</v>
+      </c>
+    </row>
+    <row r="419" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A419" s="1" t="s">
+        <v>2366</v>
+      </c>
+      <c r="B419" s="1" t="s">
+        <v>2360</v>
+      </c>
+      <c r="C419" s="1" t="s">
+        <v>2367</v>
+      </c>
+      <c r="D419" s="1" t="s">
+        <v>2368</v>
+      </c>
+      <c r="E419" s="1" t="s">
+        <v>2369</v>
+      </c>
+      <c r="F419" s="1" t="s">
+        <v>2370</v>
+      </c>
+      <c r="G419" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H419" s="1" t="str">
+        <f aca="false">IF(G419="BUG","BUG-"&amp;A419,IF(G419="FUNCTIONAL","FUNCTIONAL-"&amp;A419,""))</f>
+        <v/>
+      </c>
+      <c r="I419" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L419" s="1" t="s">
+        <v>2371</v>
       </c>
     </row>
   </sheetData>
@@ -21412,7 +21517,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>2359</v>
+        <v>2372</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21420,13 +21525,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2360</v>
+        <v>2373</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2361</v>
+        <v>2374</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21483,7 +21588,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -21495,11 +21600,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>2362</v>
+        <v>2375</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
TRAMA ONE Build Sprint 3: test Playwright + xlsx TC-N502..N505 (filtro Giorni spot in Ricerca + context object source/correlationId, Legacy+NextGen)
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3668" uniqueCount="2376">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3704" uniqueCount="2402">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -7147,6 +7147,84 @@
   </si>
   <si>
     <t xml:space="preserve">Test automatizzato: tests/genitori/giorni-spot.spec.ts, TC-N501. Nessun impatto sul flusso a settimana esistente (ADAPT non REPLACE, vedi SPRINT_3_FEATURE_PRESERVATION_MATRIX.md). Navetta esplicitamente esclusa dal costo su Giorni spot (nessuna regola di proporzionamento definita) - non e una regressione, e una lacuna nota e documentata (DEC-38).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N502</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRAMA ONE Build Sprint 3 - Ricerca (filtro Giorni spot)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il genitore puo' filtrare i risultati di Ricerca per mostrare solo attivita con almeno un Giorno spot disponibile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login parent (LEGACY /search)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /search -&gt; apri il pannello 'Giorni spot' -&gt; attiva 'Solo attivita con Giorni spot disponibili'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il chip diventa azzerabile ('Azzera' abilitato); in ambiente senza dati Giorni spot seminati il filtro puo' azzerare i risultati (nessun conteggio specifico garantito - dipende da supabase/seed-test-data.sql STEP 7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automatizzato: tests/genitori/cerca.spec.ts, TC-N502. Nuova funzione dati lib/data/activities.ts#getActivitiesWithOpenDaySpots() (query unica, no N+1, stesso pattern di getActivityAvailabilityByWeek). Filtro client-side come tutti gli altri filtri di SearchClient.tsx.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N503</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRAMA ONE Build Sprint 3 - Context object leggero (Ricerca-&gt;Dettaglio-&gt;Prenotazione)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Un correlationId e source='search' generati in Ricerca (LEGACY) propagano nel link alla scheda attivita e poi nel link 'Prenota ora'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /search -&gt; osserva il link della prima card risultato -&gt; clicca sulla card -&gt; osserva il link 'Prenota ora' nella scheda attivita</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il link della card contiene ?source=search e ?cid=&lt;uuid&gt;; la URL del dettaglio li contiene entrambi; il link 'Prenota ora' li propaga a sua volta verso /booking/[id]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automatizzato: tests/genitori/cerca.spec.ts, TC-N503. Scope minimo: solo source/correlationId, propagazione client-side via query string (ActivityCardHorizontal.tsx -&gt; DetailClient.tsx -&gt; BookingClient.tsx). Loggato server-side in actions.ts via logTelemetryEvent('booking_created'), nessun dato personale, nessuna persistenza (sistema eventi completo resta E11/Sprint 6, vedi lib/telemetry/correlation.ts).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N504</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRAMA ONE Build Sprint 3 - Ricerca NEXTGEN (filtro Giorni spot)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stesso filtro di TC-N502, nel pannello Ricerca NEXTGEN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login parent (NEXTGEN /nextgen/search)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen/search -&gt; apri il pannello 'Giorni spot' -&gt; attiva 'Solo attivita con Giorni spot disponibili' -&gt; 'Azzera'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il chip diventa azzerabile; 'Azzera' rimuove il filtro e torna a non essere presente nel DOM (stesso comportamento degli altri filtri NEXTGEN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automatizzato: tests/nextgen/search-filters-5-7.spec.ts, TC-N504. Stessa fonte dati di TC-N502 (getActivitiesWithOpenDaySpots), passata a SearchDiscoveryClient.tsx.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N505</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRAMA ONE Build Sprint 3 - Context object leggero (Ricerca NEXTGEN-&gt;Dettaglio-&gt;Prenotazione)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stesso concetto di TC-N503, con source='nextgen_search'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri /nextgen/search -&gt; osserva il link della prima card risultato -&gt; clicca -&gt; osserva il link 'Prenota ora'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il link della card contiene ?source=nextgen_search e ?cid=&lt;uuid&gt;; propagati fino al link 'Prenota ora'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automatizzato: tests/nextgen/search-filters-5-7.spec.ts, TC-N505. ActivityCard.tsx (NEXTGEN) prima non propagava alcun query param nel link al dettaglio - estensione additiva (props opzionali).</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -7986,7 +8064,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L419"/>
+  <dimension ref="A1:L423"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -21458,6 +21536,138 @@
       </c>
       <c r="L419" s="1" t="s">
         <v>2371</v>
+      </c>
+    </row>
+    <row r="420" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A420" s="1" t="s">
+        <v>2372</v>
+      </c>
+      <c r="B420" s="1" t="s">
+        <v>2373</v>
+      </c>
+      <c r="C420" s="1" t="s">
+        <v>2374</v>
+      </c>
+      <c r="D420" s="1" t="s">
+        <v>2375</v>
+      </c>
+      <c r="E420" s="1" t="s">
+        <v>2376</v>
+      </c>
+      <c r="F420" s="1" t="s">
+        <v>2377</v>
+      </c>
+      <c r="G420" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H420" s="1" t="str">
+        <f aca="false">IF(G420="BUG","BUG-"&amp;A420,IF(G420="FUNCTIONAL","FUNCTIONAL-"&amp;A420,""))</f>
+        <v/>
+      </c>
+      <c r="I420" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L420" s="1" t="s">
+        <v>2378</v>
+      </c>
+    </row>
+    <row r="421" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A421" s="1" t="s">
+        <v>2379</v>
+      </c>
+      <c r="B421" s="1" t="s">
+        <v>2380</v>
+      </c>
+      <c r="C421" s="1" t="s">
+        <v>2381</v>
+      </c>
+      <c r="D421" s="1" t="s">
+        <v>2375</v>
+      </c>
+      <c r="E421" s="1" t="s">
+        <v>2382</v>
+      </c>
+      <c r="F421" s="1" t="s">
+        <v>2383</v>
+      </c>
+      <c r="G421" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H421" s="1" t="str">
+        <f aca="false">IF(G421="BUG","BUG-"&amp;A421,IF(G421="FUNCTIONAL","FUNCTIONAL-"&amp;A421,""))</f>
+        <v/>
+      </c>
+      <c r="I421" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="L421" s="1" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="422" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A422" s="1" t="s">
+        <v>2385</v>
+      </c>
+      <c r="B422" s="1" t="s">
+        <v>2386</v>
+      </c>
+      <c r="C422" s="1" t="s">
+        <v>2387</v>
+      </c>
+      <c r="D422" s="1" t="s">
+        <v>2388</v>
+      </c>
+      <c r="E422" s="1" t="s">
+        <v>2389</v>
+      </c>
+      <c r="F422" s="1" t="s">
+        <v>2390</v>
+      </c>
+      <c r="G422" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H422" s="1" t="str">
+        <f aca="false">IF(G422="BUG","BUG-"&amp;A422,IF(G422="FUNCTIONAL","FUNCTIONAL-"&amp;A422,""))</f>
+        <v/>
+      </c>
+      <c r="I422" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L422" s="1" t="s">
+        <v>2391</v>
+      </c>
+    </row>
+    <row r="423" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A423" s="1" t="s">
+        <v>2392</v>
+      </c>
+      <c r="B423" s="1" t="s">
+        <v>2393</v>
+      </c>
+      <c r="C423" s="1" t="s">
+        <v>2394</v>
+      </c>
+      <c r="D423" s="1" t="s">
+        <v>2388</v>
+      </c>
+      <c r="E423" s="1" t="s">
+        <v>2395</v>
+      </c>
+      <c r="F423" s="1" t="s">
+        <v>2396</v>
+      </c>
+      <c r="G423" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H423" s="1" t="str">
+        <f aca="false">IF(G423="BUG","BUG-"&amp;A423,IF(G423="FUNCTIONAL","FUNCTIONAL-"&amp;A423,""))</f>
+        <v/>
+      </c>
+      <c r="I423" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="L423" s="1" t="s">
+        <v>2397</v>
       </c>
     </row>
   </sheetData>
@@ -21517,7 +21727,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>2372</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21525,13 +21735,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2373</v>
+        <v>2399</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2374</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21588,7 +21798,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -21600,11 +21810,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>2375</v>
+        <v>2401</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
test(sprint5): xlsx test matrix - righe TC-N600-606
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -907,7 +907,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L428"/>
+  <dimension ref="A1:L435"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11.83" customWidth="1" style="31" min="1" max="1"/>
@@ -21884,155 +21884,512 @@
       </c>
     </row>
     <row r="426">
-      <c r="A426" t="inlineStr">
+      <c r="A426" s="22" t="inlineStr">
         <is>
           <t>TC-508</t>
         </is>
       </c>
-      <c r="B426" t="inlineStr">
+      <c r="B426" s="22" t="inlineStr">
         <is>
           <t>TRAMA ONE Build Sprint 4 - Inbox prenotazioni Partner (risposta)</t>
         </is>
       </c>
-      <c r="C426" t="inlineStr">
+      <c r="C426" s="22" t="inlineStr">
         <is>
           <t>Il centro vede una prenotazione 'pending' nella nuova Inbox /center/prenotazioni e puo' accettarla</t>
         </is>
       </c>
-      <c r="D426" t="inlineStr">
+      <c r="D426" s="22" t="inlineStr">
         <is>
           <t>Login center_admin; supabase/seed-test-data.sql STEP 8 eseguito (prenotazione di test pending)</t>
         </is>
       </c>
-      <c r="E426" t="inlineStr">
+      <c r="E426" s="22" t="inlineStr">
         <is>
           <t>Apri /center/prenotazioni -&gt; individua la riga dell'attivita di test in 'Da rispondere' -&gt; clic 'Accetta'</t>
         </is>
       </c>
-      <c r="F426" t="inlineStr">
+      <c r="F426" s="22" t="inlineStr">
         <is>
           <t>La riga passa da badge 'Da rispondere' a 'Accettata'; bookings.partner_decision passa a 'accepted' e status a 'confirmed' (RLS: nuova policy UPDATE centro, migration_13)</t>
         </is>
       </c>
-      <c r="G426" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H426">
+      <c r="G426" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H426" s="22">
         <f>IF(G426="BUG","BUG-"&amp;A426,IF(G426="FUNCTIONAL","FUNCTIONAL-"&amp;A426,""))</f>
         <v/>
       </c>
-      <c r="I426" t="inlineStr">
+      <c r="I426" s="22" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="L426" t="inlineStr">
+      <c r="L426" s="22" t="inlineStr">
         <is>
           <t>Test automatizzato: tests/gestore/prenotazioni.spec.ts, TC-508. Nuova pagina app/center/prenotazioni/page.tsx + PrenotazioniClient.tsx, azione respondToBookingAction (app/actions/booking-response.ts), data layer lib/data/center-bookings.ts. WRAP non REPLACE (DEC-15/DEC-42): nessuna nuova tabella, colonne additive su bookings/booking_days.</t>
         </is>
       </c>
     </row>
     <row r="427">
-      <c r="A427" t="inlineStr">
+      <c r="A427" s="22" t="inlineStr">
         <is>
           <t>TC-509</t>
         </is>
       </c>
-      <c r="B427" t="inlineStr">
+      <c r="B427" s="22" t="inlineStr">
         <is>
           <t>TRAMA ONE Build Sprint 4 - Sync genitore su risposta Partner</t>
         </is>
       </c>
-      <c r="C427" t="inlineStr">
+      <c r="C427" s="22" t="inlineStr">
         <is>
           <t>Dopo l'accettazione del centro, il genitore vede la prenotazione come 'Confermata' in 'Le mie prenotazioni'</t>
         </is>
       </c>
-      <c r="D427" t="inlineStr">
+      <c r="D427" s="22" t="inlineStr">
         <is>
           <t>TC-508 gia eseguito (o comunque una prenotazione accepted per il genitore di test)</t>
         </is>
       </c>
-      <c r="E427" t="inlineStr">
+      <c r="E427" s="22" t="inlineStr">
         <is>
           <t>Login parent -&gt; apri /prenotazioni -&gt; individua la riga dell'attivita di test</t>
         </is>
       </c>
-      <c r="F427" t="inlineStr">
+      <c r="F427" s="22" t="inlineStr">
         <is>
           <t>Il badge stato mostra 'Confermata' (bookings.status = 'confirmed', propagato da partner_decision = 'accepted')</t>
         </is>
       </c>
-      <c r="G427" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H427">
+      <c r="G427" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H427" s="22">
         <f>IF(G427="BUG","BUG-"&amp;A427,IF(G427="FUNCTIONAL","FUNCTIONAL-"&amp;A427,""))</f>
         <v/>
       </c>
-      <c r="I427" t="inlineStr">
+      <c r="I427" s="22" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="L427" t="inlineStr">
+      <c r="L427" s="22" t="inlineStr">
         <is>
           <t>Test automatizzato: tests/gestore/prenotazioni.spec.ts, TC-509. lib/data/my-bookings.ts esteso con partnerDecision/partnerProposalNote/readByParent (additivo). Badge 'novita' (pallino rosso) su read_by_parent, stesso pattern di activity_inquiries.</t>
         </is>
       </c>
     </row>
     <row r="428">
-      <c r="A428" t="inlineStr">
+      <c r="A428" s="22" t="inlineStr">
         <is>
           <t>TC-510</t>
         </is>
       </c>
-      <c r="B428" t="inlineStr">
+      <c r="B428" s="22" t="inlineStr">
         <is>
           <t>TRAMA ONE Build Sprint 4 - Stato Inbox prenotazioni Partner</t>
         </is>
       </c>
-      <c r="C428" t="inlineStr">
+      <c r="C428" s="22" t="inlineStr">
         <is>
           <t>La pagina /center/prenotazioni non va mai in errore e mostra sempre le due sezioni con conteggio, anche senza prenotazioni in attesa</t>
         </is>
       </c>
-      <c r="D428" t="inlineStr">
+      <c r="D428" s="22" t="inlineStr">
         <is>
           <t>Login center_admin</t>
         </is>
       </c>
-      <c r="E428" t="inlineStr">
+      <c r="E428" s="22" t="inlineStr">
         <is>
           <t>Apri /center/prenotazioni</t>
         </is>
       </c>
-      <c r="F428" t="inlineStr">
+      <c r="F428" s="22" t="inlineStr">
         <is>
           <t>Sono visibili 'Da rispondere (N)' e 'Storico (N)' con N &gt;= 0, nessun errore a schermo</t>
         </is>
       </c>
-      <c r="G428" t="inlineStr">
-        <is>
-          <t>DA TESTARE</t>
-        </is>
-      </c>
-      <c r="H428">
+      <c r="G428" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H428" s="22">
         <f>IF(G428="BUG","BUG-"&amp;A428,IF(G428="FUNCTIONAL","FUNCTIONAL-"&amp;A428,""))</f>
         <v/>
       </c>
-      <c r="I428" t="inlineStr">
+      <c r="I428" s="22" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="L428" t="inlineStr">
+      <c r="L428" s="22" t="inlineStr">
         <is>
           <t>Test automatizzato: tests/gestore/prenotazioni.spec.ts, TC-510. Stesso principio dello stato vuoto gia' verificato per 'Le mie richieste' (TC-164).</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="22" t="inlineStr">
+        <is>
+          <t>TC-N600</t>
+        </is>
+      </c>
+      <c r="B429" s="22" t="inlineStr">
+        <is>
+          <t>TRAMA ONE Build Sprint 5 - CenterLead (Segnalazione centro, Genitore)</t>
+        </is>
+      </c>
+      <c r="C429" s="22" t="inlineStr">
+        <is>
+          <t>Genitore: una ricerca senza risultati mostra il punto di ingresso 'Suggerisci un centro'</t>
+        </is>
+      </c>
+      <c r="D429" s="22" t="inlineStr">
+        <is>
+          <t>Login parent; nessuna attivita/centro nel DB corrisponde alla query di ricerca usata nel test</t>
+        </is>
+      </c>
+      <c r="E429" s="22" t="inlineStr">
+        <is>
+          <t>Login genitore -&gt; apri /nextgen/search -&gt; cerca 'zzzznonexistentcenterzzzz9999' (query pensata per non trovare alcun risultato)</t>
+        </is>
+      </c>
+      <c r="F429" s="22" t="inlineStr">
+        <is>
+          <t>Compare il messaggio 'Nessuna attivita corrisponde ai filtri scelti.' insieme al punto di ingresso 'Non trovi il centro che cerchi?' (CTA verso il flusso di segnalazione)</t>
+        </is>
+      </c>
+      <c r="G429" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H429" s="22">
+        <f>IF(G429="BUG","BUG-"&amp;A429,IF(G429="FUNCTIONAL","FUNCTIONAL-"&amp;A429,""))</f>
+        <v/>
+      </c>
+      <c r="I429" s="22" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="L429" s="22" t="inlineStr">
+        <is>
+          <t>Test automatizzato: tests/one/center-leads.spec.ts, TC-N600 (gated su isRealDeployment: richiede un deploy con Supabase configurato e gli account di test parent/platform_admin). TRAMA ONE Build Sprint 5 - CenterLead: il genitore puo' segnalare un centro non ancora sulla piattaforma (referral). Riferimento: docs/trama-one/analysis/SPRINT_5_FEATURE_PRESERVATION_MATRIX.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="22" t="inlineStr">
+        <is>
+          <t>TC-N601</t>
+        </is>
+      </c>
+      <c r="B430" s="22" t="inlineStr">
+        <is>
+          <t>TRAMA ONE Build Sprint 5 - CenterLead (Invio segnalazione, Genitore)</t>
+        </is>
+      </c>
+      <c r="C430" s="22" t="inlineStr">
+        <is>
+          <t>Genitore: inviare una segnalazione crea SOLO una riga center_leads, mai un'attivita pubblica</t>
+        </is>
+      </c>
+      <c r="D430" s="22" t="inlineStr">
+        <is>
+          <t>Login parent; stessa ricerca senza risultati di TC-N600; migrazione additiva center_leads applicata</t>
+        </is>
+      </c>
+      <c r="E430" s="22" t="inlineStr">
+        <is>
+          <t>Da /nextgen/search (0 risultati) -&gt; 'Suggerisci un centro' -&gt; compila 'Nome del centro *' (nome univoco di test) e 'Citta / zona (indicativo)' -&gt; 'Invia segnalazione'</t>
+        </is>
+      </c>
+      <c r="F430" s="22" t="inlineStr">
+        <is>
+          <t>Messaggio di conferma 'Grazie! Abbiamo ricevuto la tua segnalazione'; viene creata una riga in center_leads; nessuna riga viene creata in activities (nessuna attivita pubblica fantasma)</t>
+        </is>
+      </c>
+      <c r="G430" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H430" s="22">
+        <f>IF(G430="BUG","BUG-"&amp;A430,IF(G430="FUNCTIONAL","FUNCTIONAL-"&amp;A430,""))</f>
+        <v/>
+      </c>
+      <c r="I430" s="22" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="L430" s="22" t="inlineStr">
+        <is>
+          <t>Test automatizzato: tests/one/center-leads.spec.ts, TC-N601 (gated su isRealDeployment: richiede un deploy con Supabase configurato e gli account di test parent/platform_admin). Serializzato con TC-N602/603/604/605 (stesso pattern gia' usato da tests/one/walkthrough-partner.spec.ts per TC-N414/415): crea una segnalazione reale che i test successivi leggono e mutano in sequenza.</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" s="22" t="inlineStr">
+        <is>
+          <t>TC-N602</t>
+        </is>
+      </c>
+      <c r="B431" s="22" t="inlineStr">
+        <is>
+          <t>TRAMA ONE Build Sprint 5 - CenterLead (I tuoi suggerimenti, Genitore)</t>
+        </is>
+      </c>
+      <c r="C431" s="22" t="inlineStr">
+        <is>
+          <t>Genitore: 'I tuoi suggerimenti' mostra la segnalazione appena inviata come 'Ricevuta'</t>
+        </is>
+      </c>
+      <c r="D431" s="22" t="inlineStr">
+        <is>
+          <t>TC-N601 gia' eseguito nella stessa run (segnalazione creata); login parent (stesso utente)</t>
+        </is>
+      </c>
+      <c r="E431" s="22" t="inlineStr">
+        <is>
+          <t>Login genitore -&gt; apri /center-leads</t>
+        </is>
+      </c>
+      <c r="F431" s="22" t="inlineStr">
+        <is>
+          <t>La riga corrispondente al nome del centro segnalato in TC-N601 mostra lo stato 'Ricevuta'</t>
+        </is>
+      </c>
+      <c r="G431" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H431" s="22">
+        <f>IF(G431="BUG","BUG-"&amp;A431,IF(G431="FUNCTIONAL","FUNCTIONAL-"&amp;A431,""))</f>
+        <v/>
+      </c>
+      <c r="I431" s="22" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="L431" s="22" t="inlineStr">
+        <is>
+          <t>Test automatizzato: tests/one/center-leads.spec.ts, TC-N602 (gated su isRealDeployment: richiede un deploy con Supabase configurato e gli account di test parent/platform_admin). Pagina /center-leads a sola lettura lato Genitore.</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="22" t="inlineStr">
+        <is>
+          <t>TC-N603</t>
+        </is>
+      </c>
+      <c r="B432" s="22" t="inlineStr">
+        <is>
+          <t>TRAMA ONE Build Sprint 5 - CenterLead (Coda Admin)</t>
+        </is>
+      </c>
+      <c r="C432" s="22" t="inlineStr">
+        <is>
+          <t>Admin: la coda 'Segnalazioni centri' mostra la nuova segnalazione tra le Attive</t>
+        </is>
+      </c>
+      <c r="D432" s="22" t="inlineStr">
+        <is>
+          <t>TC-N601 gia' eseguito (segnalazione creata); login platform_admin</t>
+        </is>
+      </c>
+      <c r="E432" s="22" t="inlineStr">
+        <is>
+          <t>Login admin -&gt; apri /admin/center-leads</t>
+        </is>
+      </c>
+      <c r="F432" s="22" t="inlineStr">
+        <is>
+          <t>La segnalazione con il nome di test compare tra le Attive con badge 'Nuova'</t>
+        </is>
+      </c>
+      <c r="G432" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H432" s="22">
+        <f>IF(G432="BUG","BUG-"&amp;A432,IF(G432="FUNCTIONAL","FUNCTIONAL-"&amp;A432,""))</f>
+        <v/>
+      </c>
+      <c r="I432" s="22" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="L432" s="22" t="inlineStr">
+        <is>
+          <t>Test automatizzato: tests/one/center-leads.spec.ts, TC-N603 (gated su isRealDeployment: richiede un deploy con Supabase configurato e gli account di test parent/platform_admin).</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" s="22" t="inlineStr">
+        <is>
+          <t>TC-N604</t>
+        </is>
+      </c>
+      <c r="B433" s="22" t="inlineStr">
+        <is>
+          <t>TRAMA ONE Build Sprint 5 - CenterLead (Coda Admin - Qualifica)</t>
+        </is>
+      </c>
+      <c r="C433" s="22" t="inlineStr">
+        <is>
+          <t>Admin: 'Qualifica' sposta lo stato della segnalazione a 'In valutazione'</t>
+        </is>
+      </c>
+      <c r="D433" s="22" t="inlineStr">
+        <is>
+          <t>TC-N603 gia' verificato (segnalazione visibile tra le Attive); login platform_admin</t>
+        </is>
+      </c>
+      <c r="E433" s="22" t="inlineStr">
+        <is>
+          <t>Apri /admin/center-leads -&gt; sulla card della segnalazione di test -&gt; 'Qualifica'</t>
+        </is>
+      </c>
+      <c r="F433" s="22" t="inlineStr">
+        <is>
+          <t>Il badge di stato della card passa a 'In valutazione'</t>
+        </is>
+      </c>
+      <c r="G433" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H433" s="22">
+        <f>IF(G433="BUG","BUG-"&amp;A433,IF(G433="FUNCTIONAL","FUNCTIONAL-"&amp;A433,""))</f>
+        <v/>
+      </c>
+      <c r="I433" s="22" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="L433" s="22" t="inlineStr">
+        <is>
+          <t>Test automatizzato: tests/one/center-leads.spec.ts, TC-N604 (gated su isRealDeployment: richiede un deploy con Supabase configurato e gli account di test parent/platform_admin).</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" s="22" t="inlineStr">
+        <is>
+          <t>TC-N605</t>
+        </is>
+      </c>
+      <c r="B434" s="22" t="inlineStr">
+        <is>
+          <t>TRAMA ONE Build Sprint 5 - CenterLead (Coda Admin - Claim)</t>
+        </is>
+      </c>
+      <c r="C434" s="22" t="inlineStr">
+        <is>
+          <t>Admin: il claim collega la segnalazione a un centro esistente e la sposta nello Storico come 'claimed'</t>
+        </is>
+      </c>
+      <c r="D434" s="22" t="inlineStr">
+        <is>
+          <t>TC-N604 gia' eseguito (segnalazione in 'In valutazione'); login platform_admin; almeno un centro reale selezionabile nella select di claim</t>
+        </is>
+      </c>
+      <c r="E434" s="22" t="inlineStr">
+        <is>
+          <t>Sulla card della segnalazione di test -&gt; seleziona un centro esistente dalla select -&gt; 'Claim'</t>
+        </is>
+      </c>
+      <c r="F434" s="22" t="inlineStr">
+        <is>
+          <t>La segnalazione risulta collegata al centro selezionato (claim, non creazione di un nuovo centro) e mostra 'Iscritto (claimed)', spostandosi nello Storico</t>
+        </is>
+      </c>
+      <c r="G434" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H434" s="22">
+        <f>IF(G434="BUG","BUG-"&amp;A434,IF(G434="FUNCTIONAL","FUNCTIONAL-"&amp;A434,""))</f>
+        <v/>
+      </c>
+      <c r="I434" s="22" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="L434" s="22" t="inlineStr">
+        <is>
+          <t>Test automatizzato: tests/one/center-leads.spec.ts, TC-N605 (gated su isRealDeployment: richiede un deploy con Supabase configurato e gli account di test parent/platform_admin). Il claim collega la segnalazione a un centro esistente, non crea nulla di nuovo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" s="22" t="inlineStr">
+        <is>
+          <t>TC-N606</t>
+        </is>
+      </c>
+      <c r="B435" s="22" t="inlineStr">
+        <is>
+          <t>TRAMA ONE Build Sprint 5 - CenterLead (Sicurezza/Autenticazione)</t>
+        </is>
+      </c>
+      <c r="C435" s="22" t="inlineStr">
+        <is>
+          <t>Un utente non autenticato che apre /center-leads o /admin/center-leads viene reindirizzato al login</t>
+        </is>
+      </c>
+      <c r="D435" s="22" t="inlineStr">
+        <is>
+          <t>Nessuna sessione attiva</t>
+        </is>
+      </c>
+      <c r="E435" s="22" t="inlineStr">
+        <is>
+          <t>Apri /center-leads senza login -&gt; poi apri /admin/center-leads senza login</t>
+        </is>
+      </c>
+      <c r="F435" s="22" t="inlineStr">
+        <is>
+          <t>Entrambe le route reindirizzano a /auth/login (comportamento proxy.ts invariato, non modificato da questa feature)</t>
+        </is>
+      </c>
+      <c r="G435" s="22" t="inlineStr">
+        <is>
+          <t>DA TESTARE</t>
+        </is>
+      </c>
+      <c r="H435" s="22">
+        <f>IF(G435="BUG","BUG-"&amp;A435,IF(G435="FUNCTIONAL","FUNCTIONAL-"&amp;A435,""))</f>
+        <v/>
+      </c>
+      <c r="I435" s="22" t="inlineStr">
+        <is>
+          <t>Bassa</t>
+        </is>
+      </c>
+      <c r="L435" s="22" t="inlineStr">
+        <is>
+          <t>Test automatizzato: tests/one/center-leads.spec.ts, TC-N606 (gated su isRealDeployment: richiede un deploy con Supabase configurato e gli account di test parent/platform_admin).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(sprint6): aggiorna matrice xlsx con TC-N609 (feature flag expiry)
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3830" uniqueCount="2497">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3839" uniqueCount="2504">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -7510,6 +7510,27 @@
   </si>
   <si>
     <t xml:space="preserve">Test automatizzato: tests/one/capacity.spec.ts, TC-N608 (gated su isRealDeployment: richiede la prenotazione creata e accettata in TC-N607 nella stessa run). Verifica il fix del bug per cui cancelBookingAction non rilasciava mai booking_weeks.capacity_decremented ne' activity_weeks.spots_left.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N609</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRAMA ONE Build Sprint 6 - Feature flag override expiry (Admin)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin crea, vede lo stato (attivo/in scadenza/scaduto) e poi elimina un override di feature flag da /admin/feature-flags</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deploy reale con Supabase configurato, migration_07_feature_flags_foundation.sql applicata, account platform_admin di test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Admin apre /admin/feature-flags, seleziona il flag TRAMA_ONE_ENABLED, aggiunge un override di test con scope 'user' e un UUID inventato (mai un utente reale, per non toccare l'eventuale override globale reale gia' usato per abilitare le route /one), verifica che appaia con badge 'Senza scadenza', poi lo elimina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'override compare nella lista con lo stato corretto; dopo l'eliminazione la riga sparisce. Verifica anche indirettamente il bug fix di TC-N409 (Gate C, ottava ondata): un override scaduto ora e' visibile con badge 'Scaduto'/'In scadenza (&lt;72h)' invece di fallire silenziosamente senza alcuna traccia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automatizzato: tests/one/feature-flags.spec.ts, TC-N609 (gated su isRealDeployment). Lo stesso file contiene anche ~15 unit test 'no browser' (findRecentlyExpiredMatchingOverride, computeOverrideStatus) eseguibili senza browser reale -- gia' verificati passanti in locale (56/56 pass).</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -8349,7 +8370,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L437"/>
+  <dimension ref="A1:L438"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -22021,7 +22042,7 @@
         <v>2409</v>
       </c>
     </row>
-    <row r="426" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="426" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A426" s="1" t="s">
         <v>2410</v>
       </c>
@@ -22054,7 +22075,7 @@
         <v>2416</v>
       </c>
     </row>
-    <row r="427" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="427" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A427" s="1" t="s">
         <v>2417</v>
       </c>
@@ -22087,7 +22108,7 @@
         <v>2423</v>
       </c>
     </row>
-    <row r="428" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="428" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A428" s="1" t="s">
         <v>2424</v>
       </c>
@@ -22120,7 +22141,7 @@
         <v>2430</v>
       </c>
     </row>
-    <row r="429" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="429" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A429" s="1" t="s">
         <v>2431</v>
       </c>
@@ -22153,7 +22174,7 @@
         <v>2437</v>
       </c>
     </row>
-    <row r="430" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="430" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A430" s="1" t="s">
         <v>2438</v>
       </c>
@@ -22186,7 +22207,7 @@
         <v>2444</v>
       </c>
     </row>
-    <row r="431" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="431" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A431" s="1" t="s">
         <v>2445</v>
       </c>
@@ -22219,7 +22240,7 @@
         <v>2451</v>
       </c>
     </row>
-    <row r="432" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="432" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A432" s="1" t="s">
         <v>2452</v>
       </c>
@@ -22252,7 +22273,7 @@
         <v>2458</v>
       </c>
     </row>
-    <row r="433" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="433" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A433" s="1" t="s">
         <v>2459</v>
       </c>
@@ -22285,7 +22306,7 @@
         <v>2465</v>
       </c>
     </row>
-    <row r="434" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="434" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A434" s="1" t="s">
         <v>2466</v>
       </c>
@@ -22318,7 +22339,7 @@
         <v>2472</v>
       </c>
     </row>
-    <row r="435" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="435" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A435" s="1" t="s">
         <v>2473</v>
       </c>
@@ -22351,7 +22372,7 @@
         <v>2478</v>
       </c>
     </row>
-    <row r="436" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="436" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A436" s="10" t="s">
         <v>2479</v>
       </c>
@@ -22384,7 +22405,7 @@
         <v>2485</v>
       </c>
     </row>
-    <row r="437" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="437" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A437" s="10" t="s">
         <v>2486</v>
       </c>
@@ -22415,6 +22436,39 @@
       </c>
       <c r="L437" s="11" t="s">
         <v>2492</v>
+      </c>
+    </row>
+    <row r="438" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A438" s="10" t="s">
+        <v>2493</v>
+      </c>
+      <c r="B438" s="10" t="s">
+        <v>2494</v>
+      </c>
+      <c r="C438" s="10" t="s">
+        <v>2495</v>
+      </c>
+      <c r="D438" s="10" t="s">
+        <v>2496</v>
+      </c>
+      <c r="E438" s="10" t="s">
+        <v>2497</v>
+      </c>
+      <c r="F438" s="10" t="s">
+        <v>2498</v>
+      </c>
+      <c r="G438" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H438" s="10" t="str">
+        <f aca="false">IF(G438="BUG","BUG-"&amp;A438,IF(G438="FUNCTIONAL","FUNCTIONAL-"&amp;A438,""))</f>
+        <v/>
+      </c>
+      <c r="I438" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="L438" s="11" t="s">
+        <v>2499</v>
       </c>
     </row>
   </sheetData>
@@ -22474,7 +22528,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>2493</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22482,13 +22536,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2494</v>
+        <v>2501</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2495</v>
+        <v>2502</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22545,7 +22599,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -22557,11 +22611,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>2496</v>
+        <v>2503</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
test(sprint6): aggiorna matrice xlsx con TC-N610 (email fire-and-forget)
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3839" uniqueCount="2504">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3848" uniqueCount="2511">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -7531,6 +7531,27 @@
   </si>
   <si>
     <t xml:space="preserve">Test automatizzato: tests/one/feature-flags.spec.ts, TC-N609 (gated su isRealDeployment). Lo stesso file contiene anche ~15 unit test 'no browser' (findRecentlyExpiredMatchingOverride, computeOverrideStatus) eseguibili senza browser reale -- gia' verificati passanti in locale (56/56 pass).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N610</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRAMA ONE Build Sprint 6 - Email fire-and-forget (stato di consegna, Gestore-&gt;Genitore)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accettare una prenotazione registra sempre un email_delivery_status noto su bookings (mai piu' silenzioso)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deploy reale con Supabase configurato, migration_19_bookings_email_delivery_status.sql applicata, SUPABASE_SERVICE_ROLE_KEY in .env.test, attivita' di test "[TEST] Attivita' BuddyKids" seminata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il genitore di test crea una prenotazione reale a settimana intera; il gestore di test la accetta da /center/prenotazioni (che internamente invoca notifyParentOfBookingResponse -&gt; sendEmail, con retry minimo se il primo tentativo fallisce)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bookings.email_delivery_status viene sempre valorizzato con uno dei 4 valori noti (sent/failed/not_configured/no_recipient), mai lasciato null come prima di questa migrazione, e bookings.email_delivery_attempted_at viene registrato (verificato via client Supabase service_role, nessuna UI mostra questo dettaglio infrastrutturale)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automatizzato: tests/one/email-delivery.spec.ts, TC-N610 (gated su isRealDeployment). Chiude il debito P2 'email fire-and-forget' (SPRINT_GOVERNANCE.md riga 151, DEC-49): prima nessuno stato di consegna era persistito e un fallimento di invio spariva senza traccia.</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -8370,7 +8391,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L438"/>
+  <dimension ref="A1:L439"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -22469,6 +22490,39 @@
       </c>
       <c r="L438" s="11" t="s">
         <v>2499</v>
+      </c>
+    </row>
+    <row r="439" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A439" s="10" t="s">
+        <v>2500</v>
+      </c>
+      <c r="B439" s="10" t="s">
+        <v>2501</v>
+      </c>
+      <c r="C439" s="10" t="s">
+        <v>2502</v>
+      </c>
+      <c r="D439" s="10" t="s">
+        <v>2503</v>
+      </c>
+      <c r="E439" s="10" t="s">
+        <v>2504</v>
+      </c>
+      <c r="F439" s="10" t="s">
+        <v>2505</v>
+      </c>
+      <c r="G439" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H439" s="10" t="str">
+        <f aca="false">IF(G439="BUG","BUG-"&amp;A439,IF(G439="FUNCTIONAL","FUNCTIONAL-"&amp;A439,""))</f>
+        <v/>
+      </c>
+      <c r="I439" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="L439" s="11" t="s">
+        <v>2506</v>
       </c>
     </row>
   </sheetData>
@@ -22528,7 +22582,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>2500</v>
+        <v>2507</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22536,13 +22590,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2501</v>
+        <v>2508</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2502</v>
+        <v>2509</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22599,7 +22653,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -22611,11 +22665,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>2503</v>
+        <v>2510</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
test(sprint6): aggiorna matrice xlsx con TC-N611 (Command Center Admin)
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3848" uniqueCount="2511">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3857" uniqueCount="2518">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -7552,6 +7552,27 @@
   </si>
   <si>
     <t xml:space="preserve">Test automatizzato: tests/one/email-delivery.spec.ts, TC-N610 (gated su isRealDeployment). Chiude il debito P2 'email fire-and-forget' (SPRINT_GOVERNANCE.md riga 151, DEC-49): prima nessuno stato di consegna era persistito e un fallimento di invio spariva senza traccia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N611</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRAMA ONE Build Sprint 6 - Command Center Admin (E08)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin: /admin/one mostra le code operative aggregate (onboarding/prenotazioni/richieste/centri-lead/certificazioni/feedback-beta/feature-flag) con priorita' ed etichette, senza rimuovere le pagine per dominio esistenti</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deploy reale con Supabase configurato, account platform_admin di test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Admin apre /admin/one</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sono visibili 7 code operative con etichetta e conteggio (Onboarding, Prenotazioni, Richieste, Centri-lead, Certificazioni, Feedback BETA, Feature flag), un riepilogo testuale in cima, e la sezione Walkthrough preesistente resta visibile sotto. Ogni coda linka alla pagina Admin per dominio gia' esistente (nessuna sostituzione)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automatizzato: tests/one/command-center.spec.ts, TC-N611 (gated su isRealDeployment) + 7 unit test 'no browser' su lib/command-center/priority.ts (computeQueuePriority/compareQueuesByPriority), gia' verificati passanti in locale (16/16 pass, incluso mobile-chrome).</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -8391,7 +8412,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L439"/>
+  <dimension ref="A1:L440"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -22492,7 +22513,7 @@
         <v>2499</v>
       </c>
     </row>
-    <row r="439" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="439" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A439" s="10" t="s">
         <v>2500</v>
       </c>
@@ -22523,6 +22544,39 @@
       </c>
       <c r="L439" s="11" t="s">
         <v>2506</v>
+      </c>
+    </row>
+    <row r="440" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A440" s="10" t="s">
+        <v>2507</v>
+      </c>
+      <c r="B440" s="10" t="s">
+        <v>2508</v>
+      </c>
+      <c r="C440" s="10" t="s">
+        <v>2509</v>
+      </c>
+      <c r="D440" s="10" t="s">
+        <v>2510</v>
+      </c>
+      <c r="E440" s="10" t="s">
+        <v>2511</v>
+      </c>
+      <c r="F440" s="10" t="s">
+        <v>2512</v>
+      </c>
+      <c r="G440" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H440" s="10" t="str">
+        <f aca="false">IF(G440="BUG","BUG-"&amp;A440,IF(G440="FUNCTIONAL","FUNCTIONAL-"&amp;A440,""))</f>
+        <v/>
+      </c>
+      <c r="I440" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="L440" s="11" t="s">
+        <v>2513</v>
       </c>
     </row>
   </sheetData>
@@ -22582,7 +22636,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>2507</v>
+        <v>2514</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22590,13 +22644,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2508</v>
+        <v>2515</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2509</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22653,7 +22707,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -22665,11 +22719,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>2510</v>
+        <v>2517</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
test(sprint6): xlsx TC-N612 (E11)
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3857" uniqueCount="2518">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3866" uniqueCount="2525">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -7573,6 +7573,27 @@
   </si>
   <si>
     <t xml:space="preserve">Test automatizzato: tests/one/command-center.spec.ts, TC-N611 (gated su isRealDeployment) + 7 unit test 'no browser' su lib/command-center/priority.ts (computeQueuePriority/compareQueuesByPriority), gia' verificati passanti in locale (16/16 pass, incluso mobile-chrome).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N612</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRAMA ONE Build Sprint 6 - Eventi analytics con correlationId (E11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visitare /one registra un evento product_events persistito, correlato da correlationId, senza mai includere dati personali</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deploy reale con Supabase configurato, migration_20_product_events.sql applicata, TRAMA_ONE_ENABLED attivo per l'utente di test, SUPABASE_SERVICE_ROLE_KEY in .env.test (RLS select su product_events e' ristretta a is_platform_admin())</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il genitore di test effettua login e visita /one (il layout genera un correlationId ed emette one_route_access sia via logTelemetryEvent, invariato, sia via persistProductEvent verso product_events)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compare in product_events una riga con event_name="one_route_access" e correlation_id valorizzato (mai null); nessuna colonna della tabella contiene nome/email/altri dati personali per costruzione (whitelist KNOWN_PRODUCT_EVENTS + shape fissa event_name/correlation_id/tenant/role/detail)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automatizzato: tests/one/product-events.spec.ts, TC-N612 (gated su isRealDeployment) + 4 unit test 'no browser' su lib/telemetry/known-events.ts (KNOWN_PRODUCT_EVENTS), gia' verificati passanti in locale (8/8 pass, incluso mobile-chrome).</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -8412,7 +8433,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L440"/>
+  <dimension ref="A1:L441"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -22546,7 +22567,7 @@
         <v>2506</v>
       </c>
     </row>
-    <row r="440" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="440" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A440" s="10" t="s">
         <v>2507</v>
       </c>
@@ -22577,6 +22598,39 @@
       </c>
       <c r="L440" s="11" t="s">
         <v>2513</v>
+      </c>
+    </row>
+    <row r="441" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A441" s="10" t="s">
+        <v>2514</v>
+      </c>
+      <c r="B441" s="10" t="s">
+        <v>2515</v>
+      </c>
+      <c r="C441" s="10" t="s">
+        <v>2516</v>
+      </c>
+      <c r="D441" s="10" t="s">
+        <v>2517</v>
+      </c>
+      <c r="E441" s="10" t="s">
+        <v>2518</v>
+      </c>
+      <c r="F441" s="10" t="s">
+        <v>2519</v>
+      </c>
+      <c r="G441" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H441" s="10" t="str">
+        <f aca="false">IF(G441="BUG","BUG-"&amp;A441,IF(G441="FUNCTIONAL","FUNCTIONAL-"&amp;A441,""))</f>
+        <v/>
+      </c>
+      <c r="I441" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="L441" s="11" t="s">
+        <v>2520</v>
       </c>
     </row>
   </sheetData>
@@ -22636,7 +22690,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>2514</v>
+        <v>2521</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22644,13 +22698,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2515</v>
+        <v>2522</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2516</v>
+        <v>2523</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22707,7 +22761,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -22719,11 +22773,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>2517</v>
+        <v>2524</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
test(sprint6): xlsx TC-N613 (hardening walkthrough)
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3866" uniqueCount="2525">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3875" uniqueCount="2532">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -7594,6 +7594,27 @@
   </si>
   <si>
     <t xml:space="preserve">Test automatizzato: tests/one/product-events.spec.ts, TC-N612 (gated su isRealDeployment) + 4 unit test 'no browser' su lib/telemetry/known-events.ts (KNOWN_PRODUCT_EVENTS), gia' verificati passanti in locale (8/8 pass, incluso mobile-chrome).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N613</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRAMA ONE Build Sprint 6 - Hardening Walkthrough (funnel/drop-off, microcopy, accessibilita, performance)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il Command Center Admin mostra il funnel Walkthrough (raggiunti/abbandono per step) e il conteggio riavvii; il componente WalkthroughCard e' accessibile (aria-live, aria-describedby, role=region) e usa microcopy piu' chiara</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deploy reale con Supabase configurato, account platform_admin di test per la vista Admin; account parent di test per WalkthroughCard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin apre /admin/one e legge la tabella funnel Walkthrough; Genitore apre /one e interagisce con Inizia/Continua/Salta per ora/Ricomincia il percorso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La tabella mostra colonne Raggiunti e Abbandono vs step prec. coerenti (nessun valore negativo, nessuna divisione per zero); il paragrafo informativo mostra il conteggio riavvii o "N/D" se migration_20 non applicata; i pulsanti Inizia/Continua restano individuabili per nome accessibile esatto (nessuna regressione su TC-N414/N415); lo screen reader annuncia il cambio di step (aria-live) senza richiedere refresh manuale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automatizzato: tests/one/walkthrough-funnel.spec.ts, TC-N613 (gated su isRealDeployment) + 6 unit test 'no browser' su lib/walkthrough/funnel.ts (computeWalkthroughFunnel), gia' verificati passanti in locale (12/12 pass, incluso mobile-chrome). Nessuna regressione: tests/one/walkthrough-partner.spec.ts (TC-N414/N415) continua a usare getByRole con nome accessibile invariato (Inizia/Continua).</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -8433,7 +8454,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L441"/>
+  <dimension ref="A1:L442"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -22600,7 +22621,7 @@
         <v>2513</v>
       </c>
     </row>
-    <row r="441" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="441" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A441" s="10" t="s">
         <v>2514</v>
       </c>
@@ -22631,6 +22652,39 @@
       </c>
       <c r="L441" s="11" t="s">
         <v>2520</v>
+      </c>
+    </row>
+    <row r="442" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A442" s="10" t="s">
+        <v>2521</v>
+      </c>
+      <c r="B442" s="10" t="s">
+        <v>2522</v>
+      </c>
+      <c r="C442" s="10" t="s">
+        <v>2523</v>
+      </c>
+      <c r="D442" s="10" t="s">
+        <v>2524</v>
+      </c>
+      <c r="E442" s="10" t="s">
+        <v>2525</v>
+      </c>
+      <c r="F442" s="10" t="s">
+        <v>2526</v>
+      </c>
+      <c r="G442" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H442" s="10" t="str">
+        <f aca="false">IF(G442="BUG","BUG-"&amp;A442,IF(G442="FUNCTIONAL","FUNCTIONAL-"&amp;A442,""))</f>
+        <v/>
+      </c>
+      <c r="I442" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="L442" s="11" t="s">
+        <v>2527</v>
       </c>
     </row>
   </sheetData>
@@ -22690,7 +22744,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>2521</v>
+        <v>2528</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22698,13 +22752,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2522</v>
+        <v>2529</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2523</v>
+        <v>2530</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22761,7 +22815,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -22773,11 +22827,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>2524</v>
+        <v>2531</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
docs(controlled-beta): xlsx test matrix - aggiornare TC-N414/N415 per il nuovo Spotlight, aggiungere TC-N416/TC-N417
TC-N414/TC-N415 riscritte per riflettere lo scenario reale (Spotlight
su /center/activities, non piu' WalkthroughCard su /center/one).
TC-N416 nuovo: avanzamento via click reale. TC-N417: unit test puri
lib/spotlight/position.ts (13/13 assert, no browser). Recalc
LibreOffice: 0 errori su 441 formule.
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3875" uniqueCount="2532">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3893" uniqueCount="2547">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -7080,31 +7080,34 @@
     <t xml:space="preserve">TC-N414</t>
   </si>
   <si>
-    <t xml:space="preserve">TRAMA ONE - Walkthrough attivita (Partner, Sprint 2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Il gestore vede in /center/one il percorso guidato 'Pubblica la tua prima attivita' con il primo step ('Crea l'attivita') pronto da iniziare</t>
+    <t xml:space="preserve">TRAMA ONE - Product Walkthrough Spotlight reale (Controlled Beta, S7-14)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il gestore vede in /center/activities lo Spotlight reale (overlay+cutout+popover ancorato) sul pulsante '+ Nuova attivita', non piu' una card testuale scollegata in /center/one</t>
   </si>
   <si>
     <t xml:space="preserve">Login center_admin; flag TRAMA_ONE_ENABLED attivo per l'utente di test (override, vedi DEC-34)</t>
   </si>
   <si>
-    <t xml:space="preserve">La card del percorso e' visibile con titolo 'Pubblica la tua prima attivita', il primo step 'Crea l'attivita' e il bottone 'Inizia'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test automatizzato: tests/one/walkthrough-partner.spec.ts, TC-N414. Riusa il motore Walkthrough generico gia' verificato in Sprint 1 (nessuna modifica al motore, solo nuova voce in lib/walkthrough/registry.ts).</t>
+    <t xml:space="preserve">Login gestore -&gt; apri /center/activities</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il pulsante '+ Nuova attivita' ha l'attributo data-spotlight="create_activity"; e' visibile un dialog (role=dialog) ancorato ad esso con titolo 'Crea l'attivita', 'Passo 1 di 6', la descrizione dello step e il bottone 'Inizia'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automatizzato: tests/one/walkthrough-partner.spec.ts, TC-N414 (riscritto per il gate Controlled Beta S7-14/DEC-60: la WalkthroughCard su /center/one e' stata rimossa, il vero Spotlight vive ora sulle pagine reali, montato in app/center/layout.tsx).</t>
   </si>
   <si>
     <t xml:space="preserve">TC-N415</t>
   </si>
   <si>
-    <t xml:space="preserve">Avviare il primo step del percorso attivita lo marca come iniziato in modo persistente (tutorial_progress), non solo nello stato locale del componente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Login gestore -&gt; apri /center/one -&gt; 'Inizia' -&gt; ricarica la pagina</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dopo il reload il bottone mostra 'Continua' (non torna a 'Inizia'), a conferma che lo stato e' scritto su Supabase via startWalkthroughStepAction e non solo nel componente client</t>
+    <t xml:space="preserve">Avviare lo step ('Inizia') lo marca 'in_progress' in modo persistente (tutorial_progress), non solo nello stato locale del componente Spotlight</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login gestore -&gt; apri /center/activities -&gt; click 'Inizia' nel popover -&gt; ricarica la pagina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il popover mostra il messaggio "Fatto? Clicca l'elemento evidenziato per continuare."; dopo il reload lo stesso messaggio ricompare (conferma scrittura reale via startWalkthroughStepAction, non solo useState)</t>
   </si>
   <si>
     <t xml:space="preserve">Test automatizzato: tests/one/walkthrough-partner.spec.ts, TC-N415.</t>
@@ -7615,6 +7618,48 @@
   </si>
   <si>
     <t xml:space="preserve">Test automatizzato: tests/one/walkthrough-funnel.spec.ts, TC-N613 (gated su isRealDeployment) + 6 unit test 'no browser' su lib/walkthrough/funnel.ts (computeWalkthroughFunnel), gia' verificati passanti in locale (12/12 pass, incluso mobile-chrome). Nessuna regressione: tests/one/walkthrough-partner.spec.ts (TC-N414/N415) continua a usare getByRole con nome accessibile invariato (Inizia/Continua).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N416</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Completare lo step con un click GENUINO sull'elemento reale dell'interfaccia (non un bottone 'Continua' dentro il tour) fa avanzare il percorso allo step successivo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login center_admin; flag TRAMA_ONE_ENABLED attivo; step 'create_activity' gia' in_progress (segue TC-N415)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login gestore -&gt; apri /center/activities -&gt; click sul VERO pulsante '+ Nuova attivita' (elemento con data-spotlight, non un bottone del tour)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La navigazione reale avviene (URL -&gt; /center/activities/new); lo step 'create_activity' risulta completato e il percorso avanza a 'configure_weeks' — poiche' quel target non esiste sulla pagina di creazione, lo Spotlight mostra il badge 'target non trovato' col titolo 'Configura le settimane' invece di restare ancorato al pulsante ormai scomparso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automatizzato: tests/one/walkthrough-partner.spec.ts, TC-N416 (nuovo per il gate Controlled Beta S7-14/DEC-60 — verifica il meccanismo di avanzamento via click reale, cuore del nuovo motore Spotlight rispetto al vecchio WalkthroughCard).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N417</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRAMA ONE - Spotlight: unit test puri lib/spotlight/position.ts [no browser]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">computePopoverPosition/computeCutoutRect/matchesSpotlightRoute producono i placement/rect/match attesi per i casi noti (spazio sopra/sotto, clamp orizzontale, wildcard singola/centrale/globale)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nessuna (funzioni pure, nessun browser/DB richiesto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">npx playwright test tests/one/spotlight-position.spec.ts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13/13 assert passano: placement top/bottom coerente con lo spazio disponibile, cutout con padding corretto, matchesSpotlightRoute coerente per pattern esatti/prefisso/prefisso+suffisso/wildcard globale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PASS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automatizzato eseguito nel sandbox Claude (26/26 passed su chromium+mobile-chrome, nessun browser reale richiesto): tests/one/spotlight-position.spec.ts.</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -8454,7 +8499,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L442"/>
+  <dimension ref="A1:L444"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -21810,10 +21855,10 @@
         <v>2351</v>
       </c>
       <c r="E416" s="1" t="s">
-        <v>2234</v>
+        <v>2352</v>
       </c>
       <c r="F416" s="1" t="s">
-        <v>2352</v>
+        <v>2353</v>
       </c>
       <c r="G416" s="1" t="s">
         <v>74</v>
@@ -21826,27 +21871,27 @@
         <v>65</v>
       </c>
       <c r="L416" s="1" t="s">
-        <v>2353</v>
+        <v>2354</v>
       </c>
     </row>
     <row r="417" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A417" s="1" t="s">
-        <v>2354</v>
+        <v>2355</v>
       </c>
       <c r="B417" s="1" t="s">
         <v>2349</v>
       </c>
       <c r="C417" s="1" t="s">
-        <v>2355</v>
+        <v>2356</v>
       </c>
       <c r="D417" s="1" t="s">
         <v>2351</v>
       </c>
       <c r="E417" s="1" t="s">
-        <v>2356</v>
+        <v>2357</v>
       </c>
       <c r="F417" s="1" t="s">
-        <v>2357</v>
+        <v>2358</v>
       </c>
       <c r="G417" s="1" t="s">
         <v>74</v>
@@ -21859,27 +21904,27 @@
         <v>65</v>
       </c>
       <c r="L417" s="1" t="s">
-        <v>2358</v>
+        <v>2359</v>
       </c>
     </row>
     <row r="418" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A418" s="1" t="s">
-        <v>2359</v>
+        <v>2360</v>
       </c>
       <c r="B418" s="1" t="s">
-        <v>2360</v>
+        <v>2361</v>
       </c>
       <c r="C418" s="1" t="s">
-        <v>2361</v>
+        <v>2362</v>
       </c>
       <c r="D418" s="1" t="s">
-        <v>2362</v>
+        <v>2363</v>
       </c>
       <c r="E418" s="1" t="s">
-        <v>2363</v>
+        <v>2364</v>
       </c>
       <c r="F418" s="1" t="s">
-        <v>2364</v>
+        <v>2365</v>
       </c>
       <c r="G418" s="1" t="s">
         <v>74</v>
@@ -21892,27 +21937,27 @@
         <v>56</v>
       </c>
       <c r="L418" s="1" t="s">
-        <v>2365</v>
+        <v>2366</v>
       </c>
     </row>
     <row r="419" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A419" s="1" t="s">
-        <v>2366</v>
+        <v>2367</v>
       </c>
       <c r="B419" s="1" t="s">
-        <v>2360</v>
+        <v>2361</v>
       </c>
       <c r="C419" s="1" t="s">
-        <v>2367</v>
+        <v>2368</v>
       </c>
       <c r="D419" s="1" t="s">
-        <v>2368</v>
+        <v>2369</v>
       </c>
       <c r="E419" s="1" t="s">
-        <v>2369</v>
+        <v>2370</v>
       </c>
       <c r="F419" s="1" t="s">
-        <v>2370</v>
+        <v>2371</v>
       </c>
       <c r="G419" s="1" t="s">
         <v>74</v>
@@ -21925,27 +21970,27 @@
         <v>56</v>
       </c>
       <c r="L419" s="1" t="s">
-        <v>2371</v>
+        <v>2372</v>
       </c>
     </row>
     <row r="420" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A420" s="1" t="s">
-        <v>2372</v>
+        <v>2373</v>
       </c>
       <c r="B420" s="1" t="s">
-        <v>2373</v>
+        <v>2374</v>
       </c>
       <c r="C420" s="1" t="s">
-        <v>2374</v>
+        <v>2375</v>
       </c>
       <c r="D420" s="1" t="s">
-        <v>2375</v>
+        <v>2376</v>
       </c>
       <c r="E420" s="1" t="s">
-        <v>2376</v>
+        <v>2377</v>
       </c>
       <c r="F420" s="1" t="s">
-        <v>2377</v>
+        <v>2378</v>
       </c>
       <c r="G420" s="1" t="s">
         <v>74</v>
@@ -21958,27 +22003,27 @@
         <v>56</v>
       </c>
       <c r="L420" s="1" t="s">
-        <v>2378</v>
+        <v>2379</v>
       </c>
     </row>
     <row r="421" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A421" s="1" t="s">
-        <v>2379</v>
+        <v>2380</v>
       </c>
       <c r="B421" s="1" t="s">
-        <v>2380</v>
+        <v>2381</v>
       </c>
       <c r="C421" s="1" t="s">
-        <v>2381</v>
+        <v>2382</v>
       </c>
       <c r="D421" s="1" t="s">
-        <v>2375</v>
+        <v>2376</v>
       </c>
       <c r="E421" s="1" t="s">
-        <v>2382</v>
+        <v>2383</v>
       </c>
       <c r="F421" s="1" t="s">
-        <v>2383</v>
+        <v>2384</v>
       </c>
       <c r="G421" s="1" t="s">
         <v>74</v>
@@ -21991,27 +22036,27 @@
         <v>65</v>
       </c>
       <c r="L421" s="1" t="s">
-        <v>2384</v>
+        <v>2385</v>
       </c>
     </row>
     <row r="422" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A422" s="1" t="s">
-        <v>2385</v>
+        <v>2386</v>
       </c>
       <c r="B422" s="1" t="s">
-        <v>2386</v>
+        <v>2387</v>
       </c>
       <c r="C422" s="1" t="s">
-        <v>2387</v>
+        <v>2388</v>
       </c>
       <c r="D422" s="1" t="s">
-        <v>2388</v>
+        <v>2389</v>
       </c>
       <c r="E422" s="1" t="s">
-        <v>2389</v>
+        <v>2390</v>
       </c>
       <c r="F422" s="1" t="s">
-        <v>2390</v>
+        <v>2391</v>
       </c>
       <c r="G422" s="1" t="s">
         <v>74</v>
@@ -22024,27 +22069,27 @@
         <v>56</v>
       </c>
       <c r="L422" s="1" t="s">
-        <v>2391</v>
+        <v>2392</v>
       </c>
     </row>
     <row r="423" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A423" s="1" t="s">
-        <v>2392</v>
+        <v>2393</v>
       </c>
       <c r="B423" s="1" t="s">
-        <v>2393</v>
+        <v>2394</v>
       </c>
       <c r="C423" s="1" t="s">
-        <v>2394</v>
+        <v>2395</v>
       </c>
       <c r="D423" s="1" t="s">
-        <v>2388</v>
+        <v>2389</v>
       </c>
       <c r="E423" s="1" t="s">
-        <v>2395</v>
+        <v>2396</v>
       </c>
       <c r="F423" s="1" t="s">
-        <v>2396</v>
+        <v>2397</v>
       </c>
       <c r="G423" s="1" t="s">
         <v>74</v>
@@ -22057,27 +22102,27 @@
         <v>65</v>
       </c>
       <c r="L423" s="1" t="s">
-        <v>2397</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="424" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A424" s="1" t="s">
-        <v>2398</v>
+        <v>2399</v>
       </c>
       <c r="B424" s="1" t="s">
-        <v>2399</v>
+        <v>2400</v>
       </c>
       <c r="C424" s="1" t="s">
-        <v>2400</v>
+        <v>2401</v>
       </c>
       <c r="D424" s="1" t="s">
-        <v>2388</v>
+        <v>2389</v>
       </c>
       <c r="E424" s="1" t="s">
-        <v>2401</v>
+        <v>2402</v>
       </c>
       <c r="F424" s="1" t="s">
-        <v>2402</v>
+        <v>2403</v>
       </c>
       <c r="G424" s="1" t="s">
         <v>74</v>
@@ -22090,27 +22135,27 @@
         <v>56</v>
       </c>
       <c r="L424" s="1" t="s">
-        <v>2403</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="425" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A425" s="1" t="s">
-        <v>2404</v>
+        <v>2405</v>
       </c>
       <c r="B425" s="1" t="s">
-        <v>2405</v>
+        <v>2406</v>
       </c>
       <c r="C425" s="1" t="s">
-        <v>2406</v>
+        <v>2407</v>
       </c>
       <c r="D425" s="1" t="s">
-        <v>2375</v>
+        <v>2376</v>
       </c>
       <c r="E425" s="1" t="s">
-        <v>2407</v>
+        <v>2408</v>
       </c>
       <c r="F425" s="1" t="s">
-        <v>2408</v>
+        <v>2409</v>
       </c>
       <c r="G425" s="1" t="s">
         <v>74</v>
@@ -22123,27 +22168,27 @@
         <v>56</v>
       </c>
       <c r="L425" s="1" t="s">
-        <v>2409</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="426" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A426" s="1" t="s">
-        <v>2410</v>
+        <v>2411</v>
       </c>
       <c r="B426" s="1" t="s">
-        <v>2411</v>
+        <v>2412</v>
       </c>
       <c r="C426" s="1" t="s">
-        <v>2412</v>
+        <v>2413</v>
       </c>
       <c r="D426" s="1" t="s">
-        <v>2413</v>
+        <v>2414</v>
       </c>
       <c r="E426" s="1" t="s">
-        <v>2414</v>
+        <v>2415</v>
       </c>
       <c r="F426" s="1" t="s">
-        <v>2415</v>
+        <v>2416</v>
       </c>
       <c r="G426" s="1" t="s">
         <v>74</v>
@@ -22156,27 +22201,27 @@
         <v>42</v>
       </c>
       <c r="L426" s="1" t="s">
-        <v>2416</v>
+        <v>2417</v>
       </c>
     </row>
     <row r="427" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A427" s="1" t="s">
-        <v>2417</v>
+        <v>2418</v>
       </c>
       <c r="B427" s="1" t="s">
-        <v>2418</v>
+        <v>2419</v>
       </c>
       <c r="C427" s="1" t="s">
-        <v>2419</v>
+        <v>2420</v>
       </c>
       <c r="D427" s="1" t="s">
-        <v>2420</v>
+        <v>2421</v>
       </c>
       <c r="E427" s="1" t="s">
-        <v>2421</v>
+        <v>2422</v>
       </c>
       <c r="F427" s="1" t="s">
-        <v>2422</v>
+        <v>2423</v>
       </c>
       <c r="G427" s="1" t="s">
         <v>74</v>
@@ -22189,27 +22234,27 @@
         <v>42</v>
       </c>
       <c r="L427" s="1" t="s">
-        <v>2423</v>
+        <v>2424</v>
       </c>
     </row>
     <row r="428" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A428" s="1" t="s">
-        <v>2424</v>
+        <v>2425</v>
       </c>
       <c r="B428" s="1" t="s">
-        <v>2425</v>
+        <v>2426</v>
       </c>
       <c r="C428" s="1" t="s">
-        <v>2426</v>
+        <v>2427</v>
       </c>
       <c r="D428" s="1" t="s">
-        <v>2427</v>
+        <v>2428</v>
       </c>
       <c r="E428" s="1" t="s">
-        <v>2428</v>
+        <v>2429</v>
       </c>
       <c r="F428" s="1" t="s">
-        <v>2429</v>
+        <v>2430</v>
       </c>
       <c r="G428" s="1" t="s">
         <v>74</v>
@@ -22222,27 +22267,27 @@
         <v>56</v>
       </c>
       <c r="L428" s="1" t="s">
-        <v>2430</v>
+        <v>2431</v>
       </c>
     </row>
     <row r="429" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A429" s="1" t="s">
-        <v>2431</v>
+        <v>2432</v>
       </c>
       <c r="B429" s="1" t="s">
-        <v>2432</v>
+        <v>2433</v>
       </c>
       <c r="C429" s="1" t="s">
-        <v>2433</v>
+        <v>2434</v>
       </c>
       <c r="D429" s="1" t="s">
-        <v>2434</v>
+        <v>2435</v>
       </c>
       <c r="E429" s="1" t="s">
-        <v>2435</v>
+        <v>2436</v>
       </c>
       <c r="F429" s="1" t="s">
-        <v>2436</v>
+        <v>2437</v>
       </c>
       <c r="G429" s="1" t="s">
         <v>74</v>
@@ -22255,27 +22300,27 @@
         <v>56</v>
       </c>
       <c r="L429" s="1" t="s">
-        <v>2437</v>
+        <v>2438</v>
       </c>
     </row>
     <row r="430" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A430" s="1" t="s">
-        <v>2438</v>
+        <v>2439</v>
       </c>
       <c r="B430" s="1" t="s">
-        <v>2439</v>
+        <v>2440</v>
       </c>
       <c r="C430" s="1" t="s">
-        <v>2440</v>
+        <v>2441</v>
       </c>
       <c r="D430" s="1" t="s">
-        <v>2441</v>
+        <v>2442</v>
       </c>
       <c r="E430" s="1" t="s">
-        <v>2442</v>
+        <v>2443</v>
       </c>
       <c r="F430" s="1" t="s">
-        <v>2443</v>
+        <v>2444</v>
       </c>
       <c r="G430" s="1" t="s">
         <v>74</v>
@@ -22288,27 +22333,27 @@
         <v>42</v>
       </c>
       <c r="L430" s="1" t="s">
-        <v>2444</v>
+        <v>2445</v>
       </c>
     </row>
     <row r="431" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A431" s="1" t="s">
-        <v>2445</v>
+        <v>2446</v>
       </c>
       <c r="B431" s="1" t="s">
-        <v>2446</v>
+        <v>2447</v>
       </c>
       <c r="C431" s="1" t="s">
-        <v>2447</v>
+        <v>2448</v>
       </c>
       <c r="D431" s="1" t="s">
-        <v>2448</v>
+        <v>2449</v>
       </c>
       <c r="E431" s="1" t="s">
-        <v>2449</v>
+        <v>2450</v>
       </c>
       <c r="F431" s="1" t="s">
-        <v>2450</v>
+        <v>2451</v>
       </c>
       <c r="G431" s="1" t="s">
         <v>74</v>
@@ -22321,27 +22366,27 @@
         <v>56</v>
       </c>
       <c r="L431" s="1" t="s">
-        <v>2451</v>
+        <v>2452</v>
       </c>
     </row>
     <row r="432" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A432" s="1" t="s">
-        <v>2452</v>
+        <v>2453</v>
       </c>
       <c r="B432" s="1" t="s">
-        <v>2453</v>
+        <v>2454</v>
       </c>
       <c r="C432" s="1" t="s">
-        <v>2454</v>
+        <v>2455</v>
       </c>
       <c r="D432" s="1" t="s">
-        <v>2455</v>
+        <v>2456</v>
       </c>
       <c r="E432" s="1" t="s">
-        <v>2456</v>
+        <v>2457</v>
       </c>
       <c r="F432" s="1" t="s">
-        <v>2457</v>
+        <v>2458</v>
       </c>
       <c r="G432" s="1" t="s">
         <v>74</v>
@@ -22354,27 +22399,27 @@
         <v>42</v>
       </c>
       <c r="L432" s="1" t="s">
-        <v>2458</v>
+        <v>2459</v>
       </c>
     </row>
     <row r="433" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A433" s="1" t="s">
-        <v>2459</v>
+        <v>2460</v>
       </c>
       <c r="B433" s="1" t="s">
-        <v>2460</v>
+        <v>2461</v>
       </c>
       <c r="C433" s="1" t="s">
-        <v>2461</v>
+        <v>2462</v>
       </c>
       <c r="D433" s="1" t="s">
-        <v>2462</v>
+        <v>2463</v>
       </c>
       <c r="E433" s="1" t="s">
-        <v>2463</v>
+        <v>2464</v>
       </c>
       <c r="F433" s="1" t="s">
-        <v>2464</v>
+        <v>2465</v>
       </c>
       <c r="G433" s="1" t="s">
         <v>74</v>
@@ -22387,27 +22432,27 @@
         <v>56</v>
       </c>
       <c r="L433" s="1" t="s">
-        <v>2465</v>
+        <v>2466</v>
       </c>
     </row>
     <row r="434" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A434" s="1" t="s">
-        <v>2466</v>
+        <v>2467</v>
       </c>
       <c r="B434" s="1" t="s">
-        <v>2467</v>
+        <v>2468</v>
       </c>
       <c r="C434" s="1" t="s">
-        <v>2468</v>
+        <v>2469</v>
       </c>
       <c r="D434" s="1" t="s">
-        <v>2469</v>
+        <v>2470</v>
       </c>
       <c r="E434" s="1" t="s">
-        <v>2470</v>
+        <v>2471</v>
       </c>
       <c r="F434" s="1" t="s">
-        <v>2471</v>
+        <v>2472</v>
       </c>
       <c r="G434" s="1" t="s">
         <v>74</v>
@@ -22420,27 +22465,27 @@
         <v>42</v>
       </c>
       <c r="L434" s="1" t="s">
-        <v>2472</v>
+        <v>2473</v>
       </c>
     </row>
     <row r="435" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A435" s="1" t="s">
-        <v>2473</v>
+        <v>2474</v>
       </c>
       <c r="B435" s="1" t="s">
-        <v>2474</v>
+        <v>2475</v>
       </c>
       <c r="C435" s="1" t="s">
-        <v>2475</v>
+        <v>2476</v>
       </c>
       <c r="D435" s="1" t="s">
         <v>1184</v>
       </c>
       <c r="E435" s="1" t="s">
-        <v>2476</v>
+        <v>2477</v>
       </c>
       <c r="F435" s="1" t="s">
-        <v>2477</v>
+        <v>2478</v>
       </c>
       <c r="G435" s="1" t="s">
         <v>74</v>
@@ -22453,27 +22498,27 @@
         <v>65</v>
       </c>
       <c r="L435" s="1" t="s">
-        <v>2478</v>
+        <v>2479</v>
       </c>
     </row>
     <row r="436" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A436" s="10" t="s">
-        <v>2479</v>
+        <v>2480</v>
       </c>
       <c r="B436" s="10" t="s">
-        <v>2480</v>
+        <v>2481</v>
       </c>
       <c r="C436" s="10" t="s">
-        <v>2481</v>
+        <v>2482</v>
       </c>
       <c r="D436" s="10" t="s">
-        <v>2482</v>
+        <v>2483</v>
       </c>
       <c r="E436" s="10" t="s">
-        <v>2483</v>
+        <v>2484</v>
       </c>
       <c r="F436" s="10" t="s">
-        <v>2484</v>
+        <v>2485</v>
       </c>
       <c r="G436" s="10" t="s">
         <v>74</v>
@@ -22486,27 +22531,27 @@
         <v>42</v>
       </c>
       <c r="L436" s="11" t="s">
-        <v>2485</v>
+        <v>2486</v>
       </c>
     </row>
     <row r="437" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A437" s="10" t="s">
-        <v>2486</v>
+        <v>2487</v>
       </c>
       <c r="B437" s="10" t="s">
-        <v>2487</v>
+        <v>2488</v>
       </c>
       <c r="C437" s="10" t="s">
-        <v>2488</v>
+        <v>2489</v>
       </c>
       <c r="D437" s="10" t="s">
-        <v>2489</v>
+        <v>2490</v>
       </c>
       <c r="E437" s="10" t="s">
-        <v>2490</v>
+        <v>2491</v>
       </c>
       <c r="F437" s="10" t="s">
-        <v>2491</v>
+        <v>2492</v>
       </c>
       <c r="G437" s="10" t="s">
         <v>74</v>
@@ -22519,27 +22564,27 @@
         <v>42</v>
       </c>
       <c r="L437" s="11" t="s">
-        <v>2492</v>
+        <v>2493</v>
       </c>
     </row>
     <row r="438" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A438" s="10" t="s">
-        <v>2493</v>
+        <v>2494</v>
       </c>
       <c r="B438" s="10" t="s">
-        <v>2494</v>
+        <v>2495</v>
       </c>
       <c r="C438" s="10" t="s">
-        <v>2495</v>
+        <v>2496</v>
       </c>
       <c r="D438" s="10" t="s">
-        <v>2496</v>
+        <v>2497</v>
       </c>
       <c r="E438" s="10" t="s">
-        <v>2497</v>
+        <v>2498</v>
       </c>
       <c r="F438" s="10" t="s">
-        <v>2498</v>
+        <v>2499</v>
       </c>
       <c r="G438" s="10" t="s">
         <v>74</v>
@@ -22552,27 +22597,27 @@
         <v>42</v>
       </c>
       <c r="L438" s="11" t="s">
-        <v>2499</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="439" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A439" s="10" t="s">
-        <v>2500</v>
+        <v>2501</v>
       </c>
       <c r="B439" s="10" t="s">
-        <v>2501</v>
+        <v>2502</v>
       </c>
       <c r="C439" s="10" t="s">
-        <v>2502</v>
+        <v>2503</v>
       </c>
       <c r="D439" s="10" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
       <c r="E439" s="10" t="s">
-        <v>2504</v>
+        <v>2505</v>
       </c>
       <c r="F439" s="10" t="s">
-        <v>2505</v>
+        <v>2506</v>
       </c>
       <c r="G439" s="10" t="s">
         <v>74</v>
@@ -22585,27 +22630,27 @@
         <v>56</v>
       </c>
       <c r="L439" s="11" t="s">
-        <v>2506</v>
+        <v>2507</v>
       </c>
     </row>
     <row r="440" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A440" s="10" t="s">
-        <v>2507</v>
+        <v>2508</v>
       </c>
       <c r="B440" s="10" t="s">
-        <v>2508</v>
+        <v>2509</v>
       </c>
       <c r="C440" s="10" t="s">
-        <v>2509</v>
+        <v>2510</v>
       </c>
       <c r="D440" s="10" t="s">
-        <v>2510</v>
+        <v>2511</v>
       </c>
       <c r="E440" s="10" t="s">
-        <v>2511</v>
+        <v>2512</v>
       </c>
       <c r="F440" s="10" t="s">
-        <v>2512</v>
+        <v>2513</v>
       </c>
       <c r="G440" s="10" t="s">
         <v>74</v>
@@ -22618,27 +22663,27 @@
         <v>42</v>
       </c>
       <c r="L440" s="11" t="s">
-        <v>2513</v>
+        <v>2514</v>
       </c>
     </row>
     <row r="441" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A441" s="10" t="s">
-        <v>2514</v>
+        <v>2515</v>
       </c>
       <c r="B441" s="10" t="s">
-        <v>2515</v>
+        <v>2516</v>
       </c>
       <c r="C441" s="10" t="s">
-        <v>2516</v>
+        <v>2517</v>
       </c>
       <c r="D441" s="10" t="s">
-        <v>2517</v>
+        <v>2518</v>
       </c>
       <c r="E441" s="10" t="s">
-        <v>2518</v>
+        <v>2519</v>
       </c>
       <c r="F441" s="10" t="s">
-        <v>2519</v>
+        <v>2520</v>
       </c>
       <c r="G441" s="10" t="s">
         <v>74</v>
@@ -22651,27 +22696,27 @@
         <v>56</v>
       </c>
       <c r="L441" s="11" t="s">
-        <v>2520</v>
-      </c>
-    </row>
-    <row r="442" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>2521</v>
+      </c>
+    </row>
+    <row r="442" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A442" s="10" t="s">
-        <v>2521</v>
+        <v>2522</v>
       </c>
       <c r="B442" s="10" t="s">
-        <v>2522</v>
+        <v>2523</v>
       </c>
       <c r="C442" s="10" t="s">
-        <v>2523</v>
+        <v>2524</v>
       </c>
       <c r="D442" s="10" t="s">
-        <v>2524</v>
+        <v>2525</v>
       </c>
       <c r="E442" s="10" t="s">
-        <v>2525</v>
+        <v>2526</v>
       </c>
       <c r="F442" s="10" t="s">
-        <v>2526</v>
+        <v>2527</v>
       </c>
       <c r="G442" s="10" t="s">
         <v>74</v>
@@ -22684,7 +22729,73 @@
         <v>56</v>
       </c>
       <c r="L442" s="11" t="s">
-        <v>2527</v>
+        <v>2528</v>
+      </c>
+    </row>
+    <row r="443" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A443" s="10" t="s">
+        <v>2529</v>
+      </c>
+      <c r="B443" s="10" t="s">
+        <v>2349</v>
+      </c>
+      <c r="C443" s="10" t="s">
+        <v>2530</v>
+      </c>
+      <c r="D443" s="10" t="s">
+        <v>2531</v>
+      </c>
+      <c r="E443" s="10" t="s">
+        <v>2532</v>
+      </c>
+      <c r="F443" s="10" t="s">
+        <v>2533</v>
+      </c>
+      <c r="G443" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H443" s="10" t="str">
+        <f aca="false">IF(G443="BUG","BUG-"&amp;A443,IF(G443="FUNCTIONAL","FUNCTIONAL-"&amp;A443,""))</f>
+        <v/>
+      </c>
+      <c r="I443" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="L443" s="11" t="s">
+        <v>2534</v>
+      </c>
+    </row>
+    <row r="444" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A444" s="10" t="s">
+        <v>2535</v>
+      </c>
+      <c r="B444" s="10" t="s">
+        <v>2536</v>
+      </c>
+      <c r="C444" s="10" t="s">
+        <v>2537</v>
+      </c>
+      <c r="D444" s="10" t="s">
+        <v>2538</v>
+      </c>
+      <c r="E444" s="10" t="s">
+        <v>2539</v>
+      </c>
+      <c r="F444" s="10" t="s">
+        <v>2540</v>
+      </c>
+      <c r="G444" s="10" t="s">
+        <v>2541</v>
+      </c>
+      <c r="H444" s="10" t="str">
+        <f aca="false">IF(G444="BUG","BUG-"&amp;A444,IF(G444="FUNCTIONAL","FUNCTIONAL-"&amp;A444,""))</f>
+        <v/>
+      </c>
+      <c r="I444" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="L444" s="11" t="s">
+        <v>2542</v>
       </c>
     </row>
   </sheetData>
@@ -22744,7 +22855,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>2528</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22752,13 +22863,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2529</v>
+        <v>2544</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2530</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22815,7 +22926,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -22827,11 +22938,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>2531</v>
+        <v>2546</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
docs(controlled-beta): xlsx test matrix - aggiungere TC-N418 (wiring Command Center)
Recalc LibreOffice: 0 errori su 442 formule.
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3893" uniqueCount="2547">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3902" uniqueCount="2554">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -7660,6 +7660,27 @@
   </si>
   <si>
     <t xml:space="preserve">Test automatizzato eseguito nel sandbox Claude (26/26 passed su chromium+mobile-chrome, nessun browser reale richiesto): tests/one/spotlight-position.spec.ts.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N418</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRAMA ONE - Controlled Publication (fase E, wiring) - Command Center in menu Admin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La voce 'Command Center' compare nel menu Admin (condizionata al flag TRAMA_ONE_ENABLED) e porta a /admin/one - chiude il gap noto in DEC-58 ('/admin/one raggiungibile solo per URL diretto, mai da una voce di menu')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login platform_admin; flag TRAMA_ONE_ENABLED attivo per l'utente di test (override, vedi DEC-34/DEC-57)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login Admin -&gt; apri /admin -&gt; cerca la voce 'Command Center' nel menu -&gt; click</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La voce e' visibile con href /admin/one; il click naviga a /admin/one senza redirect/errore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automatizzato: tests/one/command-center.spec.ts, TC-N418.</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -8499,7 +8520,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L444"/>
+  <dimension ref="A1:L445"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -22732,7 +22753,7 @@
         <v>2528</v>
       </c>
     </row>
-    <row r="443" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="443" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A443" s="10" t="s">
         <v>2529</v>
       </c>
@@ -22765,7 +22786,7 @@
         <v>2534</v>
       </c>
     </row>
-    <row r="444" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="444" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A444" s="10" t="s">
         <v>2535</v>
       </c>
@@ -22796,6 +22817,39 @@
       </c>
       <c r="L444" s="11" t="s">
         <v>2542</v>
+      </c>
+    </row>
+    <row r="445" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A445" s="10" t="s">
+        <v>2543</v>
+      </c>
+      <c r="B445" s="10" t="s">
+        <v>2544</v>
+      </c>
+      <c r="C445" s="10" t="s">
+        <v>2545</v>
+      </c>
+      <c r="D445" s="10" t="s">
+        <v>2546</v>
+      </c>
+      <c r="E445" s="10" t="s">
+        <v>2547</v>
+      </c>
+      <c r="F445" s="10" t="s">
+        <v>2548</v>
+      </c>
+      <c r="G445" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H445" s="10" t="str">
+        <f aca="false">IF(G445="BUG","BUG-"&amp;A445,IF(G445="FUNCTIONAL","FUNCTIONAL-"&amp;A445,""))</f>
+        <v/>
+      </c>
+      <c r="I445" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="L445" s="11" t="s">
+        <v>2549</v>
       </c>
     </row>
   </sheetData>
@@ -22855,7 +22909,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>2543</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22863,13 +22917,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2544</v>
+        <v>2551</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2545</v>
+        <v>2552</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22926,7 +22980,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -22938,11 +22992,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>2546</v>
+        <v>2553</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
docs(xlsx): aggiorna TC-N416 e aggiungi TC-N615 (DEC-69)
Riflette il titolo rinominato del badge (TC-N416) e il nuovo test
per il link esplicito verso il Calendario disponibilità (TC-N615).
Ricalcolato: 488 formule, 0 errori.
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3911" uniqueCount="2559">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3920" uniqueCount="2565">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -7647,10 +7647,28 @@
     <t xml:space="preserve">Login gestore -&gt; apri /center/activities -&gt; click sul VERO pulsante '+ Nuova attivita' (elemento con data-spotlight, non un bottone del tour)</t>
   </si>
   <si>
-    <t xml:space="preserve">La navigazione reale avviene (URL -&gt; /center/activities/new); lo step 'create_activity' risulta completato e il percorso avanza a 'configure_weeks' — poiche' quel target non esiste sulla pagina di creazione, lo Spotlight mostra il badge 'target non trovato' col titolo 'Configura le settimane' invece di restare ancorato al pulsante ormai scomparso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test automatizzato: tests/one/walkthrough-partner.spec.ts, TC-N416 (nuovo per il gate Controlled Beta S7-14/DEC-60 — verifica il meccanismo di avanzamento via click reale, cuore del nuovo motore Spotlight rispetto al vecchio WalkthroughCard).</t>
+    <t xml:space="preserve">La navigazione reale avviene (URL -&gt; /center/activities/new); lo step 'create_activity' risulta completato e il percorso avanza a 'configure_weeks' — poiche' quel target non esiste sulla pagina di creazione, lo Spotlight mostra il badge 'target non trovato' col titolo 'Informazioni di base' (rinominato da 'Configura le settimane', DEC-69) invece di restare ancorato al pulsante ormai scomparso; nessun link nel badge (siamo su /new, nessuna attivita' reale)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automatizzato: tests/one/walkthrough-partner.spec.ts, TC-N416 (nuovo per il gate Controlled Beta S7-14/DEC-60 — verifica il meccanismo di avanzamento via click reale, cuore del nuovo motore Spotlight rispetto al vecchio WalkthroughCard). Titolo del badge aggiornato a 'Informazioni di base' (DEC-69, Visual Acceptance Gate §15): il target reale (card 'Informazioni generali') non conteneva cio' che il vecchio testo descriveva.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N615</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il badge 'target non trovato' per lo step 'Configura i Giorni spot' mostra un link REALE verso il Calendario disponibilita', non solo testo (DEC-69)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login center_admin; flag TRAMA_ONE_ENABLED attivo; almeno un'attivita' esistente nel centro collegato; step precedenti (configure_weeks/configure_pricing/publish) completati cliccando i rispettivi elementi reali</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login gestore -&gt; apri un'attivita' esistente -&gt; click su Informazioni generali (configure_weeks) -&gt; click su Servizi extra e pasto (configure_pricing) -&gt; click su Salva modifiche (publish)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il badge 'target non trovato' mostra il titolo 'Configura i Giorni spot' e un link cliccabile 'Vai al Calendario disponibilita' →' con href verso .../calendar; il click naviga davvero li'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automatizzato: tests/one/walkthrough-partner.spec.ts, TC-N615. Bug reale trovato da Fabrizio: prima di questo fix il badge dava solo testo, l'utente doveva indovinare dove andare per configurare i Giorni spot dopo aver pubblicato. Fix: nuovo campo spotlightMissingHint in lib/walkthrough/registry.ts, reso come &lt;Link&gt; reale in components/spotlight/PartnerSpotlight.tsx.</t>
   </si>
   <si>
     <t xml:space="preserve">TC-N417</t>
@@ -8535,7 +8553,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L446"/>
+  <dimension ref="A1:L447"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -22971,65 +22989,98 @@
         <v>2540</v>
       </c>
       <c r="B445" s="10" t="s">
+        <v>2354</v>
+      </c>
+      <c r="C445" s="10" t="s">
         <v>2541</v>
       </c>
-      <c r="C445" s="10" t="s">
+      <c r="D445" s="10" t="s">
         <v>2542</v>
       </c>
-      <c r="D445" s="10" t="s">
+      <c r="E445" s="10" t="s">
         <v>2543</v>
       </c>
-      <c r="E445" s="10" t="s">
+      <c r="F445" s="10" t="s">
         <v>2544</v>
       </c>
-      <c r="F445" s="10" t="s">
-        <v>2545</v>
-      </c>
       <c r="G445" s="10" t="s">
-        <v>2546</v>
+        <v>74</v>
       </c>
       <c r="H445" s="10" t="str">
         <f aca="false">IF(G445="BUG","BUG-"&amp;A445,IF(G445="FUNCTIONAL","FUNCTIONAL-"&amp;A445,""))</f>
         <v/>
       </c>
       <c r="I445" s="10" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="L445" s="11" t="s">
-        <v>2547</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="446" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A446" s="10" t="s">
+        <v>2546</v>
+      </c>
+      <c r="B446" s="10" t="s">
+        <v>2547</v>
+      </c>
+      <c r="C446" s="10" t="s">
         <v>2548</v>
       </c>
-      <c r="B446" s="10" t="s">
+      <c r="D446" s="10" t="s">
         <v>2549</v>
       </c>
-      <c r="C446" s="10" t="s">
+      <c r="E446" s="10" t="s">
         <v>2550</v>
       </c>
-      <c r="D446" s="10" t="s">
+      <c r="F446" s="10" t="s">
         <v>2551</v>
       </c>
-      <c r="E446" s="10" t="s">
+      <c r="G446" s="10" t="s">
         <v>2552</v>
       </c>
-      <c r="F446" s="10" t="s">
-        <v>2553</v>
-      </c>
-      <c r="G446" s="10" t="s">
-        <v>74</v>
-      </c>
       <c r="H446" s="10" t="str">
-        <f aca="false">IF(G446="BUG","BUG-"&amp;A446,IF(G446="FUNCTIONAL","FUNCTIONAL-"&amp;A446,""))</f>
+        <f aca="false">IF(G445="BUG","BUG-"&amp;A445,IF(G445="FUNCTIONAL","FUNCTIONAL-"&amp;A445,""))</f>
         <v/>
       </c>
       <c r="I446" s="10" t="s">
         <v>65</v>
       </c>
       <c r="L446" s="11" t="s">
+        <v>2553</v>
+      </c>
+    </row>
+    <row r="447" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A447" s="10" t="s">
         <v>2554</v>
+      </c>
+      <c r="B447" s="10" t="s">
+        <v>2555</v>
+      </c>
+      <c r="C447" s="10" t="s">
+        <v>2556</v>
+      </c>
+      <c r="D447" s="10" t="s">
+        <v>2557</v>
+      </c>
+      <c r="E447" s="10" t="s">
+        <v>2558</v>
+      </c>
+      <c r="F447" s="10" t="s">
+        <v>2559</v>
+      </c>
+      <c r="G447" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H447" s="10" t="str">
+        <f aca="false">IF(G446="BUG","BUG-"&amp;A446,IF(G446="FUNCTIONAL","FUNCTIONAL-"&amp;A446,""))</f>
+        <v/>
+      </c>
+      <c r="I447" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="L447" s="11" t="s">
+        <v>2560</v>
       </c>
     </row>
   </sheetData>
@@ -23089,7 +23140,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>2555</v>
+        <v>2561</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23097,13 +23148,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2556</v>
+        <v>2562</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2557</v>
+        <v>2563</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23160,7 +23211,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -23172,11 +23223,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>2558</v>
+        <v>2564</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
docs(xlsx): TC-N616 per pickVisibleTargetIndex (DEC-70)
Ricalcolato: 489 formule, 0 errori.
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3920" uniqueCount="2565">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3929" uniqueCount="2570">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -7671,25 +7671,40 @@
     <t xml:space="preserve">Test automatizzato: tests/one/walkthrough-partner.spec.ts, TC-N615. Bug reale trovato da Fabrizio: prima di questo fix il badge dava solo testo, l'utente doveva indovinare dove andare per configurare i Giorni spot dopo aver pubblicato. Fix: nuovo campo spotlightMissingHint in lib/walkthrough/registry.ts, reso come &lt;Link&gt; reale in components/spotlight/PartnerSpotlight.tsx.</t>
   </si>
   <si>
+    <t xml:space="preserve">TC-N616</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRAMA ONE - Spotlight: unit test puri lib/spotlight/position.ts [no browser]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pickVisibleTargetIndex sceglie il primo rect con area non nulla tra piu' candidati con lo stesso data-spotlight (bug reale DEC-70: la voce 'dashboard' esiste sia nella sidebar desktop sia nel cassetto mobile, e su schermi &lt;768px la prima e' display:none con rect degenere 0x0x0x0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nessuna (funzione pura, nessun browser/DOM richiesto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">npx playwright test tests/one/spotlight-position.spec.ts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5/5 assert passano: nessun candidato -&gt; -1; un solo candidato nascosto -&gt; -1; primo nascosto e secondo visibile -&gt; indice 1 (caso reale mobile 390px); primo gia' visibile -&gt; indice 0 (caso desktop/tablet); tutti nascosti -&gt; -1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PASS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bug reale trovato da Fabrizio via screenshot: su mobile 390px lo step 'Monitora dalla dashboard' mostrava un popover rotto (ancorato in alto a sinistra, il vero nav item 'Dashboard' non evidenziato) mentre su 768/1440 funzionava. Causa: document.querySelector prendeva sempre la prima delle 2 copie DOM dello stesso data-spotlight, quella nascosta su mobile. Fix in components/spotlight/PartnerSpotlight.tsx: legge tutti i candidati e sceglie il primo visibile via questa funzione pura; se nessuno lo e', mostra il badge 'target non trovato' invece del popover rotto. Test eseguito nel sandbox Claude (38/38 passed su chromium+mobile-chrome).</t>
+  </si>
+  <si>
     <t xml:space="preserve">TC-N417</t>
   </si>
   <si>
-    <t xml:space="preserve">TRAMA ONE - Spotlight: unit test puri lib/spotlight/position.ts [no browser]</t>
-  </si>
-  <si>
     <t xml:space="preserve">computePopoverPosition/computeCutoutRect/matchesSpotlightRoute producono i placement/rect/match attesi per i casi noti (spazio sopra/sotto, clamp orizzontale, wildcard singola/centrale/globale)</t>
   </si>
   <si>
     <t xml:space="preserve">Nessuna (funzioni pure, nessun browser/DB richiesto)</t>
   </si>
   <si>
-    <t xml:space="preserve">npx playwright test tests/one/spotlight-position.spec.ts</t>
-  </si>
-  <si>
     <t xml:space="preserve">13/13 assert passano: placement top/bottom coerente con lo spazio disponibile, cutout con padding corretto, matchesSpotlightRoute coerente per pattern esatti/prefisso/prefisso+suffisso/wildcard globale</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PASS</t>
   </si>
   <si>
     <t xml:space="preserve">Test automatizzato eseguito nel sandbox Claude (26/26 passed su chromium+mobile-chrome, nessun browser reale richiesto): tests/one/spotlight-position.spec.ts.</t>
@@ -8553,7 +8568,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L447"/>
+  <dimension ref="A1:L448"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -23040,47 +23055,80 @@
         <v>2552</v>
       </c>
       <c r="H446" s="10" t="str">
-        <f aca="false">IF(G445="BUG","BUG-"&amp;A445,IF(G445="FUNCTIONAL","FUNCTIONAL-"&amp;A445,""))</f>
+        <f aca="false">IF(G446="BUG","BUG-"&amp;A446,IF(G446="FUNCTIONAL","FUNCTIONAL-"&amp;A446,""))</f>
         <v/>
       </c>
       <c r="I446" s="10" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="L446" s="11" t="s">
         <v>2553</v>
       </c>
     </row>
-    <row r="447" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="447" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A447" s="10" t="s">
         <v>2554</v>
       </c>
       <c r="B447" s="10" t="s">
+        <v>2547</v>
+      </c>
+      <c r="C447" s="10" t="s">
         <v>2555</v>
       </c>
-      <c r="C447" s="10" t="s">
+      <c r="D447" s="10" t="s">
         <v>2556</v>
       </c>
-      <c r="D447" s="10" t="s">
+      <c r="E447" s="10" t="s">
+        <v>2550</v>
+      </c>
+      <c r="F447" s="10" t="s">
         <v>2557</v>
       </c>
-      <c r="E447" s="10" t="s">
-        <v>2558</v>
-      </c>
-      <c r="F447" s="10" t="s">
-        <v>2559</v>
-      </c>
       <c r="G447" s="10" t="s">
-        <v>74</v>
+        <v>2552</v>
       </c>
       <c r="H447" s="10" t="str">
-        <f aca="false">IF(G446="BUG","BUG-"&amp;A446,IF(G446="FUNCTIONAL","FUNCTIONAL-"&amp;A446,""))</f>
+        <f aca="false">IF(G445="BUG","BUG-"&amp;A445,IF(G445="FUNCTIONAL","FUNCTIONAL-"&amp;A445,""))</f>
         <v/>
       </c>
       <c r="I447" s="10" t="s">
         <v>65</v>
       </c>
       <c r="L447" s="11" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="448" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A448" s="10" t="s">
+        <v>2559</v>
+      </c>
+      <c r="B448" s="10" t="s">
         <v>2560</v>
+      </c>
+      <c r="C448" s="10" t="s">
+        <v>2561</v>
+      </c>
+      <c r="D448" s="10" t="s">
+        <v>2562</v>
+      </c>
+      <c r="E448" s="10" t="s">
+        <v>2563</v>
+      </c>
+      <c r="F448" s="10" t="s">
+        <v>2564</v>
+      </c>
+      <c r="G448" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H448" s="10" t="str">
+        <f aca="false">IF(G446="BUG","BUG-"&amp;A446,IF(G446="FUNCTIONAL","FUNCTIONAL-"&amp;A446,""))</f>
+        <v/>
+      </c>
+      <c r="I448" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="L448" s="11" t="s">
+        <v>2565</v>
       </c>
     </row>
   </sheetData>
@@ -23140,7 +23188,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>2561</v>
+        <v>2566</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23148,13 +23196,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2562</v>
+        <v>2567</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2563</v>
+        <v>2568</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23223,11 +23271,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>2564</v>
+        <v>2569</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
DEC-71: aggiornare xlsx (TC-N615 riscritta, nuova TC-N617)
Riga TC-N615 riscritta per il nuovo flusso; nuova riga TC-N617 per la
verifica dedicata che un click su un campo reale non avanzi lo step.
Ricalcolato: 490 formule, 0 errori.
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3929" uniqueCount="2570">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3938" uniqueCount="2576">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -7659,16 +7659,16 @@
     <t xml:space="preserve">Il badge 'target non trovato' per lo step 'Configura i Giorni spot' mostra un link REALE verso il Calendario disponibilita', non solo testo (DEC-69)</t>
   </si>
   <si>
-    <t xml:space="preserve">Login center_admin; flag TRAMA_ONE_ENABLED attivo; almeno un'attivita' esistente nel centro collegato; step precedenti (configure_weeks/configure_pricing/publish) completati cliccando i rispettivi elementi reali</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Login gestore -&gt; apri un'attivita' esistente -&gt; click su Informazioni generali (configure_weeks) -&gt; click su Servizi extra e pasto (configure_pricing) -&gt; click su Salva modifiche (publish)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Il badge 'target non trovato' mostra il titolo 'Configura i Giorni spot' e un link cliccabile 'Vai al Calendario disponibilita' →' con href verso .../calendar; il click naviga davvero li'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test automatizzato: tests/one/walkthrough-partner.spec.ts, TC-N615. Bug reale trovato da Fabrizio: prima di questo fix il badge dava solo testo, l'utente doveva indovinare dove andare per configurare i Giorni spot dopo aver pubblicato. Fix: nuovo campo spotlightMissingHint in lib/walkthrough/registry.ts, reso come &lt;Link&gt; reale in components/spotlight/PartnerSpotlight.tsx.</t>
+    <t xml:space="preserve">Login center_admin; flag TRAMA_ONE_ENABLED attivo; almeno un'attivita' esistente nel centro collegato; step precedenti (configure_weeks/configure_pricing) completati con il flusso manuale 'Inizia' + 'Ho finito, continua -&gt;' (DEC-71), poi publish completato cliccando l'elemento reale 'Salva modifiche'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login gestore -&gt; apri un'attivita' esistente -&gt; step Informazioni di base: click 'Inizia' poi click 'Ho finito, continua -&gt;' -&gt; step Servizi extra e pasto: click 'Inizia', poi click sulla checkbox reale 'Ingresso anticipato (pre-servizio)' (verifica che lo step NON avanzi da solo), poi click 'Ho finito, continua -&gt;' -&gt; click su Salva modifiche (publish)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gli step 'manuali' (Informazioni di base, Servizi extra e pasto) NON avanzano al click su un campo reale della card: resta visibile il popover con il testo 'Compila con calma i campi di questa sezione, poi continua.' finche' non si clicca il pulsante esplicito 'Ho finito, continua -&gt;'. Dopo publish, il badge 'target non trovato' mostra il titolo 'Configura i Giorni spot' e un link cliccabile 'Vai al Calendario disponibilita' →' con href verso .../calendar; il click naviga davvero li'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automatizzato: tests/one/walkthrough-partner.spec.ts, TC-N615. Bug reale trovato da Fabrizio (DEC-69): prima di questo fix il badge dava solo testo per Giorni spot. Fix: campo spotlightMissingHint in lib/walkthrough/registry.ts, reso come &lt;Link&gt; reale in PartnerSpotlight.tsx. Aggiornato per DEC-71: secondo bug reale di Fabrizio, cliccare un campo dentro Servizi extra/Informazioni di base avanzava subito lo step impedendo di finire la configurazione. Fix: campo spotlightManualAdvance, pulsante esplicito 'Ho finito, continua -&gt;'.</t>
   </si>
   <si>
     <t xml:space="preserve">TC-N616</t>
@@ -7693,6 +7693,24 @@
   </si>
   <si>
     <t xml:space="preserve">Bug reale trovato da Fabrizio via screenshot: su mobile 390px lo step 'Monitora dalla dashboard' mostrava un popover rotto (ancorato in alto a sinistra, il vero nav item 'Dashboard' non evidenziato) mentre su 768/1440 funzionava. Causa: document.querySelector prendeva sempre la prima delle 2 copie DOM dello stesso data-spotlight, quella nascosta su mobile. Fix in components/spotlight/PartnerSpotlight.tsx: legge tutti i candidati e sceglie il primo visibile via questa funzione pura; se nessuno lo e', mostra il badge 'target non trovato' invece del popover rotto. Test eseguito nel sandbox Claude (38/38 passed su chromium+mobile-chrome).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N617</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cliccare un campo reale dentro una card multi-campo dello step tutorial (es. checkbox 'Ingresso anticipato' in Servizi extra e pasto) NON deve avanzare da solo lo step: serve il pulsante esplicito 'Ho finito, continua -&gt;' (DEC-71)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login center_admin; flag TRAMA_ONE_ENABLED attivo; almeno un'attivita' esistente nel centro collegato; step configure_weeks gia' completato (percorso arrivato allo step configure_pricing)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri un'attivita' esistente -&gt; arriva allo step 'Servizi extra e pasto' -&gt; click 'Inizia' -&gt; click sulla checkbox reale 'Ingresso anticipato (pre-servizio)' dentro la card -&gt; verifica che il popover resti sullo stesso step -&gt; click 'Ho finito, continua -&gt;'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dopo il click sulla checkbox il popover 'Servizi extra e pasto' resta visibile con il testo 'Compila con calma i campi di questa sezione, poi continua.' (lo step NON e' avanzato); solo il click esplicito su 'Ho finito, continua -&gt;' fa avanzare al passo successivo (Pubblica)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automatizzato: tests/one/walkthrough-partner.spec.ts, incluso nel test TC-N615 (stessa run seriale). Bug reale segnalato da Fabrizio: 'se clicco una delle impostazioni dello step (es. servizi extra clicco ingresso anticipato..) va direttamente nello step successivo e non permette di finire la configurazione'. Fix: campo spotlightManualAdvance in lib/walkthrough/registry.ts + lib/walkthrough/data.ts, click-capture listener disattivato per questi step in PartnerSpotlight.tsx, nuovo pulsante 'Ho finito, continua -&gt;'.</t>
   </si>
   <si>
     <t xml:space="preserve">TC-N417</t>
@@ -8568,7 +8586,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L448"/>
+  <dimension ref="A1:L449"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -23070,7 +23088,7 @@
         <v>2554</v>
       </c>
       <c r="B447" s="10" t="s">
-        <v>2547</v>
+        <v>2354</v>
       </c>
       <c r="C447" s="10" t="s">
         <v>2555</v>
@@ -23079,31 +23097,31 @@
         <v>2556</v>
       </c>
       <c r="E447" s="10" t="s">
-        <v>2550</v>
+        <v>2557</v>
       </c>
       <c r="F447" s="10" t="s">
-        <v>2557</v>
+        <v>2558</v>
       </c>
       <c r="G447" s="10" t="s">
-        <v>2552</v>
+        <v>74</v>
       </c>
       <c r="H447" s="10" t="str">
-        <f aca="false">IF(G445="BUG","BUG-"&amp;A445,IF(G445="FUNCTIONAL","FUNCTIONAL-"&amp;A445,""))</f>
+        <f aca="false">IF(G447="BUG","BUG-"&amp;A447,IF(G447="FUNCTIONAL","FUNCTIONAL-"&amp;A447,""))</f>
         <v/>
       </c>
       <c r="I447" s="10" t="s">
-        <v>65</v>
+        <v>42</v>
       </c>
       <c r="L447" s="11" t="s">
-        <v>2558</v>
-      </c>
-    </row>
-    <row r="448" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="448" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A448" s="10" t="s">
-        <v>2559</v>
+        <v>2560</v>
       </c>
       <c r="B448" s="10" t="s">
-        <v>2560</v>
+        <v>2547</v>
       </c>
       <c r="C448" s="10" t="s">
         <v>2561</v>
@@ -23112,23 +23130,56 @@
         <v>2562</v>
       </c>
       <c r="E448" s="10" t="s">
+        <v>2550</v>
+      </c>
+      <c r="F448" s="10" t="s">
         <v>2563</v>
       </c>
-      <c r="F448" s="10" t="s">
-        <v>2564</v>
-      </c>
       <c r="G448" s="10" t="s">
-        <v>74</v>
+        <v>2552</v>
       </c>
       <c r="H448" s="10" t="str">
-        <f aca="false">IF(G446="BUG","BUG-"&amp;A446,IF(G446="FUNCTIONAL","FUNCTIONAL-"&amp;A446,""))</f>
+        <f aca="false">IF(G445="BUG","BUG-"&amp;A445,IF(G445="FUNCTIONAL","FUNCTIONAL-"&amp;A445,""))</f>
         <v/>
       </c>
       <c r="I448" s="10" t="s">
         <v>65</v>
       </c>
       <c r="L448" s="11" t="s">
+        <v>2564</v>
+      </c>
+    </row>
+    <row r="449" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A449" s="10" t="s">
         <v>2565</v>
+      </c>
+      <c r="B449" s="10" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C449" s="10" t="s">
+        <v>2567</v>
+      </c>
+      <c r="D449" s="10" t="s">
+        <v>2568</v>
+      </c>
+      <c r="E449" s="10" t="s">
+        <v>2569</v>
+      </c>
+      <c r="F449" s="10" t="s">
+        <v>2570</v>
+      </c>
+      <c r="G449" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H449" s="10" t="str">
+        <f aca="false">IF(G446="BUG","BUG-"&amp;A446,IF(G446="FUNCTIONAL","FUNCTIONAL-"&amp;A446,""))</f>
+        <v/>
+      </c>
+      <c r="I449" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="L449" s="11" t="s">
+        <v>2571</v>
       </c>
     </row>
   </sheetData>
@@ -23188,7 +23239,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>2566</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23196,13 +23247,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2567</v>
+        <v>2573</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2568</v>
+        <v>2574</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23259,7 +23310,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -23271,11 +23322,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>2569</v>
+        <v>2575</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
DEC-72: aggiornare xlsx (TC-N615 riscritta, nuove TC-N618/TC-N619)
TC-N618: verifica manuale che il focus non venga rubato ai campi reali.
TC-N619: verifica che il badge target non trovato compaia sempre (con
o senza link) quando la route non combacia, nei due scenari reali
(Giorni spot dopo il salvataggio; step ancora in corso su una pagina
qualunque). Ricalcolato: 492 formule, 0 errori.
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3938" uniqueCount="2576">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3956" uniqueCount="2588">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -7659,16 +7659,16 @@
     <t xml:space="preserve">Il badge 'target non trovato' per lo step 'Configura i Giorni spot' mostra un link REALE verso il Calendario disponibilita', non solo testo (DEC-69)</t>
   </si>
   <si>
-    <t xml:space="preserve">Login center_admin; flag TRAMA_ONE_ENABLED attivo; almeno un'attivita' esistente nel centro collegato; step precedenti (configure_weeks/configure_pricing) completati con il flusso manuale 'Inizia' + 'Ho finito, continua -&gt;' (DEC-71), poi publish completato cliccando l'elemento reale 'Salva modifiche'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Login gestore -&gt; apri un'attivita' esistente -&gt; step Informazioni di base: click 'Inizia' poi click 'Ho finito, continua -&gt;' -&gt; step Servizi extra e pasto: click 'Inizia', poi click sulla checkbox reale 'Ingresso anticipato (pre-servizio)' (verifica che lo step NON avanzi da solo), poi click 'Ho finito, continua -&gt;' -&gt; click su Salva modifiche (publish)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gli step 'manuali' (Informazioni di base, Servizi extra e pasto) NON avanzano al click su un campo reale della card: resta visibile il popover con il testo 'Compila con calma i campi di questa sezione, poi continua.' finche' non si clicca il pulsante esplicito 'Ho finito, continua -&gt;'. Dopo publish, il badge 'target non trovato' mostra il titolo 'Configura i Giorni spot' e un link cliccabile 'Vai al Calendario disponibilita' →' con href verso .../calendar; il click naviga davvero li'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test automatizzato: tests/one/walkthrough-partner.spec.ts, TC-N615. Bug reale trovato da Fabrizio (DEC-69): prima di questo fix il badge dava solo testo per Giorni spot. Fix: campo spotlightMissingHint in lib/walkthrough/registry.ts, reso come &lt;Link&gt; reale in PartnerSpotlight.tsx. Aggiornato per DEC-71: secondo bug reale di Fabrizio, cliccare un campo dentro Servizi extra/Informazioni di base avanzava subito lo step impedendo di finire la configurazione. Fix: campo spotlightManualAdvance, pulsante esplicito 'Ho finito, continua -&gt;'.</t>
+    <t xml:space="preserve">Login center_admin; flag TRAMA_ONE_ENABLED attivo; almeno un'attivita' esistente nel centro collegato; step create_activity gia' completato (unico step che richiede 'Inizia' esplicito, DEC-72) cosi' che configure_weeks risulti gia' avviato in automatico all'arrivo su questa scheda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login gestore -&gt; apri un'attivita' esistente -&gt; step Informazioni di base: GIA' avviato (nessun 'Inizia', DEC-72), click 'Ho finito, continua -&gt;' -&gt; step Servizi extra e pasto: GIA' avviato, click sulla checkbox reale 'Ingresso anticipato (pre-servizio)' (verifica che lo step NON avanzi da solo e il focus non sparisca), poi click 'Ho finito, continua -&gt;' -&gt; click su Salva modifiche (publish, gia' avviato, click-based)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nessuno step dopo il primo (create_activity) mostra il pulsante 'Inizia' (DEC-72): si avviano da soli. Gli step 'manuali' (Informazioni di base, Servizi extra e pasto) NON avanzano al click su un campo reale della card: resta visibile il popover con 'Compila con calma i campi di questa sezione, poi continua.' finche' non si clicca il pulsante esplicito 'Ho finito, continua -&gt;'. Dopo publish, il badge 'target non trovato' mostra il titolo 'Configura i Giorni spot' e un link cliccabile 'Vai al Calendario disponibilita' →' con href verso .../calendar (DEC-72: prima di questo fix non compariva NULLA, bug bloccante); il click naviga davvero li'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automatizzato: tests/one/walkthrough-partner.spec.ts, TC-N615. Bug reale trovato da Fabrizio (DEC-69): prima di questo fix il badge dava solo testo per Giorni spot. Fix: campo spotlightMissingHint in lib/walkthrough/registry.ts. DEC-71: cliccare un campo dentro Servizi extra/Informazioni di base avanzava subito lo step. Fix: campo spotlightManualAdvance, pulsante 'Ho finito, continua -&gt;'. DEC-72: 3 bug reali aggiuntivi trovati da Fabrizio testando il deploy di DEC-71 -- focus rubato ogni 500ms (cursore che sparisce), booleano invertito che faceva sparire l'intero badge 'target non trovato' (righe 16/18), 'Inizia' ripetuto senza motivo per ogni step. Vedi TC-N618/TC-N619 per la copertura dedicata dei primi due.</t>
   </si>
   <si>
     <t xml:space="preserve">TC-N616</t>
@@ -7711,6 +7711,42 @@
   </si>
   <si>
     <t xml:space="preserve">Test automatizzato: tests/one/walkthrough-partner.spec.ts, incluso nel test TC-N615 (stessa run seriale). Bug reale segnalato da Fabrizio: 'se clicco una delle impostazioni dello step (es. servizi extra clicco ingresso anticipato..) va direttamente nello step successivo e non permette di finire la configurazione'. Fix: campo spotlightManualAdvance in lib/walkthrough/registry.ts + lib/walkthrough/data.ts, click-capture listener disattivato per questi step in PartnerSpotlight.tsx, nuovo pulsante 'Ho finito, continua -&gt;'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N618</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il popover NON deve rubare il focus a un campo reale mentre l'utente lo sta compilando dentro uno step 'manuale' -- il cursore non deve sparire ne' un menu a tendina nativo deve chiudersi da solo (DEC-72)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login center_admin; flag TRAMA_ONE_ENABLED attivo; step configure_pricing corrente e gia' avviato</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri un'attivita' esistente -&gt; arriva allo step 'Servizi extra e pasto' (gia' avviato) -&gt; clicca un campo di testo reale (es. un input orario di un servizio extra) e digita -&gt; attendi almeno 1-2 secondi senza cliccare altrove -&gt; verifica che il cursore/focus resti nel campo -&gt; apri il menu a tendina 'Pasto' e prova a scegliere un'opzione con calma (non un click immediato)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il cursore/focus resta nel campo di testo per tutto il tempo necessario a digitare, senza sparire da solo; il menu a tendina 'Pasto' resta aperto abbastanza a lungo da poter scegliere un'opzione con calma, senza chiudersi da solo prima del click sull'opzione</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verifica manuale (richiede timing reale, non facilmente automatizzabile in modo affidabile con Playwright headless). Bug reale segnalato da Fabrizio: 'se clicco nel campo il cursore poi sembra sparire', 'la scelta del pasto appare ma non riesco a selezionare per tempo'. Causa: components/spotlight/PartnerSpotlight.tsx, l'effetto di focus sul popover dipendeva da targetRect (nuovo oggetto ad ogni measure(), che gira ogni 500ms via setInterval), rifocalizzando il popover a ripetizione e rubando il focus al campo reale. Fix: targetRect aggiornato solo se davvero cambiato (stessa referenza altrimenti) + focus del popover una sola volta per step (focusedStepRef, stesso pattern di scrolledStepRef).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N619</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il badge 'target non trovato' deve comparire (con o senza link a seconda dello step) OGNI VOLTA che la pagina corrente non corrisponde alla route dello step corrente -- non deve sparire l'intero componente (DEC-72)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login center_admin; flag TRAMA_ONE_ENABLED attivo; step corrente con spotlightRoute che non combacia con la pagina su cui ci si trova</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caso A: dopo aver salvato un'attivita' (step passato a configure_spot_days), restare sulla pagina di modifica (senza navigare al calendario) -&gt; verificare che compaia il badge con link 'Vai al Calendario disponibilita' →'. Caso B: con lo step ancora 'Informazioni di base' o 'Servizi extra e pasto', navigare su /center/profile (pagina senza alcun target Spotlight) -&gt; verificare che compaia il badge SENZA link</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In ENTRAMBI i casi compare il badge 'target non trovato' in alto a destra con titolo e descrizione dello step corrente -- mai una pagina completamente priva di badge/overlay mentre esiste uno step Spotlight attivo e la route non combacia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bug reale segnalato da Fabrizio: 'dopo aver fatto salva non mi fa capire che devo andare nel Calendario disponibilita''. Causa: components/spotlight/PartnerSpotlight.tsx, measure() impostava targetMissing=false (invece di true) quando la route non combacia, e 'if (!targetRect &amp;&amp; !targetMissing) return null' faceva si' che l'intero componente non renderizzasse nulla -- bug presente anche per il Caso B (riga 18 della matrice Visual Acceptance), mai realmente verificabile prima d'ora perche' gli unici step verificati manualmente in precedenza (create_activity/configure_weeks) usano un pattern di route 'prefisso*' che combacia quasi sempre, mascherando il bug.</t>
   </si>
   <si>
     <t xml:space="preserve">TC-N417</t>
@@ -8586,7 +8622,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L449"/>
+  <dimension ref="A1:L451"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -23121,7 +23157,7 @@
         <v>2560</v>
       </c>
       <c r="B448" s="10" t="s">
-        <v>2547</v>
+        <v>2354</v>
       </c>
       <c r="C448" s="10" t="s">
         <v>2561</v>
@@ -23130,31 +23166,31 @@
         <v>2562</v>
       </c>
       <c r="E448" s="10" t="s">
-        <v>2550</v>
+        <v>2563</v>
       </c>
       <c r="F448" s="10" t="s">
-        <v>2563</v>
+        <v>2564</v>
       </c>
       <c r="G448" s="10" t="s">
-        <v>2552</v>
+        <v>74</v>
       </c>
       <c r="H448" s="10" t="str">
-        <f aca="false">IF(G445="BUG","BUG-"&amp;A445,IF(G445="FUNCTIONAL","FUNCTIONAL-"&amp;A445,""))</f>
+        <f aca="false">IF(G448="BUG","BUG-"&amp;A448,IF(G448="FUNCTIONAL","FUNCTIONAL-"&amp;A448,""))</f>
         <v/>
       </c>
       <c r="I448" s="10" t="s">
-        <v>65</v>
+        <v>42</v>
       </c>
       <c r="L448" s="11" t="s">
-        <v>2564</v>
-      </c>
-    </row>
-    <row r="449" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>2565</v>
+      </c>
+    </row>
+    <row r="449" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A449" s="10" t="s">
-        <v>2565</v>
+        <v>2566</v>
       </c>
       <c r="B449" s="10" t="s">
-        <v>2566</v>
+        <v>2354</v>
       </c>
       <c r="C449" s="10" t="s">
         <v>2567</v>
@@ -23172,14 +23208,80 @@
         <v>74</v>
       </c>
       <c r="H449" s="10" t="str">
-        <f aca="false">IF(G446="BUG","BUG-"&amp;A446,IF(G446="FUNCTIONAL","FUNCTIONAL-"&amp;A446,""))</f>
+        <f aca="false">IF(G449="BUG","BUG-"&amp;A449,IF(G449="FUNCTIONAL","FUNCTIONAL-"&amp;A449,""))</f>
         <v/>
       </c>
       <c r="I449" s="10" t="s">
-        <v>65</v>
+        <v>42</v>
       </c>
       <c r="L449" s="11" t="s">
         <v>2571</v>
+      </c>
+    </row>
+    <row r="450" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A450" s="10" t="s">
+        <v>2572</v>
+      </c>
+      <c r="B450" s="10" t="s">
+        <v>2547</v>
+      </c>
+      <c r="C450" s="10" t="s">
+        <v>2573</v>
+      </c>
+      <c r="D450" s="10" t="s">
+        <v>2574</v>
+      </c>
+      <c r="E450" s="10" t="s">
+        <v>2550</v>
+      </c>
+      <c r="F450" s="10" t="s">
+        <v>2575</v>
+      </c>
+      <c r="G450" s="10" t="s">
+        <v>2552</v>
+      </c>
+      <c r="H450" s="10" t="str">
+        <f aca="false">IF(G445="BUG","BUG-"&amp;A445,IF(G445="FUNCTIONAL","FUNCTIONAL-"&amp;A445,""))</f>
+        <v/>
+      </c>
+      <c r="I450" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="L450" s="11" t="s">
+        <v>2576</v>
+      </c>
+    </row>
+    <row r="451" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A451" s="10" t="s">
+        <v>2577</v>
+      </c>
+      <c r="B451" s="10" t="s">
+        <v>2578</v>
+      </c>
+      <c r="C451" s="10" t="s">
+        <v>2579</v>
+      </c>
+      <c r="D451" s="10" t="s">
+        <v>2580</v>
+      </c>
+      <c r="E451" s="10" t="s">
+        <v>2581</v>
+      </c>
+      <c r="F451" s="10" t="s">
+        <v>2582</v>
+      </c>
+      <c r="G451" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H451" s="10" t="str">
+        <f aca="false">IF(G446="BUG","BUG-"&amp;A446,IF(G446="FUNCTIONAL","FUNCTIONAL-"&amp;A446,""))</f>
+        <v/>
+      </c>
+      <c r="I451" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="L451" s="11" t="s">
+        <v>2583</v>
       </c>
     </row>
   </sheetData>
@@ -23239,7 +23341,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>2572</v>
+        <v>2584</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23247,13 +23349,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2573</v>
+        <v>2585</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2574</v>
+        <v>2586</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23310,7 +23412,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -23322,11 +23424,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>2575</v>
+        <v>2587</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
test(xlsx): add TC-N620..TC-N623 rows for DEC-73 fixes
Ricalcolato: 496 formule, 0 errori.
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3956" uniqueCount="2588">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3992" uniqueCount="2612">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -7783,6 +7783,78 @@
   </si>
   <si>
     <t xml:space="preserve">Test automatizzato: tests/one/command-center.spec.ts, TC-N418.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N620</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il badge 'target non trovato' per lo step 'Monitora dalla dashboard' mostra una nota di aiuto quando il nav item non e' visibile su mobile con il cassetto chiuso (DEC-73)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login center_admin; flag TRAMA_ONE_ENABLED attivo; percorso arrivato allo step finale 'dashboard'; viewport mobile (390px), cassetto laterale chiuso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Con lo step 'dashboard' corrente e il cassetto laterale chiuso, osservare il badge 'target non trovato' in alto a destra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il badge mostra titolo 'Monitora dalla dashboard', la descrizione originale, e in piu' una nota testuale (nessun link, non serve navigare): 'Su schermi piccoli, apri il menu (hamburger) in alto per trovare la voce Dashboard nel cassetto laterale.' Aprendo il cassetto, il nav item viene evidenziato normalmente (comportamento DEC-70 invariato).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bug reale segnalato da Fabrizio: 'nella schermata dei giorni spot c'e' qualcosa che non funziona..l'elemento dashboard non e' evidenziato..l'ho visto solo aprendo il menu laterale'. Causa: il badge di fallback per il target 'dashboard' (visibile solo a cassetto aperto su mobile, DEC-70) non dava alcun indizio su COME renderlo visibile. Fix: nuovo campo opzionale spotlightMissingNote in lib/walkthrough/registry.ts/data.ts, mostrato nel badge in components/spotlight/PartnerSpotlight.tsx. Test automatizzato 'no browser' del dato nel registry: tests/one/walkthrough-partner.spec.ts, TC-N620 (verifica manuale del rendering reale del badge su mobile nel prossimo giro di test live, troppo fragile da automatizzare in modo affidabile qui).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N621</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il riquadro (ring) del cutout attorno all'elemento evidenziato deve avere angoli visibilmente arrotondati quando l'elemento reale lo e' (es. Salva modifiche, rounded-md) -- non 'squadrato' (DEC-73)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">npx playwright test tests/one/spotlight-position.spec.ts -g padBorderRadius</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6/6 assert passano: 6px -&gt; 14px (caso reale 'Salva modifiche'); padding esplicito rispettato; 9999px (pulsante pillola) resta una pillola; shorthand a piu' valori incrementato token per token; token non in px (es. '%') invariato; stringa vuota invariata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bug reale segnalato da Fabrizio (dopo il fix DEC-70): 'Come vedi il riquadro intorno ai pulsanti e' ancora squadrato ci sono gli angoli'. Causa: il ring usa il border-radius REALE del target (getComputedStyle, DEC-70) ma il cutout e' quel rettangolo ingrandito di 8px per lato (computeCutoutRect) -- applicare lo STESSO raggio numerico a un box piu' grande appiattisce visivamente la curvatura (6px su un box alto ~56px e' quasi impercettibile). Fix: nuova funzione pura padBorderRadius in lib/spotlight/position.ts (raggio_nuovo = raggio_originale + padding), usata in components/spotlight/PartnerSpotlight.tsx. Test eseguito nel sandbox Claude (106/106 passed su chromium+mobile-chrome per l'intera suite no-browser tests/one/).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N622</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nel passaggio automatico da uno step al successivo (DEC-72), il popover/cutout non deve mostrare per un frame la posizione del target APPENA CONCLUSO sovrapposta al testo del nuovo step (DEC-73)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login center_admin; flag TRAMA_ONE_ENABLED attivo; step 'Servizi extra e pasto' corrente e completabile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Completare lo step 'Servizi extra e pasto' (click 'Ho finito, continua -&gt;') e osservare con attenzione (idealmente uno screen recording) la transizione verso lo step 'Pubblica'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nessun frame visibile in cui popover/cutout restano ancorati alla posizione del target precedente mentre mostrano gia' titolo/descrizione del nuovo step; il componente puo' sparire per un singolo frame e ricomparire correttamente posizionato, ma non deve mai mostrare una posizione sbagliata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bug reale segnalato da Fabrizio: 'Nel passaggio da step 3 a 4 la schermata del walkthrough cambia ma non son riuscito a registrarlo..comunque e' sovrapposto' (troppo rapido per uno screenshot). Causa: quando currentKey cambia, targetRect/targetMissing restavano quelli dello step concluso fino al tick successivo di measure() (schedulato via rAF, un frame dopo) -- un frame con testo nuovo e posizione vecchia. Fix: pattern React 'adjusting state while rendering' (confronto con l'ultimo currentKey renderizzato, azzeramento sincrono di targetRect/targetMissing durante il render stesso, non in un effetto) in components/spotlight/PartnerSpotlight.tsx. Verifica manuale (timing visivo di un singolo frame, non automatizzabile in modo affidabile con Playwright).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N623</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRAMA ONE - Menu Impostazioni Gestore/Genitore (ProfileSettingsSection)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il sottotitolo della voce 'Preferenze' nel menu Impostazioni del Gestore menziona anche il tour guidato (riavviabile da li'), il profilo Genitore resta invariato (nessun tour da riavviare ancora) (DEC-73)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login center_admin; flag TRAMA_ONE_ENABLED attivo (mostra il bottone di riavvio tour dentro Preferenze)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login gestore -&gt; apri /center/account -&gt; osserva il sottotitolo della voce 'Preferenze' nel menu Impostazioni. Ripetere login genitore -&gt; /profile -&gt; stesso controllo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lato Gestore il sottotitolo e' 'Lingua, tema, notifiche, tour guidato'. Lato Genitore il sottotitolo resta 'Lingua, tema, notifiche' (nessuna menzione di tour guidato: lo Spotlight Parent non e' ancora stato costruito, task #441 backlog)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Richiesta esplicita di Fabrizio: 'Nel sottotitolo del menu Preferenze va indicato anche tour guidato'. Fix: components/ProfileSettingsSection.tsx, sottotitolo condizionale su basePath (solo /center/account menziona il tour, dove vive gia' WalkthroughRestartButton dentro app/center/account/preferenze/page.tsx). Test automatizzato: tests/gestore/account.spec.ts, TC-138 aggiornato per asserire il nuovo testo completo; tests/genitori/profilo.spec.ts invariato (asserisce ancora il testo originale, corretto perche' lato Genitore non cambia).</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -8622,7 +8694,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L451"/>
+  <dimension ref="A1:L455"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -23218,7 +23290,7 @@
         <v>2571</v>
       </c>
     </row>
-    <row r="450" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="450" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A450" s="10" t="s">
         <v>2572</v>
       </c>
@@ -23251,7 +23323,7 @@
         <v>2576</v>
       </c>
     </row>
-    <row r="451" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="451" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A451" s="10" t="s">
         <v>2577</v>
       </c>
@@ -23282,6 +23354,138 @@
       </c>
       <c r="L451" s="11" t="s">
         <v>2583</v>
+      </c>
+    </row>
+    <row r="452" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A452" s="10" t="s">
+        <v>2584</v>
+      </c>
+      <c r="B452" s="10" t="s">
+        <v>2354</v>
+      </c>
+      <c r="C452" s="10" t="s">
+        <v>2585</v>
+      </c>
+      <c r="D452" s="10" t="s">
+        <v>2586</v>
+      </c>
+      <c r="E452" s="10" t="s">
+        <v>2587</v>
+      </c>
+      <c r="F452" s="10" t="s">
+        <v>2588</v>
+      </c>
+      <c r="G452" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H452" s="10" t="str">
+        <f aca="false">IF(G452="BUG","BUG-"&amp;A452,IF(G452="FUNCTIONAL","FUNCTIONAL-"&amp;A452,""))</f>
+        <v/>
+      </c>
+      <c r="I452" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="L452" s="11" t="s">
+        <v>2589</v>
+      </c>
+    </row>
+    <row r="453" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A453" s="10" t="s">
+        <v>2590</v>
+      </c>
+      <c r="B453" s="10" t="s">
+        <v>2354</v>
+      </c>
+      <c r="C453" s="10" t="s">
+        <v>2591</v>
+      </c>
+      <c r="D453" s="10" t="s">
+        <v>2549</v>
+      </c>
+      <c r="E453" s="10" t="s">
+        <v>2592</v>
+      </c>
+      <c r="F453" s="10" t="s">
+        <v>2593</v>
+      </c>
+      <c r="G453" s="10" t="s">
+        <v>2552</v>
+      </c>
+      <c r="H453" s="10" t="str">
+        <f aca="false">IF(G453="BUG","BUG-"&amp;A453,IF(G453="FUNCTIONAL","FUNCTIONAL-"&amp;A453,""))</f>
+        <v/>
+      </c>
+      <c r="I453" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="L453" s="11" t="s">
+        <v>2594</v>
+      </c>
+    </row>
+    <row r="454" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A454" s="10" t="s">
+        <v>2595</v>
+      </c>
+      <c r="B454" s="10" t="s">
+        <v>2354</v>
+      </c>
+      <c r="C454" s="10" t="s">
+        <v>2596</v>
+      </c>
+      <c r="D454" s="10" t="s">
+        <v>2597</v>
+      </c>
+      <c r="E454" s="10" t="s">
+        <v>2598</v>
+      </c>
+      <c r="F454" s="10" t="s">
+        <v>2599</v>
+      </c>
+      <c r="G454" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H454" s="10" t="str">
+        <f aca="false">IF(G454="BUG","BUG-"&amp;A454,IF(G454="FUNCTIONAL","FUNCTIONAL-"&amp;A454,""))</f>
+        <v/>
+      </c>
+      <c r="I454" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="L454" s="11" t="s">
+        <v>2600</v>
+      </c>
+    </row>
+    <row r="455" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A455" s="10" t="s">
+        <v>2601</v>
+      </c>
+      <c r="B455" s="10" t="s">
+        <v>2602</v>
+      </c>
+      <c r="C455" s="10" t="s">
+        <v>2603</v>
+      </c>
+      <c r="D455" s="10" t="s">
+        <v>2604</v>
+      </c>
+      <c r="E455" s="10" t="s">
+        <v>2605</v>
+      </c>
+      <c r="F455" s="10" t="s">
+        <v>2606</v>
+      </c>
+      <c r="G455" s="10" t="s">
+        <v>2552</v>
+      </c>
+      <c r="H455" s="10" t="str">
+        <f aca="false">IF(G455="BUG","BUG-"&amp;A455,IF(G455="FUNCTIONAL","FUNCTIONAL-"&amp;A455,""))</f>
+        <v/>
+      </c>
+      <c r="I455" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="L455" s="11" t="s">
+        <v>2607</v>
       </c>
     </row>
   </sheetData>
@@ -23341,7 +23545,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>2584</v>
+        <v>2608</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23349,13 +23553,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2585</v>
+        <v>2609</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2586</v>
+        <v>2610</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23412,7 +23616,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -23424,11 +23628,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>2587</v>
+        <v>2611</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
test(xlsx): add TC-N624 row (E2E ring radius + dashboard step, DEC-74)
Ricalcolato: 497 formule, 0 errori.
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3992" uniqueCount="2612">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4001" uniqueCount="2618">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -7855,6 +7855,24 @@
   </si>
   <si>
     <t xml:space="preserve">Richiesta esplicita di Fabrizio: 'Nel sottotitolo del menu Preferenze va indicato anche tour guidato'. Fix: components/ProfileSettingsSection.tsx, sottotitolo condizionale su basePath (solo /center/account menziona il tour, dove vive gia' WalkthroughRestartButton dentro app/center/account/preferenze/page.tsx). Test automatizzato: tests/gestore/account.spec.ts, TC-138 aggiornato per asserire il nuovo testo completo; tests/genitori/profilo.spec.ts invariato (asserisce ancora il testo originale, corretto perche' lato Genitore non cambia).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N624</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copertura E2E reale (non solo unit test) di 2 verifiche prima ritenute 'troppo fragili da automatizzare': raggio del cutout applicato davvero nel DOM, e badge/evidenziazione dello step finale 'dashboard' su mobile a cassetto chiuso/aperto (DEC-74)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login center_admin; flag TRAMA_ONE_ENABLED attivo; percorso arrivato allo step 'Configura i Giorni spot' (prosegue dallo stato lasciato da TC-N615, serial)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nel test TC-N615: prima di cliccare 'Salva modifiche', leggere via getComputedStyle il border-radius reale del ring (data-testid=spotlight-cutout-ring). Nel test TC-N624 (nuovo): completare 'Configura i Giorni spot' (Ho finito, continua), poi verificare lo step 'dashboard' -- su viewport mobile (&lt;768px) a cassetto chiuso, poi aprendolo; su desktop/tablet direttamente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il border-radius calcolato del ring e' 14px (6px reali del pulsante 'Salva modifiche' + 8px di padding del cutout, DEC-73) - prova diretta della curvatura, non solo della funzione pura. Su mobile a cassetto chiuso compare il badge con la nota 'apri il menu' (DEC-73); aprendo il cassetto (bottone 'Apri il menu') compare il popover reale ancorato alla voce Dashboard. Su desktop/tablet il popover compare subito, nessun badge necessario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Richiesta esplicita di Fabrizio dopo DEC-73: 'non c'e' modo nessuno di renderlo automatizzato il test?' -- rivisto il giudizio iniziale (TC-N620, 'troppo fragile/lento'): non lo era, serviva solo completare la sequenza fino in fondo e aggiungere un data-testid al ring per poterlo selezionare. Aggiunto data-testid='spotlight-cutout-ring' in components/spotlight/PartnerSpotlight.tsx (nessun impatto visivo/comportamentale, solo per i test). Non ancora eseguito in questo ambiente (stessa limitazione nota: Chromium senza le dipendenze di sistema nel sandbox Claude) -- verificabile da Fabrizio col prossimo bash test-deploy.sh/deploy.sh (TC-N624 gira sotto sia chromium che mobile-chrome, con INCLUDE_MOBILE=1 per includere quest'ultimo).</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -8694,7 +8712,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L455"/>
+  <dimension ref="A1:L456"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -23356,7 +23374,7 @@
         <v>2583</v>
       </c>
     </row>
-    <row r="452" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="452" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A452" s="10" t="s">
         <v>2584</v>
       </c>
@@ -23389,7 +23407,7 @@
         <v>2589</v>
       </c>
     </row>
-    <row r="453" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="453" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A453" s="10" t="s">
         <v>2590</v>
       </c>
@@ -23422,7 +23440,7 @@
         <v>2594</v>
       </c>
     </row>
-    <row r="454" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="454" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A454" s="10" t="s">
         <v>2595</v>
       </c>
@@ -23455,7 +23473,7 @@
         <v>2600</v>
       </c>
     </row>
-    <row r="455" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="455" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A455" s="10" t="s">
         <v>2601</v>
       </c>
@@ -23486,6 +23504,39 @@
       </c>
       <c r="L455" s="11" t="s">
         <v>2607</v>
+      </c>
+    </row>
+    <row r="456" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A456" s="10" t="s">
+        <v>2608</v>
+      </c>
+      <c r="B456" s="10" t="s">
+        <v>2354</v>
+      </c>
+      <c r="C456" s="10" t="s">
+        <v>2609</v>
+      </c>
+      <c r="D456" s="10" t="s">
+        <v>2610</v>
+      </c>
+      <c r="E456" s="10" t="s">
+        <v>2611</v>
+      </c>
+      <c r="F456" s="10" t="s">
+        <v>2612</v>
+      </c>
+      <c r="G456" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H456" s="10" t="str">
+        <f aca="false">IF(G456="BUG","BUG-"&amp;A456,IF(G456="FUNCTIONAL","FUNCTIONAL-"&amp;A456,""))</f>
+        <v/>
+      </c>
+      <c r="I456" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="L456" s="11" t="s">
+        <v>2613</v>
       </c>
     </row>
   </sheetData>
@@ -23545,7 +23596,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>2608</v>
+        <v>2614</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23553,13 +23604,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2609</v>
+        <v>2615</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2610</v>
+        <v>2616</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23616,7 +23667,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -23628,11 +23679,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>2611</v>
+        <v>2617</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
docs(trama-one): DEC-75 + xlsx TC-N625 - estensione Segnalazioni al portale Partner
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4001" uniqueCount="2618">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4009" uniqueCount="2625">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -7873,6 +7873,27 @@
   </si>
   <si>
     <t xml:space="preserve">Richiesta esplicita di Fabrizio dopo DEC-73: 'non c'e' modo nessuno di renderlo automatizzato il test?' -- rivisto il giudizio iniziale (TC-N620, 'troppo fragile/lento'): non lo era, serviva solo completare la sequenza fino in fondo e aggiungere un data-testid al ring per poterlo selezionare. Aggiunto data-testid='spotlight-cutout-ring' in components/spotlight/PartnerSpotlight.tsx (nessun impatto visivo/comportamentale, solo per i test). Non ancora eseguito in questo ambiente (stessa limitazione nota: Chromium senza le dipendenze di sistema nel sandbox Claude) -- verificabile da Fabrizio col prossimo bash test-deploy.sh/deploy.sh (TC-N624 gira sotto sia chromium che mobile-chrome, con INCLUDE_MOBILE=1 per includere quest'ultimo).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N625</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRAMA ONE - Segnalazioni BETA (estensione Partner)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il pulsante flottante 'Segnala un problema' (gia' presente lato genitore) e' raggiungibile anche dal portale Partner (/center/*), con area calcolata sulle rotte del menu Partner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login come gestore (center_admin), qualunque pagina sotto /center/*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apri una pagina qualunque del portale Partner (es. /center/activities) -&gt; individua il pulsante flottante viola in basso a destra (icona segnalazione) -&gt; clicca -&gt; compila un messaggio -&gt; invia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si apre il dialog 'Segnala un problema' con l'area corretta indicata (es. 'Attivita''), l'invio va a buon fine, il dialog mostra una conferma interna ('Segnalazione inviata, grazie!') e si chiude da solo; la riga compare in Admin &gt; Segnalazioni BETA con etichetta 'App gestori'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estensione richiesta da Fabrizio ('il pulsante per le segnalazioni... nel portale partner?'): app_source='gestore' gia' supportato da schema/RLS/Admin, nessuna migrazione necessaria (DEC-75). Copertura automatica solo per la funzione pura area-&gt;label (centerAreaLabelFromPath, tests/gestore/beta-feedback-center.spec.ts); l'interazione reale col pulsante (drag, apertura dialog, invio) richiede un browser reale, non eseguibile in questo sandbox.</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -8712,7 +8733,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L456"/>
+  <dimension ref="A1:L457"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -23506,7 +23527,7 @@
         <v>2607</v>
       </c>
     </row>
-    <row r="456" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="456" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A456" s="10" t="s">
         <v>2608</v>
       </c>
@@ -23537,6 +23558,36 @@
       </c>
       <c r="L456" s="11" t="s">
         <v>2613</v>
+      </c>
+    </row>
+    <row r="457" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A457" s="10" t="s">
+        <v>2614</v>
+      </c>
+      <c r="B457" s="10" t="s">
+        <v>2615</v>
+      </c>
+      <c r="C457" s="10" t="s">
+        <v>2616</v>
+      </c>
+      <c r="D457" s="10" t="s">
+        <v>2617</v>
+      </c>
+      <c r="E457" s="10" t="s">
+        <v>2618</v>
+      </c>
+      <c r="F457" s="10" t="s">
+        <v>2619</v>
+      </c>
+      <c r="H457" s="10" t="str">
+        <f aca="false">IF(G457="BUG","BUG-"&amp;A457,IF(G457="FUNCTIONAL","FUNCTIONAL-"&amp;A457,""))</f>
+        <v/>
+      </c>
+      <c r="I457" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="L457" s="11" t="s">
+        <v>2620</v>
       </c>
     </row>
   </sheetData>
@@ -23596,7 +23647,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>2614</v>
+        <v>2621</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23604,13 +23655,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2615</v>
+        <v>2622</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2616</v>
+        <v>2623</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23679,11 +23730,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>2617</v>
+        <v>2624</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
docs(trama-one): DEC-76 - fix scroll drawer mobile, toggle password, diagnosi conferma email Partner
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4009" uniqueCount="2625">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4017" uniqueCount="2632">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -7894,6 +7894,27 @@
   </si>
   <si>
     <t xml:space="preserve">Estensione richiesta da Fabrizio ('il pulsante per le segnalazioni... nel portale partner?'): app_source='gestore' gia' supportato da schema/RLS/Admin, nessuna migrazione necessaria (DEC-75). Copertura automatica solo per la funzione pura area-&gt;label (centerAreaLabelFromPath, tests/gestore/beta-feedback-center.spec.ts); l'interazione reale col pulsante (drag, apertura dialog, invio) richiede un browser reale, non eseguibile in questo sandbox.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-511</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login/Sicurezza - Visualizzazione password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'icona occhio nel campo password (login, cambio password Profilo/Account, reset password) alterna testo in chiaro/nascosto (Fabrizio: 'aggiungiamo l'opzione di visualizzare la password in tutti i punti in cui e richiesta?')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pagina /auth/login (tab Accedi o Registrati), oppure Profilo/Account &gt; Sicurezza, oppure link di reset password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scrivi una password nel campo -&gt; clicca l'icona a forma di occhio a destra del campo -&gt; osserva il testo -&gt; clicca di nuovo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il testo diventa visibile in chiaro al primo click (icona 'occhio barrato', aria-label 'Nascondi password'), torna nascosto (pallini) al secondo click (icona 'occhio', aria-label 'Mostra password'); il valore digitato non cambia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stesso toggle replicato in 3 punti indipendenti (LoginForm.tsx, ProfileSecuritySection.tsx, auth/reset-password/page.tsx) - nessun componente condiviso creato per non introdurre un'astrazione prematura su 3 stili di input leggermente diversi</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -8733,7 +8754,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L457"/>
+  <dimension ref="A1:L458"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -23588,6 +23609,36 @@
       </c>
       <c r="L457" s="11" t="s">
         <v>2620</v>
+      </c>
+    </row>
+    <row r="458" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A458" s="10" t="s">
+        <v>2621</v>
+      </c>
+      <c r="B458" s="10" t="s">
+        <v>2622</v>
+      </c>
+      <c r="C458" s="10" t="s">
+        <v>2623</v>
+      </c>
+      <c r="D458" s="10" t="s">
+        <v>2624</v>
+      </c>
+      <c r="E458" s="10" t="s">
+        <v>2625</v>
+      </c>
+      <c r="F458" s="10" t="s">
+        <v>2626</v>
+      </c>
+      <c r="H458" s="10" t="str">
+        <f aca="false">IF(G458="BUG","BUG-"&amp;A458,IF(G458="FUNCTIONAL","FUNCTIONAL-"&amp;A458,""))</f>
+        <v/>
+      </c>
+      <c r="I458" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="L458" s="11" t="s">
+        <v>2627</v>
       </c>
     </row>
   </sheetData>
@@ -23647,7 +23698,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>2621</v>
+        <v>2628</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23655,13 +23706,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2622</v>
+        <v>2629</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2623</v>
+        <v>2630</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23730,11 +23781,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>2624</v>
+        <v>2631</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
docs(trama-one): DEC-77 - Candidati come centro + xlsx TC-512..514
Chiude il gap architetturale diagnosticato in DEC-76 (nessuna
registrazione self-service per diventare gestore).
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4017" uniqueCount="2632">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4044" uniqueCount="2649">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -7915,6 +7915,57 @@
   </si>
   <si>
     <t xml:space="preserve">Stesso toggle replicato in 3 punti indipendenti (LoginForm.tsx, ProfileSecuritySection.tsx, auth/reset-password/page.tsx) - nessun componente condiviso creato per non introdurre un'astrazione prematura su 3 stili di input leggermente diversi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-512</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Candidati come centro (Partner) - Migrazione 21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il form pubblico /auth/candidati invia una candidatura e reindirizza alla pagina di conferma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nessun account/login richiesto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vai su /auth/candidati -&gt; compila Nome del centro, Città/zona, Email di contatto -&gt; clicca 'Invia candidatura'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redirect a /auth/candidati/conferma/[id]; la pagina mostra il nome del centro appena inserito e lo stato 'In revisione'; nessun account viene creato (verificabile: nessuna nuova riga in auth.users)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabrizio: 'il registrati deve essere un candidati per cui deve far partire processo di onboarding'. Scrive una riga in center_leads con lead_type='self_candidacy' e suggested_by=null (service client, lib/supabase/service.ts), mai un account. Vedi supabase/migration_21_center_candidacy.sql. Test: tests/gestore/candidati.spec.ts TC-512, non eseguito in questo sandbox (Chromium senza dipendenze di sistema), richiede anche il deploy col service role key configurato.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-513</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Un link di conferma con id inesistente/non valido mostra 'candidatura non trovata' invece di un errore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vai su /auth/candidati/conferma/00000000-0000-0000-0000-000000000000 (UUID inesistente)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pagina 'Candidatura non trovata' con spiegazione e link 'Candidati come centro' per inviarne una nuova</t>
+  </si>
+  <si>
+    <t xml:space="preserve">getCandidacyStatusPublic (lib/data/center-leads.ts) restituisce null per id inesistente o non di tipo self_candidacy: la pagina non fa mai trapelare un errore tecnico. Test: tests/gestore/candidati.spec.ts TC-513, non eseguito in questo sandbox (stessa limitazione Chromium).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-514</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il form Candidati richiede nome del centro ed email prima di poter essere inviato</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vai su /auth/candidati -&gt; clicca subito 'Invia candidatura' senza compilare nulla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validazione nativa del browser blocca l'invio (campi 'required'); si resta sulla stessa pagina, nessuna richiesta al server</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validazione minima lato client (attributi required/type=email), nessuna logica applicativa aggiuntiva. Test: tests/gestore/candidati.spec.ts TC-514, non eseguito in questo sandbox (stessa limitazione Chromium).</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -8754,7 +8805,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L458"/>
+  <dimension ref="A1:L461"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -23639,6 +23690,105 @@
       </c>
       <c r="L458" s="11" t="s">
         <v>2627</v>
+      </c>
+    </row>
+    <row r="459" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A459" s="10" t="s">
+        <v>2628</v>
+      </c>
+      <c r="B459" s="10" t="s">
+        <v>2629</v>
+      </c>
+      <c r="C459" s="10" t="s">
+        <v>2630</v>
+      </c>
+      <c r="D459" s="10" t="s">
+        <v>2631</v>
+      </c>
+      <c r="E459" s="10" t="s">
+        <v>2632</v>
+      </c>
+      <c r="F459" s="10" t="s">
+        <v>2633</v>
+      </c>
+      <c r="G459" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H459" s="10" t="str">
+        <f aca="false">IF(G459="BUG","BUG-"&amp;A459,IF(G459="FUNCTIONAL","FUNCTIONAL-"&amp;A459,""))</f>
+        <v/>
+      </c>
+      <c r="I459" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="L459" s="11" t="s">
+        <v>2634</v>
+      </c>
+    </row>
+    <row r="460" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A460" s="10" t="s">
+        <v>2635</v>
+      </c>
+      <c r="B460" s="10" t="s">
+        <v>2629</v>
+      </c>
+      <c r="C460" s="10" t="s">
+        <v>2636</v>
+      </c>
+      <c r="D460" s="10" t="s">
+        <v>2631</v>
+      </c>
+      <c r="E460" s="10" t="s">
+        <v>2637</v>
+      </c>
+      <c r="F460" s="10" t="s">
+        <v>2638</v>
+      </c>
+      <c r="G460" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H460" s="10" t="str">
+        <f aca="false">IF(G460="BUG","BUG-"&amp;A460,IF(G460="FUNCTIONAL","FUNCTIONAL-"&amp;A460,""))</f>
+        <v/>
+      </c>
+      <c r="I460" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="L460" s="11" t="s">
+        <v>2639</v>
+      </c>
+    </row>
+    <row r="461" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A461" s="10" t="s">
+        <v>2640</v>
+      </c>
+      <c r="B461" s="10" t="s">
+        <v>2629</v>
+      </c>
+      <c r="C461" s="10" t="s">
+        <v>2641</v>
+      </c>
+      <c r="D461" s="10" t="s">
+        <v>2631</v>
+      </c>
+      <c r="E461" s="10" t="s">
+        <v>2642</v>
+      </c>
+      <c r="F461" s="10" t="s">
+        <v>2643</v>
+      </c>
+      <c r="G461" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H461" s="10" t="str">
+        <f aca="false">IF(G461="BUG","BUG-"&amp;A461,IF(G461="FUNCTIONAL","FUNCTIONAL-"&amp;A461,""))</f>
+        <v/>
+      </c>
+      <c r="I461" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="L461" s="11" t="s">
+        <v>2644</v>
       </c>
     </row>
   </sheetData>
@@ -23698,7 +23848,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>2628</v>
+        <v>2645</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23706,13 +23856,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2629</v>
+        <v>2646</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2630</v>
+        <v>2647</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23769,7 +23919,7 @@
       </c>
       <c r="B6" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -23781,11 +23931,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>2631</v>
+        <v>2648</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
test(OD-02): aggiungere TC-N626..TC-N636 alla matrice di test
Righe per i test Playwright del fix bulk 'Giornata particolare' del
Calendario disponibilità Partner (tests/gestore/calendario-bulk.spec.ts):
8 test puri PASS (TC-N626..N633, eseguiti in questo sandbox) + 3 test
E2E non eseguibili qui per assenza di deploy/credenziali (TC-N634..N636,
Esito lasciato vuoto/DA TESTARE, verificabili da Fabrizio col prossimo
deploy). Formula ID Anomalia ricalcolata (recalc.py, 0 errori).
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4095" uniqueCount="2679">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4202" uniqueCount="2740">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -8056,6 +8056,189 @@
   </si>
   <si>
     <t xml:space="preserve">Requisito esplicito Addendum Sezione B: conferma rinforzata per lo scope che impatta tutti gli utenti. Non eseguito in questo sandbox (Chromium senza dipendenze di sistema), verificabile da Fabrizio col prossimo deploy.sh/test-deploy.sh.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N626</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gestore - Calendario disponibilita (OD-02 bulk)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">applyBulkPatch imposta la Giornata particolare su tutti e soli i giorni selezionati</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nessuna (funzione pura, lib/availability-bulk.ts)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Selezionare 2 giorni su 3, azione 'set' con emoji/etichetta, chiamare applyBulkPatch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I 2 giorni selezionati hanno la nuova Giornata particolare; il terzo giorno (non selezionato) resta invariato</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OD-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test A richiesto da Fabrizio (REVISIONE DECISIONE OD-02: FIX PRIMA DELLA BETA, 06/08). Test puro, nessun browser (tests/gestore/calendario-bulk.spec.ts). Eseguito con successo in questo sandbox (chromium + mobile-chrome).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N627</t>
+  </si>
+  <si>
+    <t xml:space="preserve">applyBulkPatch con azione 'remove' toglie la Giornata particolare solo dai giorni selezionati</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nessuna (funzione pura)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 giorni con Giornata particolare preesistente + 1 diverso non selezionato, azione 'remove' sui primi 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I 2 giorni selezionati perdono emoji/etichetta; il terzo giorno mantiene il proprio valore preesistente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test C richiesto da Fabrizio. Test puro. Eseguito con successo in questo sandbox.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N628</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Impostare la Giornata particolare (senza includere gli altri campi) non modifica apertura/capacita/sconto/last-minute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 giorni con valori eterogenei di isOpen/capacity/discountPercent/lastMinute, applica solo specialDayAction='set' (gli altri toggle include restano false)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">isOpen/capacity/spotsLeft/discountPercent/lastMinute restano identici ai valori di partenza su entrambi i giorni; solo la Giornata particolare cambia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test D richiesto esplicitamente da Fabrizio (root cause del bug originale: il bulk draft sovrascriveva sempre questi 4 campi). Test puro. Eseguito con successo in questo sandbox.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N629</t>
+  </si>
+  <si>
+    <t xml:space="preserve">summarizeSpecialDay segnala uno stato 'misto' quando i giorni selezionati hanno valori diversi, poi uniformita' dopo l'applicazione</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 giorni selezionati con emoji/etichetta diverse tra loro -&gt; summarizeSpecialDay -&gt; applyBulkPatch 'set' -&gt; summarizeSpecialDay di nuovo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prima: mixed=true. Dopo l'applicazione: mixed=false con l'emoji/etichetta appena impostata su tutti</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test E richiesto da Fabrizio (stato mixed/indeterminato). Include anche le varianti 'valore gia' uniforme' e 'nessuna selezione'. Test puro. Eseguito con successo in questo sandbox.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N630</t>
+  </si>
+  <si>
+    <t xml:space="preserve">applyBulkPatch non modifica alcun campo dei giorni non selezionati</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 giorno selezionato + 1 giorno non selezionato con tutti i campi valorizzati, draft con tutti i campi inclusi + azione 'remove'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il giorno non selezionato risulta esattamente identico (deep equal) a prima della chiamata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test F richiesto da Fabrizio. Test puro. Eseguito con successo in questo sandbox.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N631</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bulkDraftHasChanges e' false per il draft di default e true non appena un campo viene incluso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificare bulkDraftHasChanges su defaultBulkDraft(), poi con un include=true, poi con specialDayAction='remove'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">false sul draft vuoto, true in entrambi gli altri due casi (usato per disabilitare il bottone Applica quando non c'e' nulla da salvare)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copre il requisito 'nessun campo applicato per default'. Test puro. Eseguito con successo in questo sandbox.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N632</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Campo non modificato' di default: applicare il draft di default non cambia alcun valore, nemmeno sui giorni selezionati</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 giorno con tutti i campi valorizzati (incluso Giornata particolare), selezionato, applyBulkPatch(defaultBulkDraft())</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il giorno risultante e' identico (deep equal) a quello di partenza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verifica la semantica 'non modificato' richiesta esplicitamente da Fabrizio (nessun valore vuoto ambiguo). Test puro. Eseguito con successo in questo sandbox.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N633</t>
+  </si>
+  <si>
+    <t xml:space="preserve">applyBulkPatch non produce righe duplicate ne' perde giorni</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 giorni in ingresso, 2 selezionati, applyBulkPatch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'array in uscita ha sempre 3 elementi, stesso insieme e ordine di date dell'ingresso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test puro. Eseguito con successo in questo sandbox.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N634</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il Partner puo' applicare la Giornata particolare a piu' giorni via bulk, salvarla, e ritrovarla dopo refresh e sul giorno singolo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login Gestore di test collegato a un centro con attivita' seminata (supabase/seed-test-data.sql)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login gestore -&gt; Calendario disponibilita' -&gt; Seleziona piu' giorni -&gt; seleziona una settimana -&gt; Giornata particolare: Imposta + emoji + etichetta -&gt; Applica -&gt; Salva calendario -&gt; ricarica pagina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il badge/emoji della Giornata particolare compare su tutti i giorni della settimana selezionata, persiste dopo il refresh (letto da Supabase, non solo stato locale)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test B richiesto da Fabrizio (persistenza). Non eseguito in questo sandbox (nessun deploy/credenziali Supabase disponibili), verificabile da Fabrizio col prossimo deploy.sh/test-deploy.sh.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N635</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il pannello a giorno singolo continua a impostare/rimuovere la Giornata particolare senza modalita' bulk attiva (regressione)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login Gestore di test collegato a un centro con attivita' seminata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login gestore -&gt; Calendario disponibilita' (modalita' bulk NON attivata) -&gt; click su un giorno -&gt; imposta emoji+etichetta -&gt; Salva -&gt; poi rimuovi (bottone '-') -&gt; Salva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il pannello 'Modifica &lt;data&gt;' si apre come prima del fix; impostare e rimuovere la Giornata particolare dal giorno singolo funziona esattamente come prima</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test G richiesto da Fabrizio (nessuna regressione sul giorno singolo). Non eseguito in questo sandbox, verificabile da Fabrizio col prossimo deploy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N636</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il pannello bulk della Giornata particolare e' utilizzabile su viewport mobile 390x844</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viewport 390x844 -&gt; Login gestore -&gt; Calendario disponibilita' -&gt; Seleziona piu' giorni -&gt; seleziona un giorno -&gt; verificare che il bottone 'Imposta' sia visibile e che la pagina non abbia overflow orizzontale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il controllo e' visibile e raggiungibile, nessun overflow orizzontale (scrollWidth documento &lt;= 400px)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test H richiesto da Fabrizio (mobile). Non eseguito in questo sandbox, verificabile da Fabrizio col prossimo deploy.</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -8895,7 +9078,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L467"/>
+  <dimension ref="A1:L478"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -23941,7 +24124,7 @@
         <v>2655</v>
       </c>
     </row>
-    <row r="464" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="464" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A464" s="10" t="s">
         <v>2520</v>
       </c>
@@ -23974,7 +24157,7 @@
         <v>2661</v>
       </c>
     </row>
-    <row r="465" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="465" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A465" s="10" t="s">
         <v>2527</v>
       </c>
@@ -24007,7 +24190,7 @@
         <v>2665</v>
       </c>
     </row>
-    <row r="466" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="466" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A466" s="10" t="s">
         <v>1332</v>
       </c>
@@ -24040,7 +24223,7 @@
         <v>2669</v>
       </c>
     </row>
-    <row r="467" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="467" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A467" s="10" t="s">
         <v>2540</v>
       </c>
@@ -24068,6 +24251,393 @@
       </c>
       <c r="L467" s="11" t="s">
         <v>2674</v>
+      </c>
+    </row>
+    <row r="468" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A468" s="10" t="s">
+        <v>2675</v>
+      </c>
+      <c r="B468" s="10" t="s">
+        <v>2676</v>
+      </c>
+      <c r="C468" s="10" t="s">
+        <v>2677</v>
+      </c>
+      <c r="D468" s="10" t="s">
+        <v>2678</v>
+      </c>
+      <c r="E468" s="10" t="s">
+        <v>2679</v>
+      </c>
+      <c r="F468" s="10" t="s">
+        <v>2680</v>
+      </c>
+      <c r="G468" s="10" t="s">
+        <v>2552</v>
+      </c>
+      <c r="H468" s="10" t="str">
+        <f aca="false">IF(G468="BUG","BUG-"&amp;A468,IF(G468="FUNCTIONAL","FUNCTIONAL-"&amp;A468,""))</f>
+        <v/>
+      </c>
+      <c r="I468" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="J468" s="10" t="s">
+        <v>2681</v>
+      </c>
+      <c r="L468" s="11" t="s">
+        <v>2682</v>
+      </c>
+    </row>
+    <row r="469" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A469" s="10" t="s">
+        <v>2683</v>
+      </c>
+      <c r="B469" s="10" t="s">
+        <v>2676</v>
+      </c>
+      <c r="C469" s="10" t="s">
+        <v>2684</v>
+      </c>
+      <c r="D469" s="10" t="s">
+        <v>2685</v>
+      </c>
+      <c r="E469" s="10" t="s">
+        <v>2686</v>
+      </c>
+      <c r="F469" s="10" t="s">
+        <v>2687</v>
+      </c>
+      <c r="G469" s="10" t="s">
+        <v>2552</v>
+      </c>
+      <c r="H469" s="10" t="str">
+        <f aca="false">IF(G469="BUG","BUG-"&amp;A469,IF(G469="FUNCTIONAL","FUNCTIONAL-"&amp;A469,""))</f>
+        <v/>
+      </c>
+      <c r="I469" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="J469" s="10" t="s">
+        <v>2681</v>
+      </c>
+      <c r="L469" s="11" t="s">
+        <v>2688</v>
+      </c>
+    </row>
+    <row r="470" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A470" s="10" t="s">
+        <v>2689</v>
+      </c>
+      <c r="B470" s="10" t="s">
+        <v>2676</v>
+      </c>
+      <c r="C470" s="10" t="s">
+        <v>2690</v>
+      </c>
+      <c r="D470" s="10" t="s">
+        <v>2685</v>
+      </c>
+      <c r="E470" s="10" t="s">
+        <v>2691</v>
+      </c>
+      <c r="F470" s="10" t="s">
+        <v>2692</v>
+      </c>
+      <c r="G470" s="10" t="s">
+        <v>2552</v>
+      </c>
+      <c r="H470" s="10" t="str">
+        <f aca="false">IF(G470="BUG","BUG-"&amp;A470,IF(G470="FUNCTIONAL","FUNCTIONAL-"&amp;A470,""))</f>
+        <v/>
+      </c>
+      <c r="I470" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="J470" s="10" t="s">
+        <v>2681</v>
+      </c>
+      <c r="L470" s="11" t="s">
+        <v>2693</v>
+      </c>
+    </row>
+    <row r="471" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A471" s="10" t="s">
+        <v>2694</v>
+      </c>
+      <c r="B471" s="10" t="s">
+        <v>2676</v>
+      </c>
+      <c r="C471" s="10" t="s">
+        <v>2695</v>
+      </c>
+      <c r="D471" s="10" t="s">
+        <v>2685</v>
+      </c>
+      <c r="E471" s="10" t="s">
+        <v>2696</v>
+      </c>
+      <c r="F471" s="10" t="s">
+        <v>2697</v>
+      </c>
+      <c r="G471" s="10" t="s">
+        <v>2552</v>
+      </c>
+      <c r="H471" s="10" t="str">
+        <f aca="false">IF(G471="BUG","BUG-"&amp;A471,IF(G471="FUNCTIONAL","FUNCTIONAL-"&amp;A471,""))</f>
+        <v/>
+      </c>
+      <c r="I471" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="J471" s="10" t="s">
+        <v>2681</v>
+      </c>
+      <c r="L471" s="11" t="s">
+        <v>2698</v>
+      </c>
+    </row>
+    <row r="472" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A472" s="10" t="s">
+        <v>2699</v>
+      </c>
+      <c r="B472" s="10" t="s">
+        <v>2676</v>
+      </c>
+      <c r="C472" s="10" t="s">
+        <v>2700</v>
+      </c>
+      <c r="D472" s="10" t="s">
+        <v>2685</v>
+      </c>
+      <c r="E472" s="10" t="s">
+        <v>2701</v>
+      </c>
+      <c r="F472" s="10" t="s">
+        <v>2702</v>
+      </c>
+      <c r="G472" s="10" t="s">
+        <v>2552</v>
+      </c>
+      <c r="H472" s="10" t="str">
+        <f aca="false">IF(G472="BUG","BUG-"&amp;A472,IF(G472="FUNCTIONAL","FUNCTIONAL-"&amp;A472,""))</f>
+        <v/>
+      </c>
+      <c r="I472" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="J472" s="10" t="s">
+        <v>2681</v>
+      </c>
+      <c r="L472" s="11" t="s">
+        <v>2703</v>
+      </c>
+    </row>
+    <row r="473" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A473" s="10" t="s">
+        <v>2704</v>
+      </c>
+      <c r="B473" s="10" t="s">
+        <v>2676</v>
+      </c>
+      <c r="C473" s="10" t="s">
+        <v>2705</v>
+      </c>
+      <c r="D473" s="10" t="s">
+        <v>2685</v>
+      </c>
+      <c r="E473" s="10" t="s">
+        <v>2706</v>
+      </c>
+      <c r="F473" s="10" t="s">
+        <v>2707</v>
+      </c>
+      <c r="G473" s="10" t="s">
+        <v>2552</v>
+      </c>
+      <c r="H473" s="10" t="str">
+        <f aca="false">IF(G473="BUG","BUG-"&amp;A473,IF(G473="FUNCTIONAL","FUNCTIONAL-"&amp;A473,""))</f>
+        <v/>
+      </c>
+      <c r="I473" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="J473" s="10" t="s">
+        <v>2681</v>
+      </c>
+      <c r="L473" s="11" t="s">
+        <v>2708</v>
+      </c>
+    </row>
+    <row r="474" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A474" s="10" t="s">
+        <v>2709</v>
+      </c>
+      <c r="B474" s="10" t="s">
+        <v>2676</v>
+      </c>
+      <c r="C474" s="10" t="s">
+        <v>2710</v>
+      </c>
+      <c r="D474" s="10" t="s">
+        <v>2685</v>
+      </c>
+      <c r="E474" s="10" t="s">
+        <v>2711</v>
+      </c>
+      <c r="F474" s="10" t="s">
+        <v>2712</v>
+      </c>
+      <c r="G474" s="10" t="s">
+        <v>2552</v>
+      </c>
+      <c r="H474" s="10" t="str">
+        <f aca="false">IF(G474="BUG","BUG-"&amp;A474,IF(G474="FUNCTIONAL","FUNCTIONAL-"&amp;A474,""))</f>
+        <v/>
+      </c>
+      <c r="I474" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="J474" s="10" t="s">
+        <v>2681</v>
+      </c>
+      <c r="L474" s="11" t="s">
+        <v>2713</v>
+      </c>
+    </row>
+    <row r="475" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A475" s="10" t="s">
+        <v>2714</v>
+      </c>
+      <c r="B475" s="10" t="s">
+        <v>2676</v>
+      </c>
+      <c r="C475" s="10" t="s">
+        <v>2715</v>
+      </c>
+      <c r="D475" s="10" t="s">
+        <v>2685</v>
+      </c>
+      <c r="E475" s="10" t="s">
+        <v>2716</v>
+      </c>
+      <c r="F475" s="10" t="s">
+        <v>2717</v>
+      </c>
+      <c r="G475" s="10" t="s">
+        <v>2552</v>
+      </c>
+      <c r="H475" s="10" t="str">
+        <f aca="false">IF(G475="BUG","BUG-"&amp;A475,IF(G475="FUNCTIONAL","FUNCTIONAL-"&amp;A475,""))</f>
+        <v/>
+      </c>
+      <c r="I475" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="J475" s="10" t="s">
+        <v>2681</v>
+      </c>
+      <c r="L475" s="11" t="s">
+        <v>2718</v>
+      </c>
+    </row>
+    <row r="476" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A476" s="10" t="s">
+        <v>2719</v>
+      </c>
+      <c r="B476" s="10" t="s">
+        <v>2676</v>
+      </c>
+      <c r="C476" s="10" t="s">
+        <v>2720</v>
+      </c>
+      <c r="D476" s="10" t="s">
+        <v>2721</v>
+      </c>
+      <c r="E476" s="10" t="s">
+        <v>2722</v>
+      </c>
+      <c r="F476" s="10" t="s">
+        <v>2723</v>
+      </c>
+      <c r="H476" s="10" t="str">
+        <f aca="false">IF(G476="BUG","BUG-"&amp;A476,IF(G476="FUNCTIONAL","FUNCTIONAL-"&amp;A476,""))</f>
+        <v/>
+      </c>
+      <c r="I476" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="J476" s="10" t="s">
+        <v>2681</v>
+      </c>
+      <c r="L476" s="11" t="s">
+        <v>2724</v>
+      </c>
+    </row>
+    <row r="477" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A477" s="10" t="s">
+        <v>2725</v>
+      </c>
+      <c r="B477" s="10" t="s">
+        <v>2676</v>
+      </c>
+      <c r="C477" s="10" t="s">
+        <v>2726</v>
+      </c>
+      <c r="D477" s="10" t="s">
+        <v>2727</v>
+      </c>
+      <c r="E477" s="10" t="s">
+        <v>2728</v>
+      </c>
+      <c r="F477" s="10" t="s">
+        <v>2729</v>
+      </c>
+      <c r="H477" s="10" t="str">
+        <f aca="false">IF(G477="BUG","BUG-"&amp;A477,IF(G477="FUNCTIONAL","FUNCTIONAL-"&amp;A477,""))</f>
+        <v/>
+      </c>
+      <c r="I477" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="J477" s="10" t="s">
+        <v>2681</v>
+      </c>
+      <c r="L477" s="11" t="s">
+        <v>2730</v>
+      </c>
+    </row>
+    <row r="478" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A478" s="10" t="s">
+        <v>2731</v>
+      </c>
+      <c r="B478" s="10" t="s">
+        <v>2676</v>
+      </c>
+      <c r="C478" s="10" t="s">
+        <v>2732</v>
+      </c>
+      <c r="D478" s="10" t="s">
+        <v>2727</v>
+      </c>
+      <c r="E478" s="10" t="s">
+        <v>2733</v>
+      </c>
+      <c r="F478" s="10" t="s">
+        <v>2734</v>
+      </c>
+      <c r="H478" s="10" t="str">
+        <f aca="false">IF(G478="BUG","BUG-"&amp;A478,IF(G478="FUNCTIONAL","FUNCTIONAL-"&amp;A478,""))</f>
+        <v/>
+      </c>
+      <c r="I478" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="J478" s="10" t="s">
+        <v>2681</v>
+      </c>
+      <c r="L478" s="11" t="s">
+        <v>2735</v>
       </c>
     </row>
   </sheetData>
@@ -24127,7 +24697,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>2675</v>
+        <v>2736</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24135,13 +24705,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2676</v>
+        <v>2737</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2677</v>
+        <v>2738</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24210,11 +24780,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>2678</v>
+        <v>2739</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>466</v>
+        <v>477</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
test(xlsx): TC-N637/N638 nuovi bug fixati + PASS live OD-02 (TC-N634..636) + nota fix TC-N609
- TC-N634/635/636: Esito aggiornato a PASS, verificati dal vivo da
  Fabrizio il 06/08 dopo deploy 24464bf
- TC-N609: nota sul secondo bug del test (locator) e relativo fix
- TC-N637 (nuovo): verifica identità Admin invisibile - RISOLTA
- TC-N638 (nuovo): menu Scatta foto coperto da Torna a V1 - RISOLTA
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4202" uniqueCount="2740">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4225" uniqueCount="2755">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -7548,7 +7548,7 @@
     <t xml:space="preserve">L'override compare nella lista con lo stato corretto; dopo l'eliminazione la riga sparisce. Verifica anche indirettamente il bug fix di TC-N409 (Gate C, ottava ondata): un override scaduto ora e' visibile con badge 'Scaduto'/'In scadenza (&lt;72h)' invece di fallire silenziosamente senza alcuna traccia</t>
   </si>
   <si>
-    <t xml:space="preserve">Test automatizzato: tests/one/feature-flags.spec.ts, TC-N609 (gated su isRealDeployment). Lo stesso file contiene anche ~15 unit test 'no browser' (findRecentlyExpiredMatchingOverride, computeOverrideStatus) eseguibili senza browser reale -- gia' verificati passanti in locale (56/56 pass).</t>
+    <t xml:space="preserve">Test automatizzato: tests/one/feature-flags.spec.ts, TC-N609 (gated su isRealDeployment). Lo stesso file contiene anche ~15 unit test 'no browser' (findRecentlyExpiredMatchingOverride, computeOverrideStatus) eseguibili senza browser reale -- gia' verificati passanti in locale (56/56 pass). AGGIORNAMENTO 06/08/2026: nel run critical post-deploy (commit 24464bf) il test è fallito di nuovo con un diverso strict-mode violation (il locator div+hasText+first() ora intercetta anche il &lt;select&gt; di BatchBetaControls, aggiunto da Addendum Sezione B sopra la card del flag). Root cause: assunzione di struttura DOM non più valida (bug del test, non della pagina Admin). Fix: aggiunto data-testid="flag-card-TRAMA_ONE_ENABLED" alla card in FeatureFlagsAdminClient.tsx e il test ora usa page.getByTestId(...) invece del locator fragile. Non rieseguibile in questo sandbox (richiede browser + deploy reale) — verificabile da Fabrizio al prossimo giro di test-deploy.sh.</t>
   </si>
   <si>
     <t xml:space="preserve">TC-N610</t>
@@ -8205,7 +8205,7 @@
     <t xml:space="preserve">Il badge/emoji della Giornata particolare compare su tutti i giorni della settimana selezionata, persiste dopo il refresh (letto da Supabase, non solo stato locale)</t>
   </si>
   <si>
-    <t xml:space="preserve">Test B richiesto da Fabrizio (persistenza). Non eseguito in questo sandbox (nessun deploy/credenziali Supabase disponibili), verificabile da Fabrizio col prossimo deploy.sh/test-deploy.sh.</t>
+    <t xml:space="preserve">Test B richiesto da Fabrizio (persistenza). VERIFICATO DAL VIVO da Fabrizio il 06/08/2026 dopo deploy commit 24464bf: PASS (persistenza confermata dopo refresh e sul giorno singolo).</t>
   </si>
   <si>
     <t xml:space="preserve">TC-N635</t>
@@ -8223,7 +8223,7 @@
     <t xml:space="preserve">Il pannello 'Modifica &lt;data&gt;' si apre come prima del fix; impostare e rimuovere la Giornata particolare dal giorno singolo funziona esattamente come prima</t>
   </si>
   <si>
-    <t xml:space="preserve">Test G richiesto da Fabrizio (nessuna regressione sul giorno singolo). Non eseguito in questo sandbox, verificabile da Fabrizio col prossimo deploy.</t>
+    <t xml:space="preserve">Test G richiesto da Fabrizio (nessuna regressione sul giorno singolo). VERIFICATO DAL VIVO da Fabrizio il 06/08/2026 dopo deploy commit 24464bf: PASS.</t>
   </si>
   <si>
     <t xml:space="preserve">TC-N636</t>
@@ -8238,7 +8238,52 @@
     <t xml:space="preserve">Il controllo e' visibile e raggiungibile, nessun overflow orizzontale (scrollWidth documento &lt;= 400px)</t>
   </si>
   <si>
-    <t xml:space="preserve">Test H richiesto da Fabrizio (mobile). Non eseguito in questo sandbox, verificabile da Fabrizio col prossimo deploy.</t>
+    <t xml:space="preserve">Test H richiesto da Fabrizio (mobile). VERIFICATO DAL VIVO da Fabrizio il 06/08/2026 dopo deploy commit 24464bf: PASS (pannello bulk Calendario ok su mobile; durante questo test è emerso un bug distinto e non correlato nel menu 'Scatta foto' della pagina Profilo, registrato come TC-N638 e fixato separatamente in questo stesso passaggio).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N637</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin - Onboarding centri (TRAMA ONE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Admin vede e puo' agire su una verifica identita' 'pending' anche se il centro non e' ancora in stato SUBMITTED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Un centro con una richiesta di verifica identita' sottomessa dal Partner (nota/documento) mentre il centro e' ancora CLAIMED/CHANGES_REQUESTED (non SUBMITTED)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partner: onboarding -&gt; scheda 'Verifica identita'' -&gt; scrive nota + allega documento (senza premere 'Invia per verifica' sull'intero onboarding) -&gt; Admin: /admin/one/onboarding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il centro compare in 'Altri stati' con la riga 'Identita: pending', la nota, il link 'Vedi documento' e i bottoni 'Verifica identita''/'Rifiuta identita'' — non piu' invisibile come prima del fix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RISOLTA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bug reale scoperto da Fabrizio il 06/08/2026 (screenshot: centro 'Centro estivo prova candidatura', identita' 'Sono io' sottomessa, centro CLAIMED, invisibile in Admin sia in 'In revisione' che in 'Altri stati'). Root cause: submitIdentityVerificationAction (app/actions/onboarding.ts) e' indipendente dallo stato onboarding generale; il blocco identita' in AdminOnboardingReviewClient.tsx era renderizzato solo nel loop 'In revisione' (status===SUBMITTED). Fix: blocco identita'/documento/bottoni aggiunto anche al loop 'Altri stati', condizionato su identity.status, senza toccare la state machine onboarding generale. Verificato: tsc/eslint puliti, nessun test E2E dedicato in questo sandbox (richiede un centro di test in stato CLAIMED con identita' pending — non presente nei fixture attuali), verificabile da Fabrizio al prossimo deploy con lo stesso centro dello screenshot.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N638</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Genitore - Profilo (foto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il menu 'Scatta foto'/'Galleria' non e' coperto dal bottone globale 'Torna a V1' su mobile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login Genitore, viewport mobile (~390px)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profilo -&gt; tap sull'icona fotocamera sull'avatar per aprire il menu 'Scatta foto'/'Scegli dalla galleria'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il menu si apre completamente visibile sotto l'avatar, sopra qualunque altro elemento fisso della pagina (incluso il bottone 'Torna a V1'/'Passa a NextGen')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bug reale segnalato da Fabrizio con screenshot il 06/08/2026 (scoperto durante il test mobile di OD-02, non correlato). Root cause: components/AvatarUploadButton.tsx e components/VersionToggle.tsx usavano entrambi z-50; VersionToggle (position:fixed, montato dopo nel DOM radice in app/layout.tsx) vinceva a parita' di z-index e copriva il menu quando le due zone si sovrapponevano in alto sullo schermo. Fix: z-index del menu portato a z-[60] (sopra il toggle). Verificato: tsc/eslint puliti. Fix puramente CSS (z-index), non testabile in modo significativo senza screenshot/visual regression — verificabile da Fabrizio al prossimo deploy sullo stesso screenshot.</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -9078,7 +9123,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L478"/>
+  <dimension ref="A1:L480"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -24253,7 +24298,7 @@
         <v>2674</v>
       </c>
     </row>
-    <row r="468" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="468" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A468" s="10" t="s">
         <v>2675</v>
       </c>
@@ -24289,7 +24334,7 @@
         <v>2682</v>
       </c>
     </row>
-    <row r="469" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="469" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A469" s="10" t="s">
         <v>2683</v>
       </c>
@@ -24325,7 +24370,7 @@
         <v>2688</v>
       </c>
     </row>
-    <row r="470" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="470" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A470" s="10" t="s">
         <v>2689</v>
       </c>
@@ -24361,7 +24406,7 @@
         <v>2693</v>
       </c>
     </row>
-    <row r="471" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="471" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A471" s="10" t="s">
         <v>2694</v>
       </c>
@@ -24397,7 +24442,7 @@
         <v>2698</v>
       </c>
     </row>
-    <row r="472" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="472" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A472" s="10" t="s">
         <v>2699</v>
       </c>
@@ -24433,7 +24478,7 @@
         <v>2703</v>
       </c>
     </row>
-    <row r="473" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="473" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A473" s="10" t="s">
         <v>2704</v>
       </c>
@@ -24469,7 +24514,7 @@
         <v>2708</v>
       </c>
     </row>
-    <row r="474" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="474" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A474" s="10" t="s">
         <v>2709</v>
       </c>
@@ -24505,7 +24550,7 @@
         <v>2713</v>
       </c>
     </row>
-    <row r="475" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="475" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A475" s="10" t="s">
         <v>2714</v>
       </c>
@@ -24541,7 +24586,7 @@
         <v>2718</v>
       </c>
     </row>
-    <row r="476" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="476" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A476" s="10" t="s">
         <v>2719</v>
       </c>
@@ -24560,6 +24605,9 @@
       <c r="F476" s="10" t="s">
         <v>2723</v>
       </c>
+      <c r="G476" s="10" t="s">
+        <v>2552</v>
+      </c>
       <c r="H476" s="10" t="str">
         <f aca="false">IF(G476="BUG","BUG-"&amp;A476,IF(G476="FUNCTIONAL","FUNCTIONAL-"&amp;A476,""))</f>
         <v/>
@@ -24574,7 +24622,7 @@
         <v>2724</v>
       </c>
     </row>
-    <row r="477" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="477" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A477" s="10" t="s">
         <v>2725</v>
       </c>
@@ -24593,6 +24641,9 @@
       <c r="F477" s="10" t="s">
         <v>2729</v>
       </c>
+      <c r="G477" s="10" t="s">
+        <v>2552</v>
+      </c>
       <c r="H477" s="10" t="str">
         <f aca="false">IF(G477="BUG","BUG-"&amp;A477,IF(G477="FUNCTIONAL","FUNCTIONAL-"&amp;A477,""))</f>
         <v/>
@@ -24607,7 +24658,7 @@
         <v>2730</v>
       </c>
     </row>
-    <row r="478" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="478" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A478" s="10" t="s">
         <v>2731</v>
       </c>
@@ -24626,6 +24677,9 @@
       <c r="F478" s="10" t="s">
         <v>2734</v>
       </c>
+      <c r="G478" s="10" t="s">
+        <v>2552</v>
+      </c>
       <c r="H478" s="10" t="str">
         <f aca="false">IF(G478="BUG","BUG-"&amp;A478,IF(G478="FUNCTIONAL","FUNCTIONAL-"&amp;A478,""))</f>
         <v/>
@@ -24638,6 +24692,78 @@
       </c>
       <c r="L478" s="11" t="s">
         <v>2735</v>
+      </c>
+    </row>
+    <row r="479" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A479" s="10" t="s">
+        <v>2736</v>
+      </c>
+      <c r="B479" s="10" t="s">
+        <v>2737</v>
+      </c>
+      <c r="C479" s="10" t="s">
+        <v>2738</v>
+      </c>
+      <c r="D479" s="10" t="s">
+        <v>2739</v>
+      </c>
+      <c r="E479" s="10" t="s">
+        <v>2740</v>
+      </c>
+      <c r="F479" s="10" t="s">
+        <v>2741</v>
+      </c>
+      <c r="G479" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="H479" s="10" t="str">
+        <f aca="false">IF(G479="BUG","BUG-"&amp;A479,IF(G479="FUNCTIONAL","FUNCTIONAL-"&amp;A479,""))</f>
+        <v>BUG-TC-N637</v>
+      </c>
+      <c r="I479" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="K479" s="11" t="s">
+        <v>2742</v>
+      </c>
+      <c r="L479" s="11" t="s">
+        <v>2743</v>
+      </c>
+    </row>
+    <row r="480" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A480" s="10" t="s">
+        <v>2744</v>
+      </c>
+      <c r="B480" s="10" t="s">
+        <v>2745</v>
+      </c>
+      <c r="C480" s="10" t="s">
+        <v>2746</v>
+      </c>
+      <c r="D480" s="10" t="s">
+        <v>2747</v>
+      </c>
+      <c r="E480" s="10" t="s">
+        <v>2748</v>
+      </c>
+      <c r="F480" s="10" t="s">
+        <v>2749</v>
+      </c>
+      <c r="G480" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="H480" s="10" t="str">
+        <f aca="false">IF(G480="BUG","BUG-"&amp;A480,IF(G480="FUNCTIONAL","FUNCTIONAL-"&amp;A480,""))</f>
+        <v>BUG-TC-N638</v>
+      </c>
+      <c r="I480" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="K480" s="11" t="s">
+        <v>2742</v>
+      </c>
+      <c r="L480" s="11" t="s">
+        <v>2750</v>
       </c>
     </row>
   </sheetData>
@@ -24697,7 +24823,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>2736</v>
+        <v>2751</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24705,13 +24831,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2737</v>
+        <v>2752</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2738</v>
+        <v>2753</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24736,7 +24862,7 @@
       </c>
       <c r="B4" s="20" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"BUG")</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>114</v>
@@ -24780,11 +24906,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>2739</v>
+        <v>2754</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
test(xlsx): TC-N638 - nota sul secondo fix (portale) per il menu Scatta foto
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -8283,7 +8283,7 @@
     <t xml:space="preserve">Il menu si apre completamente visibile sotto l'avatar, sopra qualunque altro elemento fisso della pagina (incluso il bottone 'Torna a V1'/'Passa a NextGen')</t>
   </si>
   <si>
-    <t xml:space="preserve">Bug reale segnalato da Fabrizio con screenshot il 06/08/2026 (scoperto durante il test mobile di OD-02, non correlato). Root cause: components/AvatarUploadButton.tsx e components/VersionToggle.tsx usavano entrambi z-50; VersionToggle (position:fixed, montato dopo nel DOM radice in app/layout.tsx) vinceva a parita' di z-index e copriva il menu quando le due zone si sovrapponevano in alto sullo schermo. Fix: z-index del menu portato a z-[60] (sopra il toggle). Verificato: tsc/eslint puliti. Fix puramente CSS (z-index), non testabile in modo significativo senza screenshot/visual regression — verificabile da Fabrizio al prossimo deploy sullo stesso screenshot.</t>
+    <t xml:space="preserve">Bug reale segnalato da Fabrizio con screenshot il 06/08/2026 (scoperto durante il test mobile di OD-02, non correlato). Root cause: components/AvatarUploadButton.tsx e components/VersionToggle.tsx usavano entrambi z-50; VersionToggle (position:fixed, montato dopo nel DOM radice in app/layout.tsx) vinceva a parita' di z-index e copriva il menu quando le due zone si sovrapponevano in alto sullo schermo. Fix: z-index del menu portato a z-[60] (sopra il toggle). Verificato: tsc/eslint puliti. Fix puramente CSS (z-index), non testabile in modo significativo senza screenshot/visual regression — verificabile da Fabrizio al prossimo deploy sullo stesso screenshot. AGGIORNAMENTO 06/08/2026 (stesso giorno): il fix z-index non copriva questo caso — Fabrizio ha rimandato un secondo screenshot che mostra il menu tagliato da un overflow-hidden DIVERSO (DecorativeIntroCard, wrapper della pagina Profilo NEXTGEN attorno a ProfileHeaderClient), non dal bottone Torna a V1. Root cause: qualunque antenato con overflow-hidden può tagliare un menu absolute. Fix definitivo: il menu è ora un React portal su document.body (position:fixed, coordinate da getBoundingClientRect), immune per costruzione a overflow/z-index di QUALUNQUE antenato presente o futuro. Si chiude su scroll/resize per evitare posizione stale.</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -24694,7 +24694,7 @@
         <v>2735</v>
       </c>
     </row>
-    <row r="479" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="479" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A479" s="10" t="s">
         <v>2736</v>
       </c>
@@ -24730,7 +24730,7 @@
         <v>2743</v>
       </c>
     </row>
-    <row r="480" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="480" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A480" s="10" t="s">
         <v>2744</v>
       </c>

</xml_diff>

<commit_message>
fix: rinomina test in TC-N658 (evita collisione ID con TC-N502 esistente) + xlsx
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4567" uniqueCount="2957">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4577" uniqueCount="2965">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -8890,6 +8890,30 @@
   </si>
   <si>
     <t xml:space="preserve">Verifica STATICA (lettura policy), non un test Playwright eseguito. Prova comportamentale reale richiederebbe 2 account Parent di test con bambini reciprocamente noti (fixture TEST-marked non create) — deferita a Fabrizio o a una futura estensione E2E.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-N658</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Genitore - Modifica prenotazione Giorni spot (add/remove)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Segnalazione Fabrizio 25/08/2026 ('Modifica prenotazione... perche' non da opzioni?'): il genitore puo' aggiungere e rimuovere giorni singoli da una prenotazione a Giorni spot gia' effettuata, non solo annullarla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login parent; prenotazione a Giorni spot esistente (creata via TC-N501/TC-N500), fuori dalla finestra di preavviso del centro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Da /prenotazioni apri 'Modifica' sulla prenotazione a giorni -&gt; osserva la griglia Lun-Ven interattiva -&gt; aggiungi un giorno disponibile -&gt; 'Salva modifiche'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'avviso 'La modifica delle date non e' ancora supportata' e' sparito; la griglia mostra i giorni gia' prenotati come 'Incluso' e permette di aggiungerne/rimuoverne; dopo il salvataggio il totale e i giorni prenotati (booking_days) riflettono la nuova selezione, con prezzo congelato sui giorni mantenuti e prezzo fresco sui giorni nuovi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#602-604</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automatizzato: tests/genitori/giorni-spot.spec.ts, TC-N658 (gated su isRealDeployment + dati STEP 7 seed-test-data.sql). Nuova server action updateBookingDaysAction (app/actions/bookings.ts) + editor in ModificaPrenotazioneClient.tsx. Rimozione rilascia capacita' se gia' decrementata; aggiunta richiede disponibilita' residua sul giorno. Nessuna granularita' aggiuntiva sulla finestra di cancellazione (stesso gate singolo gia' usato per le settimane, vedi checkCancellationWindowForDays).</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -9739,7 +9763,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L516"/>
+  <dimension ref="A1:L517"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -26068,7 +26092,7 @@
         <v>2858</v>
       </c>
     </row>
-    <row r="501" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="501" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A501" s="10" t="s">
         <v>2859</v>
       </c>
@@ -26104,7 +26128,7 @@
         <v>2865</v>
       </c>
     </row>
-    <row r="502" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="502" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A502" s="10" t="s">
         <v>2866</v>
       </c>
@@ -26140,7 +26164,7 @@
         <v>2870</v>
       </c>
     </row>
-    <row r="503" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="503" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A503" s="10" t="s">
         <v>2871</v>
       </c>
@@ -26176,7 +26200,7 @@
         <v>2870</v>
       </c>
     </row>
-    <row r="504" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="504" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A504" s="10" t="s">
         <v>2875</v>
       </c>
@@ -26212,7 +26236,7 @@
         <v>2882</v>
       </c>
     </row>
-    <row r="505" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="505" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A505" s="10" t="s">
         <v>2883</v>
       </c>
@@ -26248,7 +26272,7 @@
         <v>2870</v>
       </c>
     </row>
-    <row r="506" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="506" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A506" s="10" t="s">
         <v>2887</v>
       </c>
@@ -26284,7 +26308,7 @@
         <v>2891</v>
       </c>
     </row>
-    <row r="507" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="507" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A507" s="10" t="s">
         <v>2892</v>
       </c>
@@ -26320,7 +26344,7 @@
         <v>2896</v>
       </c>
     </row>
-    <row r="508" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="508" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A508" s="10" t="s">
         <v>2897</v>
       </c>
@@ -26356,7 +26380,7 @@
         <v>2870</v>
       </c>
     </row>
-    <row r="509" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="509" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A509" s="10" t="s">
         <v>2901</v>
       </c>
@@ -26392,7 +26416,7 @@
         <v>2908</v>
       </c>
     </row>
-    <row r="510" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="510" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A510" s="10" t="s">
         <v>2909</v>
       </c>
@@ -26428,7 +26452,7 @@
         <v>2908</v>
       </c>
     </row>
-    <row r="511" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="511" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A511" s="10" t="s">
         <v>2913</v>
       </c>
@@ -26464,7 +26488,7 @@
         <v>2919</v>
       </c>
     </row>
-    <row r="512" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="512" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A512" s="10" t="s">
         <v>2920</v>
       </c>
@@ -26500,7 +26524,7 @@
         <v>2924</v>
       </c>
     </row>
-    <row r="513" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="513" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A513" s="10" t="s">
         <v>2925</v>
       </c>
@@ -26536,7 +26560,7 @@
         <v>2932</v>
       </c>
     </row>
-    <row r="514" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="514" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A514" s="10" t="s">
         <v>2933</v>
       </c>
@@ -26572,7 +26596,7 @@
         <v>2939</v>
       </c>
     </row>
-    <row r="515" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="515" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A515" s="10" t="s">
         <v>2940</v>
       </c>
@@ -26608,7 +26632,7 @@
         <v>2947</v>
       </c>
     </row>
-    <row r="516" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="516" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A516" s="10" t="s">
         <v>2948</v>
       </c>
@@ -26642,6 +26666,42 @@
       </c>
       <c r="L516" s="11" t="s">
         <v>2952</v>
+      </c>
+    </row>
+    <row r="517" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A517" s="10" t="s">
+        <v>2953</v>
+      </c>
+      <c r="B517" s="10" t="s">
+        <v>2954</v>
+      </c>
+      <c r="C517" s="10" t="s">
+        <v>2955</v>
+      </c>
+      <c r="D517" s="10" t="s">
+        <v>2956</v>
+      </c>
+      <c r="E517" s="10" t="s">
+        <v>2957</v>
+      </c>
+      <c r="F517" s="10" t="s">
+        <v>2958</v>
+      </c>
+      <c r="G517" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H517" s="10" t="str">
+        <f aca="false">IF(G517="BUG","BUG-"&amp;A517,IF(G517="FUNCTIONAL","FUNCTIONAL-"&amp;A517,""))</f>
+        <v/>
+      </c>
+      <c r="I517" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="J517" s="10" t="s">
+        <v>2959</v>
+      </c>
+      <c r="L517" s="11" t="s">
+        <v>2960</v>
       </c>
     </row>
   </sheetData>
@@ -26701,7 +26761,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="20" t="s">
-        <v>2953</v>
+        <v>2961</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26709,13 +26769,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2954</v>
+        <v>2962</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2955</v>
+        <v>2963</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26772,7 +26832,7 @@
       </c>
       <c r="B6" s="21" t="n">
         <f aca="false">COUNTIF('Test Case'!G:G,"DA TESTARE")</f>
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>201</v>
@@ -26784,11 +26844,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>2956</v>
+        <v>2964</v>
       </c>
       <c r="B7" s="22" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
feat(parent): onboarding carousel Private Beta (5 slide, riuso walkthrough)
Carousel di benvenuto Genitore (Benvenuto/Vedo/Trovo/Chiedo e organizzo/Ora provo), mostrato automaticamente solo alla prima esperienza Parent dopo login ed eventuale Legal Gate. Zero nuova migration: riusa 100% l'infrastruttura tutorial_progress/Server Action esistente (nuova voce registry a step singolo 'parent_beta_onboarding'). Parent-only per costruzione (montato solo in app/nextgen/layout.tsx) + guardia esplicita realRole. Nessuna modifica a Home/Planner/Search/Activity Detail/Booking/Auth/Legal/Partner/Admin. Vedi docs/trama-one/analysis/TRAMA_PARENT_ONBOARDING_IMPLEMENTATION.md.
</commit_message>
<xml_diff>
--- a/BuddyKids_Test_Case.xlsx
+++ b/BuddyKids_Test_Case.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4656" uniqueCount="3020">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4776" uniqueCount="3083">
   <si>
     <t xml:space="preserve">BuddyKids — Matrice di Test</t>
   </si>
@@ -9079,6 +9079,195 @@
   </si>
   <si>
     <t xml:space="preserve">Wiring UI mancante colmato in app/nextgen/planner/PlannerClient.tsx: stato locale dismissedOverrides (optimistic update) + router.refresh() dopo il salvataggio per riallineare priorityIndex/coveredNeededCount calcolati server-side in page.tsx. Test gated isRealDeployment (richiede browser reale, non eseguibile in questo sandbox).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ONB-P01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEXTGEN - Onboarding Parent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parent prima esperienza -&gt; carousel di onboarding visibile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Account genitore di test in cohort TRAMA_ONE_ENABLED, tutorial 'parent_beta_onboarding' mai risolto (not_started)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login come genitore -&gt; vai su /nextgen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il carousel (role=dialog, aria-modal) appare automaticamente con titolo 'Benvenuto in TRAMA', progress 1/5, CTA 'Continua' e 'Salta' visibili</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Onboarding Carousel Beta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test in tests/nextgen/onboarding-carousel.spec.ts, gated isRealDeployment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ONB-P02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parent con onboarding gia' risolto -&gt; il carousel non compare piu'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Come ONB-P01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se il carousel e' visibile, clicca 'Salta' -&gt; ricarica la pagina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dopo il reload il carousel NON ricompare (stato persistito su tutorial_progress, non solo useState locale)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Idem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ONB-P03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Salta' persiste il completamento (nessuna conferma richiesta)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carousel visibile (prima esperienza)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clicca 'Salta' su una slide qualsiasi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il carousel si chiude immediatamente (nessun popup di conferma) e resta chiuso dopo reload</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ONB-P04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Completare le 5 slide (Continua x4 + CTA finale) persiste il completamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clicca 'Continua' su slide 1-4, poi 'Inizia a esplorare' sulla slide 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il carousel si chiude e resta chiuso dopo reload (stato 'completed' su tutorial_progress)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ONB-P05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partner non vede mai il carousel Parent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Account gestore di test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login come gestore -&gt; vai su /center</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nessun dialog 'Benvenuto in TRAMA' ne' testo 'Adesso prova TRAMA' in pagina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Componente montato solo in app/nextgen/layout.tsx, mai in app/center/layout.tsx.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ONB-P06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin non vede mai il carousel Parent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Account platform admin di test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login come admin -&gt; vai su /admin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Componente montato solo in app/nextgen/layout.tsx, mai in app/admin/layout.tsx.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ONB-P07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legal Gate pending impedisce di raggiungere l'onboarding carousel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deploy dedicato con LEGAL_TERMS_GATE=ON (mai attivato globalmente in questa sessione) + account senza legal_acceptances</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login come genitore -&gt; tentare di raggiungere /nextgen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redirect a /auth/legal-pending PRIMA di qualunque possibilita' di vedere il carousel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ordinamento garantito per costruzione: redirect legale avviene in app/auth/callback/route.ts, prima di app/nextgen/layout.tsx. Non eseguibile nella suite ordinaria (flag resta OFF).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ONB-P08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La slide 4 (richiesta) contiene testualmente 'In attesa'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nessuna (dati puri)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verifica diretta di ONBOARDING_REQUEST_FLOW e del titolo della slide 4 in lib/nextgen/onboarding-slides.ts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'In attesa' presente nel flow; slide4.title === 'Tu chiedi. Il centro risponde.'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test [no browser], eseguito con successo in questa sessione (npx playwright test --project=chromium).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ONB-P09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nessuna slide menziona scoring/AI ranking ('Match 99%' o simili)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verifica regex su titolo/body/microcopy di tutte le 5 slide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nessuna occorrenza di 'match NN%', 'scoring', 'ranking'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test [no browser], eseguito con successo in questa sessione.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ONB-P10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nessuna slide menziona pagamento/checkout/carta/transazione</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nessuna occorrenza di pagamento/checkout/carta di credito/transazione/totale da pagare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ONB-P11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">390px: nessun overflow orizzontale evidente nel carousel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carousel visibile (prima esperienza), viewport 390x844</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login come genitore -&gt; vai su /nextgen a 390px -&gt; misura document.documentElement.scrollWidth vs window.innerWidth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Overflow orizzontale &lt;= 1px (tolleranza subpixel)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ONB-P12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tastiera/focus di base: focus iniziale sul dialog, freccia destra avanza, Escape salta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vai su /nextgen -&gt; verifica focus sul dialog -&gt; premi ArrowRight -&gt; verifica progress 2/5 -&gt; premi Escape</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il dialog ha il focus alla comparsa; ArrowRight avanza alla slide successiva; Escape chiude il carousel (equivalente a 'Salta')</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo per Esito</t>
@@ -9928,7 +10117,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L525"/>
+  <dimension ref="A1:L537"/>
   <sheetFormatPr defaultColWidth="39.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="11.83"/>
@@ -27121,7 +27310,7 @@
         <v>3008</v>
       </c>
     </row>
-    <row r="525" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="525" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A525" s="10" t="s">
         <v>3009</v>
       </c>
@@ -27152,6 +27341,438 @@
       </c>
       <c r="L525" s="11" t="s">
         <v>3015</v>
+      </c>
+    </row>
+    <row r="526" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A526" s="10" t="s">
+        <v>3016</v>
+      </c>
+      <c r="B526" s="10" t="s">
+        <v>3017</v>
+      </c>
+      <c r="C526" s="10" t="s">
+        <v>3018</v>
+      </c>
+      <c r="D526" s="10" t="s">
+        <v>3019</v>
+      </c>
+      <c r="E526" s="10" t="s">
+        <v>3020</v>
+      </c>
+      <c r="F526" s="10" t="s">
+        <v>3021</v>
+      </c>
+      <c r="G526" s="10" t="s">
+        <v>2908</v>
+      </c>
+      <c r="H526" s="10" t="str">
+        <f aca="false">IF(G526="BUG","BUG-"&amp;A526,IF(G526="FUNCTIONAL","FUNCTIONAL-"&amp;A526,""))</f>
+        <v/>
+      </c>
+      <c r="I526" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="J526" s="10" t="s">
+        <v>3022</v>
+      </c>
+      <c r="L526" s="11" t="s">
+        <v>3023</v>
+      </c>
+    </row>
+    <row r="527" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A527" s="10" t="s">
+        <v>3024</v>
+      </c>
+      <c r="B527" s="10" t="s">
+        <v>3017</v>
+      </c>
+      <c r="C527" s="10" t="s">
+        <v>3025</v>
+      </c>
+      <c r="D527" s="10" t="s">
+        <v>3026</v>
+      </c>
+      <c r="E527" s="10" t="s">
+        <v>3027</v>
+      </c>
+      <c r="F527" s="10" t="s">
+        <v>3028</v>
+      </c>
+      <c r="G527" s="10" t="s">
+        <v>2908</v>
+      </c>
+      <c r="H527" s="10" t="str">
+        <f aca="false">IF(G527="BUG","BUG-"&amp;A527,IF(G527="FUNCTIONAL","FUNCTIONAL-"&amp;A527,""))</f>
+        <v/>
+      </c>
+      <c r="I527" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="J527" s="10" t="s">
+        <v>3022</v>
+      </c>
+      <c r="L527" s="11" t="s">
+        <v>3029</v>
+      </c>
+    </row>
+    <row r="528" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A528" s="10" t="s">
+        <v>3030</v>
+      </c>
+      <c r="B528" s="10" t="s">
+        <v>3017</v>
+      </c>
+      <c r="C528" s="10" t="s">
+        <v>3031</v>
+      </c>
+      <c r="D528" s="10" t="s">
+        <v>3032</v>
+      </c>
+      <c r="E528" s="10" t="s">
+        <v>3033</v>
+      </c>
+      <c r="F528" s="10" t="s">
+        <v>3034</v>
+      </c>
+      <c r="G528" s="10" t="s">
+        <v>2908</v>
+      </c>
+      <c r="H528" s="10" t="str">
+        <f aca="false">IF(G528="BUG","BUG-"&amp;A528,IF(G528="FUNCTIONAL","FUNCTIONAL-"&amp;A528,""))</f>
+        <v/>
+      </c>
+      <c r="I528" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="J528" s="10" t="s">
+        <v>3022</v>
+      </c>
+      <c r="L528" s="11" t="s">
+        <v>3029</v>
+      </c>
+    </row>
+    <row r="529" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A529" s="10" t="s">
+        <v>3035</v>
+      </c>
+      <c r="B529" s="10" t="s">
+        <v>3017</v>
+      </c>
+      <c r="C529" s="10" t="s">
+        <v>3036</v>
+      </c>
+      <c r="D529" s="10" t="s">
+        <v>3032</v>
+      </c>
+      <c r="E529" s="10" t="s">
+        <v>3037</v>
+      </c>
+      <c r="F529" s="10" t="s">
+        <v>3038</v>
+      </c>
+      <c r="G529" s="10" t="s">
+        <v>2908</v>
+      </c>
+      <c r="H529" s="10" t="str">
+        <f aca="false">IF(G529="BUG","BUG-"&amp;A529,IF(G529="FUNCTIONAL","FUNCTIONAL-"&amp;A529,""))</f>
+        <v/>
+      </c>
+      <c r="I529" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="J529" s="10" t="s">
+        <v>3022</v>
+      </c>
+      <c r="L529" s="11" t="s">
+        <v>3029</v>
+      </c>
+    </row>
+    <row r="530" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A530" s="10" t="s">
+        <v>3039</v>
+      </c>
+      <c r="B530" s="10" t="s">
+        <v>3017</v>
+      </c>
+      <c r="C530" s="10" t="s">
+        <v>3040</v>
+      </c>
+      <c r="D530" s="10" t="s">
+        <v>3041</v>
+      </c>
+      <c r="E530" s="10" t="s">
+        <v>3042</v>
+      </c>
+      <c r="F530" s="10" t="s">
+        <v>3043</v>
+      </c>
+      <c r="G530" s="10" t="s">
+        <v>2908</v>
+      </c>
+      <c r="H530" s="10" t="str">
+        <f aca="false">IF(G530="BUG","BUG-"&amp;A530,IF(G530="FUNCTIONAL","FUNCTIONAL-"&amp;A530,""))</f>
+        <v/>
+      </c>
+      <c r="I530" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="J530" s="10" t="s">
+        <v>3022</v>
+      </c>
+      <c r="L530" s="11" t="s">
+        <v>3044</v>
+      </c>
+    </row>
+    <row r="531" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A531" s="10" t="s">
+        <v>3045</v>
+      </c>
+      <c r="B531" s="10" t="s">
+        <v>3017</v>
+      </c>
+      <c r="C531" s="10" t="s">
+        <v>3046</v>
+      </c>
+      <c r="D531" s="10" t="s">
+        <v>3047</v>
+      </c>
+      <c r="E531" s="10" t="s">
+        <v>3048</v>
+      </c>
+      <c r="F531" s="10" t="s">
+        <v>3043</v>
+      </c>
+      <c r="G531" s="10" t="s">
+        <v>2908</v>
+      </c>
+      <c r="H531" s="10" t="str">
+        <f aca="false">IF(G531="BUG","BUG-"&amp;A531,IF(G531="FUNCTIONAL","FUNCTIONAL-"&amp;A531,""))</f>
+        <v/>
+      </c>
+      <c r="I531" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="J531" s="10" t="s">
+        <v>3022</v>
+      </c>
+      <c r="L531" s="11" t="s">
+        <v>3049</v>
+      </c>
+    </row>
+    <row r="532" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A532" s="10" t="s">
+        <v>3050</v>
+      </c>
+      <c r="B532" s="10" t="s">
+        <v>3017</v>
+      </c>
+      <c r="C532" s="10" t="s">
+        <v>3051</v>
+      </c>
+      <c r="D532" s="10" t="s">
+        <v>3052</v>
+      </c>
+      <c r="E532" s="10" t="s">
+        <v>3053</v>
+      </c>
+      <c r="F532" s="10" t="s">
+        <v>3054</v>
+      </c>
+      <c r="G532" s="10" t="s">
+        <v>2908</v>
+      </c>
+      <c r="H532" s="10" t="str">
+        <f aca="false">IF(G532="BUG","BUG-"&amp;A532,IF(G532="FUNCTIONAL","FUNCTIONAL-"&amp;A532,""))</f>
+        <v/>
+      </c>
+      <c r="I532" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="J532" s="10" t="s">
+        <v>3022</v>
+      </c>
+      <c r="L532" s="11" t="s">
+        <v>3055</v>
+      </c>
+    </row>
+    <row r="533" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A533" s="10" t="s">
+        <v>3056</v>
+      </c>
+      <c r="B533" s="10" t="s">
+        <v>3017</v>
+      </c>
+      <c r="C533" s="10" t="s">
+        <v>3057</v>
+      </c>
+      <c r="D533" s="10" t="s">
+        <v>3058</v>
+      </c>
+      <c r="E533" s="10" t="s">
+        <v>3059</v>
+      </c>
+      <c r="F533" s="10" t="s">
+        <v>3060</v>
+      </c>
+      <c r="G533" s="10" t="s">
+        <v>2864</v>
+      </c>
+      <c r="H533" s="10" t="str">
+        <f aca="false">IF(G533="BUG","BUG-"&amp;A533,IF(G533="FUNCTIONAL","FUNCTIONAL-"&amp;A533,""))</f>
+        <v/>
+      </c>
+      <c r="I533" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="J533" s="10" t="s">
+        <v>3022</v>
+      </c>
+      <c r="L533" s="11" t="s">
+        <v>3061</v>
+      </c>
+    </row>
+    <row r="534" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A534" s="10" t="s">
+        <v>3062</v>
+      </c>
+      <c r="B534" s="10" t="s">
+        <v>3017</v>
+      </c>
+      <c r="C534" s="10" t="s">
+        <v>3063</v>
+      </c>
+      <c r="D534" s="10" t="s">
+        <v>3058</v>
+      </c>
+      <c r="E534" s="10" t="s">
+        <v>3064</v>
+      </c>
+      <c r="F534" s="10" t="s">
+        <v>3065</v>
+      </c>
+      <c r="G534" s="10" t="s">
+        <v>2864</v>
+      </c>
+      <c r="H534" s="10" t="str">
+        <f aca="false">IF(G534="BUG","BUG-"&amp;A534,IF(G534="FUNCTIONAL","FUNCTIONAL-"&amp;A534,""))</f>
+        <v/>
+      </c>
+      <c r="I534" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="J534" s="10" t="s">
+        <v>3022</v>
+      </c>
+      <c r="L534" s="11" t="s">
+        <v>3066</v>
+      </c>
+    </row>
+    <row r="535" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A535" s="10" t="s">
+        <v>3067</v>
+      </c>
+      <c r="B535" s="10" t="s">
+        <v>3017</v>
+      </c>
+      <c r="C535" s="10" t="s">
+        <v>3068</v>
+      </c>
+      <c r="D535" s="10" t="s">
+        <v>3058</v>
+      </c>
+      <c r="E535" s="10" t="s">
+        <v>3064</v>
+      </c>
+      <c r="F535" s="10" t="s">
+        <v>3069</v>
+      </c>
+      <c r="G535" s="10" t="s">
+        <v>2864</v>
+      </c>
+      <c r="H535" s="10" t="str">
+        <f aca="false">IF(G535="BUG","BUG-"&amp;A535,IF(G535="FUNCTIONAL","FUNCTIONAL-"&amp;A535,""))</f>
+        <v/>
+      </c>
+      <c r="I535" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="J535" s="10" t="s">
+        <v>3022</v>
+      </c>
+      <c r="L535" s="11" t="s">
+        <v>3066</v>
+      </c>
+    </row>
+    <row r="536" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A536" s="10" t="s">
+        <v>3070</v>
+      </c>
+      <c r="B536" s="10" t="s">
+        <v>3017</v>
+      </c>
+      <c r="C536" s="10" t="s">
+        <v>3071</v>
+      </c>
+      <c r="D536" s="10" t="s">
+        <v>3072</v>
+      </c>
+      <c r="E536" s="10" t="s">
+        <v>3073</v>
+      </c>
+      <c r="F536" s="10" t="s">
+        <v>3074</v>
+      </c>
+      <c r="G536" s="10" t="s">
+        <v>2908</v>
+      </c>
+      <c r="H536" s="10" t="str">
+        <f aca="false">IF(G536="BUG","BUG-"&amp;A536,IF(G536="FUNCTIONAL","FUNCTIONAL-"&amp;A536,""))</f>
+        <v/>
+      </c>
+      <c r="I536" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="J536" s="10" t="s">
+        <v>3022</v>
+      </c>
+      <c r="L536" s="11" t="s">
+        <v>3023</v>
+      </c>
+    </row>
+    <row r="537" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A537" s="10" t="s">
+        <v>3075</v>
+      </c>
+      <c r="B537" s="10" t="s">
+        <v>3017</v>
+      </c>
+      <c r="C537" s="10" t="s">
+        <v>3076</v>
+      </c>
+      <c r="D537" s="10" t="s">
+        <v>3032</v>
+      </c>
+      <c r="E537" s="10" t="s">
+        <v>3077</v>
+      </c>
+      <c r="F537" s="10" t="s">
+        <v>3078</v>
+      </c>
+      <c r="G537" s="10" t="s">
+        <v>2908</v>
+      </c>
+      <c r="H537" s="10" t="str">
+        <f aca="false">IF(G537="BUG","BUG-"&amp;A537,IF(G537="FUNCTIONAL","FUNCTIONAL-"&amp;A537,""))</f>
+        <v/>
+      </c>
+      <c r="I537" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="J537" s="10" t="s">
+        <v>3022</v>
+      </c>
+      <c r="L537" s="11" t="s">
+        <v>3029</v>
       </c>
     </row>
   </sheetData>
@@ -27211,7 +27832,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="20" t="s">
-        <v>3016</v>
+        <v>3079</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27219,13 +27840,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>3017</v>
+        <v>3080</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>3018</v>
+        <v>3081</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27294,11 +27915,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>3019</v>
+        <v>3082</v>
       </c>
       <c r="B7" s="22" t="n">
         <f aca="false">COUNTA('Test Case'!A2:A10000)</f>
-        <v>524</v>
+        <v>536</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>226</v>

</xml_diff>